<commit_message>
graphe exp ok, vp regimes m pas ok
</commit_message>
<xml_diff>
--- a/Simulations.xlsx
+++ b/Simulations.xlsx
@@ -536,11 +536,11 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>[0.0, 5.942398898115364e-07, 1.1884797796230727e-06, 7.130878677738436e-06, 1.30732775758538e-05, 3.086116630045566e-05, 4.864905502505752e-05, 6.643694374965938e-05, 0.00011040843194583058, 0.00015437992014200177, 0.00019835140833817297, 0.00041359264505891867, 0.0006288338817796643, 0.00084407511850041, 0.0016937044987897058, 0.0025433338790790015, 0.0033929632593682974, 0.004427474068214024, 0.00546198487705975, 0.006496495685905476, 0.0075310064947512025, 0.009552645183663267, 0.011574283872575333, 0.013595922561487398, 0.015617561250399464, 0.01763919993931153, 0.023194020427178014, 0.0287488409150445, 0.03430366140291098, 0.03985848189077747, 0.04541330237864395, 0.053644968616577596, 0.06187663485451124, 0.07010830109244488, 0.07833996733037853, 0.08657163356831217, 0.09480329980624581, 0.10243737020367691, 0.110071440601108, 0.1177055109985391, 0.12533958139597018, 0.13297365179340126, 0.14060772219083234, 0.14712940096172236, 0.15365107973261238, 0.1601727585035024, 0.16669443727439243, 0.17321611604528245, 0.17973779481617247, 0.1860348654165764, 0.19233193601698034, 0.19862900661738428, 0.20324295563956638, 0.20785690466174847, 0.21247085368393057, 0.21708480270611266, 0.22169875172829476, 0.2296372904067486, 0.23426738429100052, 0.23889747817525245, 0.24352757205950437, 0.2481576659437563, 0.2527877598280082, 0.2574178537122601, 0.2627761314867376, 0.2681344092612151, 0.2734926870356926, 0.27885096481017013, 0.28420924258464764, 0.28956752035912514, 0.29465283996894953, 0.2997381595787739, 0.3048234791885983, 0.3099087987984227, 0.3149941184082471, 0.3200794380180715, 0.33162567825543476, 0.33920431186736466, 0.34678294547929456, 0.35436157909122445, 0.36194021270315435, 0.36951884631508425, 0.3788376333657225, 0.3881564204163608, 0.39567694615488974, 0.4031974718934187, 0.41071799763194766, 0.4182385233704766, 0.4257590491090056, 0.43327957484753454, 0.44137224801838676, 0.449464921189239, 0.4575575943600912, 0.4656502675309434, 0.4737429407017956, 0.48183561387264784, 0.4930252910295104, 0.504214968186373, 0.5154046453432356, 0.5265943225000982, 0.5377839996569608, 0.5489736768138234, 0.5640392954058023, 0.5791049139977813, 0.5941705325897603, 0.6092361511817392, 0.6243017697737182, 0.6393673883656972, 0.6610621159335563, 0.6827568435014155, 0.7044515710692747, 0.7261462986371339, 0.747841026204993, 0.7695357537728522, 0.7991497215821098, 0.8287636893913675, 0.8583776572006251, 0.8879916250098827, 0.9176055928191403, 0.947219560628398, 0.9857283723063492, 1.0242371839843005, 1.0627459956622518, 1.101254807340203, 1.1397636190181544, 1.1819182413847158, 1.2240728637512772, 1.2662274861178386, 1.3083821084844, 1.3505367308509615, 1.4027777315006829, 1.4550187321504042, 1.5072597328001256, 1.559500733449847, 1.6117417340995683, 1.6639827347492897, 1.7492059039818504, 1.834429073214411, 1.9196522424469717, 2.0048754116795324, 2.090098580912093, 2.1753217501446533, 2.279174789368914, 2.3830278285931747, 2.4868808678174354, 2.590733907041696, 2.694586946265957, 2.7984399854902176, 2.968341086128742, 3.1382421867672665, 3.308143287405791, 3.4780443880443155, 3.64794548868284, 3.8178465893213644, 4.125309676978027, 4.43277276463469, 4.740235852291352, 5.047698939948015, 5.355162027604678, 6.196160808937055, 7.037159590269432, 7.87815837160181, 8.719157152934187, 10.0]</t>
+          <t>[0.0, 5.942398898115364e-07, 1.1884797796230727e-06, 7.130878677738436e-06, 1.30732775758538e-05, 3.086116629746793e-05, 4.8649055019082065e-05, 6.64369437406962e-05, 0.0001104084314030158, 0.0001543799190653354, 0.000198351406727655, 0.00041359161972225517, 0.0006288318327168554, 0.0008440720457114556, 0.0016945630968747479, 0.00254505414803804, 0.003395545199201332, 0.004429735890258312, 0.005463926581315292, 0.006498117272372272, 0.0075323079634292515, 0.009551494891329488, 0.011570681819229725, 0.013589868747129962, 0.015609055675030199, 0.017628242602930437, 0.023132208131512455, 0.028636173660094473, 0.03414013918867649, 0.03964410471725851, 0.04514807024584053, 0.05318726614513808, 0.06122646204443563, 0.06926565794373318, 0.07730485384303074, 0.08534404974232829, 0.09338324564162584, 0.10136814410897318, 0.10935304257632053, 0.11733794104366788, 0.12374425315853846, 0.13015056527340904, 0.13655687738827962, 0.1429631895031502, 0.1493695016180208, 0.15598472064441063, 0.16259993967080047, 0.1692151586971903, 0.17583037772358015, 0.18244559674997, 0.18906081577635983, 0.1950778992872281, 0.20109498279809637, 0.20711206630896464, 0.2131291498198329, 0.21914623333070118, 0.225204470531308, 0.2312627077319148, 0.2373209449325216, 0.2433791821331284, 0.2494374193337352, 0.25549565653434203, 0.26134679034775843, 0.2671979241611748, 0.2730490579745912, 0.2789001917880076, 0.284751325601424, 0.2906024594148404, 0.29640380926051835, 0.3022051591061963, 0.3080065089518742, 0.31380785879755213, 0.31960920864323006, 0.325410558488908, 0.3343234593124836, 0.3432363601360592, 0.3521492609596348, 0.3610621617832104, 0.369975062606786, 0.3797599486122817, 0.3895448346177774, 0.3993297206232731, 0.4091146066287688, 0.4188994926342645, 0.4286843786397602, 0.44053022533717645, 0.4523760720345927, 0.4642219187320089, 0.47606776542942514, 0.48791361212684137, 0.4997594588242576, 0.5161377980398125, 0.5325161372553675, 0.5488944764709225, 0.5652728156864775, 0.5816511549020325, 0.605525089946702, 0.6293990249913715, 0.653272960036041, 0.6771468950807105, 0.70102083012538, 0.7356128001360817, 0.7702047701467833, 0.804796740157485, 0.8393887101681867, 0.8739806801788884, 0.9109644386055772, 0.947948197032266, 0.9849319554589547, 1.0219157138856434, 1.0588994723123322, 1.119373938218426, 1.1798484041245199, 1.2403228700306137, 1.3007973359367075, 1.3612718018428014, 1.4217462677488952, 1.4885083577761762, 1.5552704478034571, 1.622032537830738, 1.688794627858019, 1.7555567178853, 1.8565894205444984, 1.9576221232036968, 2.058654825862895, 2.1596875285220936, 2.260720231181292, 2.3617529338404903, 2.4904804680800705, 2.6192080023196507, 2.747935536559231, 2.876663070798811, 3.005390605038391, 3.1341181392779713, 3.28178437946316, 3.4294506196483487, 3.5771168598335374, 3.724783100018726, 3.872449340203915, 4.0201155803891035, 4.255248153640831, 4.490380726892558, 4.725513300144285, 4.960645873396012, 5.195778446647739, 5.430911019899466, 5.714016645812256, 5.997122271725046, 6.280227897637836, 6.563333523550626, 6.846439149463416, 7.129544775376206, 7.516444016041985, 7.903343256707765, 8.290242497373544, 8.677141738039325, 9.064040978705105, 9.450940219370885, 9.986702326513964, 10.0]</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>0.3003580509018594</v>
+        <v>0.6284314395283689</v>
       </c>
       <c r="D2" t="n">
         <v>9.81</v>
@@ -567,13 +567,13 @@
         <v>2</v>
       </c>
       <c r="L2" t="n">
-        <v>3.003580509018594</v>
+        <v>6.284314395283689</v>
       </c>
       <c r="M2" t="n">
-        <v>0.02216927245657052</v>
+        <v>0.005064238931586606</v>
       </c>
       <c r="N2" t="n">
-        <v>0.1108463622828526</v>
+        <v>0.02532119465793303</v>
       </c>
       <c r="O2" t="n">
         <v>19.6199</v>
@@ -603,11 +603,11 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>[0.0, 5.942402908483678e-07, 1.1884805816967355e-06, 7.130883490180414e-06, 1.307328639866409e-05, 3.086118715436224e-05, 4.864908791006039e-05, 6.643698866575854e-05, 0.00011040850756487432, 0.0001543800264639901, 0.00019835154536310587, 0.0004135935000634241, 0.0006288354547637424, 0.0008440774094640607, 0.0016935906700766097, 0.0025431039306891587, 0.0033926171913017077, 0.004427096643618324, 0.00546157609593494, 0.006496055548251556, 0.007530535000568172, 0.009552272575107717, 0.011574010149647262, 0.013595747724186808, 0.015617485298726353, 0.0176392228732659, 0.023194016780228224, 0.028748810687190547, 0.03430360459415287, 0.03985839850111519, 0.04541319240807751, 0.053645167153829096, 0.061877141899580684, 0.07010911664533227, 0.07834109139108386, 0.08657306613683545, 0.09480504088258704, 0.10243893653933142, 0.1100728321960758, 0.11770672785282019, 0.12534062350956457, 0.13297451916630895, 0.14060841482305333, 0.1471303734218029, 0.15365233202055248, 0.16017429061930205, 0.16669624921805162, 0.1732182078168012, 0.17974016641555077, 0.18603763408414314, 0.19233510175273552, 0.1986325694213279, 0.20324628787445384, 0.20786000632757978, 0.21247372478070572, 0.21708744323383167, 0.2217011616869576, 0.2296352023703069, 0.23426492584894257, 0.23889464932757823, 0.2435243728062139, 0.24815409628484955, 0.2527838197634852, 0.25741354324212085, 0.2627927834955154, 0.2681720237489099, 0.27355126400230445, 0.278930504255699, 0.2843097445090935, 0.28968898476248806, 0.2947795122080763, 0.29987003965366454, 0.3049605670992528, 0.31005109454484103, 0.3151416219904293, 0.3202321494360175, 0.3316856740464036, 0.33924260567922143, 0.3467995373120393, 0.3543564689448571, 0.36191340057767496, 0.3694703322104928, 0.37881976039885745, 0.3881691885872221, 0.395696060405963, 0.4032229322247039, 0.4107498040434448, 0.4182766758621857, 0.4258035476809266, 0.4333304194996675, 0.44142621037598895, 0.4495220012523104, 0.45761779212863185, 0.4657135830049533, 0.47380937388127475, 0.4819051647575962, 0.4931070178915512, 0.5043088710255061, 0.5155107241594611, 0.526712577293416, 0.537914430427371, 0.5491162835613259, 0.5641978538762233, 0.5792794241911208, 0.5943609945060182, 0.6094425648209156, 0.6245241351358131, 0.6396057054507105, 0.6613174598195075, 0.6830292141883045, 0.7047409685571016, 0.7264527229258986, 0.7481644772946956, 0.7698762316634926, 0.7994684935332794, 0.8290607554030662, 0.858653017272853, 0.8882452791426398, 0.9178375410124266, 0.9474298028822135, 0.9859700383548214, 1.0245102738274294, 1.0630505093000373, 1.1015907447726452, 1.140130980245253, 1.182295322842675, 1.2244596654400968, 1.2666240080375186, 1.3087883506349405, 1.3509526932323623, 1.4032268617297046, 1.4555010302270468, 1.507775198724389, 1.5600493672217313, 1.6123235357190735, 1.6645977042164157, 1.7476035440352637, 1.8306093838541118, 1.9136152236729598, 1.9966210634918078, 2.079626903310656, 2.162632743129504, 2.266242644278102, 2.3698525454267, 2.473462446575298, 2.577072347723896, 2.680682248872494, 2.784292150021092, 2.953122462532354, 3.1219527750436162, 3.2907830875548783, 3.4596134000661403, 3.6284437125774023, 4.135189135956406, 4.641934559335409, 5.1486799827144125, 5.655425406093416, 7.346141815899059, 9.036858225704702, 10.0]</t>
+          <t>[0.0, 5.942402908483678e-07, 1.1884805816967355e-06, 7.130883490180414e-06, 1.307328639866409e-05, 3.086118715137464e-05, 4.864908790408519e-05, 6.643698865679574e-05, 0.00011040850702206408, 0.00015438002538733242, 0.00019835154375260077, 0.0004135924747165978, 0.0006288334056805949, 0.000844074336644592, 0.0016944487960028499, 0.002544823255361108, 0.003395197714719366, 0.004429356880527615, 0.005463516046335864, 0.006497675212144113, 0.0075318343779523615, 0.009551119768839161, 0.01157040515972596, 0.01358969055061276, 0.01560897594149956, 0.01762826133238636, 0.023132200576280102, 0.028636139820173843, 0.03414007906406759, 0.03964401830796133, 0.04514795755185508, 0.053187421718595, 0.061226885885334925, 0.06926635005207485, 0.07730581421881477, 0.0853452783855547, 0.09338474255229462, 0.10136899319471987, 0.10935324383714512, 0.11733749447957037, 0.12374366816704216, 0.13014984185451395, 0.13655601554198574, 0.14296218922945753, 0.14936836291692931, 0.15598267293222168, 0.16259698294751404, 0.1692112929628064, 0.17582560297809877, 0.18243991299339113, 0.1890542230086835, 0.19507326769589334, 0.20109231238310318, 0.20711135707031303, 0.21313040175752287, 0.21914944644473272, 0.22521091012391095, 0.23127237380308918, 0.2373338374822674, 0.24339530116144564, 0.24945676484062387, 0.2555182285198021, 0.2613706438835017, 0.26722305924720124, 0.2730754746109008, 0.2789278899746004, 0.28478030533829995, 0.2906327207019995, 0.29643381515585115, 0.3022349096097028, 0.3080360040635544, 0.31383709851740604, 0.3196381929712577, 0.3254392874251093, 0.33433789027380706, 0.3432364931225048, 0.35213509597120257, 0.36103369881990033, 0.3699323016685981, 0.3797149580339743, 0.38949761439935054, 0.3992802707647268, 0.409062927130103, 0.41884558349547923, 0.42862823986085546, 0.4404682674011607, 0.4523082949414659, 0.4641483224817711, 0.47598835002207635, 0.48782837756238157, 0.4996684051026868, 0.5160414344943797, 0.5324144638860726, 0.5487874932777655, 0.5651605226694585, 0.5815335520611514, 0.6054019913841876, 0.6292704307072238, 0.6531388700302599, 0.6770073093532961, 0.7008757486763323, 0.7354598857274778, 0.7700440227786233, 0.8046281598297688, 0.8392122968809143, 0.8737964339320597, 0.9107715871737254, 0.9477467404153911, 0.9847218936570568, 1.0216970468987223, 1.0586722001403879, 1.1191373601074568, 1.1796025200745257, 1.2400676800415946, 1.3005328400086635, 1.3609979999757325, 1.4214631599428014, 1.4882101247467525, 1.5549570895507037, 1.6217040543546548, 1.688451019158606, 1.755197983962557, 1.8562070918419498, 1.9572161997213424, 2.0582253076007353, 2.159234415480128, 2.260243523359521, 2.361252631238914, 2.4899513072576966, 2.6186499832764794, 2.747348659295262, 2.8760473353140448, 3.0047460113328275, 3.13344468735161, 3.2810779766043034, 3.4287112658569967, 3.57634455510969, 3.723977844362383, 3.8716111336150765, 4.01924442286777, 4.2543242325061135, 4.489404042144457, 4.724483851782801, 4.959563661421145, 5.194643471059488, 5.429723280697832, 5.71276419718481, 5.995805113671787, 6.278846030158765, 6.561886946645743, 6.84492786313272, 7.127968779619698, 7.5147790390802625, 7.901589298540827, 8.288399558001391, 8.675209817461955, 9.062020076922519, 9.448830336383082, 9.984465874599545, 10.0]</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>0.3003573308535942</v>
+        <v>0.6284033769873318</v>
       </c>
       <c r="D3" t="n">
         <v>9.81</v>
@@ -634,13 +634,13 @@
         <v>2</v>
       </c>
       <c r="L3" t="n">
-        <v>3.003573308535942</v>
+        <v>6.284033769873318</v>
       </c>
       <c r="M3" t="n">
-        <v>0.02216937874973315</v>
+        <v>0.005064691248016657</v>
       </c>
       <c r="N3" t="n">
-        <v>0.1108468937486658</v>
+        <v>0.02532345624008328</v>
       </c>
       <c r="O3" t="n">
         <v>19.61987351447831</v>
@@ -670,11 +670,11 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>[0.0, 5.942407981030446e-07, 1.1884815962060891e-06, 7.130889577236535e-06, 1.3073297558266982e-05, 3.086121353159444e-05, 4.86491295049219e-05, 6.643704547824935e-05, 0.00011040860321223327, 0.0001543801609462172, 0.00019835171868020114, 0.00041359458153223023, 0.0006288374443842594, 0.0008440803072362885, 0.0016934467848553586, 0.0025428132624744286, 0.0033921797400934986, 0.004426619562714922, 0.005461059385336345, 0.006495499207957768, 0.007529939030579191, 0.009551801715410056, 0.011573664400240921, 0.013595527085071786, 0.015617389769902651, 0.017639252454733516, 0.023194012743923784, 0.02874877303311405, 0.03430353332230432, 0.03985829361149459, 0.045413053900684855, 0.05364540994171538, 0.0618777659827459, 0.07011012202377642, 0.07834247806480694, 0.08657483410583747, 0.09480719014686799, 0.10244086812192293, 0.11007454609697788, 0.11770822407203282, 0.12534190204708778, 0.13297558002214274, 0.1406092579971977, 0.14713084489527692, 0.15365243179335614, 0.16017401869143535, 0.16669560558951457, 0.1732171924875938, 0.179738779385673, 0.1860365075548579, 0.1923342357240428, 0.19863196389322768, 0.2032452987243326, 0.20785863355543754, 0.21247196838654248, 0.2170853032176474, 0.22169863804875234, 0.22965388453842897, 0.2342846323723775, 0.23891538020632605, 0.2435461280402746, 0.24817687587422313, 0.25280762370817167, 0.25743837154212024, 0.2627954190267434, 0.2681524665113666, 0.2735095139959898, 0.27886656148061295, 0.28422360896523613, 0.2895806564498593, 0.2946647337292333, 0.2997488110086073, 0.3048328882879813, 0.30991696556735526, 0.31500104284672925, 0.32008512012610324, 0.3316383895530376, 0.3392159050536099, 0.34679342055418216, 0.35437093605475445, 0.36194845155532673, 0.369525967055899, 0.3788700310177856, 0.3882140949796722, 0.3957385479936051, 0.403263001007538, 0.4107874540214709, 0.4183119070354038, 0.42583636004933667, 0.43336081306326957, 0.44145538129021694, 0.4495499495171643, 0.4576445177441117, 0.46573908597105906, 0.47383365419800644, 0.4819282224249538, 0.493137187615811, 0.5043461528066682, 0.5155551179975253, 0.5267640831883824, 0.5379730483792395, 0.5491820135700967, 0.5642742273753645, 0.5793664411806323, 0.5944586549859001, 0.6095508687911679, 0.6246430825964358, 0.6397352964017036, 0.6614721445995324, 0.6832089927973612, 0.7049458409951901, 0.7266826891930189, 0.7484195373908478, 0.7701563855886766, 0.7997818519286933, 0.8294073182687101, 0.8590327846087268, 0.8886582509487435, 0.9182837172887602, 0.947909183628777, 0.9864537146727665, 1.0249982457167561, 1.0635427767607457, 1.1020873078047353, 1.1406318388487249, 1.1828117625556243, 1.2249916862625236, 1.267171609969423, 1.3093515336763224, 1.3515314573832218, 1.403817093385269, 1.456102729387316, 1.5083883653893633, 1.5606740013914104, 1.6129596373934576, 1.6652452733955048, 1.7505216434991402, 1.8357980136027756, 1.921074383706411, 2.0063507538100467, 2.0916271239136823, 2.176903494017318, 2.280820668119605, 2.3847378422218917, 2.4886550163241785, 2.5925721904264654, 2.696489364528752, 2.800406538631039, 2.970443786122599, 3.140481033614159, 3.3105182811057188, 3.4805555285972787, 3.6505927760888386, 3.8206300235803985, 4.128342299233844, 4.436054574887289, 4.743766850540735, 5.05147912619418, 5.359191401847625, 6.200701855796121, 7.042212309744616, 7.883722763693111, 8.725233217641605, 10.0]</t>
+          <t>[0.0, 5.942407981030446e-07, 1.1884815962060891e-06, 7.130889577236535e-06, 1.3073297558266982e-05, 3.0861213528606995e-05, 4.864912949894701e-05, 6.643704546928703e-05, 0.00011040860266942747, 0.0001543801598695679, 0.00019835171706970834, 0.00041359355617251914, 0.0006288353952753299, 0.0008440772343781407, 0.0016943043142248365, 0.0025445313940715324, 0.0033947584739182283, 0.004428877796895411, 0.0054629971198725934, 0.006497116442849776, 0.007531235765826958, 0.009550645734219518, 0.011570055702612079, 0.01358946567100464, 0.0156088756393972, 0.01762828560778976, 0.02313219177205894, 0.028636097936328122, 0.0341400041005973, 0.03964391026486648, 0.04514781642913566, 0.053187614193155805, 0.06122741195717595, 0.0692672097211961, 0.07730700748521624, 0.08534680524923638, 0.09338660301325652, 0.10137003727722849, 0.10935347154120045, 0.11733690580517242, 0.12374270567882788, 0.13014850555248333, 0.13655430542613878, 0.14296010529979422, 0.14936590517344966, 0.15598111765859754, 0.16259633014374542, 0.1692115426288933, 0.17582675511404117, 0.18244196759918904, 0.18905718008433692, 0.19507360549516423, 0.20109003090599153, 0.20710645631681884, 0.21312288172764615, 0.21913930713847346, 0.2251960191932164, 0.23125273124795936, 0.23730944330270232, 0.24336615535744527, 0.24942286741218822, 0.2554795794669312, 0.26133110998717934, 0.2671826405074275, 0.2730341710276757, 0.27888570154792386, 0.28473723206817203, 0.2905887625884202, 0.296389911240585, 0.3021910598927498, 0.3079922085449146, 0.3137933571970794, 0.3195945058492442, 0.325395654501409, 0.3343077475832697, 0.3432198406651304, 0.3521319337469911, 0.3610440268288518, 0.3699561199107125, 0.37974078860663923, 0.389525457302566, 0.39931012599849275, 0.4090947946944195, 0.41887946339034626, 0.428664132086273, 0.4405094969687854, 0.45235486185129775, 0.4642002267338101, 0.4760455916163225, 0.48789095649883485, 0.4997363213813472, 0.5161142372559808, 0.5324921531306144, 0.5488700690052479, 0.5652479848798815, 0.581625900754515, 0.6054989826372299, 0.6293720645199448, 0.6532451464026596, 0.6771182282853745, 0.7009913101680894, 0.7355819360825078, 0.7701725619969262, 0.8047631879113446, 0.839353813825763, 0.8739444397401814, 0.9109267097570395, 0.9479089797738975, 0.9848912497907556, 1.0218735198076137, 1.0588557898244717, 1.1193279055358787, 1.1798000212472857, 1.2402721369586927, 1.3007442526700996, 1.3612163683815066, 1.4216884840929136, 1.4884478799884635, 1.5552072758840134, 1.6219666717795633, 1.6887260676751132, 1.7554854635706632, 1.8565141473316564, 1.9575428310926497, 2.058571514853643, 2.159600198614636, 2.260628882375629, 2.361657566136622, 2.4903799653024934, 2.6191023644683646, 2.747824763634236, 2.876547162800107, 3.0052695619659784, 3.1339919611318496, 3.2816523697541817, 3.429312778376514, 3.576973186998846, 3.724633595621178, 3.87229400424351, 4.019954412865842, 4.255077678568674, 4.490200944271506, 4.725324209974338, 4.96044747567717, 5.195570741380002, 5.430694007082834, 5.713788582927359, 5.996883158771884, 6.279977734616409, 6.563072310460934, 6.846166886305459, 7.129261462149985, 7.51614564212528, 7.903029822100575, 8.289914002075871, 8.676798182051169, 9.063682362026466, 9.450566542001763, 9.986306879437356, 10.0]</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>0.3003564316594717</v>
+        <v>0.6283678912018534</v>
       </c>
       <c r="D4" t="n">
         <v>9.81</v>
@@ -701,13 +701,13 @@
         <v>2</v>
       </c>
       <c r="L4" t="n">
-        <v>3.003564316594717</v>
+        <v>6.283678912018534</v>
       </c>
       <c r="M4" t="n">
-        <v>0.02216951148939051</v>
+        <v>0.005065263300231435</v>
       </c>
       <c r="N4" t="n">
-        <v>0.1108475574469525</v>
+        <v>0.02532631650115717</v>
       </c>
       <c r="O4" t="n">
         <v>19.61984001412804</v>
@@ -737,11 +737,11 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>[0.0, 5.942414397086066e-07, 1.1884828794172133e-06, 7.13089727650328e-06, 1.3073311673589347e-05, 3.08612468950699e-05, 4.864918211655045e-05, 6.6437117338031e-05, 0.00011040872419264435, 0.0001543803310472577, 0.00019835193790187103, 0.00041359594945237203, 0.000628839961002873, 0.000844083972553374, 0.0016932649372261048, 0.0025424459018988355, 0.0033916268665715663, 0.004426016614762648, 0.0054604063629537306, 0.006494796111144813, 0.007529185859335895, 0.009551206851399202, 0.01157322784346251, 0.013595248835525818, 0.015617269827589125, 0.01763929081965243, 0.02319400941668599, 0.028748728013719548, 0.0343034466107531, 0.03985816520778666, 0.04541288380482021, 0.053645731984476315, 0.06187858016413242, 0.07011142834378853, 0.07834427652344464, 0.08657712470310075, 0.09480997288275686, 0.1024433722851153, 0.11007677168747373, 0.11771017108983217, 0.1253435704921906, 0.13297696989454905, 0.14061036929690748, 0.14713221207630367, 0.15365405485569986, 0.16017589763509604, 0.16669774041449223, 0.17321958319388842, 0.1797414259732846, 0.18603972595176277, 0.19233802593024094, 0.1986363259087191, 0.20324926847595148, 0.20786221104318386, 0.21247515361041625, 0.21708809617764863, 0.221701038744881, 0.22965612074640152, 0.23428666627045303, 0.23891721179450454, 0.24354775731855605, 0.24817830284260756, 0.25280884836665907, 0.2574393938907106, 0.26281724616733937, 0.26819509844396816, 0.27357295072059695, 0.27895080299722574, 0.28432865527385454, 0.2897065075504833, 0.2947955154891009, 0.29988452342771843, 0.304973531366336, 0.31006253930495353, 0.3151515472435711, 0.32024055518218864, 0.33162793634386045, 0.3391810918234181, 0.34673424730297575, 0.3542874027825334, 0.36184055826209105, 0.3693937137416487, 0.37866565514559153, 0.38793759654953436, 0.3972095379534772, 0.40648147935742, 0.41575342076136285, 0.4250253621653057, 0.4341153235036919, 0.44320528484207816, 0.4522952461804644, 0.46138520751885065, 0.4704751688572369, 0.47956513019562313, 0.489797402710398, 0.5000296752251729, 0.5102619477399479, 0.5204942202547229, 0.5307264927694979, 0.5409587652842729, 0.5544482413504134, 0.5679377174165539, 0.5814271934826943, 0.5949166695488348, 0.6084061456149753, 0.6218956216811158, 0.6418875962857212, 0.6618795708903267, 0.6818715454949321, 0.7018635200995376, 0.721855494704143, 0.7418474693087485, 0.7729560280298092, 0.80406458675087, 0.8351731454719308, 0.8662817041929916, 0.8973902629140523, 0.9284988216351131, 0.9668790085599935, 1.005259195484874, 1.0436393824097543, 1.0820195693346346, 1.120399756259515, 1.1587799431843953, 1.2091565391496808, 1.2595331351149663, 1.3099097310802519, 1.3602863270455374, 1.410662923010823, 1.4610395189761085, 1.5312817070505984, 1.6015238951250883, 1.6717660831995782, 1.742008271274068, 1.812250459348558, 1.882492647423048, 1.9642020089996401, 2.045911370576232, 2.127620732152824, 2.209330093729416, 2.2910394553060076, 2.3727488168825994, 2.5008553282912915, 2.6289618396999836, 2.7570683511086758, 2.885174862517368, 3.01328137392606, 3.141387885334752, 3.3554301153027426, 3.569472345270733, 3.7835145752387236, 3.997556805206714, 4.211599035174705, 5.5875762570691965, 6.963553478963688, 8.33953070085818, 9.715507922752671, 10.0]</t>
+          <t>[0.0, 5.942414397086066e-07, 1.1884828794172133e-06, 7.13089727650328e-06, 1.3073311673589347e-05, 3.086124689208264e-05, 4.864918211057593e-05, 6.643711732906922e-05, 0.00011040872364984249, 0.00015438032997061574, 0.000198351936291389, 0.00041359492407584876, 0.0006288379118603085, 0.0008440808996447683, 0.001694121713095992, 0.0025441625265472155, 0.0033942033399984393, 0.004428272319203938, 0.005462341298409437, 0.006496410277614936, 0.007530479256820434, 0.009550046856469808, 0.011569614456119181, 0.013589182055768555, 0.015608749655417928, 0.0176283172550673, 0.023132182208890895, 0.02863604716271449, 0.03413991211653808, 0.039643777070361666, 0.04514764202418525, 0.053187868259874434, 0.061228094495563615, 0.0692683207312528, 0.07730854696694199, 0.08534877320263118, 0.09338899943832037, 0.1013713984239307, 0.10935379740954103, 0.11733619639515136, 0.12374172208136586, 0.13014724776758035, 0.13655277345379485, 0.14295829914000935, 0.14936382482622385, 0.15597812602899122, 0.1625924272317586, 0.16920672843452597, 0.17582102963729335, 0.18243533084006072, 0.1890496320428281, 0.1950678518234736, 0.20108607160411912, 0.20710429138476463, 0.21312251116541014, 0.21914073094605566, 0.22520027455635958, 0.2312598181666635, 0.2373193617769674, 0.24337890538727133, 0.24943844899757525, 0.2554979926078792, 0.2613509175345455, 0.26720384246121176, 0.27305676738787804, 0.2789096923145443, 0.2847626172412106, 0.2906155421678769, 0.2964163827557066, 0.3022172233435363, 0.308018063931366, 0.3138189045191957, 0.3196197451070254, 0.3254205856948551, 0.33431812318411586, 0.3432156606733766, 0.35211319816263736, 0.3610107356518981, 0.36990827314115887, 0.37969064075840747, 0.38947300837565607, 0.39925537599290467, 0.40903774361015327, 0.41882011122740187, 0.42860247884465047, 0.4404418845002776, 0.45228129015590474, 0.46412069581153187, 0.475960101467159, 0.48779950712278614, 0.49963891277841327, 0.5160113871176936, 0.5323838614569738, 0.548756335796254, 0.5651288101355343, 0.5815012844748145, 0.6053686240918275, 0.6292359637088404, 0.6531033033258533, 0.6769706429428662, 0.7008379825598792, 0.7354203943702238, 0.7700028061805684, 0.804585217990913, 0.8391676298012576, 0.8737500416116022, 0.9107232865805254, 0.9476965315494486, 0.9846697765183717, 1.021643021487295, 1.0586162664562182, 1.1190784216065648, 1.1795405767569114, 1.240002731907258, 1.3004648870576045, 1.3609270422079511, 1.4213891973582977, 1.4881327073995854, 1.554876217440873, 1.6216197274821607, 1.6883632375234483, 1.755106747564736, 1.856110698684157, 1.9571146498035779, 2.058118600922999, 2.1591225520424198, 2.2601265031618407, 2.3611304542812617, 2.489822548450549, 2.6185146426198367, 2.747206736789124, 2.8758988309584117, 3.004590925127699, 3.1332830192969867, 3.2809088339495487, 3.4285346486021107, 3.5761604632546726, 3.7237862779072346, 3.8714120925597966, 4.0190379072123585, 4.254105784169638, 4.489173661126917, 4.724241538084196, 4.959309415041475, 5.194377291998754, 5.4294451689560335, 5.712471957962157, 5.99549874696828, 6.278525535974403, 6.561552324980526, 6.844579113986649, 7.127605902992772, 7.514396846368352, 7.901187789743932, 8.287978733119512, 8.674769676495092, 9.061560619870672, 9.448351563246252, 9.983959218548776, 10.0]</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>0.3003552791819071</v>
+        <v>0.6283230206563284</v>
       </c>
       <c r="D5" t="n">
         <v>9.81</v>
@@ -768,13 +768,13 @@
         <v>2</v>
       </c>
       <c r="L5" t="n">
-        <v>3.003552791819071</v>
+        <v>6.283230206563283</v>
       </c>
       <c r="M5" t="n">
-        <v>0.02216968162066769</v>
+        <v>0.005065986779192006</v>
       </c>
       <c r="N5" t="n">
-        <v>0.1108484081033384</v>
+        <v>0.02532993389596003</v>
       </c>
       <c r="O5" t="n">
         <v>19.61979764103523</v>
@@ -804,11 +804,11 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>[0.0, 5.942422512496885e-07, 1.188484502499377e-06, 7.130907014996262e-06, 1.3073329527493148e-05, 3.0861289095188775e-05, 4.8649248662884406e-05, 6.643720823058004e-05, 0.00011040887721590429, 0.00015438054620122853, 0.00019835221518655277, 0.0004135976797034373, 0.0006288431442203218, 0.0008440886087372063, 0.001693035160174211, 0.0025419817116112157, 0.0033909282630482204, 0.0044252547558400026, 0.005459581248631785, 0.006493907741423568, 0.00752823423421535, 0.009550455553587677, 0.011572676872960003, 0.01359489819233233, 0.015617119511704657, 0.01763934083107698, 0.023194007190171513, 0.028748673549266045, 0.034303339908360576, 0.03985800626745511, 0.04541267262654964, 0.05364613490696913, 0.06187959718738862, 0.0701130594678081, 0.0783465217482276, 0.08657998402864708, 0.09481344630906657, 0.10244649676444431, 0.11007954721982205, 0.11771259767519979, 0.12534564813057752, 0.13297869858595526, 0.140611749041333, 0.14713318913135312, 0.15365462922137324, 0.16017606931139336, 0.16669750940141348, 0.1732189494914336, 0.17974038958145372, 0.18603917117877813, 0.19233795277610255, 0.19863673437342697, 0.2032490871508309, 0.20786143992823483, 0.21247379270563876, 0.2170861454830427, 0.22169849826044663, 0.2296811217612328, 0.23431296135732144, 0.23894480095341009, 0.24357664054949874, 0.24820848014558738, 0.25284031974167603, 0.2574721593377647, 0.2628271993204229, 0.26818223930308116, 0.2735372792857394, 0.27889231926839764, 0.2842473592510559, 0.2896023992337141, 0.2946844198739828, 0.2997664405142515, 0.3048484611545202, 0.3099304817947889, 0.3150125024350576, 0.32009452307532626, 0.3316339158908484, 0.3392090767032969, 0.34678423751574544, 0.35435939832819396, 0.3619345591406425, 0.369509719953091, 0.3788587555911084, 0.38820779122912574, 0.3957355569980556, 0.4032633227669855, 0.4107910885359154, 0.4183188543048453, 0.42584662007377516, 0.43337438584270505, 0.4414730835120107, 0.44957178118131635, 0.457670478850622, 0.46576917651992766, 0.4738678741892333, 0.481966571858539, 0.4931843732064604, 0.5044021745543819, 0.5156199759023032, 0.5268377772502246, 0.538055578598146, 0.5492733799460674, 0.5643826189080688, 0.5794918578700703, 0.5946010968320717, 0.6097103357940732, 0.6248195747560746, 0.6399288137180761, 0.6616975965677225, 0.683466379417369, 0.7052351622670154, 0.7270039451166619, 0.7487727279663083, 0.7705415108159548, 0.8001810895094091, 0.8298206682028635, 0.8594602468963178, 0.8890998255897722, 0.9187394042832265, 0.9483789829766809, 0.9869392014290108, 1.0254994198813407, 1.0640596383336707, 1.1026198567860006, 1.1411800752383305, 1.1833678602612048, 1.225555645284079, 1.2677434303069532, 1.3099312153298275, 1.3521190003527017, 1.4044239681688062, 1.4567289359849107, 1.5090339038010152, 1.5613388716171197, 1.6136438394332242, 1.6659488072493287, 1.7512374761722151, 1.8365261450951016, 1.921814814017988, 2.0071034829408747, 2.0923921518637614, 2.177680820786648, 2.2815703184247558, 2.3854598160628635, 2.4893493137009712, 2.593238811339079, 2.6971283089771867, 2.8010178066152944, 2.970998084515729, 3.1409783624161633, 3.310958640316598, 3.4809389182170323, 3.6509191961174667, 3.820899474017901, 4.1283608048125515, 4.435822135607202, 4.743283466401852, 5.0507447971965025, 5.358206127991153, 6.200006754291846, 7.041807380592539, 7.883608006893232, 8.725408633193926, 10.0]</t>
+          <t>[0.0, 5.942422512496885e-07, 1.188484502499377e-06, 7.130907014996262e-06, 1.3073329527493148e-05, 3.086128909220172e-05, 4.864924865691029e-05, 6.643720822161886e-05, 0.00011040887667311251, 0.00015438054512460618, 0.00019835221357609984, 0.0004135966543057189, 0.0006288410950353379, 0.0008440855357649569, 0.0016938909845901707, 0.0025436964334153845, 0.0033935018822405984, 0.004427507265925544, 0.00546151264961049, 0.006495518033295436, 0.007529523416980382, 0.009549290490165075, 0.011569057563349769, 0.013588824636534462, 0.015608591709719155, 0.01762835878290385, 0.023132172254101017, 0.028635985725298185, 0.03413979919649535, 0.03964361266769252, 0.04514742613888969, 0.053188189071997, 0.061228952005104316, 0.06926971493821163, 0.07731047787131895, 0.08535124080442627, 0.09339200373753359, 0.10137309647928391, 0.10935418922103424, 0.11733528196278456, 0.12374026252124617, 0.1301452430797078, 0.1365502236381694, 0.14295520419663102, 0.14936018475509263, 0.1559753874117719, 0.16259059006845114, 0.1692057927251304, 0.17582099538180965, 0.1824361980384889, 0.18905140069516815, 0.19506676829711803, 0.2010821358990679, 0.20709750350101777, 0.21311287110296764, 0.21912823870491752, 0.22518250572042572, 0.23123677273593393, 0.23729103975144214, 0.24334530676695035, 0.24939957378245856, 0.25545384079796674, 0.26130600486382716, 0.2671581689296876, 0.273010332995548, 0.2788624970614084, 0.28471466112726884, 0.29056682519312926, 0.2963676519267012, 0.3021684786602732, 0.30796930539384515, 0.3137701321274171, 0.3195709588609891, 0.32537178559456104, 0.33428260111696084, 0.34319341663936065, 0.35210423216176046, 0.36101504768416026, 0.36992586320656007, 0.3797101883855316, 0.38949451356450315, 0.3992788387434747, 0.40906316392244624, 0.4188474891014178, 0.4286318142803893, 0.4404764140592879, 0.45232101383818646, 0.464165613617085, 0.4760102133959836, 0.48785481317488216, 0.49969941295378073, 0.5160766584118801, 0.5324539038699795, 0.5488311493280789, 0.5652083947861782, 0.5815856402442776, 0.6054573646492596, 0.6293290890542416, 0.6532008134592235, 0.6770725378642055, 0.7009442622691875, 0.7355327478134575, 0.7701212333577274, 0.8047097189019974, 0.8392982044462673, 0.8738866899905373, 0.9108665896304758, 0.9478464892704144, 0.9848263889103529, 1.0218062885502914, 1.05878618819023, 1.119254556308346, 1.179722924426462, 1.240191292544578, 1.300659660662694, 1.3611280287808099, 1.4215963968989258, 1.4883515015314053, 1.5551066061638847, 1.6218617107963642, 1.6886168154288437, 1.7553719200613231, 1.8563942137657414, 1.9574165074701597, 2.058438801174578, 2.1594610948789965, 2.260483388583415, 2.3615056822878335, 2.4902199089802117, 2.61893413567259, 2.747648362364968, 2.8763625890573463, 3.0050768157497245, 3.1337910424421027, 3.281442181986878, 3.4290933215316537, 3.576744461076429, 3.7243956006212047, 3.87204674016598, 4.019697879710756, 4.254806341594869, 4.489914803478983, 4.725023265363096, 4.96013172724721, 5.195240189131323, 5.430348651015437, 5.713425662583056, 5.996502674150675, 6.279579685718295, 6.562656697285914, 6.845733708853533, 7.128810720421153, 7.515670944995857, 7.902531169570561, 8.289391394145266, 8.67625161871997, 9.063111843294674, 9.449972067869378, 9.985677775883676, 10.0]</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>0.3003538408637317</v>
+        <v>0.6282662890152124</v>
       </c>
       <c r="D6" t="n">
         <v>9.81</v>
@@ -835,13 +835,13 @@
         <v>2</v>
       </c>
       <c r="L6" t="n">
-        <v>3.003538408637317</v>
+        <v>6.282662890152124</v>
       </c>
       <c r="M6" t="n">
-        <v>0.02216989395111284</v>
+        <v>0.005066901724733047</v>
       </c>
       <c r="N6" t="n">
-        <v>0.1108494697555642</v>
+        <v>0.02533450862366523</v>
       </c>
       <c r="O6" t="n">
         <v>19.61974404520773</v>
@@ -871,11 +871,11 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>[0.0, 5.942432777363632e-07, 1.1884865554727263e-06, 7.130919332836359e-06, 1.307335211019999e-05, 3.0861342472474006e-05, 4.864933283474802e-05, 6.643732319702203e-05, 0.00011040907076906653, 0.00015438081834111104, 0.00019835256591315556, 0.0004135998682685408, 0.000628847170623926, 0.0008440944729793112, 0.001692744898814662, 0.0025413953246500127, 0.0033900457504853635, 0.004424292365106065, 0.0054585389797267665, 0.006492785594347468, 0.0075270322089681695, 0.009549507065620444, 0.011571981922272719, 0.013594456778924994, 0.015616931635577268, 0.017639406492229545, 0.023194008399857243, 0.02874861030748494, 0.034303212215112636, 0.03985781412274033, 0.045412416030368025, 0.05364666582074197, 0.061880915611115916, 0.07011516540148986, 0.07834941519186381, 0.08658366498223775, 0.0948179147726117, 0.1024505207209947, 0.1100831266693777, 0.1177157326177607, 0.1253483385661437, 0.1329809445145267, 0.1406135504629097, 0.147135208229364, 0.1536568659958183, 0.1601785237622726, 0.1667001815287269, 0.1732218392951812, 0.1797434970616355, 0.18604313085667387, 0.19234276465171224, 0.1986423984467506, 0.20325410062120758, 0.20786580279566455, 0.21247750497012152, 0.2170892071445785, 0.22170090931903547, 0.22969068697151795, 0.23432262038639196, 0.23895455380126596, 0.24358648721613996, 0.24821842063101396, 0.25285035404588796, 0.25748228746076196, 0.2628578665006092, 0.26823344554045647, 0.27360902458030373, 0.278984603620151, 0.28436018265999824, 0.2897357616998455, 0.2948222316743412, 0.2999087016488369, 0.30499517162333256, 0.31008164159782825, 0.31516811157232394, 0.3202545815468196, 0.3315098616905881, 0.33905705371846845, 0.3466042457463488, 0.35415143777422914, 0.3616986298021095, 0.36924582182998983, 0.37837825477490517, 0.3875106877198205, 0.39664312066473584, 0.4057755536096512, 0.4149079865545665, 0.42404041949948185, 0.4331447464699158, 0.44224907344034975, 0.4513534004107837, 0.46045772738121765, 0.4695620543516516, 0.47866638132208555, 0.48890166395660706, 0.49913694659112856, 0.5093722292256501, 0.5196075118601715, 0.529842794494693, 0.5400780771292144, 0.5534949280077356, 0.5669117788862568, 0.580328629764778, 0.5937454806432991, 0.6071623315218203, 0.6205791824003415, 0.6403887186252941, 0.6601982548502467, 0.6800077910751994, 0.699817327300152, 0.7196268635251046, 0.7394363997500573, 0.7703047137228498, 0.8011730276956424, 0.8320413416684349, 0.8629096556412275, 0.89377796961402, 0.9246462835868126, 0.962962404634053, 1.0012785256812935, 1.039594646728534, 1.0779107677757744, 1.116226888823015, 1.1545430098702554, 1.2046491989403394, 1.2547553880104234, 1.3048615770805074, 1.3549677661505914, 1.4050739552206755, 1.4551801442907595, 1.5249451006577108, 1.5947100570246622, 1.6644750133916135, 1.7342399697585649, 1.8040049261255162, 1.8737698824924676, 1.955002936316254, 2.0362359901400406, 2.117469043963827, 2.1987020977876135, 2.2799351516114, 2.3611682054351864, 2.488124813413509, 2.6150814213918316, 2.7420380293701543, 2.868994637348477, 2.9959512453267996, 3.122907853305122, 3.3341313375508217, 3.545354821796521, 3.7565783060422206, 3.96780179028792, 4.17902527453362, 5.197933996377317, 6.216842718221013, 7.23575144006471, 8.254660161908406, 10.0]</t>
+          <t>[0.0, 5.942432777363632e-07, 1.1884865554727263e-06, 7.130919332836359e-06, 1.307335211019999e-05, 3.086134246948727e-05, 4.864933282877455e-05, 6.643732318806183e-05, 0.00011040907022628473, 0.0001543808172645076, 0.0001983525643027305, 0.00041359884284429614, 0.0006288451213858618, 0.0008440913999274275, 0.0016935995224422668, 0.002543107644957106, 0.0033926157674719452, 0.004426540843516299, 0.005460465919560653, 0.0064943909956050065, 0.00752831607164936, 0.009548335599899024, 0.011568355128148688, 0.013588374656398353, 0.015608394184648017, 0.01762841371289768, 0.02313216346091664, 0.028635913208935597, 0.03413966295695456, 0.03964341270497352, 0.04514716245299248, 0.05318861152484993, 0.06123006059670738, 0.06927150966856482, 0.07731295874042227, 0.08535440781227971, 0.09339585688413715, 0.10137529507868724, 0.10935473327323733, 0.11733417146778742, 0.12373866076179606, 0.13014315005580468, 0.1365476393498133, 0.1429521286438219, 0.1493566179378305, 0.15597090605952574, 0.16258519418122097, 0.1691994823029162, 0.17581377042461144, 0.18242805854630667, 0.1890423466680019, 0.19505923883072881, 0.20107613099345573, 0.20709302315618264, 0.21310991531890955, 0.21912680748163646, 0.2251832711660634, 0.23123973485049035, 0.2372961985349173, 0.24335266221934423, 0.24940912590377118, 0.2554655895881981, 0.26131932796949536, 0.26717306635079263, 0.2730268047320899, 0.27888054311338717, 0.28473428149468444, 0.2905880198759817, 0.2963884542585285, 0.3021888886410753, 0.3079893230236221, 0.3137897574061689, 0.31959019178871567, 0.32539062617126246, 0.3342864826371019, 0.3431823391029414, 0.35207819556878084, 0.3609740520346203, 0.36986990850045975, 0.3796518207781606, 0.3894337330558615, 0.39921564533356235, 0.4089975576112632, 0.4187794698889641, 0.42856138216666495, 0.44039980197613177, 0.4522382217855986, 0.4640766415950654, 0.4759150614045322, 0.48775348121399903, 0.49959190102346585, 0.5159634982870246, 0.5323350955505833, 0.5487066928141421, 0.5650782900777008, 0.5814498873412596, 0.6053154794927107, 0.6291810716441618, 0.6530466637956129, 0.6769122559470641, 0.7007778480985152, 0.7353575156581483, 0.7699371832177815, 0.8045168507774146, 0.8390965183370478, 0.873676185896681, 0.9106463948349163, 0.9476166037731516, 0.9845868127113869, 1.0215570216496221, 1.0585272305878575, 1.1189845992374159, 1.1794419678869743, 1.2398993365365327, 1.3003567051860911, 1.3608140738356496, 1.421271442485208, 1.4880094556218617, 1.5547474687585154, 1.6214854818951692, 1.688223495031823, 1.7549615081684766, 1.8559572585191118, 1.9569530088697469, 2.0579487592203822, 2.1589445095710174, 2.2599402599216525, 2.3609360102722876, 2.4896176289633836, 2.6182992476544795, 2.7469808663455755, 2.8756624850366714, 3.0043441037277674, 3.1330257224188633, 3.2806396448134088, 3.428253567207954, 3.5758674896024996, 3.723481411997045, 3.8710953343915904, 4.018709256786136, 4.253758147239042, 4.488807037691948, 4.723855928144854, 4.95890481859776, 5.193953709050666, 5.429002599503572, 5.712006856053182, 5.995011112602792, 6.278015369152402, 6.561019625702012, 6.844023882251622, 7.127028138801232, 7.513788343964114, 7.900548549126996, 8.287308754289878, 8.674068959452761, 9.060829164615644, 9.447589369778527, 9.983152612781113, 10.0]</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>0.3003520011421242</v>
+        <v>0.6281945676476332</v>
       </c>
       <c r="D7" t="n">
         <v>9.81</v>
@@ -902,13 +902,13 @@
         <v>2</v>
       </c>
       <c r="L7" t="n">
-        <v>3.003520011421242</v>
+        <v>6.281945676476331</v>
       </c>
       <c r="M7" t="n">
-        <v>0.02217016554282986</v>
+        <v>0.005068058773472081</v>
       </c>
       <c r="N7" t="n">
-        <v>0.1108508277141493</v>
+        <v>0.0253402938673604</v>
       </c>
       <c r="O7" t="n">
         <v>19.61967625424572</v>
@@ -938,11 +938,11 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>[0.0, 5.942445761009135e-07, 1.188489152201827e-06, 7.130934913210962e-06, 1.3073380674220097e-05, 3.08614099874032e-05, 4.8649439300586306e-05, 6.643746861376941e-05, 0.0001104093155872215, 0.00015438116256067357, 0.00019835300953412562, 0.0004136026365634725, 0.0006288522635928194, 0.0008441018906221663, 0.0016923783560319056, 0.002540654821441645, 0.003388931286851384, 0.004423077075323437, 0.005457222863795489, 0.006491368652267542, 0.007525514440739595, 0.009548310224311955, 0.011571106007884316, 0.013593901791456676, 0.015616697575029037, 0.017639493358601398, 0.023194015647964285, 0.028748537937327172, 0.03430306022669006, 0.039857582516052946, 0.04541210480541583, 0.053647347817834326, 0.06188259083025282, 0.07011783384267131, 0.0783530768550898, 0.08658831986750828, 0.09482356287992677, 0.10245560870458469, 0.1100876545292426, 0.11771970035390052, 0.12535174617855843, 0.13298379200321636, 0.1406158378278743, 0.14713736511311015, 0.15365889239834601, 0.16018041968358188, 0.16670194696881774, 0.1732234742540536, 0.17974500153928946, 0.1860455791595979, 0.19234615677990635, 0.1986467344002148, 0.20325756106730952, 0.20786838773440425, 0.21247921440149897, 0.2170900410685937, 0.22170086773568842, 0.22971595802045813, 0.23434892819032255, 0.23898189836018696, 0.24361486853005138, 0.2482478386999158, 0.2528808088697802, 0.2575137790396446, 0.26288771181394754, 0.26826164458825047, 0.2736355773625534, 0.2790095101368563, 0.28438344291115925, 0.28975737568546217, 0.29484196900345155, 0.29992656232144094, 0.3050111556394303, 0.3100957489574197, 0.3151803422754091, 0.32026493559339847, 0.33141216870486273, 0.3389546401834831, 0.34649711166210345, 0.3540395831407238, 0.3615820546193442, 0.36912452609796453, 0.3781524518641568, 0.38718037763034907, 0.39620830339654134, 0.4052362291627336, 0.4142641549289259, 0.42329208069511814, 0.4324081479424621, 0.441524215189806, 0.45064028243714993, 0.45975634968449386, 0.4688724169318378, 0.4779884841791817, 0.4882257362031365, 0.49846298822709123, 0.508700240251046, 0.5189374922750007, 0.5291747442989555, 0.5394119963229103, 0.5527759916092685, 0.5661399868956267, 0.579503982181985, 0.5928679774683432, 0.6062319727547014, 0.6195959680410597, 0.6392727276446353, 0.6589494872482109, 0.6786262468517865, 0.6983030064553621, 0.7179797660589378, 0.7376565256625134, 0.7683473395142394, 0.7990381533659654, 0.8297289672176914, 0.8604197810694174, 0.8911105949211434, 0.9218014087728694, 0.9600684396324304, 0.9983354704919913, 1.0366025013515523, 1.0748695322111133, 1.1131365630706742, 1.1514035939302352, 1.2013139968972002, 1.2512243998641652, 1.3011348028311303, 1.3510452057980953, 1.4009556087650603, 1.4508660117320253, 1.5202844552826058, 1.5897028988331863, 1.6591213423837667, 1.7285397859343472, 1.7979582294849277, 1.8673766730355081, 1.9482638548992595, 2.029151036763011, 2.1100382186267623, 2.1909254004905137, 2.271812582354265, 2.3526997642180163, 2.478825175136798, 2.6049505860555797, 2.7310759969743614, 2.857201407893143, 2.983326818811925, 3.1094522297307066, 3.318647665097651, 3.5278431004645956, 3.73703853583154, 3.9462339711984846, 4.155429406565429, 5.112536316104592, 6.0696432256437545, 7.026750135182917, 7.98385704472208, 10.0]</t>
+          <t>[0.0, 5.942445761009135e-07, 1.188489152201827e-06, 7.130934913210962e-06, 1.3073380674220097e-05, 3.08614099844169e-05, 4.864943929461371e-05, 6.643746860481051e-05, 0.00011040931504445142, 0.0001543811614840923, 0.0001983530079237332, 0.00041360161110568064, 0.000628850214287628, 0.0008440988174695755, 0.0016932314650892418, 0.0025423641127089083, 0.0033914967603285748, 0.004425320468321392, 0.005459144176314209, 0.006492967884307026, 0.0075267915922998425, 0.00954713067850141, 0.011567469764702978, 0.013587808850904546, 0.015608147937106114, 0.01762848702330768, 0.02313215808853593, 0.028635829153764177, 0.034139500218992425, 0.03964317128422067, 0.04514684234944892, 0.05318915790848166, 0.0612314734675144, 0.06927378902654713, 0.07731610458557986, 0.08535842014461259, 0.09340073570364532, 0.10137808363621975, 0.10935543156879418, 0.11733277950136861, 0.12373653694234917, 0.13014029438332972, 0.1365440518243103, 0.14294780926529085, 0.14935156670627142, 0.1559658463431947, 0.16258012598011795, 0.16919440561704122, 0.17580868525396448, 0.18242296489088775, 0.189037244527811, 0.19505319302335797, 0.20106914151890493, 0.20708509001445188, 0.21310103850999884, 0.2191169870055458, 0.22517126922462236, 0.2312255514436989, 0.23727983366277547, 0.24333411588185203, 0.24938839810092858, 0.25544268032000517, 0.2612969919847635, 0.2671513036495219, 0.27300561531428025, 0.2788599269790386, 0.28471423864379697, 0.29056855030855533, 0.29636869771710556, 0.3021688451256558, 0.307968992534206, 0.31376913994275624, 0.31956928735130646, 0.3253694347598567, 0.33426412082699913, 0.3431588068941416, 0.352053492961284, 0.36094817902842646, 0.3698428650955689, 0.37962446056334426, 0.3894060560311196, 0.39918765149889496, 0.4089692469666703, 0.41875084243444566, 0.428532437902221, 0.44037016792953715, 0.4522078979568533, 0.46404562798416943, 0.47588335801148557, 0.4877210880388017, 0.49955881806611785, 0.5159298037223513, 0.5323007893785847, 0.5486717750348181, 0.5650427606910515, 0.5814137463472849, 0.605278112752132, 0.629142479156979, 0.653006845561826, 0.676871211966673, 0.70073557837152, 0.7353133188349535, 0.7698910592983871, 0.8044687997618206, 0.8390465402252542, 0.8736242806886877, 0.9105923569803318, 0.9475604332719759, 0.98452850956362, 1.0214965858552643, 1.0584646621469085, 1.1189186622423266, 1.1793726623377447, 1.2398266624331629, 1.300280662528581, 1.3607346626239991, 1.4211886627194172, 1.487922814263889, 1.5546569658083607, 1.6213911173528324, 1.688125268897304, 1.7548594204417758, 1.8558494069035554, 1.956839393365335, 2.0578293798271146, 2.158819366288894, 2.2598093527506737, 2.3607993392124533, 2.489473598753463, 2.618147858294473, 2.7468221178354826, 2.8754963773764923, 3.004170636917502, 3.132844896458512, 3.2804504638721306, 3.4280560312857493, 3.575661598699368, 3.723267166112987, 3.8708727335266055, 4.018478300940224, 4.2535138545388875, 4.488549408137551, 4.723584961736215, 4.958620515334879, 5.193656068933542, 5.428691622532206, 5.711680032021765, 5.994668441511324, 6.277656851000883, 6.560645260490443, 6.843633669980002, 7.126622079469561, 7.513360696994241, 7.90009931451892, 8.2868379320436, 8.67357654956828, 9.06031516709296, 9.447053784617639, 9.982585815666416, 10.0]</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>0.300349685184086</v>
+        <v>0.6281039087644976</v>
       </c>
       <c r="D8" t="n">
         <v>9.81</v>
@@ -969,13 +969,13 @@
         <v>2</v>
       </c>
       <c r="L8" t="n">
-        <v>3.00349685184086</v>
+        <v>6.281039087644976</v>
       </c>
       <c r="M8" t="n">
-        <v>0.02217050744677442</v>
+        <v>0.00506952189987717</v>
       </c>
       <c r="N8" t="n">
-        <v>0.1108525372338721</v>
+        <v>0.02534760949938585</v>
       </c>
       <c r="O8" t="n">
         <v>19.61959050849376</v>
@@ -1005,11 +1005,11 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>[0.0, 5.942462183561271e-07, 1.1884924367122541e-06, 7.130954620273526e-06, 1.3073416803834797e-05, 3.086149538464003e-05, 4.864957396544526e-05, 6.643765254625049e-05, 0.00011040962524902647, 0.00015438159795180245, 0.00019835357065457843, 0.00041360613817857585, 0.0006288587057025732, 0.0008441112732265706, 0.001691915682687794, 0.0025397200921490177, 0.0033875245016102415, 0.004421543091760744, 0.0054555616819112465, 0.006489580272061749, 0.0075235988622122515, 0.00954680095503433, 0.011570003047856409, 0.013593205140678487, 0.015616407233500565, 0.017639609326322643, 0.02319403408571982, 0.028748458845116995, 0.03430288360451417, 0.03985730836391134, 0.04541173312330851, 0.0536482320161126, 0.06188473090891669, 0.07012122980172078, 0.07835772869452487, 0.08659422758732896, 0.09483072648013305, 0.10246206572425823, 0.11009340496838341, 0.11772474421250859, 0.12535608345663377, 0.13298742270075894, 0.14061876194488412, 0.14713980235331098, 0.15366084276173783, 0.16018188317016469, 0.16670292357859154, 0.1732239639870184, 0.17974500439544525, 0.18604667047914722, 0.1923483365628492, 0.19865000264655117, 0.2032596780591498, 0.20786935347174842, 0.21247902888434705, 0.21708870429694568, 0.2216983797095443, 0.22976010382297063, 0.23439522867507667, 0.23903035352718272, 0.24366547837928876, 0.2483006032313948, 0.25293572808350084, 0.2575708529356069, 0.2629411862592761, 0.2683115195829453, 0.2736818529066145, 0.2790521862302837, 0.2844225195539529, 0.28979285287762213, 0.2948743706467891, 0.2999558884159561, 0.3050374061851231, 0.3101189239542901, 0.31520044172345707, 0.32028195949262406, 0.3314439431588417, 0.3389780012062703, 0.34651205925369893, 0.35404611730112756, 0.3615801753485562, 0.3691142333959848, 0.3782532851389739, 0.38739233688196295, 0.396531388624952, 0.4056704403679411, 0.41480949211093016, 0.4239485438539192, 0.43305237070924013, 0.44215619756456104, 0.45126002441988194, 0.46036385127520285, 0.46946767813052376, 0.47857150498584466, 0.48881304261336916, 0.49905458024089366, 0.5092961178684181, 0.5195376554959426, 0.529779193123467, 0.5400207307509914, 0.5534534148414668, 0.5668860989319422, 0.5803187830224176, 0.593751467112893, 0.6071841512033683, 0.6206168352938437, 0.6404572023945865, 0.6602975694953293, 0.680137936596072, 0.6999783036968148, 0.7198186707975576, 0.7396590378983003, 0.7705391604916023, 0.8014192830849043, 0.8322994056782063, 0.8631795282715082, 0.8940596508648102, 0.9249397734581122, 0.9632314902882532, 1.0015232071183942, 1.0398149239485353, 1.0781066407786764, 1.1163983576088174, 1.1546900744389585, 1.2048226093376735, 1.2549551442363884, 1.3050876791351034, 1.3552202140338183, 1.4053527489325333, 1.4554852838312482, 1.5251870180492382, 1.5948887522672281, 1.6645904864852181, 1.734292220703208, 1.803993954921198, 1.873695689139188, 1.9548210542904583, 2.0359464194417285, 2.1170717845929987, 2.198197149744269, 2.279322514895539, 2.3604478800468094, 2.487226322084995, 2.6140047641231803, 2.7407832061613657, 2.867561648199551, 2.9943400902377366, 3.121118532275922, 3.331670845497544, 3.5422231587191657, 3.7527754719407875, 3.9633277851624094, 4.173880098384031, 5.160026155652637, 6.146172212921242, 7.132318270189848, 8.118464327458454, 10.0]</t>
+          <t>[0.0, 5.942462183561271e-07, 1.1884924367122541e-06, 7.130954620273526e-06, 1.3073416803834797e-05, 3.086149538165419e-05, 4.8649573959473585e-05, 6.643765253729297e-05, 0.00011040962470627208, 0.0001543815968752512, 0.00019835356904423032, 0.0004136051126777584, 0.0006288566563112865, 0.0008441081999448145, 0.0016927668827192537, 0.0025414255654936926, 0.0033900842482681316, 0.004423780074558494, 0.005457475900848857, 0.00649117172713922, 0.007524867553429583, 0.009545611216546701, 0.01156635487966382, 0.013587098542780939, 0.015607842205898058, 0.017628585869015174, 0.023132160534993583, 0.02863573520097199, 0.0341393098669504, 0.03964288453292881, 0.04514645919890722, 0.05318987124880683, 0.06123328329870644, 0.06927669534860606, 0.07732010739850567, 0.08536351944840528, 0.0934069314983049, 0.10138163825260178, 0.10935634500689867, 0.11733105176119556, 0.12373379686869124, 0.1301365419761869, 0.13653928708368257, 0.14294203219117824, 0.1493447772986739, 0.15595995711798946, 0.16257513693730502, 0.16919031675662058, 0.17580549657593614, 0.1824206763952517, 0.18903585621456725, 0.19504830497473263, 0.201060753734898, 0.2070732024950634, 0.21308565125522877, 0.21909810001539415, 0.22514566178568657, 0.231193223555979, 0.2372407853262714, 0.24328834709656383, 0.24933590886685625, 0.25538347063714867, 0.2612373570975627, 0.2670912435579767, 0.2729451300183907, 0.27879901647880473, 0.28465290293921874, 0.29050678939963276, 0.2963067371027996, 0.3021066848059664, 0.30790663250913325, 0.3137065802123001, 0.3195065279154669, 0.32530647561863374, 0.33421389324099304, 0.34312131086335235, 0.35202872848571165, 0.36093614610807095, 0.36984356373043026, 0.3796269765397787, 0.3894103893491272, 0.39919380215847566, 0.40897721496782413, 0.4187606277771726, 0.42854404058652107, 0.4403865866405074, 0.4522291326944937, 0.46407167874848004, 0.47591422480246637, 0.4877567708564527, 0.499599316910439, 0.5159747741851581, 0.5323502314598773, 0.5487256887345964, 0.5651011460093155, 0.5814766032840346, 0.6053446675966764, 0.6292127319093181, 0.6530807962219599, 0.6769488605346017, 0.7008169248472434, 0.7353996282063476, 0.7699823315654518, 0.804565034924556, 0.8391477382836602, 0.8737304416427644, 0.9107039345907404, 0.9476774275387164, 0.9846509204866924, 1.0216244134346684, 1.0585979063826443, 1.119056127149816, 1.1795143479169878, 1.2399725686841596, 1.3004307894513314, 1.3608890102185032, 1.421347230985675, 1.4880907370530727, 1.5548342431204705, 1.6215777491878682, 1.688321255255266, 1.7550647613226638, 1.8560697552846244, 1.957074749246585, 2.0580797432085456, 2.159084737170506, 2.2600897311324664, 2.3610947250944267, 2.489786849644444, 2.6184789741944616, 2.747171098744479, 2.8758632232944965, 3.004555347844514, 3.1332474723945314, 3.2808735280995123, 3.428499583804493, 3.576125639509474, 3.723751695214455, 3.871377750919436, 4.019003806624417, 4.25407221892094, 4.489140631217463, 4.724209043513986, 4.9592774558105095, 5.194345868107033, 5.429414280403556, 5.712443824986355, 5.995473369569154, 6.278502914151954, 6.561532458734753, 6.844562003317552, 7.1275915479003515, 7.514386998294119, 7.901182448687887, 8.287977899081655, 8.674773349475423, 9.06156879986919, 9.448364250262959, 9.983976371374482, 10.0]</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>0.3003467578390057</v>
+        <v>0.6279893313195548</v>
       </c>
       <c r="D9" t="n">
         <v>9.81</v>
@@ -1036,13 +1036,13 @@
         <v>2</v>
       </c>
       <c r="L9" t="n">
-        <v>3.003467578390056</v>
+        <v>6.279893313195548</v>
       </c>
       <c r="M9" t="n">
-        <v>0.02217093962085646</v>
+        <v>0.005071371949953078</v>
       </c>
       <c r="N9" t="n">
-        <v>0.1108546981042823</v>
+        <v>0.02535685974976539</v>
       </c>
       <c r="O9" t="n">
         <v>19.61948205253208</v>
@@ -1072,11 +1072,11 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>[0.0, 5.942482955904618e-07, 1.1884965911809236e-06, 7.1309795470855415e-06, 1.3073462502990159e-05, 3.0861603400782615e-05, 4.864974429857507e-05, 6.643788519636753e-05, 0.0001104100169300298, 0.0001543821486636921, 0.00019835428039735437, 0.00041361056741198493, 0.0006288668544266155, 0.000844123141441246, 0.0016913319820572145, 0.002538540822673183, 0.003385749663289152, 0.004419607895796719, 0.005453466128304286, 0.0064873243608118535, 0.007521182593319421, 0.009544899225982761, 0.011568615858646101, 0.013592332491309441, 0.015616049123972782, 0.017639765756636124, 0.023194072755818376, 0.02874837975500063, 0.03430268675418288, 0.039856993753365134, 0.04541130075254739, 0.053649403470012305, 0.06188750618747722, 0.07012560890494214, 0.07836371162240706, 0.08660181433987198, 0.0948399170573369, 0.10247035995416441, 0.11010080285099193, 0.11773124574781944, 0.12536168864464697, 0.1329921315414745, 0.140622574438302, 0.14714372889144714, 0.15366488334459227, 0.1601860377977374, 0.16670719225088254, 0.17322834670402767, 0.1797495011571728, 0.18605278989183965, 0.1923560786265065, 0.19865936736117334, 0.20326768917002708, 0.2078760109788808, 0.21248433278773454, 0.21709265459658827, 0.221700976405442, 0.2297925765264089, 0.23442879452393156, 0.23906501252145423, 0.2437012305189769, 0.24833744851649958, 0.25297366651402226, 0.25760988451154493, 0.2629789044154486, 0.2683479243193522, 0.2737169442232559, 0.2790859641271595, 0.2844549840310632, 0.2898240039349668, 0.2949119463017786, 0.29999988866859034, 0.3050878310354021, 0.31017577340221386, 0.3152637157690256, 0.3203516581358374, 0.3311910170165942, 0.3387105769551246, 0.34623013689365495, 0.3537496968321853, 0.3612692567707157, 0.36878881670924607, 0.37761124666196744, 0.3864336766146888, 0.39525610656741017, 0.40407853652013154, 0.4129009664728529, 0.42172339642557427, 0.4308632424625913, 0.4400030884996083, 0.4491429345366253, 0.4582827805736423, 0.4674226266106593, 0.4765624726476763, 0.48680509756510715, 0.497047722482538, 0.5072903473999688, 0.5175329723173996, 0.5277755972348304, 0.5380182221522611, 0.5512873042583835, 0.5645563863645058, 0.5778254684706281, 0.5910945505767504, 0.6043636326828727, 0.6176327147889951, 0.637065216294268, 0.656497717799541, 0.675930219304814, 0.695362720810087, 0.71479522231536, 0.734227723820633, 0.7645689305957067, 0.7949101373707805, 0.8252513441458543, 0.8555925509209281, 0.8859337576960019, 0.9162749644710757, 0.9544241703626588, 0.9925733762542419, 1.030722582145825, 1.0688717880374081, 1.1070209939289912, 1.1451701998205743, 1.1947113532166516, 1.2442525066127288, 1.293793660008806, 1.3433348134048833, 1.3928759668009605, 1.4424171201970377, 1.5111362729214028, 1.579855425645768, 1.648574578370133, 1.7172937310944982, 1.7860128838188634, 1.8547320365432285, 1.934897318970196, 2.0150626013971635, 2.095227883824131, 2.175393166251099, 2.2555584486780664, 2.335723731105034, 2.4590171633453455, 2.582310595585657, 2.7056040278259683, 2.8288974600662797, 2.952190892306591, 3.168011122575144, 3.383831352843697, 3.59965158311225, 3.815471813380803, 5.105141246063979, 6.394810678747154, 7.68448011143033, 10.0]</t>
+          <t>[0.0, 5.942482955904618e-07, 1.1884965911809236e-06, 7.1309795470855415e-06, 1.3073462502990159e-05, 3.0861603397797434e-05, 4.864974429260471e-05, 6.643788518741198e-05, 0.0001104100163872948, 0.00015438214758717761, 0.00019835427878706042, 0.0004136095418573381, 0.0006288648049276157, 0.0008441200679978933, 0.0016921807781542795, 0.0025402414883106657, 0.003388302198467052, 0.004421836805876193, 0.005455371413285334, 0.006488906020694476, 0.007522440628103617, 0.009543696635413945, 0.011564952642724273, 0.013586208650034601, 0.01560746465734493, 0.01762872066465526, 0.02313217861258009, 0.028635636560504923, 0.03413909450842975, 0.03964255245635458, 0.0451460104042794, 0.053190820541146995, 0.06123563067801459, 0.06928044081488219, 0.07732525095174979, 0.08537006108861739, 0.09341487122548499, 0.1013862367089923, 0.10935760219249961, 0.11732896767600692, 0.12373062967945868, 0.13013229168291043, 0.13653395368636217, 0.14293561568981392, 0.14933727769326566, 0.15595153648932863, 0.1625657952853916, 0.1691800540814546, 0.17579431287751757, 0.18240857167358054, 0.18902283046964352, 0.1950360487072489, 0.20104926694485425, 0.20706248518245962, 0.213075703420065, 0.21908892165767035, 0.22513692884266928, 0.2311849360276682, 0.23723294321266714, 0.24328095039766606, 0.249328957582665, 0.2553769647676639, 0.26123291254355496, 0.267088860319446, 0.27294480809533705, 0.2788007558712281, 0.28465670364711915, 0.2905126514230102, 0.29631197659665665, 0.3021113017703031, 0.30791062694394955, 0.313709952117596, 0.31950927729124246, 0.3253086024648889, 0.33420001159929713, 0.34309142073370535, 0.3519828298681136, 0.3608742390025218, 0.36976564813693, 0.3795463576618128, 0.38932706718669563, 0.39910777671157843, 0.40888848623646123, 0.41866919576134404, 0.42844990528622684, 0.44028568872695, 0.4521214721676732, 0.46395725560839635, 0.4757930390491195, 0.4876288224898427, 0.49946460593056585, 0.5158338750716965, 0.5322031442128272, 0.5485724133539579, 0.5649416824950886, 0.5813109516362193, 0.6051718454895616, 0.6290327393429039, 0.6528936331962463, 0.6767545270495886, 0.7006154209029309, 0.7351876927622334, 0.7697599646215358, 0.8043322364808383, 0.8389045083401407, 0.8734767801994432, 0.9104388023363853, 0.9474008244733274, 0.9843628466102695, 1.0213248687472116, 1.0582868908841538, 1.118731316606788, 1.1791757423294222, 1.2396201680520564, 1.3000645937746906, 1.3605090194973248, 1.420953445219959, 1.4876766345365764, 1.5543998238531938, 1.6211230131698111, 1.6878462024864285, 1.7545693918030458, 1.8555430295250037, 1.9565166672469616, 2.0574903049689195, 2.1584639426908776, 2.2594375804128357, 2.360411218134794, 2.4890645869231802, 2.6177179557115666, 2.746371324499953, 2.8750246932883394, 3.003678062076726, 3.1323314308651122, 3.2799132939676405, 3.427495157070169, 3.575077020172697, 3.7226588832752254, 3.8702407463777537, 4.017822609480282, 4.252820311195249, 4.487818012910216, 4.722815714625183, 4.95781341634015, 5.192811118055117, 5.427808819770084, 5.710752357544079, 5.993695895318075, 6.27663943309207, 6.559582970866066, 6.842526508640061, 7.125470046414057, 7.512147416171787, 7.898824785929518, 8.285502155687249, 8.67217952544498, 9.05885689520271, 9.445534264960441, 9.980977841230501, 10.0]</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>0.3003430501950728</v>
+        <v>0.627844555184058</v>
       </c>
       <c r="D10" t="n">
         <v>9.81</v>
@@ -1103,13 +1103,13 @@
         <v>2</v>
       </c>
       <c r="L10" t="n">
-        <v>3.003430501950728</v>
+        <v>6.27844555184058</v>
       </c>
       <c r="M10" t="n">
-        <v>0.02217148701129614</v>
+        <v>0.005073711058506403</v>
       </c>
       <c r="N10" t="n">
-        <v>0.1108574350564807</v>
+        <v>0.02536855529253201</v>
       </c>
       <c r="O10" t="n">
         <v>19.61934487144314</v>
@@ -1139,11 +1139,11 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>[0.0, 5.942509230219617e-07, 1.1885018460439234e-06, 7.131011076263541e-06, 1.3073520306483159e-05, 3.08617400271673e-05, 4.864995974785144e-05, 6.643817946853558e-05, 0.00011041051235563705, 0.00015438284524273854, 0.00019835517812984003, 0.00041361617006575874, 0.0006288771620016774, 0.0008441381539375961, 0.0016905960955732506, 0.002537054037208905, 0.0033835119788445597, 0.004417168225220889, 0.005450824471597218, 0.006484480717973547, 0.007518136964349876, 0.009542505398820636, 0.011566873833291396, 0.013591242267762156, 0.015615610702232916, 0.017639979136703676, 0.023194145418830765, 0.028748311700957853, 0.034302477983084945, 0.039856644265212036, 0.04541081054733913, 0.05365094618528237, 0.06189108182322561, 0.07013121746116885, 0.07837135309911208, 0.08661148873705532, 0.09485162437499856, 0.10248093649244873, 0.1101102486098989, 0.11773956072734908, 0.12536887284479925, 0.1329981849622494, 0.14062749707969957, 0.14714838902820399, 0.1536692809767084, 0.16019017292521281, 0.16671106487371723, 0.17323195682222164, 0.17975284877072606, 0.18605805895821625, 0.19236326914570645, 0.19866847933319665, 0.2032750346935202, 0.20788159005384377, 0.21248814541416733, 0.2170947007744909, 0.22170125613481445, 0.22985082344317811, 0.23448897324842513, 0.23912712305367215, 0.24376527285891916, 0.24840342266416618, 0.25304157246941317, 0.2576797222746602, 0.26255745740142594, 0.2674351925281917, 0.27231292765495746, 0.2771906627817232, 0.282068397908489, 0.28694613303525474, 0.29200201722446906, 0.2970579014136834, 0.3021137856028977, 0.307169669792112, 0.31222555398132634, 0.31728143817054066, 0.32496667659298, 0.33265191501541935, 0.3403371534378587, 0.34802239186029804, 0.35316029274676763, 0.3582981936332372, 0.3634360945197068, 0.3685739954061764, 0.373711896292646, 0.3798798737943376, 0.38604785129602914, 0.3922158287977207, 0.3983838062994123, 0.40455178380110385, 0.4107197613027954, 0.42007340483019967, 0.4294270483576039, 0.4387806918850082, 0.44813433541241243, 0.4574879789398167, 0.46684162246722094, 0.4770046348821429, 0.48716764729706485, 0.4973306597119868, 0.5074936721269088, 0.5176566845418307, 0.5278196969567526, 0.5404758299249415, 0.5531319628931304, 0.5657880958613193, 0.5784442288295082, 0.5911003617976971, 0.603756494765886, 0.6216994504445965, 0.639642406123307, 0.6575853618020175, 0.6755283174807281, 0.6934712731594386, 0.7204635730187802, 0.7474558728781218, 0.7744481727374634, 0.801440472596805, 0.8284327724561465, 0.8625240495791059, 0.8966153267020652, 0.9307066038250246, 0.9647978809479839, 0.9988891580709433, 1.0395693676859974, 1.0802495773010516, 1.120929786916106, 1.1616099965311601, 1.2022902061462144, 1.2429704157612687, 1.3048652909951937, 1.3667601662291187, 1.4286550414630437, 1.4905499166969687, 1.5524447919308937, 1.6143396671648187, 1.6891987393794932, 1.7640578115941676, 1.838916883808842, 1.9137759560235166, 1.988635028238191, 2.0634941004528655, 2.165748503390066, 2.268002906327266, 2.3702573092644665, 2.472511712201667, 2.574766115138867, 2.6770205180760676, 2.831366884011291, 2.985713249946514, 3.1400596158817375, 3.294405981816961, 3.448752347752184, 3.6030987136874075, 3.87729078512904, 4.151482856570672, 4.425674928012304, 4.699866999453937, 4.974059070895569, 5.796719382012618, 6.619379693129668, 7.442040004246717, 8.264700315363767, 10.0]</t>
+          <t>[0.0, 5.942509230219617e-07, 1.1885018460439234e-06, 7.131011076263541e-06, 1.3073520306483159e-05, 3.08617400241829e-05, 4.8649959741882634e-05, 6.643817945958237e-05, 0.0001104105118129267, 0.000154382844166271, 0.00019835517651961532, 0.00041361514444324544, 0.0006288751123668756, 0.0008441350802905057, 0.0016914418679977903, 0.002538748655705075, 0.0033860554434123596, 0.004419386980488469, 0.0054527185175645785, 0.006486050054640688, 0.007519381591716797, 0.00954128662034704, 0.011563191648977284, 0.013585096677607527, 0.01560700170623777, 0.017628906734868013, 0.02313222505040221, 0.028635543365936406, 0.0341388616814706, 0.0396421799970048, 0.045145498312538994, 0.0531920815994982, 0.06123866488645741, 0.06928524817341662, 0.07733183146037584, 0.08537841474733505, 0.09342499803429427, 0.10139214264149127, 0.10935928724868826, 0.11732643185588526, 0.1237266146861277, 0.13012679751637013, 0.13652698034661256, 0.142927163176855, 0.14932734600709743, 0.15594159318168896, 0.16255584035628048, 0.169170087530872, 0.17578433470546354, 0.18239858188005506, 0.1890128290546466, 0.19502409455617095, 0.20103536005769532, 0.20704662555921968, 0.21305789106074405, 0.2190691565622684, 0.2251127091941974, 0.2311562618261264, 0.23719981445805538, 0.24324336708998437, 0.24928691972191336, 0.2553304723538423, 0.2611875702389803, 0.2670446681241183, 0.2729017660092563, 0.2787588638943943, 0.2846159617795323, 0.2904730596646703, 0.29627180393602887, 0.30207054820738743, 0.307869292478746, 0.3136680367501046, 0.31946678102146314, 0.3252655252928217, 0.33415468530283055, 0.3430438453128394, 0.3519330053228482, 0.36082216533285705, 0.3697113253428659, 0.3794914278438147, 0.3892715303447635, 0.39905163284571227, 0.40883173534666106, 0.41861183784760986, 0.42839194034855865, 0.4402263741384946, 0.4520608079284305, 0.46389524171836644, 0.47572967550830236, 0.4875641092982383, 0.4993985430881742, 0.5157666303448002, 0.5321347176014262, 0.5485028048580521, 0.5648708921146781, 0.5812389793713041, 0.6050974535997763, 0.6289559278282485, 0.6528144020567207, 0.6766728762851929, 0.7005313505136651, 0.7350998036060068, 0.7696682566983485, 0.8042367097906902, 0.8388051628830319, 0.8733736159753736, 0.9103314086732172, 0.9472892013710608, 0.9842469940689044, 1.021204786766748, 1.0581625794645917, 1.1186002984899155, 1.1790380175152393, 1.239475736540563, 1.2999134555658869, 1.3603511745912107, 1.4207888936165345, 1.4875044238149169, 1.5542199540132993, 1.6209354842116817, 1.687651014410064, 1.7543665446084464, 1.8553287749184164, 1.9562910052283864, 2.057253235538356, 2.158215465848326, 2.2591776961582957, 2.3601399264682654, 2.4887787032246957, 2.617417479981126, 2.7460562567375564, 2.8746950334939867, 3.003333810250417, 3.1319725870068473, 3.2795378923345293, 3.4271031976622113, 3.5746685029898932, 3.722233808317575, 3.869799113645257, 4.017364418972939, 4.252335683658167, 4.487306948343395, 4.722278213028623, 4.957249477713852, 5.19222074239908, 5.427192007084308, 5.710104214005361, 5.9930164209264145, 6.275928627847468, 6.558840834768521, 6.841753041689574, 7.124665248610627, 7.511299866400934, 7.897934484191241, 8.284569101981548, 8.671203719771855, 9.057838337562162, 9.444472955352468, 9.979854738547234, 10.0]</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>0.3003383626789455</v>
+        <v>0.6276616710166519</v>
       </c>
       <c r="D11" t="n">
         <v>9.81</v>
@@ -1170,13 +1170,13 @@
         <v>2</v>
       </c>
       <c r="L11" t="n">
-        <v>3.003383626789454</v>
+        <v>6.276616710166519</v>
       </c>
       <c r="M11" t="n">
-        <v>0.02217217909746881</v>
+        <v>0.0050766681822198</v>
       </c>
       <c r="N11" t="n">
-        <v>0.1108608954873441</v>
+        <v>0.025383340911099</v>
       </c>
       <c r="O11" t="n">
         <v>19.61917135722715</v>
@@ -1206,11 +1206,11 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>[0.0, 5.942542463917016e-07, 1.1885084927834032e-06, 7.13105095670042e-06, 1.3073593420617436e-05, 3.086191284232796e-05, 4.8650232264038484e-05, 6.643855168574901e-05, 0.00011041113900665433, 0.00015438372632755964, 0.00019835631364846496, 0.0004136232571157099, 0.0006288902005829549, 0.0008441571440501998, 0.001689669137418599, 0.0025351811307869985, 0.003380693124155398, 0.0044140952281158585, 0.005447497332076319, 0.006480899436036779, 0.007514301539997239, 0.009539495985085772, 0.011564690430174305, 0.013589884875262838, 0.015615079320351371, 0.017640273765439904, 0.023194275288396946, 0.028748276811353987, 0.03430227833431103, 0.03985627985726807, 0.04541028138022511, 0.05365299944910189, 0.06189571751797866, 0.07013843558685544, 0.07838115365573221, 0.08662387172460899, 0.09486658979348576, 0.10249447492053076, 0.11012236004757577, 0.11775024517462077, 0.12537813030166578, 0.1330060154287108, 0.1406339005557558, 0.14715413711274833, 0.15367437366974085, 0.16019461022673337, 0.1667148467837259, 0.1732350833407184, 0.17975531989771093, 0.18606285992689692, 0.1923703999560829, 0.1986779399852689, 0.20328221439924016, 0.20788648881321142, 0.2124907632271827, 0.21709503764115395, 0.22169931205512522, 0.2299442055971994, 0.23458756402652378, 0.23923092245584815, 0.24387428088517252, 0.24851763931449689, 0.2531609977438213, 0.2578043561731457, 0.26316301827851396, 0.26852168038388224, 0.27388034248925053, 0.2792390045946188, 0.2845976666999871, 0.2899563288053554, 0.2950236433188693, 0.30009095783238326, 0.3051582723458972, 0.31022558685941115, 0.3152929013729251, 0.32036021588643904, 0.3318730437899504, 0.3394025392208422, 0.34693203465173394, 0.3544615300826257, 0.3619910255135175, 0.36952052094440924, 0.3793991252732584, 0.3892777296021076, 0.39687554889053517, 0.40447336817896273, 0.4120711874673903, 0.41966900675581786, 0.42726682604424543, 0.434864645332673, 0.44302168846326145, 0.4511787315938499, 0.4593357747244384, 0.46749281785502683, 0.4756498609856153, 0.48547063657226336, 0.4952914121589114, 0.5051121877455595, 0.5149329633322077, 0.5247537389188559, 0.53731105843755, 0.5498683779562441, 0.5624256974749382, 0.5749830169936323, 0.5875403365123264, 0.6049512869686203, 0.6223622374249143, 0.6397731878812082, 0.6571841383375021, 0.674595088793796, 0.7003212914599092, 0.7260474941260223, 0.7517736967921355, 0.7774998994582486, 0.8032261021243617, 0.833555283930169, 0.8638844657359762, 0.8942136475417835, 0.9245428293475907, 0.9548720111533979, 0.9903933162022734, 1.025914621251149, 1.0614359263000246, 1.0969572313489002, 1.1324785363977758, 1.1756086539223953, 1.2187387714470148, 1.2618688889716343, 1.3049990064962538, 1.3481291240208733, 1.3912592415454927, 1.4611566658844233, 1.5310540902233538, 1.6009515145622844, 1.6708489389012149, 1.7407463632401454, 1.810643787579076, 1.8894722733031961, 1.9683007590273163, 2.0471292447514364, 2.1259577304755566, 2.2047862161996767, 2.283614701923797, 2.401076375736902, 2.5185380495500067, 2.6359997233631116, 2.7534613971762165, 2.8709230709893214, 2.9883847448024263, 3.180226588207398, 3.37206843161237, 3.5639102750173417, 3.7557521184223135, 3.9475939618272853, 4.641016268024108, 5.334438574220931, 6.027860880417753, 6.721283186614576, 9.361130365429531, 10.0]</t>
+          <t>[0.0, 5.942542463917016e-07, 1.1885084927834032e-06, 7.13105095670042e-06, 1.3073593420617436e-05, 3.086191283934457e-05, 4.86502322580717e-05, 6.643855167679882e-05, 0.00011041113846397605, 0.00015438372525115328, 0.00019835631203833051, 0.00041362223140662053, 0.0006288881507749105, 0.0008441540701432006, 0.0016905111122795112, 0.002536868154415822, 0.0033832251965521328, 0.00441630122798287, 0.005449377259413607, 0.006482453290844344, 0.007515529322275082, 0.009538256838342528, 0.011560984354409973, 0.01358371187047742, 0.015606439386544865, 0.017629166902612313, 0.0231323213774089, 0.028635475852205487, 0.034138630327002074, 0.03964178480179866, 0.04514493927659525, 0.0531937756836251, 0.06124261209065495, 0.0692914484976848, 0.07734028490471465, 0.08538912131174449, 0.09343795771877433, 0.1013997708628615, 0.10936158400694868, 0.11732339715103585, 0.12372162445103722, 0.1301198517510386, 0.13651807905103996, 0.14291630635104133, 0.1493145336510427, 0.15592968517690114, 0.1625448367027596, 0.16915998822861805, 0.1757751397544765, 0.18239029128033496, 0.1890054428061934, 0.19501184529142077, 0.20101824777664812, 0.20702465026187547, 0.21303105274710282, 0.21903745523233017, 0.22507132309518857, 0.23110519095804696, 0.23713905882090536, 0.24317292668376375, 0.24920679454662215, 0.2552406624094805, 0.26109800124945953, 0.26695534008943855, 0.2728126789294176, 0.2786700177693966, 0.2845273566093756, 0.29038469544935464, 0.29618286380622344, 0.30198103216309224, 0.30777920051996105, 0.31357736887682985, 0.31937553723369866, 0.32517370559056746, 0.33407462717123987, 0.3429755487519123, 0.3518764703325847, 0.3607773919132571, 0.3696783134939295, 0.379459988516545, 0.3892416635391605, 0.399023338561776, 0.40880501358439153, 0.41858668860700704, 0.42836836362962255, 0.44020690160759196, 0.45204543958556137, 0.4638839775635308, 0.4757225155415002, 0.4875610535194696, 0.499399591497439, 0.5157716083363638, 0.5321436251752887, 0.5485156420142135, 0.5648876588531384, 0.5812596756920633, 0.6051205278150351, 0.628981379938007, 0.6528422320609788, 0.6767030841839506, 0.7005639363069225, 0.7351351976863375, 0.7697064590657525, 0.8042777204451675, 0.8388489818245826, 0.8734202432039976, 0.9103810462405703, 0.9473418492771429, 0.9843026523137156, 1.0212634553502884, 1.0582242583868613, 1.1186622804406305, 1.1791003024943998, 1.239538324548169, 1.2999763466019383, 1.3604143686557075, 1.4208523907094768, 1.4875729187086268, 1.554293446707777, 1.621013974706927, 1.687734502706077, 1.7544550307052271, 1.8554257987406166, 1.9563965667760062, 2.0573673348113957, 2.158338102846785, 2.2593088708821742, 2.3602796389175635, 2.4889279882154294, 2.617576337513295, 2.746224686811161, 2.874873036109027, 3.0035213854068927, 3.1321697347047586, 3.279746111783442, 3.427322488862125, 3.5748988659408085, 3.722475243019492, 3.870051620098175, 4.0176279971768585, 4.252617100258853, 4.487606203340847, 4.722595306422841, 4.957584409504835, 5.192573512586829, 5.4275626156688235, 5.710498229672117, 5.993433843675411, 6.276369457678705, 6.559305071681998, 6.842240685685292, 7.125176299688586, 7.511843601760332, 7.898510903832078, 8.285178205903826, 8.671845507975572, 9.058512810047318, 9.445180112119065, 9.980606978721621, 10.0]</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>0.3003324587766139</v>
+        <v>0.6274307264766951</v>
       </c>
       <c r="D12" t="n">
         <v>9.81</v>
@@ -1237,13 +1237,13 @@
         <v>2</v>
       </c>
       <c r="L12" t="n">
-        <v>3.003324587766139</v>
+        <v>6.27430726476695</v>
       </c>
       <c r="M12" t="n">
-        <v>0.02217305082253666</v>
+        <v>0.005080406107450482</v>
       </c>
       <c r="N12" t="n">
-        <v>0.1108652541126833</v>
+        <v>0.02540203053725241</v>
       </c>
       <c r="O12" t="n">
         <v>19.61895188686585</v>
@@ -1273,11 +1273,11 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>[0.0, 5.942584500521307e-07, 1.1885169001042613e-06, 7.131101400625569e-06, 1.3073685901146876e-05, 3.08621314325892e-05, 4.865057696403153e-05, 6.643902249547386e-05, 0.00011041193164442831, 0.00015438484079338276, 0.0001983577499423372, 0.00041363222201434786, 0.0006289066940863585, 0.0008441811661583692, 0.0016885027508724902, 0.002532824335586611, 0.0033771459203007317, 0.004410228700037035, 0.005443311479773338, 0.006476394259509642, 0.0075094770392459455, 0.009535718794638322, 0.0115619605500307, 0.013588202305423076, 0.015614444060815453, 0.01764068581620783, 0.02319450032632943, 0.028748314836451027, 0.034302129346572625, 0.03985594385669422, 0.045409758366815815, 0.05365577249042954, 0.06190178661404327, 0.070147800737657, 0.07839381486127073, 0.08663982898488445, 0.09488584310849818, 0.10251192436692975, 0.11013800562536133, 0.1177640868837929, 0.12539016814222448, 0.13301624940065604, 0.1406423306590876, 0.14716214895951318, 0.15368196725993877, 0.16020178556036435, 0.16672160386078994, 0.17324142216121552, 0.1797612404616411, 0.1860718746144676, 0.19238250876729407, 0.19869314292012055, 0.20329459879738104, 0.20789605467464153, 0.21249751055190202, 0.21709896642916252, 0.221700422306423, 0.23005650953777015, 0.2347046463870348, 0.23935278323629947, 0.24400092008556412, 0.24864905693482878, 0.25329719378409343, 0.2579453306333581, 0.2633013224449591, 0.26865731425656003, 0.274013306068161, 0.27936929787976195, 0.2847252896913629, 0.29008128150296386, 0.2951486041294846, 0.3002159267560054, 0.30528324938252616, 0.3103505720090469, 0.3154178946355677, 0.32048521726208845, 0.3315239802252866, 0.3390229790324625, 0.34652197783963834, 0.3540209766468142, 0.36151997545399006, 0.3690189742611659, 0.3782565154274503, 0.3874940565937347, 0.3967315977600191, 0.4059691389263035, 0.4152066800925879, 0.42444422125887227, 0.4335624576196947, 0.4426806939805171, 0.45179893034133956, 0.460917166702162, 0.4700354030629844, 0.47915363942380684, 0.48944391840473817, 0.4997341973856695, 0.5100244763666009, 0.5203147553475322, 0.5306050343284636, 0.540895313309395, 0.5544614368276244, 0.5680275603458538, 0.5815936838640832, 0.5951598073823126, 0.608725930900542, 0.6222920544187713, 0.6424248963839891, 0.662557738349207, 0.6826905803144248, 0.7028234222796426, 0.7229562642448604, 0.7430891062100782, 0.7742506683488408, 0.8054122304876035, 0.8365737926263661, 0.8677353547651288, 0.8988969169038914, 0.930058479042654, 0.968513924868307, 1.00696937069396, 1.045424816519613, 1.083880262345266, 1.1223357081709189, 1.1607911539965718, 1.211224456705214, 1.261657759413856, 1.3120910621224982, 1.3625243648311403, 1.4129576675397824, 1.4633909702484245, 1.5331934928182145, 1.6029960153880045, 1.6727985379577945, 1.7426010605275846, 1.8124035830973746, 1.8822061056671646, 1.9634152837324217, 2.044624461797679, 2.125833639862936, 2.207042817928193, 2.28825199599345, 2.3694611740587073, 2.495203621106951, 2.6209460681551944, 2.746688515203438, 2.8724309622516815, 2.998173409299925, 3.2213240500554083, 3.4444746908108916, 3.667625331566375, 3.8907759723218582, 6.122282379876691, 8.353788787431524, 10.0]</t>
+          <t>[0.0, 5.942584500521307e-07, 1.1885169001042613e-06, 7.131101400625569e-06, 1.3073685901146876e-05, 3.0862131429607124e-05, 4.865057695806737e-05, 6.643902248652762e-05, 0.00011041193110178897, 0.00015438483971705032, 0.00019835774833231167, 0.0004136311961961234, 0.0006289046440599352, 0.0008441780919237469, 0.0016893399649361525, 0.002534501837948558, 0.0033796637109609635, 0.004412418706631742, 0.005445173702302521, 0.0064779286979733, 0.007510683693644079, 0.009534454051360827, 0.011558224409077575, 0.013581994766794322, 0.01560576512451107, 0.01762953548222782, 0.023132503167290253, 0.028635470852352688, 0.03413843853741512, 0.039641406222477554, 0.04514437390753999, 0.0531960844750011, 0.06124779504246221, 0.06929950560992332, 0.07735121617738443, 0.08540292674484554, 0.09345463731230665, 0.10140971522498142, 0.1093647931376562, 0.11731987105033097, 0.12371573602468237, 0.1301116009990338, 0.1365074659733852, 0.1429033309477366, 0.149299195922088, 0.15591434222501913, 0.16252948852795024, 0.16914463483088135, 0.17575978113381246, 0.18237492743674358, 0.1889900737396747, 0.19499570091993967, 0.20100132810020466, 0.20700695528046964, 0.21301258246073462, 0.2190182096409996, 0.225046991303107, 0.23107577296521442, 0.23710455462732183, 0.24313333628942924, 0.24916211795153664, 0.25519089961364405, 0.2610522411338983, 0.26691358265415255, 0.2727749241744068, 0.27863626569466104, 0.2844976072149153, 0.29035894873516954, 0.2961561068891586, 0.3019532650431477, 0.30775042319713675, 0.3135475813511258, 0.3193447395051149, 0.32514189765910395, 0.3340253613742367, 0.3429088250893695, 0.35179228880450225, 0.360675752519635, 0.3695592162347678, 0.3793364766874348, 0.38911373714010183, 0.39889099759276886, 0.4086682580454359, 0.4184455184981029, 0.42822277895076993, 0.44005393805299925, 0.45188509715522857, 0.4637162562574579, 0.4755474153596872, 0.4873785744619165, 0.49920973356414583, 0.5155736498150107, 0.5319375660658756, 0.5483014823167405, 0.5646653985676053, 0.5810293148184702, 0.6048799020531079, 0.6287304892877457, 0.6525810765223834, 0.6764316637570211, 0.7002822509916589, 0.7348390193295004, 0.7693957876673418, 0.8039525560051833, 0.8385093243430248, 0.8730660926808663, 0.9100112574427247, 0.9469564222045831, 0.9839015869664415, 1.0208467517282998, 1.057791916490158, 1.1182089003772144, 1.178625884264271, 1.2390428681513275, 1.299459852038384, 1.3598768359254405, 1.420293819812497, 1.4869862016035653, 1.5536785833946336, 1.620370965185702, 1.6870633469767702, 1.7537557287678385, 1.854683567348713, 1.9556114059295875, 2.056539244510462, 2.1574670830913365, 2.258394921672211, 2.3593227602530855, 2.487917340524319, 2.6165119207955523, 2.7451065010667857, 2.873701081338019, 3.0022956616092524, 3.130890241880486, 3.278405445644533, 3.4259206494085803, 3.5734358531726276, 3.720951056936675, 3.868466260700722, 4.015981464464769, 4.2508727051924, 4.485763945920031, 4.720655186647662, 4.9555464273752925, 5.190437668102923, 5.425328908830554, 5.708146038727102, 5.990963168623649, 6.2737802985201965, 6.556597428416744, 6.839414558313291, 7.122231688209839, 7.5087365395283, 7.895241390846762, 8.281746242165223, 8.668251093483684, 9.054755944802146, 9.441260796120607, 9.976455220977437, 10.0]</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>0.3003249533319581</v>
+        <v>0.6271392160900274</v>
       </c>
       <c r="D13" t="n">
         <v>9.81</v>
@@ -1304,13 +1304,13 @@
         <v>2</v>
       </c>
       <c r="L13" t="n">
-        <v>3.003249533319581</v>
+        <v>6.271392160900274</v>
       </c>
       <c r="M13" t="n">
-        <v>0.02217415909331765</v>
+        <v>0.005085130211165047</v>
       </c>
       <c r="N13" t="n">
-        <v>0.1108707954665882</v>
+        <v>0.02542565105582523</v>
       </c>
       <c r="O13" t="n">
         <v>19.61867428863441</v>
@@ -1340,11 +1340,11 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>[0.0, 5.942637672001492e-07, 1.1885275344002983e-06, 7.13116520640179e-06, 1.3073802878403282e-05, 3.086240792418739e-05, 4.8651012969971504e-05, 6.643961801575562e-05, 0.0001104129342403982, 0.0001543862504650408, 0.0001983595666896834, 0.00041364356260389543, 0.0006289275585181075, 0.0008442115544323195, 0.0016870370723733462, 0.002529862590314373, 0.0033726881082553994, 0.004405370362842437, 0.005438052617429474, 0.006470734872016512, 0.007503417126603549, 0.009530987624444263, 0.011558558122284977, 0.013586128620125692, 0.015613699117966406, 0.01764126961580712, 0.023194881299481933, 0.028748492983156744, 0.034302104666831555, 0.039855716350506366, 0.04540932803418118, 0.05365955443670569, 0.061909780839230204, 0.07016000724175472, 0.07841023364427924, 0.08666046004680375, 0.09491068644932826, 0.10253448934813511, 0.11015829224694196, 0.1177820951457488, 0.12540589804455565, 0.1330297009433625, 0.14065350384216935, 0.14717312284986728, 0.1536927418575652, 0.16021236086526314, 0.16673197987296107, 0.173251598880659, 0.17977121788835693, 0.18608589081678933, 0.19240056374522174, 0.19871523667365415, 0.20331319421483454, 0.20791115175601493, 0.21250910929719533, 0.21710706683837572, 0.2217050243795561, 0.23019896200316026, 0.23485365768479918, 0.2395083533664381, 0.24416304904807704, 0.24881774472971596, 0.25347244041135486, 0.25812713609299376, 0.2629871858862958, 0.2678472356795979, 0.27270728547289996, 0.27756733526620203, 0.2824273850595041, 0.28728743485280617, 0.2923026098027831, 0.29731778475276005, 0.302332959702737, 0.30734813465271393, 0.3123633096026909, 0.3173784845526678, 0.3261638814753926, 0.3349492783981174, 0.3416850303714577, 0.348420782344798, 0.3551565343181383, 0.3618922862914786, 0.36862803826481894, 0.3797628526110417, 0.38838235000567717, 0.39700184740031264, 0.4056213447949481, 0.41424084218958357, 0.42286033958421904, 0.4314798369788545, 0.4398762272369323, 0.44827261749501013, 0.45666900775308794, 0.46506539801116575, 0.47346178826924357, 0.4818581785273214, 0.4923278297628614, 0.5027974809984014, 0.5132671322339414, 0.5237367834694814, 0.5342064347050214, 0.5446760859405614, 0.5593467072088821, 0.5740173284772029, 0.5886879497455236, 0.6033585710138444, 0.6180291922821651, 0.6326998135504859, 0.6546560693389385, 0.6766123251273911, 0.6985685809158437, 0.7205248367042963, 0.742481092492749, 0.7644373482812016, 0.7956518690564259, 0.8268663898316503, 0.8580809106068746, 0.889295431382099, 0.9205099521573233, 0.9517244729325477, 0.9896904388984132, 1.027656404864279, 1.0656223708301447, 1.1035883367960104, 1.1415543027618762, 1.1836404724461844, 1.2257266421304926, 1.2678128118148009, 1.309898981499109, 1.3519851511834173, 1.4037434870999574, 1.4555018230164976, 1.5072601589330377, 1.5590184948495778, 1.6107768307661179, 1.662535166682658, 1.7477738237738085, 1.833012480864959, 1.9182511379561096, 2.00348979504726, 2.088728452138411, 2.1739671092295616, 2.2764794987281434, 2.378991888226725, 2.481504277725307, 2.5840166672238887, 2.6865290567224704, 2.789041446221052, 2.9558997451930766, 3.122758044165101, 3.2896163431371255, 3.45647464210915, 3.6233329410811743, 3.7901912400531987, 4.088573720169514, 4.3869562002858284, 4.685338680402143, 4.983721160518458, 5.282103640634773, 6.1229355981910265, 6.96376755574728, 7.8045995133035335, 8.645431470859787, 10.0]</t>
+          <t>[0.0, 5.942637672001492e-07, 1.1885275344002983e-06, 7.13116520640179e-06, 1.3073802878403282e-05, 3.0862407921206894e-05, 4.8651012964010506e-05, 6.643961800681412e-05, 0.00011041293369780844, 0.00015438624938880275, 0.00019835956507979706, 0.0004136425366476901, 0.0006289255082155831, 0.0008442084797834761, 0.0016878683318436263, 0.0025315281839037767, 0.003375188035963927, 0.004407540361768098, 0.005439892687572268, 0.006472245013376439, 0.007504597339180609, 0.009529690768076185, 0.01155478419697176, 0.013579877625867336, 0.015604971054762912, 0.01763006448365849, 0.023132828214330013, 0.028635591945001537, 0.03413835567567306, 0.039641119406344585, 0.04514388313701611, 0.053199265215676264, 0.06125464729433642, 0.06931002937299657, 0.07736541145165673, 0.0854207935303169, 0.09347617560897706, 0.10142274936026323, 0.1093693231115494, 0.11731589686283557, 0.12370886163024221, 0.13010182639764883, 0.13649479116505547, 0.1428877559324621, 0.14928072069986875, 0.15589494811598378, 0.16250917553209882, 0.16912340294821385, 0.17573763036432888, 0.1823518577804439, 0.18896608519655894, 0.1949675157651727, 0.20096894633378648, 0.20697037690240025, 0.21297180747101402, 0.2189732380396278, 0.22499478456551097, 0.23101633109139416, 0.23703787761727735, 0.24305942414316054, 0.24908097066904372, 0.25510251719492694, 0.2609651675705683, 0.2668278179462097, 0.27269046832185106, 0.27855311869749244, 0.2844157690731338, 0.2902784194487752, 0.29607432413021534, 0.3018702288116555, 0.30766613349309563, 0.3134620381745358, 0.3192579428559759, 0.32505384753741606, 0.3339327320761989, 0.3428116166149817, 0.35169050115376455, 0.3605693856925474, 0.3694482702313302, 0.3792256136652968, 0.38900295709926336, 0.39878030053322994, 0.4085576439671965, 0.4183349874011631, 0.4281123308351297, 0.43994044554357453, 0.4517685602520194, 0.46359667496046425, 0.4754247896689091, 0.48725290437735397, 0.4990810190857988, 0.5154436668739836, 0.5318063146621683, 0.5481689624503531, 0.5645316102385378, 0.5808942580267226, 0.60474127514624, 0.6285882922657574, 0.6524353093852748, 0.6762823265047923, 0.7001293436243097, 0.7346796233948168, 0.769229903165324, 0.8037801829358312, 0.8383304627063384, 0.8728807424768456, 0.9098183832391178, 0.94675602400139, 0.9836936647636623, 1.0206313055259346, 1.057568946288207, 1.1179745396382668, 1.1783801329883266, 1.2387857263383864, 1.2991913196884461, 1.359596913038506, 1.4200025063885657, 1.4866815382040937, 1.5533605700196216, 1.6200396018351495, 1.6867186336506774, 1.7533976654662053, 1.854305533822971, 1.9552134021797367, 2.0561212705365026, 2.1570291388932685, 2.2579370072500344, 2.3588448756068003, 2.4874141169728627, 2.615983358338925, 2.7445525997049875, 2.87312184107105, 3.0016910824371124, 3.1302603238031748, 3.2777467240404827, 3.4252331242777907, 3.5727195245150987, 3.7202059247524066, 3.8676923249897146, 4.015178725227022, 4.250024016113912, 4.484869307000801, 4.719714597887691, 4.954559888774581, 5.18940517966147, 5.42425047054836, 5.70701345324849, 5.98977643594862, 6.27253941864875, 6.5553024013488805, 6.838065384049011, 7.120828366749141, 7.50725945336041, 7.893690539971679, 8.280121626582948, 8.666552713194218, 9.052983799805487, 9.439414886416756, 9.974502396105677, 10.0]</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>0.3003154763950147</v>
+        <v>0.6267714562091956</v>
       </c>
       <c r="D14" t="n">
         <v>9.81</v>
@@ -1371,13 +1371,13 @@
         <v>2</v>
       </c>
       <c r="L14" t="n">
-        <v>3.003154763950147</v>
+        <v>6.267714562091956</v>
       </c>
       <c r="M14" t="n">
-        <v>0.02217555859777027</v>
+        <v>0.005091099390224257</v>
       </c>
       <c r="N14" t="n">
-        <v>0.1108777929888513</v>
+        <v>0.02545549695112129</v>
       </c>
       <c r="O14" t="n">
         <v>19.61832316706319</v>
@@ -1407,11 +1407,11 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>[0.0, 5.942704928244625e-07, 1.188540985648925e-06, 7.13124591389355e-06, 1.3073950842138175e-05, 3.0862757656532745e-05, 4.8651564470927315e-05, 6.644037128532189e-05, 0.00011041420241744758, 0.00015438803354957326, 0.00019836186468169894, 0.0004136579088727343, 0.0006289539530637696, 0.000844249997254805, 0.0016851984161146381, 0.0025261468349744715, 0.0033670952538343048, 0.004399276234603275, 0.005431457215372245, 0.006463638196141215, 0.007495819176910185, 0.009525076823460675, 0.011554334470011165, 0.013583592116561655, 0.015612849763112144, 0.017642107409662634, 0.023195515270178393, 0.028748923130694153, 0.03430233099120991, 0.03985573885172567, 0.04540914671224143, 0.053664753865003786, 0.06192036101776614, 0.0701759681705285, 0.07843157532329086, 0.08668718247605321, 0.09494278962881557, 0.10256372186501311, 0.11018465410121066, 0.1178055863374082, 0.12542651857360576, 0.13304745080980332, 0.14066838304600088, 0.14718701327374292, 0.15370564350148497, 0.160224273729227, 0.16674290395696906, 0.1732615341847111, 0.17978016441245315, 0.18609972515411244, 0.19241928589577173, 0.19873884663743102, 0.20333226673031551, 0.2079256868232, 0.2125191069160845, 0.217112527008969, 0.22170594710185348, 0.2304653917595096, 0.23513418931818464, 0.23980298687685966, 0.2444717844355347, 0.24914058199420971, 0.25380937955288474, 0.25847817711155974, 0.2638124064546601, 0.26914663579776044, 0.2744808651408608, 0.27981509448396114, 0.2851493238270615, 0.29048355317016183, 0.29551710094358785, 0.30055064871701387, 0.3055841964904399, 0.3106177442638659, 0.3156512920372919, 0.32068483981071794, 0.33075042789579945, 0.33819260736145035, 0.34563478682710125, 0.35307696629275215, 0.36051914575840305, 0.36796132522405395, 0.3764456043962684, 0.38492988356848284, 0.3934141627406973, 0.40189844191291174, 0.4103827210851262, 0.41886700025734064, 0.42808296993072736, 0.4372989396041141, 0.4465149092775008, 0.45573087895088754, 0.46494684862427427, 0.474162818297661, 0.48447142570992363, 0.49478003312218627, 0.5050886405344489, 0.5153972479467115, 0.5257058553589741, 0.5360144627712367, 0.5492340386929202, 0.5624536146146037, 0.5756731905362873, 0.5888927664579708, 0.6021123423796544, 0.6153319183013379, 0.6345692180181485, 0.653806517734959, 0.6730438174517696, 0.6922811171685801, 0.7115184168853906, 0.7307557166022012, 0.760710657124212, 0.7906655976462229, 0.8206205381682338, 0.8505754786902446, 0.8805304192122555, 0.9104853597342664, 0.9484372662545036, 0.9863891727747409, 1.0243410792949783, 1.0622929858152157, 1.100244892335453, 1.1381967988556905, 1.1875193695538373, 1.2368419402519841, 1.286164510950131, 1.3354870816482778, 1.3848096523464246, 1.4341322230445714, 1.5019977898641617, 1.5698633566837519, 1.637728923503342, 1.7055944903229323, 1.7734600571425225, 1.8413256239621127, 1.9201339646460258, 1.9989423053299389, 2.077750646013852, 2.1565589866977657, 2.235367327381679, 2.3141756680655927, 2.4337877405036163, 2.55339981294164, 2.6730118853796636, 2.7926239578176872, 2.912236030255711, 3.1133796704460797, 3.3145233106364484, 3.5156669508268172, 3.716810591017186, 4.469231874600465, 5.221653158183743, 5.974074441767022, 10.0]</t>
+          <t>[0.0, 5.942704928244625e-07, 1.188540985648925e-06, 7.13124591389355e-06, 1.3073950842138175e-05, 3.086275765355432e-05, 4.8651564464970464e-05, 6.644037127638661e-05, 0.00011041420187492108, 0.00015438803247345555, 0.00019836186307199002, 0.0004136568827420112, 0.0006289519024120324, 0.0008442469220820535, 0.0016860222493675007, 0.002527797576652948, 0.0033695729039383954, 0.004401421274911052, 0.005433269645883709, 0.006465118016856365, 0.007496966387829021, 0.009523739764058322, 0.011550513140287622, 0.013577286516516922, 0.015604059892746222, 0.01763083326897552, 0.023133389819421406, 0.028635946369867292, 0.034138502920313174, 0.039641059470759056, 0.04514361602120494, 0.05320368912892416, 0.061263762236643385, 0.06932383534436261, 0.07738390845208183, 0.08544398155980105, 0.09350405466752028, 0.10143990125220309, 0.1093757478368859, 0.11731159442156872, 0.12370070493308874, 0.13008981544460876, 0.1364789259561288, 0.1428680364676488, 0.14925714697916884, 0.15587231495463738, 0.16248748293010593, 0.16910265090557447, 0.17571781888104301, 0.18233298685651156, 0.1889481548319801, 0.19494429893557205, 0.200940443039164, 0.20693658714275595, 0.2129327312463479, 0.21892887534993985, 0.2249367777121689, 0.23094468007439797, 0.23695258243662704, 0.2429604847988561, 0.24896838716108516, 0.2549762895233142, 0.26084277524226673, 0.2667092609612193, 0.2725757466801718, 0.27844223239912436, 0.2843087181180769, 0.29017520383702944, 0.29596969203881757, 0.3017641802406057, 0.3075586684423938, 0.31335315664418195, 0.3191476448459701, 0.3249421330477582, 0.33381667753552124, 0.3426912220232843, 0.3515657665110473, 0.36044031099881035, 0.3693148554865734, 0.37908974477723045, 0.3888646340678875, 0.3986395233585446, 0.40841441264920164, 0.4181893019398587, 0.42796419123051577, 0.4397896889607187, 0.4516151866909216, 0.4634406844211245, 0.47526618215132743, 0.48709167988153035, 0.49891717761173326, 0.5152763295218917, 0.5316354814320502, 0.5479946333422087, 0.5643537852523671, 0.5807129371625256, 0.6045531507445571, 0.6283933643265885, 0.65223357790862, 0.6760737914906515, 0.699914005072683, 0.734454216974251, 0.7689944288758189, 0.8035346407773869, 0.8380748526789549, 0.8726150645805228, 0.9095418439591773, 0.9464686233378317, 0.9833954027164861, 1.0203221820951405, 1.0572489614737948, 1.1176364666980176, 1.1780239719222405, 1.2384114771464634, 1.2987989823706863, 1.3591864875949091, 1.419573992819132, 1.486233071709133, 1.552892150599134, 1.619551229489135, 1.686210308379136, 1.752869387269137, 1.8537476647795348, 1.9546259422899326, 2.0555042198003304, 2.1563824973107284, 2.2572607748211264, 2.3581390523315244, 2.4866701899173056, 2.6152013275030868, 2.743732465088868, 2.872263602674649, 3.0007947402604302, 3.1293258778462114, 3.276769099916204, 3.4242123219861966, 3.5716555440561892, 3.719098766126182, 3.8665419881961745, 4.013985210266167, 4.248761538967815, 4.4835378676694635, 4.718314196371112, 4.95309052507276, 5.187866853774408, 5.422643182476056, 5.705324358169977, 5.988005533863898, 6.270686709557819, 6.55336788525174, 6.836049060945661, 7.118730236639582, 7.505049654876734, 7.891369073113886, 8.277688491351038, 8.66400790958819, 9.050327327825341, 9.436646746062493, 9.97157295669432, 10.0]</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>0.3003034906987335</v>
+        <v>0.6263078174142976</v>
       </c>
       <c r="D15" t="n">
         <v>9.81</v>
@@ -1438,13 +1438,13 @@
         <v>2</v>
       </c>
       <c r="L15" t="n">
-        <v>3.003034906987335</v>
+        <v>6.263078174142976</v>
       </c>
       <c r="M15" t="n">
-        <v>0.02217732877242716</v>
+        <v>0.005098639787460646</v>
       </c>
       <c r="N15" t="n">
-        <v>0.1108866438621358</v>
+        <v>0.02549319893730323</v>
       </c>
       <c r="O15" t="n">
         <v>19.61787904911208</v>
@@ -1474,11 +1474,11 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>[0.0, 5.942790000884973e-07, 1.1885580001769946e-06, 7.131348001061967e-06, 1.307413800194694e-05, 3.086320003412169e-05, 4.8652262066296447e-05, 6.64413240984712e-05, 0.00011041580653909673, 0.00015439028897972228, 0.00019836477142034782, 0.0004136760581315663, 0.0006289873448427849, 0.0008442986315540034, 0.0016828967384314767, 0.00252149484530895, 0.0033600929521864233, 0.004391648297714235, 0.005423203643242046, 0.006454758988769857, 0.0074863143342976685, 0.009517716380392217, 0.011549118426486765, 0.013580520472581313, 0.015611922518675861, 0.01764332456477041, 0.023196558278473202, 0.028749791992175994, 0.03430302570587879, 0.03985625941958158, 0.04540949313328438, 0.05367201133446495, 0.061934529535645516, 0.07019704773682608, 0.07845956593800665, 0.08672208413918722, 0.09498460234036779, 0.10260191443954286, 0.11021922653871793, 0.117836538637893, 0.12545385073706808, 0.13307116283624315, 0.14068847493541822, 0.14720627501057076, 0.1537240750857233, 0.16024187516087585, 0.1667596752360284, 0.17327747531118093, 0.17979527538633347, 0.1861211904082478, 0.1924471054301621, 0.19877302045207643, 0.20336080088729286, 0.2079485813225093, 0.21253636175772572, 0.21712414219294215, 0.2217119226281586, 0.22777074931366242, 0.23382957599916626, 0.2398884026846701, 0.24594722937017394, 0.2520060560556778, 0.2580648827411816, 0.26395777395552295, 0.2698506651698643, 0.2757435563842056, 0.28163644759854695, 0.2875293388128883, 0.2934222300272296, 0.2985837961230642, 0.30374536221889875, 0.3089069283147333, 0.3140684944105679, 0.31923006050640246, 0.324391626602237, 0.33236473460122096, 0.3403378426002049, 0.3456457579592725, 0.3509536733183401, 0.3562615886774077, 0.3615695040364753, 0.3668774193955429, 0.37310671220686886, 0.3793360050181948, 0.38556529782952076, 0.3917945906408467, 0.39802388345217266, 0.4042531762634986, 0.41367064789024205, 0.4230881195169855, 0.43250559114372894, 0.4419230627704724, 0.45134053439721583, 0.4607580060239593, 0.4691289371726949, 0.4774998683214305, 0.4858707994701661, 0.4942417306189017, 0.5026126617676373, 0.5109835929163729, 0.5218517738271735, 0.5327199547379742, 0.5435881356487748, 0.5544563165595755, 0.5653244974703762, 0.5785911024001027, 0.5918577073298292, 0.6051243122595558, 0.6183909171892823, 0.6316575221190088, 0.6500432388555225, 0.6684289555920362, 0.6868146723285499, 0.7052003890650635, 0.7235861058015772, 0.7531558179159155, 0.7827255300302537, 0.8122952421445919, 0.8418649542589302, 0.8714346663732684, 0.906728761112376, 0.9420228558514836, 0.9773169505905912, 1.0126110453296988, 1.0479051400688064, 1.090750129348274, 1.1335951186277415, 1.176440107907209, 1.2192850971866767, 1.2621300864661442, 1.3049750757456118, 1.3691734694091706, 1.4333718630727295, 1.4975702567362883, 1.5617686503998471, 1.625967044063406, 1.6901654377269648, 1.7684820108123562, 1.8467985838977476, 1.925115156983139, 2.0034317300685305, 2.0817483031539217, 2.160064876239313, 2.2680183494212964, 2.37597182260328, 2.4839252957852636, 2.591878768967247, 2.6998322421492307, 2.8077857153312142, 2.973641472067533, 3.1394972288038514, 3.30535298554017, 3.4712087422764886, 3.637064499012807, 4.103604610513339, 4.570144722013872, 5.036684833514404, 5.503224945014937, 7.375877072741212, 9.248529200467487, 10.0]</t>
+          <t>[0.0, 5.942790000884973e-07, 1.1885580001769946e-06, 7.131348001061967e-06, 1.307413800194694e-05, 3.086320003114589e-05, 4.865226206034484e-05, 6.644132408954379e-05, 0.00011041580599665126, 0.00015439028790375874, 0.00019836476981086623, 0.00041367503177989985, 0.0006289852937489335, 0.0008442955557179671, 0.0016837113435611798, 0.0025231271314043926, 0.0033625429192476056, 0.004393762313354324, 0.005424981707461043, 0.006456201101567761, 0.00748742049567448, 0.009516329112996047, 0.011545237730317615, 0.013574146347639184, 0.015603054964960752, 0.01763196358228232, 0.023134338328118714, 0.028636713073955107, 0.0341390878197915, 0.03964146256562789, 0.04514383731146428, 0.053209932612646935, 0.06127602791382959, 0.06934212321501225, 0.07740821851619491, 0.08547431381737756, 0.09354040911856022, 0.10146272959019667, 0.10938505006183312, 0.11730737053346957, 0.12369172190223544, 0.13007607327100132, 0.1364604246397672, 0.1428447760085331, 0.149229127377299, 0.1558443435276413, 0.1624595596779836, 0.1690747758283259, 0.1756899919786682, 0.1823052081290105, 0.1889204242793528, 0.19490961160169748, 0.20089879892404217, 0.20688798624638685, 0.21287717356873154, 0.21886636089107622, 0.22485937449550158, 0.23085238809992695, 0.2368454017043523, 0.24283841530877767, 0.24883142891320303, 0.25482444251762837, 0.2606944951557817, 0.266564547793935, 0.27243460043208834, 0.27830465307024166, 0.284174705708395, 0.2900447583465483, 0.2958373629578382, 0.3016299675691281, 0.30742257218041796, 0.31321517679170785, 0.31900778140299774, 0.3248003860142876, 0.33366913499398293, 0.34253788397367824, 0.35140663295337354, 0.36027538193306885, 0.36914413091276416, 0.37891749601027613, 0.3886908611077881, 0.3984642262053001, 0.40823759130281206, 0.41801095640032404, 0.427784321497836, 0.4396060167171285, 0.451427711936421, 0.4632494071557135, 0.475071102375006, 0.4868927975942985, 0.498714492813591, 0.5150705192047365, 0.531426545595882, 0.5477825719870275, 0.564138598378173, 0.5804946247693186, 0.604327776637123, 0.6281609285049274, 0.6519940803727319, 0.6758272322405363, 0.6996603841083407, 0.7341892562710167, 0.7687181284336927, 0.8032470005963687, 0.8377758727590446, 0.8723047449217206, 0.9092189142955618, 0.946133083669403, 0.9830472530432441, 1.0199614224170852, 1.0568755917909263, 1.1172427525417674, 1.1776099132926086, 1.2379770740434497, 1.2983442347942908, 1.358711395545132, 1.4190785562959731, 1.485714790112642, 1.5523510239293108, 1.6189872577459796, 1.6856234915626485, 1.7522597253793173, 1.8531040467379862, 1.9539483680966552, 2.054792689455324, 2.155637010813993, 2.256481332172662, 2.3573256535313307, 2.4858132811264073, 2.614300908721484, 2.7427885363165605, 2.871276163911637, 2.9997637915067137, 3.1282514191017903, 3.275645274254631, 3.4230391294074716, 3.570432984560312, 3.717826839713153, 3.8652206948659935, 4.012614550018834, 4.247312080940791, 4.482009611862748, 4.7167071427847045, 4.951404673706661, 5.186102204628618, 5.420799735550575, 5.703387755289615, 5.985975775028655, 6.2685637947676955, 6.551151814506736, 6.833739834245776, 7.116327853984816, 7.502520264982358, 7.8887126759799004, 8.274905086977443, 8.661097497974986, 9.047289908972528, 9.433482319970071, 9.968224735933836, 10.0]</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>0.3002883384633226</v>
+        <v>0.6257238035141243</v>
       </c>
       <c r="D16" t="n">
         <v>9.81</v>
@@ -1505,13 +1505,13 @@
         <v>2</v>
       </c>
       <c r="L16" t="n">
-        <v>3.002883384633226</v>
+        <v>6.257238035141242</v>
       </c>
       <c r="M16" t="n">
-        <v>0.02217956691851089</v>
+        <v>0.0051081617717145</v>
       </c>
       <c r="N16" t="n">
-        <v>0.1108978345925544</v>
+        <v>0.0255408088585725</v>
       </c>
       <c r="O16" t="n">
         <v>19.61731730420472</v>
@@ -1541,11 +1541,11 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>[0.0, 5.942897610626422e-07, 1.1885795221252844e-06, 7.131477132751707e-06, 1.307437474337813e-05, 3.0863759604614295e-05, 4.865314446585046e-05, 6.644252932708662e-05, 0.00011041783561880067, 0.0001543931419105147, 0.00019836844820222873, 0.00041369901960653613, 0.0006290295910108435, 0.0008443601624151508, 0.001680023016401738, 0.002515685870388325, 0.003351348724374912, 0.004382125923408578, 0.005412903122442243, 0.006443680321475909, 0.007474457520509574, 0.0095085886154742, 0.011542719710438826, 0.013576850805403452, 0.015610981900368078, 0.017645112995332703, 0.023198257492163327, 0.028751401988993952, 0.03430454648582458, 0.03985769098265521, 0.04541083547948584, 0.053682259298497514, 0.06195368311750919, 0.07022510693652087, 0.07849653075553255, 0.08676795457454423, 0.0950393783935559, 0.10265213094512965, 0.1102648834967034, 0.11787763604827714, 0.1254903885998509, 0.13310314115142466, 0.14071589370299842, 0.14723298937378373, 0.15375008504456905, 0.16026718071535437, 0.16678427638613968, 0.173301372056925, 0.17981846772771032, 0.1861525748955225, 0.1924866820633347, 0.19882078923114688, 0.2034015589775158, 0.20798232872388472, 0.21256309847025365, 0.21714386821662257, 0.2217246379629915, 0.22795621350187545, 0.2341877890407594, 0.23837971668567895, 0.2425716443305985, 0.24676357197551804, 0.2509554996204376, 0.2551474272653572, 0.2593393549102768, 0.2649115958064376, 0.27048383670259835, 0.2760560775987591, 0.28162831849491987, 0.28720055939108063, 0.2927728002872414, 0.2978490708467809, 0.30292534140632044, 0.30800161196585996, 0.3130778825253995, 0.318154153084939, 0.3232304236444785, 0.3305963225310651, 0.33796222141765164, 0.3453281203042382, 0.35269401919082477, 0.36005991807741133, 0.36763038670720477, 0.3752008553369982, 0.38277132396679164, 0.3903417925965851, 0.3979122612263785, 0.40548272985617195, 0.41379671266395457, 0.4221106954717372, 0.4304246782795198, 0.4387386610873024, 0.44705264389508503, 0.45536662670286765, 0.46420751340820826, 0.4730484001135489, 0.4818892868188895, 0.4907301735242301, 0.4995710602295707, 0.5084119469349113, 0.5193067331901202, 0.5302015194453291, 0.541096305700538, 0.5519910919557469, 0.5628858782109558, 0.5737806644661647, 0.5885820285996469, 0.6033833927331291, 0.6181847568666113, 0.6329861210000935, 0.6477874851335758, 0.662588849267058, 0.686811377771015, 0.711033906274972, 0.735256434778929, 0.759478963282886, 0.783701491786843, 0.8079240202908, 0.8438011769841993, 0.8796783336775986, 0.9155554903709979, 0.9514326470643972, 0.9873098037577965, 1.0231869604511958, 1.0659694450367627, 1.1087519296223296, 1.1515344142078965, 1.1943168987934634, 1.2370993833790302, 1.2798818679645971, 1.33737698963687, 1.3948721113091427, 1.4523672329814155, 1.5098623546536882, 1.567357476325961, 1.6248525979982338, 1.7012449146245292, 1.7776372312508246, 1.85402954787712, 1.9304218645034155, 2.0068141811297107, 2.083206497756006, 2.184547192017343, 2.2858878862786804, 2.3872285805400177, 2.488569274801355, 2.5899099690626923, 2.6912506633240296, 2.8461829235422544, 3.0011151837604793, 3.156047443978704, 3.310979704196929, 3.4659119644151537, 3.6208442246333785, 3.8892942248679936, 4.157744225102609, 4.426194225337223, 4.694644225571838, 4.9630942258064525, 5.780736332362926, 6.598378438919399, 7.416020545475872, 8.233662652032345, 10.0]</t>
+          <t>[0.0, 5.942897610626422e-07, 1.1885795221252844e-06, 7.131477132751707e-06, 1.307437474337813e-05, 3.086375960164175e-05, 4.865314445990537e-05, 6.644252931816899e-05, 0.00011041783507645372, 0.00015439314083473844, 0.00019836844659302318, 0.0004136979929749022, 0.0006290275393567812, 0.0008443570857386603, 0.0016808262056964437, 0.002517295325654227, 0.00335376444561201, 0.004384201543432314, 0.005414638641252618, 0.006445075739072922, 0.007475512836893227, 0.009507138838365046, 0.011538764839836865, 0.013570390841308684, 0.015602016842780503, 0.017633642844252322, 0.023135913411315677, 0.02863818397837903, 0.034140454545442386, 0.039642725112505744, 0.0451449956795691, 0.05321884731716068, 0.061292698954752256, 0.06936655059234384, 0.07744040222993542, 0.08551425386752701, 0.09358810550511859, 0.1014933887027156, 0.1093986719003126, 0.11730395509790961, 0.12368238286140135, 0.13006081062489308, 0.13643923838838481, 0.14281766615187655, 0.14919609391536828, 0.1558104708394862, 0.16242484776360414, 0.16903922468772206, 0.17565360161184, 0.18226797853595791, 0.18888235546007584, 0.19486239760366958, 0.20084243974726332, 0.20682248189085706, 0.2128025240344508, 0.21878256617804454, 0.22475873019264225, 0.23073489420723997, 0.2367110582218377, 0.2426872222364354, 0.24866338625103312, 0.25463955026563084, 0.26051305489897836, 0.2663865595323259, 0.2722600641656734, 0.2781335687990209, 0.2840070734323684, 0.28988057806571593, 0.295670750243918, 0.30146092242212, 0.30725109460032207, 0.3130412667785241, 0.31883143895672617, 0.3246216111349282, 0.3334827064947573, 0.3423438018545864, 0.3512048972144155, 0.3600659925742446, 0.3689270879340737, 0.37869973853009686, 0.38847238912612003, 0.3982450397221432, 0.40801769031816637, 0.41779034091418954, 0.4275629915102127, 0.43937948900266827, 0.4511959864951238, 0.4630124839875794, 0.47482898148003494, 0.4866454789724905, 0.49846197646494605, 0.514815042648103, 0.5311681088312599, 0.5475211750144168, 0.5638742411975737, 0.5802273073807306, 0.6040527180747886, 0.6278781287688465, 0.6517035394629045, 0.6755289501569625, 0.6993543608510204, 0.7338699732462007, 0.768385585641381, 0.8029011980365613, 0.8374168104317417, 0.871932422826922, 0.9088315217462293, 0.9457306206655366, 0.9826297195848439, 1.0195288185041513, 1.0564279174234588, 1.1167713166184596, 1.1771147158134605, 1.2374581150084614, 1.2978015142034622, 1.358144913398463, 1.418488312593464, 1.4850975114108327, 1.5517067102282014, 1.61831590904557, 1.6849251078629388, 1.7515343066803075, 1.85233835834095, 1.9531424100015926, 2.0539464616622354, 2.1547505133228784, 2.2555545649835214, 2.3563586166441643, 2.484794842238503, 2.6132310678328414, 2.74166729342718, 2.8701035190215185, 2.998539744615857, 3.1269759702101956, 3.2743114492597845, 3.4216469283093733, 3.568982407358962, 3.716317886408551, 3.86365336545814, 4.010988844507729, 4.245593236855971, 4.480197629204213, 4.714802021552455, 4.949406413900697, 5.1840108062489385, 5.41861519859718, 5.701093372679198, 5.983571546761215, 6.266049720843233, 6.54852789492525, 6.831006069007268, 7.113484243089285, 7.499527022211169, 7.8855698013330535, 8.271612580454939, 8.657655359576824, 9.043698138698709, 9.429740917820594, 9.964266511957172, 10.0]</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>0.3002690495012409</v>
+        <v>0.6249889514692164</v>
       </c>
       <c r="D17" t="n">
         <v>9.81</v>
@@ -1572,13 +1572,13 @@
         <v>2</v>
       </c>
       <c r="L17" t="n">
-        <v>3.002690495012409</v>
+        <v>6.249889514692164</v>
       </c>
       <c r="M17" t="n">
-        <v>0.02218241659327667</v>
+        <v>0.005120181023928462</v>
       </c>
       <c r="N17" t="n">
-        <v>0.1109120829663833</v>
+        <v>0.02560090511964231</v>
       </c>
       <c r="O17" t="n">
         <v>19.6166067782281</v>
@@ -1608,11 +1608,11 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>[0.0, 5.943033729638898e-07, 1.1886067459277797e-06, 7.131640475566679e-06, 1.3074674205205577e-05, 3.086446742329745e-05, 4.865426064138932e-05, 6.64440538594812e-05, 0.00011042040226775095, 0.0001543967506760207, 0.00019837309908429045, 0.00041372807101599585, 0.0006290830429477013, 0.0008444380148794067, 0.0016764467877421212, 0.0025084555606048357, 0.00334046433346755, 0.004370277898251714, 0.005400091463035878, 0.006429905027820042, 0.007459718592604206, 0.00949732836557628, 0.011534938138548355, 0.01357254791152043, 0.015610157684492504, 0.01764776745746458, 0.023201003260308325, 0.02875423906315207, 0.03430747486599582, 0.039860710668839575, 0.04541394647168333, 0.05369688499915789, 0.06197982352663245, 0.070262762054107, 0.07854570058158156, 0.08682863910905611, 0.09511157763653066, 0.10271859950940421, 0.11032562138227775, 0.11793264325515129, 0.12553966512802484, 0.13314668700089838, 0.14075370887377192, 0.14726951173634226, 0.1537853145989126, 0.16030111746148293, 0.16681692032405326, 0.1733327231866236, 0.17984852604919394, 0.1861929070790122, 0.19253728810883047, 0.19888166913864874, 0.2034535665787797, 0.20802546401891064, 0.2125973614590416, 0.21716925889917255, 0.2217411563393035, 0.22973501322417697, 0.23475155115412882, 0.23976808908408068, 0.24478462701403253, 0.24980116494398438, 0.25481770287393624, 0.25983424080388806, 0.2649308829512067, 0.27002752509852535, 0.275124167245844, 0.28022080939316263, 0.28531745154048127, 0.2904140936877999, 0.2960355798191351, 0.30165706595047026, 0.30727855208180543, 0.3129000382131406, 0.3185215243444758, 0.32414301047581096, 0.33316436536681404, 0.33955716523472684, 0.34594996510263964, 0.35234276497055245, 0.35873556483846525, 0.36512836470637805, 0.375078398673473, 0.3850284326405679, 0.39209330569787704, 0.39915817875518617, 0.4062230518124953, 0.4132879248698044, 0.42035279792711355, 0.4274176709844227, 0.4355370693162262, 0.44365646764802974, 0.45177586597983327, 0.4598952643116368, 0.4680146626434403, 0.47679277328521674, 0.48557088392699316, 0.4943489945687696, 0.5031271052105459, 0.5119052158523223, 0.524006185283668, 0.5361071547150138, 0.5482081241463596, 0.5603090935777053, 0.5724100630090511, 0.587378148264822, 0.602346233520593, 0.617314318776364, 0.632282404032135, 0.647250489287906, 0.6687791769707505, 0.6903078646535951, 0.7118365523364396, 0.7333652400192842, 0.7548939277021287, 0.783193275426358, 0.8114926231505872, 0.8397919708748165, 0.8680913185990458, 0.896390666323275, 0.932868978807631, 0.9693472912919869, 1.005825603776343, 1.0423039162606988, 1.0787822287450548, 1.12253467697415, 1.1662871252032452, 1.2100395734323404, 1.2537920216614356, 1.2975444698905307, 1.341296918119626, 1.4068196124647292, 1.4723423068098325, 1.5378650011549357, 1.603387695500039, 1.6689103898451423, 1.7344330841902456, 1.8148349765909821, 1.8952368689917187, 1.9756387613924553, 2.056040653793192, 2.1364425461939285, 2.216844438594665, 2.3282777737653073, 2.4397111089359496, 2.551144444106592, 2.662577779277234, 2.7740111144478763, 2.8854444496185185, 3.05743042159234, 3.229416393566161, 3.4014023655399823, 3.5733883375138036, 3.745374309487625, 4.2491368078062335, 4.752899306124842, 5.256661804443451, 5.760424302762059, 7.472300311910043, 9.184176321058027, 10.0]</t>
+          <t>[0.0, 5.943033729638898e-07, 1.1886067459277797e-06, 7.131640475566679e-06, 1.3074674205205577e-05, 3.0864467420329094e-05, 4.865426063545261e-05, 6.644405385057613e-05, 0.00011042040172553449, 0.00015439674960049285, 0.00019837309747545122, 0.0004137270440302829, 0.0006290809905851145, 0.0008444349371399462, 0.0016772359334238658, 0.0025100369297077854, 0.0033428379259917047, 0.004372306259310561, 0.005401774592629418, 0.006431242925948274, 0.00746071125926713, 0.00949580105364961, 0.011530890848032091, 0.013565980642414571, 0.015601070436797052, 0.017636160231179532, 0.02313849515644479, 0.028640830081710048, 0.034143165006975305, 0.03964549993224056, 0.04514783485750582, 0.053231711556639236, 0.06131558825577265, 0.06939946495490606, 0.07748334165403947, 0.08556721835317288, 0.09365109505230629, 0.10153495075319009, 0.1094188064540739, 0.1173026621549577, 0.12367351871623906, 0.13004437527752044, 0.13641523183880183, 0.14278608840008322, 0.1491569449613646, 0.15577150227758207, 0.16238605959379954, 0.169000616910017, 0.17561517422623446, 0.18222973154245192, 0.18884428885866938, 0.19481233052795274, 0.2007803721972361, 0.20674841386651946, 0.21271645553580282, 0.21868449720508618, 0.22463664602897887, 0.23058879485287156, 0.23654094367676426, 0.24249309250065695, 0.24844524132454965, 0.2543973901484423, 0.2602763565576615, 0.2661553229668807, 0.2720342893760999, 0.2779132557853191, 0.2837922221945383, 0.2896711886037575, 0.2954583765743828, 0.30124556454500806, 0.30703275251563333, 0.3128199404862586, 0.3186071284568839, 0.32439431642750916, 0.33324730174743783, 0.3421002870673665, 0.3509532723872952, 0.35980625770722385, 0.36865924302715253, 0.3784298034352914, 0.3882003638434303, 0.3979709242515692, 0.4077414846597081, 0.417512045067847, 0.4272826054759859, 0.4390934994539378, 0.45090439343188965, 0.4627152874098415, 0.4745261813877934, 0.4863370753657453, 0.49814796934369715, 0.5144966012837227, 0.5308452332237481, 0.5471938651637736, 0.563542497103799, 0.5798911290438244, 0.6037058823859182, 0.6275206357280119, 0.6513353890701056, 0.6751501424121993, 0.698964895754293, 0.7334632394873316, 0.7679615832203702, 0.8024599269534088, 0.8369582706864475, 0.8714566144194861, 0.9083364712379564, 0.9452163280564266, 0.9820961848748969, 1.0189760416933673, 1.0558558985118376, 1.1161679348525113, 1.176479971193185, 1.2367920075338588, 1.2971040438745325, 1.3574160802152062, 1.41772811655588, 1.4843024413747983, 1.5508767661937166, 1.617451091012635, 1.6840254158315533, 1.7505997406504716, 1.8513520241287775, 1.9521043076070834, 2.0528565910853893, 2.1536088745636954, 2.2543611580420015, 2.3551134415203077, 2.4834832503201905, 2.6118530591200733, 2.740222867919956, 2.868592676719839, 2.9969624855197217, 3.1253322943196045, 3.272592431175997, 3.4198525680323897, 3.5671127048887823, 3.714372841745175, 3.8616329786015675, 4.00889311545796, 4.243377262560738, 4.477861409663516, 4.712345556766294, 4.9468297038690725, 5.181313850971851, 5.415797998074629, 5.698134200499881, 5.980470402925134, 6.262806605350386, 6.545142807775639, 6.827479010200891, 7.109815212626144, 7.495664540739935, 7.881513868853727, 8.26736319696752, 8.653212525081312, 9.039061853195104, 9.424911181308897, 9.959156572618273, 10.0]</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>0.3002448264158245</v>
+        <v>0.624065547267972</v>
       </c>
       <c r="D18" t="n">
         <v>9.81</v>
@@ -1639,13 +1639,13 @@
         <v>2</v>
       </c>
       <c r="L18" t="n">
-        <v>3.002448264158244</v>
+        <v>6.24065547267972</v>
       </c>
       <c r="M18" t="n">
-        <v>0.02218599599381758</v>
+        <v>0.005135344477834043</v>
       </c>
       <c r="N18" t="n">
-        <v>0.1109299799690879</v>
+        <v>0.02567672238917022</v>
       </c>
       <c r="O18" t="n">
         <v>19.61570806573987</v>
@@ -1675,11 +1675,11 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>[0.0, 5.943205913713719e-07, 1.1886411827427437e-06, 7.131847096456462e-06, 1.307505301017018e-05, 3.086536278029582e-05, 4.8655672550421456e-05, 6.64459823205471e-05, 0.00011042364895812493, 0.00015440131559570276, 0.00019837898223328058, 0.0004137648303998568, 0.0006291506785664331, 0.0008445365267330093, 0.0016720142580838294, 0.002499491989434649, 0.003326969720785469, 0.004355596433944618, 0.005384223147103767, 0.0064128498602629164, 0.007441476573422066, 0.009483529557634509, 0.011525582541846952, 0.013567635526059395, 0.015609688510271839, 0.017651741494484282, 0.023205409762061174, 0.028759078029638067, 0.03431274629721496, 0.039866414564791855, 0.04542008283236875, 0.05371799149060475, 0.06201590014884075, 0.07031380880707674, 0.07861171746531273, 0.08690962612354872, 0.0952075347817847, 0.10280736720066495, 0.1104071996195452, 0.11800703203842546, 0.1256068644573057, 0.13320669687618597, 0.14080652929506624, 0.14732038131648928, 0.15383423333791232, 0.16034808535933537, 0.1668619373807584, 0.17337578940218146, 0.1798896414236045, 0.18624693615001253, 0.19260423087642056, 0.1989615256028286, 0.20352224285395315, 0.2080829601050777, 0.21264367735620227, 0.21720439460732682, 0.22176511185845138, 0.22792362936795305, 0.2340821468774547, 0.24024066438695638, 0.24639918189645804, 0.25255769940595973, 0.2587162169154614, 0.2647938880041683, 0.2708715590928752, 0.2769492301815821, 0.28302690127028896, 0.28910457235899584, 0.2951822434477027, 0.30035227063031744, 0.30552229781293216, 0.3106923249955469, 0.3158623521781616, 0.32103237936077633, 0.32620240654339105, 0.3336059289462049, 0.3410094513490187, 0.34841297375183256, 0.3558164961546464, 0.3632200185574602, 0.37016092480541213, 0.37710183105336403, 0.38404273730131594, 0.39098364354926785, 0.39792454979721975, 0.40486545604517166, 0.41483578302299995, 0.42480611000082824, 0.43477643697865653, 0.4447467639564848, 0.4547170909343131, 0.4646874179121414, 0.47505383162030085, 0.4854202453284603, 0.4957866590366197, 0.5061530727447792, 0.5165194864529385, 0.5268859001610979, 0.5396268100010959, 0.5523677198410939, 0.5651086296810919, 0.5778495395210899, 0.5905904493610878, 0.6033313592010858, 0.6219144344707666, 0.6404975097404473, 0.659080585010128, 0.6776636602798087, 0.6962467355494895, 0.723757528930985, 0.7512683223124805, 0.7787791156939761, 0.8062899090754716, 0.8338007024569671, 0.8677682671204971, 0.9017358317840272, 0.9357033964475572, 0.9696709611110872, 1.0036385257746172, 1.0440886506246743, 1.0845387754747313, 1.1249889003247884, 1.1654390251748454, 1.2058891500249025, 1.2463392748749595, 1.3085804315950176, 1.3708215883150756, 1.4330627450351336, 1.4953039017551917, 1.5575450584752497, 1.6197862151953077, 1.6933785915527373, 1.7669709679101668, 1.8405633442675964, 1.914155720625026, 1.9877480969824555, 2.061340473339885, 2.1610945508310455, 2.260848628322206, 2.3606027058133665, 2.460356783304527, 2.5601108607956875, 2.659864938286848, 2.8074061594552, 2.954947380623552, 3.102488601791904, 3.250029822960256, 3.397571044128608, 3.54511226529696, 3.7993021152559976, 4.053491965215035, 4.307681815174073, 4.56187166513311, 4.816061515092148, 5.678628006002765, 6.541194496913382, 7.403760987824, 8.266327478734617, 10.0]</t>
+          <t>[0.0, 5.943205913713719e-07, 1.1886411827427437e-06, 7.131847096456462e-06, 1.307505301017018e-05, 3.086536277733265e-05, 4.8655672544495126e-05, 6.64459823116576e-05, 0.0001104236484160707, 0.0001544013145204838, 0.0001983789806248969, 0.00041376380296641156, 0.0006291486253079263, 0.0008445334476494409, 0.0016727862461141762, 0.0025010390445789118, 0.0033292918430436473, 0.004357567017007446, 0.005385842190971246, 0.006414117364935045, 0.007442392538898845, 0.009481906498921418, 0.011521420458943991, 0.013560934418966565, 0.015600448378989138, 0.01763996233901171, 0.02314268309575527, 0.02864540385249883, 0.03414812460924239, 0.03965084536598595, 0.045153566122729506, 0.05325046906998747, 0.06134737201724543, 0.0694442749645034, 0.07754117791176135, 0.0856380808590193, 0.09373498380627726, 0.10159193949611176, 0.10944889518594625, 0.11730585087578074, 0.12366709754832321, 0.13002834422086568, 0.13638959089340813, 0.14275083756595058, 0.14911208423849304, 0.15572793181870376, 0.16234377939891448, 0.1689596269791252, 0.17557547455933592, 0.18219132213954664, 0.18880716971975736, 0.19475924664895256, 0.20071132357814775, 0.20666340050734294, 0.21261547743653814, 0.21856755436573333, 0.22448701470639007, 0.2304064750470468, 0.23632593538770355, 0.2422453957283603, 0.24816485606901703, 0.25408431640967377, 0.25997092868778837, 0.26585754096590297, 0.27174415324401757, 0.2776307655221322, 0.2835173778002468, 0.2894039900783614, 0.29518746442138577, 0.30097093876441017, 0.30675441310743456, 0.31253788745045896, 0.31832136179348336, 0.32410483613650776, 0.33294951268190254, 0.3417941892272973, 0.3506388657726921, 0.3594835423180869, 0.36832821886348166, 0.3780954425411234, 0.3878626662187652, 0.39762988989640696, 0.40739711357404873, 0.4171643372516905, 0.42693156092933227, 0.43873637956290346, 0.45054119819647465, 0.46234601683004584, 0.474150835463617, 0.4859556540971882, 0.4977604727307594, 0.5141032945680182, 0.530446116405277, 0.5467889382425357, 0.5631317600797945, 0.5794745819170533, 0.6032755617153271, 0.627076541513601, 0.6508775213118749, 0.6746785011101488, 0.6984794809084227, 0.7329560937017023, 0.767432706494982, 0.8019093192882616, 0.8363859320815412, 0.8708625448748208, 0.9077184483740621, 0.9445743518733034, 0.9814302553725447, 1.018286158871786, 1.0551420623710273, 1.115414087363703, 1.1756861123563789, 1.2359581373490547, 1.2962301623417305, 1.3565021873344063, 1.4167742123270821, 1.4833048465884149, 1.5498354808497476, 1.6163661151110804, 1.6828967493724132, 1.749427383633746, 1.8501149979109093, 1.9508026121880726, 2.051490226465236, 2.1521778407423997, 2.2528654550195633, 2.353553069296727, 2.4818396002651917, 2.6101261312336566, 2.7384126622021214, 2.8666991931705863, 2.994985724139051, 3.123272255107516, 3.270437983574877, 3.417603712042238, 3.5647694405095987, 3.7119351689769595, 3.8591008974443204, 4.006266625911682, 4.2406000870881115, 4.474933548264541, 4.709267009440971, 4.943600470617401, 5.177933931793831, 5.412267392970261, 5.694425739755077, 5.9765840865398925, 6.258742433324708, 6.540900780109524, 6.82305912689434, 7.105217473679156, 7.490824396055646, 7.876431318432136, 8.262038240808625, 8.647645163185114, 9.033252085561603, 9.418859007938092, 9.95275332075595, 10.0]</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>0.3002141969250957</v>
+        <v>0.622907163309016</v>
       </c>
       <c r="D19" t="n">
         <v>9.81</v>
@@ -1706,13 +1706,13 @@
         <v>2</v>
       </c>
       <c r="L19" t="n">
-        <v>3.002141969250956</v>
+        <v>6.229071633090159</v>
       </c>
       <c r="M19" t="n">
-        <v>0.0221905232975297</v>
+        <v>0.005154462035770834</v>
       </c>
       <c r="N19" t="n">
-        <v>0.1109526164876485</v>
+        <v>0.02577231017885417</v>
       </c>
       <c r="O19" t="n">
         <v>19.61457132456068</v>
@@ -1742,11 +1742,11 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>[0.0, 5.943423722811132e-07, 1.1886847445622265e-06, 7.132108467373359e-06, 1.3075532190184492e-05, 3.086649538742376e-05, 4.865745858466303e-05, 6.64484217819023e-05, 0.00011042775595309682, 0.00015440709012429134, 0.00019838642429548587, 0.0004138113474062103, 0.0006292362705169347, 0.0008446611936276592, 0.001666547585162013, 0.002488433976696367, 0.003310320368230721, 0.00433749523411577, 0.00536467010000082, 0.00639184496588587, 0.00741901983177092, 0.009466762532450546, 0.011514505233130171, 0.013562247933809796, 0.015609990634489422, 0.017657733335169047, 0.023212437802248253, 0.02876714226932746, 0.03432184673640666, 0.03987655120348586, 0.045431255670565066, 0.05374876900563992, 0.062066282340714776, 0.07038379567578963, 0.07870130901086449, 0.08701882234593934, 0.0953363356810142, 0.10292716699426416, 0.11051799830751412, 0.11810882962076408, 0.12569966093401402, 0.13329049224726397, 0.14088132356051392, 0.14739353369190353, 0.15390574382329314, 0.16041795395468275, 0.16693016408607236, 0.17344237421746198, 0.1799545843488516, 0.18632838482887742, 0.19270218530890326, 0.1990759857889291, 0.2036230358141515, 0.2081700858393739, 0.2127171358645963, 0.21726418588981872, 0.22181123591504112, 0.23026816130081945, 0.23487847390680427, 0.2394887865127891, 0.24409909911877392, 0.24870941172475874, 0.25331972433074357, 0.2579300369367284, 0.2627891469835743, 0.2676482570304202, 0.27250736707726614, 0.27736647712411205, 0.28222558717095797, 0.2870846972178039, 0.29209770034316296, 0.29711070346852203, 0.3021237065938811, 0.3071367097192402, 0.31214971284459925, 0.3171627159699583, 0.32711745633103, 0.3349467503834356, 0.34277604443584114, 0.3506053384882467, 0.35632991576058876, 0.3620544930329308, 0.36777907030527285, 0.3735036475776149, 0.37922822484995694, 0.3864456268330452, 0.3936630288161334, 0.40088043079922164, 0.4080978327823099, 0.4153152347653981, 0.42253263674848635, 0.43207348466491163, 0.4416143325813369, 0.4511551804977622, 0.4606960284141875, 0.4702368763306128, 0.4797777242470381, 0.4906806899201074, 0.5015836555931767, 0.5124866212662461, 0.5233895869393155, 0.5342925526123848, 0.5451955182854542, 0.559264600677816, 0.5733336830701778, 0.5874027654625397, 0.6014718478549015, 0.6155409302472633, 0.6296100126396251, 0.6503613302455399, 0.6711126478514546, 0.6918639654573694, 0.7126152830632841, 0.7333666006691989, 0.7629720324642654, 0.7925774642593318, 0.8221828960543983, 0.8517883278494648, 0.8813937596445313, 0.9136878994636148, 0.9459820392826984, 0.978276179101782, 1.0105703189208657, 1.0428644587399494, 1.082317222558793, 1.1217699863776365, 1.16122275019648, 1.2006755140153236, 1.2401282778341671, 1.2795810416530107, 1.3419588947825298, 1.404336747912049, 1.4667146010415681, 1.5290924541710873, 1.5914703073006065, 1.6538481604301256, 1.7227743825661614, 1.7917006047021973, 1.860626826838233, 1.929553048974269, 1.9984792711103048, 2.0674054932463406, 2.1571350814151136, 2.2468646695838865, 2.3365942577526595, 2.4263238459214325, 2.5160534340902054, 2.6057830222589784, 2.748796661588486, 2.891810300917993, 3.0348239402475006, 3.177837579577008, 3.3208512189065154, 3.5944919748388298, 3.868132730771144, 4.141773486703459, 4.415414242635773, 5.654727081315668, 6.8940399199955635, 8.133352758675459, 10.0]</t>
+          <t>[0.0, 5.943423722811132e-07, 1.1886847445622265e-06, 7.132108467373359e-06, 1.3075532190184492e-05, 3.086649538446723e-05, 4.865745857874997e-05, 6.644842177303272e-05, 0.00011042775541124608, 0.00015440708904945944, 0.0001983864226876728, 0.00041381031940627505, 0.0006292342161248773, 0.0008446581128434797, 0.001667298787345858, 0.0024899394618482363, 0.0033125801363506147, 0.004339395758452765, 0.005366211380554916, 0.006393027002657066, 0.007419842624759217, 0.009465021842616845, 0.011510201060474474, 0.013555380278332103, 0.015600559496189732, 0.01764573871404736, 0.023149417003231067, 0.028653095292414773, 0.03415677358159848, 0.03966045187078218, 0.045164130159965885, 0.053278075888028, 0.061392021616090114, 0.06950596734415224, 0.07761991307221436, 0.08573385880027648, 0.0938478045283386, 0.10167107046694498, 0.10949433640555137, 0.11731760234415775, 0.12514086828276413, 0.13136124524178824, 0.13758162220081235, 0.14380199915983646, 0.15002237611886057, 0.15624275307788468, 0.1629813251997675, 0.1697198973216503, 0.1764584694435331, 0.1831970415654159, 0.18993561368729872, 0.19667418580918153, 0.2020389604691196, 0.20740373512905766, 0.21276850978899572, 0.2181332844489338, 0.22349805910887185, 0.22886283376880992, 0.23411615535704372, 0.23936947694527752, 0.24462279853351132, 0.24987612012174512, 0.2551294417099789, 0.26038276329821275, 0.266730558117281, 0.2730783529363493, 0.2794261477554176, 0.28577394257448585, 0.2921217373935541, 0.2984695322126224, 0.30379863606192675, 0.3091277399112311, 0.31445684376053545, 0.3197859476098398, 0.32511505145914416, 0.3304441553084485, 0.33863981792315984, 0.34683548053787117, 0.3550311431525825, 0.3632268057672938, 0.37142246838200516, 0.3796181309967165, 0.38771978809467833, 0.3958214451926402, 0.403923102290602, 0.41202475938856387, 0.4201264164865257, 0.42822807358448756, 0.4377467616411536, 0.4472654496978197, 0.45678413775448573, 0.4663028258111518, 0.47582151386781785, 0.4853402019244839, 0.500149931814611, 0.5149596617047381, 0.5297693915948651, 0.5445791214849922, 0.5593888513751193, 0.5845205851024482, 0.6096523188297771, 0.634784052557106, 0.6599157862844349, 0.6850475200117638, 0.7154623693155998, 0.7458772186194358, 0.7762920679232718, 0.8067069172271077, 0.8371217665309437, 0.879748944489607, 0.9223761224482704, 0.9650033004069337, 1.0076304783655972, 1.0502576563242605, 1.0928848342829238, 1.1404806383342019, 1.18807644238548, 1.235672246436758, 1.283268050488036, 1.330863854539314, 1.3784596585905922, 1.4580375869283202, 1.5376155152660482, 1.6171934436037763, 1.6967713719415043, 1.7763493002792323, 1.8559272286169604, 1.9456666164153504, 2.0354060042137405, 2.1251453920121306, 2.2148847798105207, 2.3046241676089108, 2.394363555407301, 2.530145538446349, 2.665927521485397, 2.801709504524445, 2.937491487563493, 3.0732734706025413, 3.2090554536415894, 3.3887960341603542, 3.568536614679119, 3.748277195197884, 3.928017775716649, 4.107758356235413, 4.287498936754178, 4.497240812773783, 4.7069826887933885, 4.916724564812994, 5.1264664408325995, 5.336208316852205, 5.5459501928718105, 5.8530841854265585, 6.1602181779813066, 6.467352170536055, 6.774486163090803, 7.081620155645551, 7.388754148200299, 7.7961950667518565, 8.203635985303414, 8.611076903854972, 9.01851782240653, 9.425958740958087, 9.833399659509645, 10.0]</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>0.3001753405057772</v>
+        <v>0.6214570178944209</v>
       </c>
       <c r="D20" t="n">
         <v>9.81</v>
@@ -1773,13 +1773,13 @@
         <v>2</v>
       </c>
       <c r="L20" t="n">
-        <v>3.001753405057772</v>
+        <v>6.214570178944208</v>
       </c>
       <c r="M20" t="n">
-        <v>0.02219626860681205</v>
+        <v>0.005178545569311519</v>
       </c>
       <c r="N20" t="n">
-        <v>0.1109813430340602</v>
+        <v>0.0258927278465576</v>
       </c>
       <c r="O20" t="n">
         <v>19.61313351154996</v>
@@ -1809,11 +1809,11 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>[0.0, 5.943699253663023e-07, 1.1887398507326046e-06, 7.132439104395627e-06, 1.307613835805865e-05, 3.086792814772781e-05, 4.8659717937396974e-05, 6.645150772706614e-05, 0.00011043295134992061, 0.0001544143949727751, 0.0001983958385956296, 0.00041387021945097345, 0.0006293446003063172, 0.000844818981161661, 0.0016598461818584423, 0.0024748733825552234, 0.0032899005832520045, 0.00431531448695094, 0.0053407283906498765, 0.006366142294348813, 0.007391556198047749, 0.00944660842455517, 0.01150166065106259, 0.01355671287757001, 0.01561176510407743, 0.017666817330584852, 0.023223580232947773, 0.028780343135310693, 0.03433710603767361, 0.039893868940036534, 0.045450631842399454, 0.053793994675642914, 0.062137357508886375, 0.07048072034212984, 0.07882408317537329, 0.08716744600861674, 0.0955108088418602, 0.10309041988320718, 0.11067003092455416, 0.11824964196590114, 0.12582925300724812, 0.1334088640485951, 0.14098847508994206, 0.14749789000284957, 0.1540073049157571, 0.1605167198286646, 0.16702613474157213, 0.17353554965447965, 0.18004496456738717, 0.18643898800859468, 0.1928330114498022, 0.1992270348910097, 0.203756980412593, 0.20828692593417628, 0.21281687145575956, 0.21734681697734284, 0.22187676249892613, 0.22953828620895184, 0.23407590901711617, 0.2386135318252805, 0.24315115463344483, 0.24768877744160916, 0.2522264002497735, 0.25676402305793783, 0.26213631154915756, 0.2675086000403773, 0.27288088853159703, 0.27825317702281677, 0.2836254655140365, 0.28899775400525624, 0.29412823968261964, 0.29925872535998305, 0.30438921103734645, 0.30951969671470986, 0.31465018239207326, 0.31978066806943667, 0.3286996165516419, 0.3376185650338472, 0.34419857123750147, 0.35077857744115576, 0.35735858364481005, 0.36393858984846433, 0.3705185960521186, 0.37906849303369733, 0.38761839001527604, 0.39616828699685475, 0.40471818397843345, 0.41326808096001216, 0.42181797794159087, 0.4312893918621722, 0.4407608057827535, 0.4502322197033348, 0.45970363362391614, 0.46917504754449746, 0.4786464614650788, 0.4893962754048839, 0.500146089344689, 0.510895903284494, 0.521645717224299, 0.532395531164104, 0.543145345103909, 0.5572746869613969, 0.5714040288188849, 0.5855333706763728, 0.5996627125338607, 0.6137920543913487, 0.6346227218681556, 0.6554533893449626, 0.6762840568217695, 0.6971147242985765, 0.7179453917753834, 0.7470757539787904, 0.7762061161821975, 0.8053364783856045, 0.8344668405890115, 0.8635972027924186, 0.8954099480417002, 0.9272226932909817, 0.9590354385402633, 0.9908481837895449, 1.0226609290388264, 1.0611568244207605, 1.0996527198026946, 1.1381486151846287, 1.1766445105665628, 1.215140405948497, 1.253636301330431, 1.3168589149768999, 1.3800815286233687, 1.4433041422698376, 1.5065267559163065, 1.5697493695627753, 1.6329719832092442, 1.7000556232775084, 1.7671392633457725, 1.8342229034140367, 1.9013065434823009, 1.968390183550565, 2.0354738236188292, 2.1228101435749247, 2.21014646353102, 2.2974827834871157, 2.384819103443211, 2.4721554233993066, 2.559491743355402, 2.695784471952117, 2.832077200548832, 2.968369929145547, 3.1046626577422622, 3.2409553863389773, 3.4856415872451163, 3.7303277881512553, 3.9750139890573943, 4.219700189963533, 5.948021447917138, 7.676342705870742, 9.404663963824348, 10.0]</t>
+          <t>[0.0, 5.943699253663023e-07, 1.1887398507326046e-06, 7.132439104395627e-06, 1.307613835805865e-05, 3.086792814477967e-05, 4.865971793150069e-05, 6.645150771822172e-05, 0.00011043295080832854, 0.00015441439389843537, 0.0001983958369885422, 0.00041386919073265025, 0.0006293425444767584, 0.0008448158982208665, 0.0016605724604978867, 0.002476329022774907, 0.0032920855850519276, 0.004317130907827829, 0.005342176230603731, 0.006367221553379633, 0.007392266876155535, 0.009444724064889774, 0.011497181253624013, 0.013549638442358252, 0.01560209563109249, 0.01765455281982673, 0.023160160229403263, 0.028665767638979794, 0.03417137504855633, 0.039676982458132865, 0.0451825898677094, 0.05331898571073464, 0.061455381553759875, 0.06959177739678511, 0.07772817323981035, 0.08586456908283559, 0.09400096492586082, 0.10178218625602098, 0.10956340758618113, 0.11734462891634129, 0.12512585024650144, 0.1313343647426142, 0.13754287923872696, 0.14375139373483972, 0.14995990823095248, 0.15616842272706524, 0.16290740205860296, 0.16964638139014068, 0.1763853607216784, 0.18312434005321612, 0.18986331938475384, 0.19660229871629156, 0.20196506296400854, 0.20732782721172552, 0.2126905914594425, 0.21805335570715947, 0.22341611995487645, 0.22877888420259343, 0.23401705917136267, 0.23925523414013192, 0.24449340910890116, 0.2497315840776704, 0.25496975904643965, 0.2602079340152089, 0.26660083980367266, 0.2729937455921364, 0.27938665138060015, 0.2857795571690639, 0.29217246295752763, 0.2985653687459914, 0.3038995517433609, 0.30923373474073046, 0.3145679177381, 0.31990210073546954, 0.3252362837328391, 0.3305704667302086, 0.3388054188080464, 0.34704037088588413, 0.3552753229637219, 0.36351027504155964, 0.3717452271193974, 0.37998017919723515, 0.3896571682505123, 0.3993341573037894, 0.40901114635706654, 0.41868813541034366, 0.4283651244636208, 0.4380421135168979, 0.45001070403391524, 0.46197929455093256, 0.4739478850679499, 0.4859164755849672, 0.4978850661019845, 0.5098536566190018, 0.5283300461345777, 0.5468064356501535, 0.5652828251657294, 0.5837592146813052, 0.602235604196881, 0.6207119937124569, 0.6453123204894058, 0.6699126472663547, 0.6945129740433036, 0.7191133008202525, 0.7437136275972014, 0.7812622486217224, 0.8188108696462435, 0.8563594906707646, 0.8939081116952856, 0.9314567327198067, 0.9712047136155396, 1.0109526945112726, 1.0507006754070054, 1.0904486563027382, 1.130196637198471, 1.1942380221189546, 1.258279407039438, 1.3223207919599216, 1.386362176880405, 1.4504035618008886, 1.514444946721372, 1.5861374395877403, 1.6578299324541086, 1.7295224253204768, 1.801214918186845, 1.8729074110532133, 1.9813608111483194, 2.0898142112434255, 2.1982676113385313, 2.306721011433637, 2.415174411528743, 2.523627811623849, 2.6618948418258923, 2.8001618720279358, 2.938428902229979, 3.0766959324320227, 3.214962962634066, 3.3532299928361096, 3.5116989098756672, 3.670167826915225, 3.8286367439547826, 3.9871056609943403, 4.145574578033898, 4.304043495073456, 4.556528668108851, 4.809013841144246, 5.061499014179641, 5.313984187215036, 5.566469360250431, 5.818954533285826, 6.123483674496567, 6.428012815707309, 6.73254195691805, 7.037071098128791, 7.341600239339533, 7.646129380550274, 8.062570162294703, 8.479010944039132, 8.89545172578356, 9.31189250752799, 9.728333289272419, 10.0]</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>0.3001261668971899</v>
+        <v>0.6196464980170189</v>
       </c>
       <c r="D21" t="n">
         <v>9.81</v>
@@ -1840,13 +1840,13 @@
         <v>2</v>
       </c>
       <c r="L21" t="n">
-        <v>3.001261668971899</v>
+        <v>6.196464980170188</v>
       </c>
       <c r="M21" t="n">
-        <v>0.02220354261461239</v>
+        <v>0.005208851742882068</v>
       </c>
       <c r="N21" t="n">
-        <v>0.1110177130730619</v>
+        <v>0.02604425871441034</v>
       </c>
       <c r="O21" t="n">
         <v>19.61131488626249</v>
@@ -1876,11 +1876,11 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>[0.0, 5.944047814512516e-07, 1.1888095629025031e-06, 7.13285737741502e-06, 1.3076905191927536e-05, 3.0869740664146225e-05, 4.866257613636491e-05, 6.64554116085836e-05, 0.00011043952380334257, 0.00015442363599810154, 0.0001984077481928605, 0.0004139447397612804, 0.0006294817313297003, 0.0008450187228981203, 0.0016516910925255899, 0.0024583634621530596, 0.0032650358317805293, 0.004288336395796579, 0.0053116369598126285, 0.006334937523828678, 0.007358238087844728, 0.009422719480668714, 0.011487200873492701, 0.013551682266316688, 0.015616163659140675, 0.017680645051964664, 0.023241147109854417, 0.02880164916774417, 0.03436215122563392, 0.03992265328352367, 0.04548315534141342, 0.05386094900627552, 0.06223874267113762, 0.07061653633599971, 0.0789943300008618, 0.08737212366572389, 0.09574991733058598, 0.1033156048822794, 0.11088129243397281, 0.11844697998566622, 0.12601266753735962, 0.13357835508905302, 0.14114404264074643, 0.14765086354300555, 0.15415768444526468, 0.1606645053475238, 0.16717132624978293, 0.17367814715204205, 0.18018496805430118, 0.18601995956865894, 0.1918549510830167, 0.19768994259737446, 0.20352493411173223, 0.20935992562609, 0.21539180496358054, 0.2214236843010711, 0.22745556363856165, 0.2334874429760522, 0.23951932231354275, 0.2455512016510333, 0.2511062203214203, 0.25666123899180737, 0.2622162576621944, 0.26777127633258146, 0.2733262950029685, 0.27838260152227434, 0.2834389080415802, 0.288495214560886, 0.29355152108019184, 0.29860782759949767, 0.3036641341188035, 0.3105598129347871, 0.31745549175077076, 0.3243511705667544, 0.331246849382738, 0.33814252819872165, 0.3450382070147053, 0.3555462703978924, 0.3660543337810795, 0.3765623971642666, 0.38468120710672865, 0.3928000170491907, 0.40091882699165277, 0.4090376369341148, 0.4171564468765769, 0.42527525681903894, 0.4336614277177424, 0.4420475986164459, 0.45043376951514935, 0.4588199404138528, 0.4672061113125563, 0.47559228221125976, 0.4868561778753583, 0.4981200735394568, 0.5093839692035553, 0.5206478648676538, 0.5319117605317523, 0.5431756561958507, 0.5587527350712365, 0.5743298139466222, 0.5899068928220079, 0.6054839716973937, 0.6210610505727794, 0.6366381294481651, 0.6595939526387494, 0.6825497758293337, 0.705505599019918, 0.7284614222105024, 0.7514172454010867, 0.774373068591671, 0.8041929787038229, 0.8340128888159748, 0.8638327989281267, 0.8936527090402786, 0.9234726191524305, 0.9532925292645824, 0.9916031332544986, 1.0299137372444147, 1.0682243412343309, 1.106534945224247, 1.1448455492141631, 1.1862369760338445, 1.2276284028535258, 1.2690198296732071, 1.3104112564928885, 1.3518026833125698, 1.4036562430517174, 1.455509802790865, 1.5073633625300127, 1.5592169222691603, 1.611070482008308, 1.6629240417474556, 1.7426876005553587, 1.8224511593632617, 1.9022147181711648, 1.981978276979068, 2.061741835786971, 2.1415053945948737, 2.2369061631185274, 2.332306931642181, 2.427707700165835, 2.5231084686894887, 2.6185092372131424, 2.713910005736796, 2.8610755396490744, 3.0082410735613525, 3.1554066074736307, 3.302572141385909, 3.449737675298187, 3.7386381969445996, 4.027538718591012, 4.316439240237425, 4.6053397618838385, 5.8521328271691555, 7.0989258924544725, 8.34571895773979, 10.0]</t>
+          <t>[0.0, 5.944047814512516e-07, 1.1888095629025031e-06, 7.13285737741502e-06, 1.3076905191927536e-05, 3.086974066120871e-05, 4.8662576130489876e-05, 6.645541159977104e-05, 0.00011043952326207938, 0.00015442363492438772, 0.00019840774658669606, 0.00041394371013290073, 0.0006294796736791054, 0.00084501563722531, 0.0016523878551712855, 0.002459760073117261, 0.0032671322910632367, 0.004290053061574974, 0.005312973832086711, 0.006335894602598448, 0.0073588153731101846, 0.009420660752844477, 0.011482506132578769, 0.013544351512313061, 0.015606196892047354, 0.017668042271781648, 0.023177179287398382, 0.028686316303015116, 0.03419545331863185, 0.039704590334248585, 0.04521372734986532, 0.05337998264407202, 0.061546237938278715, 0.0697124932324854, 0.0778787485266921, 0.0860450038208988, 0.0942112591151055, 0.10194024302075337, 0.10966922692640124, 0.11739821083204911, 0.12512719473769698, 0.13132072669115877, 0.13751425864462055, 0.14370779059808234, 0.14990132255154412, 0.1560948545050059, 0.1628281488049083, 0.16956144310481072, 0.17629473740471313, 0.18302803170461554, 0.18976132600451795, 0.19649462030442036, 0.20185444259249488, 0.2072142648805694, 0.21257408716864393, 0.21793390945671845, 0.22329373174479297, 0.2286535540328675, 0.23387416320026322, 0.23909477236765894, 0.24431538153505467, 0.2495359907024504, 0.2547565998698461, 0.25997720903724186, 0.2664283837171494, 0.2728795583970569, 0.27933073307696443, 0.28578190775687196, 0.2922330824367795, 0.298684257116687, 0.3040330400457232, 0.30938182297475936, 0.31473060590379554, 0.3200793888328317, 0.3254281717618679, 0.33077695469090407, 0.33906714181540487, 0.3473573289399057, 0.3556475160644065, 0.3639377031889073, 0.3722278903134081, 0.3805180774379089, 0.3885766640335553, 0.3966352506292017, 0.4046938372248481, 0.4127524238204945, 0.4208110104161409, 0.4288695970117873, 0.43931964897986514, 0.449769700947943, 0.46021975291602085, 0.4706698048840987, 0.48111985685217656, 0.4915699088202544, 0.5087969414155172, 0.52602397401078, 0.5432510066060429, 0.5604780392013057, 0.5777050717965685, 0.5949321043918313, 0.6226347530278941, 0.6503374016639568, 0.6780400503000196, 0.7057426989360823, 0.7334453475721451, 0.7611479962082078, 0.7985098739251743, 0.8358717516421407, 0.8732336293591071, 0.9105955070760735, 0.9479573847930399, 0.9928328053148034, 1.037708225836567, 1.0825836463583307, 1.1274590668800943, 1.172334487401858, 1.2378614411234716, 1.3033883948450853, 1.368915348566699, 1.4344423022883126, 1.4999692560099263, 1.56549620973154, 1.6474235253646992, 1.7293508409978584, 1.8112781566310177, 1.893205472264177, 1.9751327878973362, 2.0693470753520353, 2.1635613628067345, 2.2577756502614337, 2.351989937716133, 2.446204225170832, 2.540418512625531, 2.685324634985187, 2.830230757344843, 2.975136879704499, 3.120043002064155, 3.264949124423811, 3.409855246783467, 3.5836095769314036, 3.7573639070793403, 3.931118237227277, 4.104872567375214, 4.27862689752315, 4.452381227671086, 4.689105985130383, 4.92583074258968, 5.162555500048977, 5.3992802575082735, 5.63600501496757, 5.872729772426867, 6.196575815323581, 6.5204218582202955, 6.84426790111701, 7.168113944013724, 7.491959986910438, 7.8158060298071526, 8.248578551884396, 8.68135107396164, 9.114123596038883, 9.546896118116127, 9.97966864019337, 10.0]</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>0.3000641221480619</v>
+        <v>0.6173931247993982</v>
       </c>
       <c r="D22" t="n">
         <v>9.81</v>
@@ -1907,13 +1907,13 @@
         <v>2</v>
       </c>
       <c r="L22" t="n">
-        <v>3.000641221480619</v>
+        <v>6.173931247993982</v>
       </c>
       <c r="M22" t="n">
-        <v>0.02221272568953041</v>
+        <v>0.005246943864066328</v>
       </c>
       <c r="N22" t="n">
-        <v>0.111063628447652</v>
+        <v>0.02623471932033164</v>
       </c>
       <c r="O22" t="n">
         <v>19.60901458858012</v>
@@ -1943,11 +1943,11 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>[0.0, 5.944488780282292e-07, 1.1888977560564584e-06, 7.133386536338751e-06, 1.3077875316621043e-05, 3.087203368640678e-05, 4.8666192056192514e-05, 6.646035042597826e-05, 0.00011044783865152601, 0.00015443532687707377, 0.00019842281510262154, 0.00041403908642394574, 0.00062965535774527, 0.0008452716290665941, 0.0016418535987404496, 0.002438435568414305, 0.00323501753808816, 0.004255815233719049, 0.005276612929349937, 0.006297410624980826, 0.007318208320611714, 0.009394917298926109, 0.011471626277240504, 0.013548335255554898, 0.015625044233869293, 0.017701753212183688, 0.023268692647643183, 0.028835632083102677, 0.03440257151856217, 0.03996951095402167, 0.04553645038948116, 0.0539606071985058, 0.062384764007530444, 0.07080892081655508, 0.07923307762557973, 0.08765723443460437, 0.09608139124362901, 0.10362993088485606, 0.11117847052608311, 0.11872701016731016, 0.12627554980853722, 0.1338240894497643, 0.14137262909099135, 0.14787593200509708, 0.1543792349192028, 0.16088253783330853, 0.16738584074741425, 0.17388914366151997, 0.1803924465756257, 0.18625167010408938, 0.19211089363255307, 0.19797011716101676, 0.20382934068948044, 0.20968856421794413, 0.2158624602343267, 0.22203635625070928, 0.22821025226709185, 0.23438414828347442, 0.240558044299857, 0.24673194031623957, 0.25204094381644265, 0.25734994731664573, 0.2626589508168488, 0.2679679543170519, 0.273276957817255, 0.27885871108579874, 0.2844404643543425, 0.29002221762288627, 0.29560397089143003, 0.3011857241599738, 0.30676747742851757, 0.31263853634986694, 0.3185095952712163, 0.3243806541925657, 0.33025171311391505, 0.3361227720352644, 0.3419938309566138, 0.35063394752147004, 0.3592740640863263, 0.36791418065118253, 0.3765542972160388, 0.38519441378089503, 0.3938345303457513, 0.40224047504093086, 0.41064641973611044, 0.41905236443129, 0.4274583091264696, 0.4358642538216492, 0.44427019851682875, 0.4540421112643585, 0.46381402401188826, 0.473585936759418, 0.48335784950694777, 0.4931297622544775, 0.5029016750020072, 0.5155202178248479, 0.5281387606476886, 0.5407573034705293, 0.55337584629337, 0.5659943891162107, 0.5786129319390514, 0.5962727565811514, 0.6139325812232515, 0.6315924058653515, 0.6492522305074515, 0.6669120551495515, 0.6845718797916516, 0.710404259560032, 0.7362366393284123, 0.7620690190967927, 0.7879013988651731, 0.8137337786335535, 0.8395661584019338, 0.8727077553521618, 0.9058493523023898, 0.9389909492526178, 0.9721325462028458, 1.0052741431530738, 1.0384157401033018, 1.0826380667187943, 1.1268603933342867, 1.171082719949779, 1.2153050465652715, 1.259527373180764, 1.3037496997962563, 1.364070452108181, 1.4243912044201057, 1.4847119567320304, 1.545032709043955, 1.6053534613558798, 1.6656742136678044, 1.7328405081578075, 1.8000068026478107, 1.8671730971378138, 1.9343393916278169, 2.00150568611782, 2.0686719806078235, 2.166184469271081, 2.2636969579343384, 2.361209446597596, 2.4587219352608534, 2.556234423924111, 2.6537469125873683, 2.7831724099387576, 2.912597907290147, 3.042023404641536, 3.1714489019929255, 3.300874399344315, 3.430299896695704, 3.657832238537285, 3.885364580378866, 4.112896922220447, 4.340429264062028, 4.567961605903609, 5.593569271842922, 6.619176937782235, 7.644784603721549, 8.670392269660862, 10.0]</t>
+          <t>[0.0, 5.944488780282292e-07, 1.1888977560564584e-06, 7.133386536338751e-06, 1.3077875316621043e-05, 3.087203368348269e-05, 4.866619205034434e-05, 6.646035041720599e-05, 0.00011044783811067776, 0.00015443532580414952, 0.00019842281349762128, 0.00041403805564296705, 0.0006296532977883129, 0.0008452685399336587, 0.0016425159212537816, 0.0024397633025739045, 0.0032370106838940276, 0.004257415261249784, 0.00527781983860554, 0.006298224415961296, 0.007318628993317052, 0.00939264829230413, 0.01146666759129121, 0.01354068689027829, 0.01561470618926537, 0.017688725488252448, 0.0232039652241127, 0.028719204959972953, 0.034234444695833206, 0.03974968443169346, 0.04526492416755371, 0.05347131729000547, 0.061677710412457225, 0.06988410353490898, 0.07809049665736073, 0.08629688977981248, 0.09450328290226423, 0.10218031029233846, 0.10985733768241268, 0.11753436507248691, 0.12521139246256113, 0.13288841985263536, 0.14056544724270958, 0.1471557981074257, 0.15374614897214184, 0.16033649983685797, 0.1669268507015741, 0.17351720156629022, 0.18010755243100635, 0.1860609114584641, 0.19201427048592185, 0.1979676295133796, 0.20392098854083734, 0.2098743475682951, 0.21595781269785097, 0.22204127782740685, 0.22812474295696272, 0.2342082080865186, 0.24029167321607448, 0.24637513834563035, 0.2522363983306096, 0.2580976583155889, 0.26395891830056817, 0.26982017828554744, 0.2756814382705267, 0.28105719943111324, 0.28643296059169976, 0.2918087217522863, 0.2971844829128728, 0.30256024407345933, 0.30793600523404585, 0.31587654760122275, 0.32381708996839964, 0.33175763233557654, 0.33969817470275343, 0.3476387170699303, 0.3555792594371072, 0.36574950412827895, 0.37591974881945067, 0.3860899935106224, 0.3962602382017941, 0.40643048289296585, 0.4166007275841376, 0.42757462824477294, 0.4385485289054083, 0.44952242956604366, 0.460496330226679, 0.4714702308873144, 0.48244413154794974, 0.49873194391693876, 0.5150197562859278, 0.5313075686549168, 0.5475953810239058, 0.5638831933928948, 0.5801710057618839, 0.6016949883924486, 0.6232189710230134, 0.6447429536535781, 0.6662669362841429, 0.6877909189147077, 0.7214200693555332, 0.7550492197963586, 0.7886783702371841, 0.8223075206780096, 0.8559366711188351, 0.892004563037527, 0.9280724549562188, 0.9641403468749107, 1.0002082387936024, 1.0362761307122943, 1.1009918878064133, 1.1657076449005324, 1.2304234019946514, 1.2951391590887704, 1.3598549161828895, 1.4245706732770085, 1.4907119341653312, 1.556853195053654, 1.6229944559419767, 1.6891357168302994, 1.7552769777186221, 1.8214182386069449, 1.9073671068179952, 1.9933159750290455, 2.0792648432400958, 2.165213711451146, 2.2511625796621964, 2.3371114478732467, 2.458178796713657, 2.5792461455540674, 2.7003134943944778, 2.821380843234888, 2.9424481920752985, 3.063515540915709, 3.225670033651935, 3.3878245263881612, 3.5499790191243874, 3.7121335118606136, 3.8742880045968398, 4.036442497333066, 4.253900534930774, 4.471358572528482, 4.68881661012619, 4.906274647723897, 5.123732685321605, 5.341190722919313, 5.631615181210967, 5.922039639502621, 6.2124640977942756, 6.50288855608593, 6.793313014377584, 7.083737472669238, 7.474434513872108, 7.865131555074978, 8.255828596277848, 8.646525637480718, 9.037222678683587, 9.427919719886457, 9.955595105529621, 10.0]</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>0.2999855750195113</v>
+        <v>0.6145995938683858</v>
       </c>
       <c r="D23" t="n">
         <v>9.81</v>
@@ -1974,13 +1974,13 @@
         <v>2</v>
       </c>
       <c r="L23" t="n">
-        <v>2.999855750195113</v>
+        <v>6.145995938683858</v>
       </c>
       <c r="M23" t="n">
-        <v>0.02222435941051196</v>
+        <v>0.005294749984958232</v>
       </c>
       <c r="N23" t="n">
-        <v>0.1111217970525598</v>
+        <v>0.02647374992479116</v>
       </c>
       <c r="O23" t="n">
         <v>19.60610504505627</v>
@@ -2010,11 +2010,11 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>[0.0, 5.945046676994561e-07, 1.1890093353989121e-06, 7.134056012393473e-06, 1.3079102689388034e-05, 3.0874934750047205e-05, 4.8670766810706376e-05, 6.646659887136555e-05, 0.00011045835836529723, 0.0001544501178592289, 0.00019844187735316057, 0.00041415856440619396, 0.0006298752514592274, 0.0008455919385122608, 0.0016419068463995243, 0.002438221754286788, 0.0032345366621740514, 0.004030851570061314, 0.005631888814103608, 0.007232926058145902, 0.008833963302188195, 0.010435000546230488, 0.01203603779027278, 0.01706180269619669, 0.022087567602120602, 0.027113332508044513, 0.03213909741396842, 0.03716486231989233, 0.04433351831384311, 0.051502174307793885, 0.058670830301744664, 0.06583948629569544, 0.07300814228964622, 0.080176798283597, 0.08851396777219964, 0.09685113726080227, 0.10518830674940491, 0.1110967150860051, 0.1170051234226053, 0.1229135317592055, 0.1288219400958057, 0.1347303484324059, 0.14167123800376996, 0.14861212757513403, 0.1555530171464981, 0.16249390671786218, 0.16943479628922625, 0.17637568586059033, 0.18270187426185097, 0.18902806266311162, 0.19535425106437226, 0.2016804394656329, 0.20800662786689356, 0.2143328162681542, 0.22087412076851906, 0.22741542526888392, 0.23180776519184296, 0.236200105114802, 0.24059244503776103, 0.24498478496072007, 0.2493771248836791, 0.25376946480663815, 0.2595576580317539, 0.26534585125686966, 0.2711340444819854, 0.27692223770710117, 0.2827104309322169, 0.2884986241573327, 0.29362112352587966, 0.29874362289442663, 0.3038661222629736, 0.3089886216315206, 0.31411112100006755, 0.3192336203686145, 0.326876088658367, 0.33451855694811944, 0.3421610252378719, 0.34980349352762435, 0.3574459618173768, 0.36528255018583494, 0.3731191385542931, 0.3809557269227512, 0.38879231529120933, 0.39662890365966746, 0.4044654920281256, 0.4139868374142343, 0.423508182800343, 0.43302952818645174, 0.44255087357256045, 0.45207221895866917, 0.4615935643447779, 0.4721708928148341, 0.4827482212848903, 0.4933255497549465, 0.5039028782250028, 0.5144802066950591, 0.5250575351651154, 0.5385249827915999, 0.5519924304180843, 0.5654598780445688, 0.5789273256710532, 0.5923947732975376, 0.6058622209240221, 0.6257432306104618, 0.6456242402969015, 0.6655052499833412, 0.6853862596697808, 0.7052672693562205, 0.7336452305371566, 0.7620231917180926, 0.7904011528990287, 0.8187791140799647, 0.8471570752609008, 0.8781476209571081, 0.9091381666533154, 0.9401287123495227, 0.97111925804573, 1.0021098037419374, 1.0395924752759504, 1.0770751468099635, 1.1145578183439766, 1.1520404898779897, 1.1895231614120028, 1.2270058329460158, 1.2875440116291879, 1.3480821903123599, 1.408620368995532, 1.469158547678704, 1.529696726361876, 1.590234905045048, 1.6539793874139663, 1.7177238697828847, 1.781468352151803, 1.8452128345207215, 1.9089573168896399, 1.9727017992585583, 2.063463573931537, 2.1542253486045158, 2.2449871232774945, 2.3357488979504732, 2.426510672623452, 2.5172724472964307, 2.6338319114068383, 2.7503913755172458, 2.8669508396276533, 2.983510303738061, 3.1000697678484683, 3.216629231958876, 3.412273032372439, 3.607916832786002, 3.803560633199565, 3.999204433613128, 4.194848234026691, 4.750125589155526, 5.305402944284361, 5.860680299413196, 6.415957654542031, 8.350982842551176, 10.0]</t>
+          <t>[0.0, 5.945046676994561e-07, 1.1890093353989121e-06, 7.134056012393473e-06, 1.3079102689388034e-05, 3.087493474714006e-05, 4.8670766804892084e-05, 6.646659886264411e-05, 0.00011045835782497391, 0.00015445011678730372, 0.00019844187574963353, 0.0004141575321633959, 0.0006298731885771582, 0.0008455888449909205, 0.0016413683311895383, 0.002437147817388156, 0.003232927303586774, 0.0040287067897853916, 0.005628657681912624, 0.0072286085740398565, 0.008828559466167089, 0.010428510358294322, 0.012028461250421554, 0.017014693520785565, 0.022000925791149574, 0.026987158061513583, 0.03197339033187759, 0.0369596226022416, 0.04403336667449801, 0.05110711074675442, 0.05818085481901083, 0.06525459889126724, 0.07232834296352364, 0.07940208703578004, 0.08813937367631304, 0.09687666031684604, 0.10328030602942907, 0.1096839517420121, 0.11608759745459514, 0.12249124316717817, 0.1288948888797612, 0.1359802262474419, 0.14306556361512263, 0.15015090098280334, 0.15723623835048406, 0.16432157571816478, 0.1714069130858455, 0.1783247391576919, 0.1852425652295383, 0.1921603913013847, 0.19907821737323111, 0.20599604344507752, 0.21291386951692393, 0.2193308342510943, 0.22574779898526465, 0.232164763719435, 0.23858172845360537, 0.24499869318777573, 0.2514156579219461, 0.25628552513598685, 0.2611553923500276, 0.26602525956406836, 0.2708951267781091, 0.2757649939921499, 0.28063486120619063, 0.2870822155652922, 0.2935295699243937, 0.29997692428349526, 0.3064242786425968, 0.31287163300169835, 0.3193189873607999, 0.33097656873708575, 0.3397026475856276, 0.3484287264341695, 0.3571548052827114, 0.36588088413125325, 0.3746069629797951, 0.38447200241696333, 0.39433704185413154, 0.40420208129129975, 0.41406712072846796, 0.4239321601656362, 0.4337971996028044, 0.4468789137202124, 0.4599606278376204, 0.47304234195502837, 0.48612405607243636, 0.49920577018984436, 0.5122874843072523, 0.5281589193034397, 0.5440303542996271, 0.5599017892958145, 0.5757732242920018, 0.5916446592881892, 0.6160523308668864, 0.6404600024455835, 0.6648676740242807, 0.6892753456029779, 0.713683017181675, 0.7488215004260178, 0.7839599836703606, 0.8190984669147033, 0.8542369501590461, 0.8893754334033889, 0.9272048054446156, 0.9650341774858423, 1.002863549527069, 1.0406929215682958, 1.0785222936095227, 1.1393978778454164, 1.20027346208131, 1.2611490463172037, 1.3220246305530974, 1.382900214788991, 1.4437757990248847, 1.5118480942757162, 1.5799203895265477, 1.6479926847773791, 1.7160649800282106, 1.784137275279042, 1.8898132353754833, 1.9954891954719245, 2.1011651555683657, 2.206841115664807, 2.312517075761248, 2.4181930358576893, 2.5496873429402727, 2.681181650022856, 2.8126759571054394, 2.9441702641880227, 3.075664571270606, 3.2071588783531895, 3.3586472861313283, 3.5101356939094672, 3.661624101687606, 3.813112509465745, 3.964600917243884, 4.116089325022022, 4.357203061593634, 4.598316798165246, 4.8394305347368585, 5.0805442713084705, 5.321658007880083, 5.562771744451695, 5.853350136926949, 6.143928529402203, 6.434506921877457, 6.725085314352711, 7.015663706827965, 7.306242099303219, 7.703469219102929, 8.100696338902639, 8.497923458702349, 8.89515057850206, 9.29237769830177, 9.68960481810148, 10.0]</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>0.2998864968054452</v>
+        <v>0.611153500492971</v>
       </c>
       <c r="D24" t="n">
         <v>9.81</v>
@@ -2041,13 +2041,13 @@
         <v>2</v>
       </c>
       <c r="L24" t="n">
-        <v>2.998864968054451</v>
+        <v>6.11153500492971</v>
       </c>
       <c r="M24" t="n">
-        <v>0.0222390470580653</v>
+        <v>0.005354629033341843</v>
       </c>
       <c r="N24" t="n">
-        <v>0.1111952352903265</v>
+        <v>0.02677314516670921</v>
       </c>
       <c r="O24" t="n">
         <v>19.60242489375145</v>
@@ -2077,11 +2077,11 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>[0.0, 5.94575255782134e-07, 1.189150511564268e-06, 7.1349030693856085e-06, 1.3080655627206949e-05, 3.087860533193518e-05, 4.867655503666342e-05, 6.647450474139165e-05, 0.00011047166849727146, 0.00015446883225315127, 0.00019846599600903107, 0.00041430991634560635, 0.0006301538366821816, 0.0008459977570187568, 0.0016477385081952174, 0.002449479259371678, 0.0032512200105481383, 0.004052960761724599, 0.00565569874189281, 0.007258436722061021, 0.008861174702229233, 0.010463912682397443, 0.012066650662565653, 0.017144195801292117, 0.02222174094001858, 0.027299286078745044, 0.03237683121747151, 0.03745437635619797, 0.044674304035130785, 0.0518942317140636, 0.05911415939299641, 0.06633408707192923, 0.07355401475086204, 0.08077394242979485, 0.0889704308291293, 0.09716691922846374, 0.10536340762779818, 0.1112263240124021, 0.11708924039700601, 0.12295215678160992, 0.12881507316621382, 0.13467798955081772, 0.14161828937923057, 0.14855858920764342, 0.15549888903605627, 0.16243918886446912, 0.16937948869288197, 0.17631978852129482, 0.18204489795013168, 0.18777000737896854, 0.1934951168078054, 0.19922022623664226, 0.20494533566547912, 0.2106870880048945, 0.21642884034430987, 0.22217059268372524, 0.22791234502314062, 0.233654097362556, 0.23939584970197136, 0.2458943190380882, 0.2502429813340863, 0.25459164363008435, 0.2589403059260824, 0.2632889682220805, 0.26763763051807854, 0.2731743125432981, 0.27871099456851767, 0.28424767659373723, 0.2897843586189568, 0.29532104064417636, 0.3008577226693959, 0.30659984958500014, 0.31234197650060436, 0.3180841034162086, 0.3238262303318128, 0.329568357247417, 0.3353104841630212, 0.3432404550468971, 0.35117042593077297, 0.35910039681464884, 0.3670303676985247, 0.3749603385824006, 0.38289030946627645, 0.3905920175831976, 0.3982937257001188, 0.40599543381703995, 0.4136971419339611, 0.4213988500508823, 0.42910055816780346, 0.4377805161589219, 0.4464604741500403, 0.45514043214115874, 0.46382039013227716, 0.4725003481233956, 0.481180306114514, 0.49202567062683605, 0.5028710351391581, 0.5137163996514802, 0.5245617641638023, 0.5354071286761244, 0.5462524931884465, 0.5608620608297878, 0.5754716284711292, 0.5900811961124706, 0.6046907637538119, 0.6193003313951533, 0.6339098990364946, 0.6568034654586912, 0.6796970318808877, 0.7025905983030842, 0.7254841647252808, 0.7483777311474773, 0.7712712975696738, 0.8032902642282833, 0.8353092308868928, 0.8673281975455023, 0.8993471642041118, 0.9313661308627212, 0.9633850975213307, 1.0029139815053216, 1.0424428654893125, 1.0819717494733034, 1.1215006334572943, 1.1610295174412852, 1.2005584014252761, 1.2541447545539737, 1.3077311076826712, 1.3613174608113687, 1.4149038139400663, 1.4684901670687638, 1.5220765201974613, 1.5893908927795803, 1.6567052653616994, 1.7240196379438184, 1.7913340105259374, 1.8586483831080565, 1.9259627556901755, 2.0135136606660153, 2.101064565641855, 2.188615470617695, 2.276166375593535, 2.3637172805693747, 2.4512681855452145, 2.572853146483106, 2.6944381074209973, 2.8160230683588887, 2.93760802929678, 3.0591929902346715, 3.180777951172563, 3.3645051683881766, 3.5482323856037903, 3.731959602819404, 3.9156868200350177, 4.099414037250631, 4.283141254466245, 4.599207608356067, 4.915273962245888, 5.23134031613571, 5.547406670025532, 5.863473023915353, 6.794256576790874, 7.725040129666394, 8.655823682541914, 9.586607235417436, 10.0]</t>
+          <t>[0.0, 5.94575255782134e-07, 1.189150511564268e-06, 7.1349030693856085e-06, 1.3080655627206949e-05, 3.087860532904964e-05, 4.867655503089233e-05, 6.647450473273503e-05, 0.0001104716679576113, 0.00015446883118248756, 0.00019846599440736382, 0.0004143088822493571, 0.0006301517700913504, 0.0008459946579333437, 0.0016471818873487188, 0.0024483691167640938, 0.0032495563461794686, 0.004050743575594843, 0.005652384037579536, 0.007254024499564228, 0.00885566496154892, 0.010457305423533611, 0.012058945885518303, 0.017094714900042964, 0.022130483914567626, 0.027166252929092288, 0.032202021943616946, 0.0372377909581416, 0.04435875984730785, 0.051479728736474106, 0.05860069762564036, 0.06572166651480661, 0.07284263540397287, 0.07996360429313913, 0.0885722500892998, 0.09718089588546046, 0.10350923489936502, 0.10983757391326958, 0.11616591292717414, 0.1224942519410787, 0.12882259095498327, 0.13589088224719797, 0.14295917353941268, 0.15002746483162738, 0.15709575612384208, 0.16416404741605678, 0.17123233870827148, 0.178090432649844, 0.18494852659141653, 0.19180662053298905, 0.19866471447456158, 0.2055228084161341, 0.21238090235770662, 0.21890622435954268, 0.22543154636137874, 0.2319568683632148, 0.23848219036505086, 0.24500751236688692, 0.251532834368723, 0.2564386731464192, 0.26134451192411545, 0.2662503507018117, 0.2711561894795079, 0.27606202825720416, 0.2809678670349004, 0.28736716925491146, 0.2937664714749225, 0.3001657736949336, 0.30656507591494464, 0.3129643781349557, 0.31936368035496676, 0.3308549858581892, 0.3394872009418228, 0.3481194160254564, 0.35675163110909, 0.36538384619272357, 0.37401606127635717, 0.38499952872651305, 0.39598299617666893, 0.4069664636268248, 0.4179499310769807, 0.4289333985271366, 0.43991686597729246, 0.45286600667830074, 0.465815147379309, 0.4787642880803173, 0.49171342878132557, 0.5046625694823339, 0.5176117101833422, 0.5344062419065181, 0.551200773629694, 0.5679953053528699, 0.5847898370760458, 0.6015843687992217, 0.6270357956152892, 0.6524872224313567, 0.6779386492474242, 0.7033900760634917, 0.7288415028795592, 0.7652648528153895, 0.8016882027512198, 0.8381115526870501, 0.8745349026228804, 0.9109582525587107, 0.9497889972628736, 0.9886197419670365, 1.0274504866711993, 1.066281231375362, 1.1051119760795247, 1.16782420857826, 1.2305364410769952, 1.2932486735757305, 1.3559609060744657, 1.418673138573201, 1.4813853710719362, 1.551432945720271, 1.6214805203686056, 1.6915280950169402, 1.761575669665275, 1.8316232443136096, 1.9376392509890839, 2.0436552576645584, 2.149671264340033, 2.255687271015508, 2.3617032776909825, 2.4677192843664573, 2.602797378922311, 2.737875473478165, 2.872953568034019, 3.0080316625898726, 3.1431097571457265, 3.2781878517015803, 3.4330552335274476, 3.587922615353315, 3.742789997179182, 3.8976573790050493, 4.0525247608309165, 4.207392142656784, 4.4540983700118275, 4.700804597366871, 4.947510824721915, 5.194217052076959, 5.440923279432003, 5.687629506787046, 5.985125660106362, 6.282621813425677, 6.580117966744992, 6.877614120064307, 7.1751102733836225, 7.472606426702938, 7.879385302875142, 8.286164179047347, 8.692943055219551, 9.099721931391755, 9.50650080756396, 9.913279683736164, 10.0]</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>0.2997605260611548</v>
+        <v>0.6069268253021186</v>
       </c>
       <c r="D25" t="n">
         <v>9.81</v>
@@ -2108,13 +2108,13 @@
         <v>2</v>
       </c>
       <c r="L25" t="n">
-        <v>2.997605260611548</v>
+        <v>6.069268253021185</v>
       </c>
       <c r="M25" t="n">
-        <v>0.02225774236787723</v>
+        <v>0.005429468645042354</v>
       </c>
       <c r="N25" t="n">
-        <v>0.1112887118393861</v>
+        <v>0.02714734322521177</v>
       </c>
       <c r="O25" t="n">
         <v>19.59777003517474</v>
@@ -2144,11 +2144,11 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>[0.0, 5.946645750668049e-07, 1.1893291501336098e-06, 7.135974900801659e-06, 1.3082620651469708e-05, 3.088324993779976e-05, 4.8683879224129816e-05, 6.648450851045988e-05, 0.00011048851063806105, 0.00015449251276566223, 0.0001984965148932634, 0.0004145017232300062, 0.0006305069315667491, 0.0008465121399034919, 0.0016553762070344276, 0.0024642402741653635, 0.003273104341296299, 0.004081968408427235, 0.005687092586546127, 0.0072922167646650195, 0.008897340942783912, 0.010502465120902804, 0.012107589299021696, 0.01725508658576028, 0.02240258387249886, 0.027550081159237443, 0.032697578445976025, 0.0378450757327146, 0.045134333205105084, 0.052423590677495566, 0.05971284814988605, 0.06700210562227653, 0.07429136309466701, 0.08158062056705749, 0.08960153148708465, 0.0976224424071118, 0.10564335332713896, 0.11203117315053208, 0.1184189929739252, 0.12480681279731833, 0.13119463262071146, 0.1375824524441046, 0.14466193977133024, 0.15174142709855587, 0.1588209144257815, 0.16590040175300713, 0.17297988908023276, 0.1800593764074584, 0.18596650273660237, 0.19187362906574634, 0.19778075539489032, 0.2036878817240343, 0.20959500805317827, 0.21621576420725216, 0.22283652036132606, 0.2271230119818325, 0.23140950360233892, 0.23569599522284534, 0.23998248684335177, 0.2442689784638582, 0.24855547008436463, 0.2537586710962606, 0.2589618721081566, 0.26416507312005255, 0.2693682741319485, 0.2745714751438445, 0.2797746761557405, 0.2849184359759758, 0.2900621957962112, 0.2952059556164465, 0.3003497154366819, 0.3054934752569172, 0.3106372350771526, 0.3185860290641203, 0.32653482305108805, 0.3344836170380558, 0.34243241102502353, 0.35038120501199127, 0.3608515961090777, 0.3713219872061641, 0.37955669602508824, 0.38779140484401237, 0.3960261136629365, 0.4042608224818606, 0.41249553130078476, 0.4207302401197089, 0.4293591266340593, 0.4379880131484097, 0.4466168996627601, 0.4552457861771105, 0.4638746726914609, 0.4725035592058113, 0.48467924021787934, 0.4968549212299474, 0.5090306022420155, 0.5212062832540836, 0.5333819642661517, 0.5455576452782198, 0.562970347051807, 0.5803830488253943, 0.5977957505989815, 0.6152084523725687, 0.6326211541461559, 0.6500338559197432, 0.6754534157403584, 0.7008729755609737, 0.726292535381589, 0.7517120952022043, 0.7771316550228196, 0.8025512148434348, 0.8337122717641441, 0.8648733286848533, 0.8960343856055626, 0.9271954425262718, 0.9583564994469811, 0.9932754313605171, 1.0281943632740531, 1.063113295187589, 1.098032227101125, 1.1329511590146608, 1.1744141179995937, 1.2158770769845266, 1.2573400359694595, 1.2988029949543924, 1.3402659539393253, 1.3817289129242583, 1.4486032508879074, 1.5154775888515566, 1.5823519268152058, 1.649226264778855, 1.716100602742504, 1.7829749407061533, 1.854645408292769, 1.9263158758793848, 1.9979863434660006, 2.0696568110526163, 2.141327278639232, 2.212997746225848, 2.3068289293387454, 2.400660112451643, 2.4944912955645404, 2.588322478677438, 2.6821536617903354, 2.775984844903233, 2.9046689313315928, 3.0333530177599526, 3.1620371041883124, 3.2907211906166722, 3.419405277045032, 3.548089363473392, 3.7506358425453894, 3.953182321617387, 4.155728800689385, 4.358275279761383, 4.560821758833381, 5.184711314857959, 5.808600870882538, 6.432490426907116, 7.056379982931695, 9.3050878139521, 10.0]</t>
+          <t>[0.0, 5.946645750668049e-07, 1.1893291501336098e-06, 7.135974900801659e-06, 1.3082620651469708e-05, 3.0883249934941384e-05, 4.868387921841306e-05, 6.648450850188473e-05, 0.00011048851009924339, 0.00015449251169660205, 0.0001984965132939607, 0.00041450068677916733, 0.0006305048602643739, 0.0008465090337495805, 0.0016547950760173635, 0.0024630811182851466, 0.0032713671605529297, 0.004079653202820712, 0.005683664397223858, 0.007287675591627003, 0.008891686786030148, 0.010495697980433294, 0.012099709174836439, 0.017202237272468904, 0.02230476537010137, 0.027407293467733837, 0.032509821565366304, 0.03761234966299877, 0.04479693101075478, 0.051981512358510784, 0.05916609370626679, 0.0663506750540228, 0.0735352564017788, 0.0807198377495348, 0.08914308958042756, 0.09756634141132033, 0.10598959324221309, 0.11195124776229236, 0.11791290228237163, 0.1238745568024509, 0.12983621132253015, 0.1357978658426094, 0.14282186817713954, 0.1498458705116697, 0.15686987284619985, 0.16389387518073, 0.17091787751526016, 0.17794187984979032, 0.18387387343678202, 0.18980586702377372, 0.19573786061076542, 0.20166985419775713, 0.20760184778474883, 0.21373641270509317, 0.2198709776254375, 0.22600554254578184, 0.23214010746612618, 0.23827467238647052, 0.24440923730681485, 0.25011063170527414, 0.25581202610373344, 0.26151342050219273, 0.267214814900652, 0.2729162092991113, 0.27827990730283925, 0.2836436053065672, 0.2890073033102951, 0.29437100131402305, 0.299734699317751, 0.3050983973214789, 0.312844921106111, 0.3205914448907431, 0.3283379686753752, 0.33608449246000727, 0.34383101624463935, 0.35157754002927144, 0.3609198466985441, 0.37026215336781676, 0.3796044600370894, 0.3889467667063621, 0.39828907337563474, 0.4076313800449074, 0.4184350991146627, 0.429238818184418, 0.4400425372541733, 0.4508462563239286, 0.4616499753936839, 0.4724536944634392, 0.487919601913995, 0.5033855093645508, 0.5188514168151066, 0.5343173242656624, 0.5497832317162181, 0.5652491391667739, 0.5880131119835803, 0.6107770848003867, 0.6335410576171931, 0.6563050304339996, 0.679069003250806, 0.7018329760676124, 0.7308413645816199, 0.7598497530956273, 0.7888581416096347, 0.8178665301236422, 0.8468749186376496, 0.8914122908990302, 0.9359496631604107, 0.9804870354217913, 1.0250244076831718, 1.0695617799445523, 1.1213400519356587, 1.173118323926765, 1.2248965959178715, 1.2766748679089779, 1.3284531399000843, 1.3802314118911907, 1.440505363108637, 1.5007793143260835, 1.5610532655435299, 1.6213272167609762, 1.6816011679784226, 1.7698304699875391, 1.8580597719966556, 1.9462890740057721, 2.034518376014889, 2.1227476780240053, 2.210976980033122, 2.3329934069148686, 2.4550098337966153, 2.577026260678362, 2.699042687560109, 2.8210591144418555, 2.9430755413236023, 3.094868663069726, 3.24666178481585, 3.398454906561974, 3.550248028308098, 3.702041150054222, 3.8538342718003458, 4.081307269933646, 4.308780268066946, 4.536253266200246, 4.763726264333546, 4.991199262466846, 5.2186722606001466, 5.514823073229999, 5.810973885859851, 6.107124698489703, 6.403275511119555, 6.699426323749408, 6.99557713637926, 7.345843532695868, 7.696109929012477, 8.046376325329085, 8.396642721645694, 8.746909117962304, 9.097175514278913, 9.615250878718088, 10.0]</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>0.299601481437283</v>
+        <v>0.6017789637713979</v>
       </c>
       <c r="D26" t="n">
         <v>9.81</v>
@@ -2175,13 +2175,13 @@
         <v>2</v>
       </c>
       <c r="L26" t="n">
-        <v>2.99601481437283</v>
+        <v>6.017789637713979</v>
       </c>
       <c r="M26" t="n">
-        <v>0.02228137986026059</v>
+        <v>0.005522757719390599</v>
       </c>
       <c r="N26" t="n">
-        <v>0.1114068993013029</v>
+        <v>0.02761378859695299</v>
       </c>
       <c r="O26" t="n">
         <v>19.59188231302026</v>
@@ -2211,11 +2211,11 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>[0.0, 5.947776079968284e-07, 1.1895552159936568e-06, 7.137331295961941e-06, 1.3085107375930226e-05, 3.0889127655718666e-05, 4.869314793550711e-05, 6.649716821529556e-05, 0.00011050982431657245, 0.00015452248041784934, 0.00019853513651912623, 0.0004147449234716011, 0.000630954710424076, 0.0008471644973765508, 0.0016654894114383231, 0.0024838143255000956, 0.003302139239561868, 0.004120464153623641, 0.005729002870470927, 0.007337541587318213, 0.008946080304165499, 0.010554619021012785, 0.01216315773786007, 0.017407312465840208, 0.022651467193820343, 0.02789562192180048, 0.033139776649780614, 0.03838393137776075, 0.04576918547867298, 0.05315443957958521, 0.06053969368049744, 0.06792494778140967, 0.0753102018823219, 0.08269545598323413, 0.09050532597715925, 0.09831519597108437, 0.1061250659650095, 0.11243967297172838, 0.11875427997844727, 0.12506888698516616, 0.13138349399188504, 0.1376981009986039, 0.14477985928672513, 0.15186161757484634, 0.15894337586296756, 0.16602513415108877, 0.17310689243921, 0.1801886507273312, 0.1861009593762018, 0.1920132680250724, 0.197925576673943, 0.2038378853228136, 0.2097501939716842, 0.21648158575312043, 0.22321297753455666, 0.22747261523096537, 0.2317322529273741, 0.2359918906237828, 0.24025152832019153, 0.24451116601660025, 0.24877080371300897, 0.25400755604900105, 0.2592443083849931, 0.2644810607209852, 0.2697178130569773, 0.27495456539296936, 0.28019131772896144, 0.28532822716229306, 0.2904651365956247, 0.2956020460289563, 0.3007389554622879, 0.3058758648956195, 0.31101277432895114, 0.32084308002085066, 0.3306733857127502, 0.3377120108276401, 0.34475063594252997, 0.35178926105741987, 0.35882788617230976, 0.36586651128719966, 0.37429897550664465, 0.38273143972608964, 0.39116390394553463, 0.3995963681649796, 0.4080288323844246, 0.4164612966038696, 0.426721834773614, 0.43698237294335834, 0.4472429111131027, 0.4575034492828471, 0.46776398745259146, 0.4780245256223358, 0.4898522588257186, 0.5016799920291013, 0.513507725232484, 0.5253354584358667, 0.5371631916392494, 0.5489909248426321, 0.5655475695290162, 0.5821042142154003, 0.5986608589017843, 0.6152175035881684, 0.6317741482745525, 0.656468127568879, 0.6811621068632054, 0.7058560861575319, 0.7305500654518584, 0.7552440447461849, 0.7834083306549363, 0.8115726165636877, 0.8397369024724392, 0.8679011883811906, 0.896065474289942, 0.92915185246612, 0.962238230642298, 0.995324608818476, 1.028410986994654, 1.0614973651708322, 1.1011699599219569, 1.1408425546730816, 1.1805151494242063, 1.220187744175331, 1.2598603389264558, 1.2995329336775805, 1.3568029004016817, 1.414072867125783, 1.4713428338498842, 1.5286128005739854, 1.5858827672980866, 1.6431527340221879, 1.70762186096676, 1.772090987911332, 1.836560114855904, 1.9010292418004762, 1.9654983687450482, 2.02996749568962, 2.1148727378719205, 2.199777980054221, 2.2846832222365214, 2.369588464418822, 2.4544937066011223, 2.5393989487834228, 2.647784456445623, 2.7561699641078237, 2.864555471770024, 2.9729409794322246, 3.081326487094425, 3.1897119947566255, 3.351509343159418, 3.51330669156221, 3.6751040399650026, 3.836901388367795, 3.9986987367705873, 4.16049608517338, 4.451818257159662, 4.743140429145944, 5.034462601132226, 5.325784773118508, 5.617106945104791, 7.208792041233089, 8.800477137361387, 10.0]</t>
+          <t>[0.0, 5.947776079968284e-07, 1.1895552159936568e-06, 7.137331295961941e-06, 1.3085107375930226e-05, 3.0889127652894774e-05, 4.8693147929859324e-05, 6.649716820682387e-05, 0.00011050982377881893, 0.000154522479350814, 0.00019853513492280905, 0.00041474388402821166, 0.0006309526331336143, 0.0008471613822390168, 0.0016648743937297044, 0.002482587405220392, 0.0033003004167110796, 0.004118013428201768, 0.005725417244525171, 0.007332821060848574, 0.008940224877171978, 0.01054762869349538, 0.012155032509818784, 0.01734948528815081, 0.022543938066482836, 0.027738390844814862, 0.032932843623146885, 0.03812729640147891, 0.045399475432279277, 0.05267165446307964, 0.05994383349388001, 0.06721601252468037, 0.07448819155548074, 0.0817603705862811, 0.0899408020790275, 0.09812123357177388, 0.10630166506452027, 0.11277451103914929, 0.11924735701377831, 0.12572020298840733, 0.13219304896303635, 0.13866589493766537, 0.14583038955191555, 0.15299488416616572, 0.1601593787804159, 0.16732387339466606, 0.17448836800891623, 0.1816528626231664, 0.1877153826863763, 0.1937779027495862, 0.1998404228127961, 0.205902942876006, 0.2119654629392159, 0.21820372372381325, 0.2244419845084106, 0.23068024529300796, 0.2369185060776053, 0.24315676686220267, 0.24939502764680002, 0.2552783871635632, 0.26116174668032643, 0.26704510619708965, 0.2729284657138529, 0.2788118252306161, 0.2846951847473793, 0.29046423511539404, 0.29623328548340877, 0.3020023358514235, 0.3077713862194382, 0.31354043658745295, 0.3193094869554677, 0.32759349505284224, 0.3358775031502168, 0.34416151124759137, 0.35244551934496593, 0.3607295274423405, 0.3702590779087829, 0.37978862837522526, 0.38931817884166764, 0.39884772930811, 0.4083772797745524, 0.4179068302409948, 0.42953052950704196, 0.44115422877308913, 0.4527779280391363, 0.4644016273051835, 0.47602532657123064, 0.4876490258372778, 0.5037565295143963, 0.5198640331915148, 0.5359715368686332, 0.5520790405457516, 0.5681865442228701, 0.591547269961761, 0.6149079957006519, 0.6382687214395428, 0.6616294471784337, 0.6849901729173247, 0.7188264983706762, 0.7526628238240278, 0.7864991492773794, 0.820335474730731, 0.8541718001840826, 0.8903373243732055, 0.9265028485623283, 0.9626683727514512, 0.9988338969405741, 1.034999421129697, 1.09413092158135, 1.153262422033003, 1.212393922484656, 1.271525422936309, 1.3306569233879622, 1.3897884238396152, 1.455052740268698, 1.5203170566977806, 1.5855813731268633, 1.650845689555946, 1.7161100059850287, 1.8171699997560318, 1.9182299935270348, 2.0192899872980377, 2.1203499810690403, 2.221409974840043, 2.3224699686110455, 2.4485727938155097, 2.574675619019974, 2.7007784442244382, 2.8268812694289025, 2.9529840946333668, 3.079086919837831, 3.2243552938362425, 3.369623667834654, 3.5148920418330656, 3.660160415831477, 3.8054287898298886, 3.9506971638283, 4.181862887990856, 4.413028612153411, 4.644194336315967, 4.875360060478522, 5.106525784641078, 5.337691508803633, 5.616137580573091, 5.894583652342549, 6.1730297241120065, 6.451475795881464, 6.729921867650922, 7.0083679394203795, 7.388918994134857, 7.769470048849335, 8.150021103563812, 8.53057215827829, 8.911123212992766, 9.291674267707243, 9.818218147090521, 10.0]</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>0.2994004184477449</v>
+        <v>0.5955610137429067</v>
       </c>
       <c r="D27" t="n">
         <v>9.81</v>
@@ -2242,13 +2242,13 @@
         <v>2</v>
       </c>
       <c r="L27" t="n">
-        <v>2.994004184477449</v>
+        <v>5.955610137429066</v>
       </c>
       <c r="M27" t="n">
-        <v>0.02231131612509685</v>
+        <v>0.005638680337490636</v>
       </c>
       <c r="N27" t="n">
-        <v>0.1115565806254842</v>
+        <v>0.02819340168745318</v>
       </c>
       <c r="O27" t="n">
         <v>19.58443519693777</v>
@@ -2278,11 +2278,11 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>[0.0, 5.949206695156695e-07, 1.189841339031339e-06, 7.139048034188033e-06, 1.3088254729344728e-05, 3.089656686442745e-05, 4.8704878999510175e-05, 6.65131911345929e-05, 0.00011053680034358905, 0.0001545604095525852, 0.00019858401876158134, 0.00041505348948016324, 0.0006315229601987452, 0.0008479924309173271, 0.0016790846153543894, 0.0025101767997914516, 0.003341268984228514, 0.004172361168665576, 0.005785900852742552, 0.007399440536819528, 0.009012980220896505, 0.01062651990497348, 0.012240059589050457, 0.017622253363036265, 0.02300444713702207, 0.028386640911007878, 0.033768834684993684, 0.03915102845897949, 0.04667397840435491, 0.054196928349730326, 0.061719878295105744, 0.06924282824048117, 0.07676577818585659, 0.084288728131232, 0.09185414398632408, 0.09941955984141615, 0.10698497569650822, 0.1145503915516003, 0.1206513233985502, 0.1267522552455001, 0.13285318709245, 0.1389541189393999, 0.1450550507863498, 0.15156134355518275, 0.1580676363240157, 0.16457392909284863, 0.17108022186168156, 0.1775865146305145, 0.18409280739934744, 0.1895251075231026, 0.19495740764685773, 0.20038970777061288, 0.20582200789436803, 0.21125430801812317, 0.21714929311253817, 0.22304427820695316, 0.22893926330136816, 0.23483424839578315, 0.24072923349019815, 0.24662421858461314, 0.2522447474349365, 0.2578652762852599, 0.2634858051355833, 0.26910633398590666, 0.27472686283623005, 0.2803473916865534, 0.28567708802416164, 0.29100678436176985, 0.29633648069937807, 0.3016661770369863, 0.3069958733745945, 0.3123255697122027, 0.32222203140354694, 0.33006196365312845, 0.33790189590270997, 0.3457418281522915, 0.353581760401873, 0.3614216926514545, 0.36989814591646675, 0.378374599181479, 0.3868510524464912, 0.39532750571150344, 0.40380395897651566, 0.4122804122415279, 0.42266194057194356, 0.43304346890235923, 0.4434249972327749, 0.45380652556319057, 0.46418805389360623, 0.4745695822240219, 0.48664173109148606, 0.4987138799589502, 0.5107860288264143, 0.5228581776938784, 0.5349303265613425, 0.5470024754288066, 0.5638673272986554, 0.5807321791685042, 0.5975970310383529, 0.6144618829082017, 0.6313267347780505, 0.6562844996115109, 0.6812422644449714, 0.7062000292784318, 0.7311577941118923, 0.7561155589453528, 0.7844152112650659, 0.812714863584779, 0.841014515904492, 0.8693141682242052, 0.8976138205439183, 0.9309483393811737, 0.9642828582184292, 0.9976173770556847, 1.0309518958929402, 1.0642864147301958, 1.1042630466141266, 1.1442396784980573, 1.184216310381988, 1.2241929422659188, 1.2641695741498495, 1.3041462060337803, 1.361405493233342, 1.4186647804329036, 1.4759240676324652, 1.5331833548320268, 1.5904426420315885, 1.64770192923115, 1.7124786738464581, 1.7772554184617662, 1.8420321630770742, 1.9068089076923822, 1.9715856523076902, 2.036362396922998, 2.1215500054818333, 2.2067376140406685, 2.2919252225995037, 2.377112831158339, 2.462300439717174, 2.5474880482760094, 2.668110016739958, 2.7887319852039063, 2.9093539536678548, 3.0299759221318032, 3.1505978905957517, 3.2712198590597, 3.448013616432819, 3.624807373805938, 3.8016011311790567, 3.9783948885521756, 4.1551886459252945, 4.331982403298413, 4.626336417410132, 4.92069043152185, 5.215044445633568, 5.509398459745286, 5.8037524738570045, 6.098106487968723, 6.622283380829749, 7.146460273690776, 7.670637166551803, 8.19481405941283, 8.718990952273856, 9.946579410090706, 10.0]</t>
+          <t>[0.0, 5.949206695156695e-07, 1.189841339031339e-06, 7.139048034188033e-06, 1.3088254729344728e-05, 3.089656686164719e-05, 4.8704878993949655e-05, 6.651319112625212e-05, 0.00011053679980718213, 0.00015456040848811213, 0.00019858401716904214, 0.00041505244622941443, 0.0006315208752897867, 0.000847989304350159, 0.0016784213712643047, 0.0025088534381784502, 0.0033392855050925958, 0.004169717572006741, 0.005782090361472542, 0.007394463150938343, 0.009006835940404145, 0.010619208729869947, 0.01223158151933575, 0.01755662975138012, 0.022881677983424487, 0.028206726215468856, 0.03353177444751322, 0.03885682267955759, 0.046253624096727106, 0.05365042551389662, 0.06104722693106614, 0.06844402834823565, 0.07584082976540517, 0.08323763118257468, 0.09112604487375935, 0.09901445856494401, 0.10690287225612867, 0.11327546101976312, 0.11964804978339756, 0.126020638547032, 0.13239322731066644, 0.13876581607430089, 0.14527747927024626, 0.15178914246619163, 0.158300805662137, 0.16481246885808237, 0.17132413205402774, 0.17783579524997312, 0.18386675662248442, 0.18989771799499572, 0.19592867936750702, 0.20195964074001832, 0.20799060211252962, 0.21414280304746997, 0.2202950039824103, 0.22644720491735065, 0.232599405852291, 0.23875160678723134, 0.24490380772217168, 0.2505268594348396, 0.2561499111475075, 0.26177296286017543, 0.26739601457284334, 0.27301906628551126, 0.2786421179981792, 0.28443268029855795, 0.2902232425989367, 0.2960138048993155, 0.3018043671996943, 0.30759492950007306, 0.31338549180045183, 0.3235334120536877, 0.33368133230692354, 0.3415282745222533, 0.3493752167375831, 0.35722215895291287, 0.36506910116824265, 0.3729160433835724, 0.38445529397186584, 0.39599454456015926, 0.40753379514845267, 0.4190730457367461, 0.4306122963250395, 0.4421515469133329, 0.45569433202517945, 0.469237117137026, 0.4827799022488725, 0.49632268736071905, 0.5098654724725655, 0.523408257584412, 0.5412383897135585, 0.5590685218427051, 0.5768986539718516, 0.5947287861009981, 0.6125589182301446, 0.6370443646076405, 0.6615298109851363, 0.6860152573626321, 0.710500703740128, 0.7349861501176238, 0.7725142804678948, 0.8100424108181659, 0.8475705411684369, 0.8850986715187079, 0.9226268018689789, 0.9698089350709698, 1.0169910682729606, 1.0641732014749514, 1.1113553346769423, 1.158537467878933, 1.214944844665161, 1.2713522214513888, 1.3277595982376167, 1.3841669750238446, 1.4405743518100724, 1.4969817285963003, 1.5770800362242132, 1.6571783438521261, 1.737276651480039, 1.817374959107952, 1.897473266735865, 2.00132892344557, 2.1051845801552744, 2.209040236864979, 2.3128958935746837, 2.4167515502843884, 2.520607206994093, 2.661493232398292, 2.8023792578024906, 2.9432652832066895, 3.0841513086108883, 3.225037334015087, 3.365923359419286, 3.555220391136062, 3.744517422852838, 3.9338144545696143, 4.1231114862863905, 4.312408518003167, 4.501705549719944, 4.716579334298278, 4.931453118876613, 5.1463269034549475, 5.361200688033282, 5.576074472611617, 5.790948257189951, 6.111534900964932, 6.432121544739912, 6.752708188514893, 7.073294832289873, 7.393881476064854, 7.714468119839834, 8.141300835084728, 8.568133550329621, 8.994966265574515, 9.421798980819409, 9.848631696064302, 10.0]</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>0.2991464599245831</v>
+        <v>0.5881225521416606</v>
       </c>
       <c r="D28" t="n">
         <v>9.81</v>
@@ -2309,13 +2309,13 @@
         <v>2</v>
       </c>
       <c r="L28" t="n">
-        <v>2.991464599245831</v>
+        <v>5.881225521416606</v>
       </c>
       <c r="M28" t="n">
-        <v>0.02234921431058936</v>
+        <v>0.005782216242443789</v>
       </c>
       <c r="N28" t="n">
-        <v>0.1117460715529468</v>
+        <v>0.02891108121221894</v>
       </c>
       <c r="O28" t="n">
         <v>19.57501567331031</v>
@@ -2345,11 +2345,11 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>[0.0, 5.951017677552405e-07, 1.190203535510481e-06, 7.141221213062886e-06, 1.3092238890615292e-05, 3.0905983989516844e-05, 4.8719729088418395e-05, 6.653347418731994e-05, 0.00011057094883918546, 0.000154608423491051, 0.00019864589814291652, 0.00041544531618901623, 0.000632244734235116, 0.0008490441522812157, 0.0016977580571497643, 0.002546471962018313, 0.0033951858668868616, 0.00424389977175541, 0.0058649744310133, 0.00748604909027119, 0.00910712374952908, 0.010728198408786969, 0.012349273068044859, 0.01793896931108704, 0.023528665554129222, 0.029118361797171404, 0.03470805804021358, 0.04029775428325576, 0.048029611240807735, 0.05576146819835971, 0.06349332515591169, 0.07122518211346367, 0.07895703907101564, 0.08668889602856762, 0.09413357449233176, 0.10157825295609589, 0.10902293141986003, 0.11646760988362416, 0.1239122883473883, 0.13135696681115244, 0.1378076631491422, 0.14425835948713195, 0.1507090558251217, 0.15715975216311145, 0.1636104485011012, 0.17006114483909096, 0.1763467549424446, 0.18263236504579822, 0.18891797514915185, 0.19349679899963323, 0.19807562285011462, 0.202654446700596, 0.2072332705510774, 0.2118120944015588, 0.2200540443051771, 0.224700689656602, 0.2293473350080269, 0.2339939803594518, 0.23864062571087669, 0.24328727106230158, 0.24793391641372647, 0.25337993500253836, 0.25882595359135024, 0.26427197218016213, 0.269717990768974, 0.2751640093577859, 0.2806100279465978, 0.28585596329289825, 0.2911018986391987, 0.2963478339854992, 0.30159376933179965, 0.3068397046781001, 0.3120856400244006, 0.3201521075136866, 0.32821857500297263, 0.33628504249225866, 0.3443515099815447, 0.3524179774708307, 0.3617453597346359, 0.3710727419984411, 0.3804001242622463, 0.3897275065260515, 0.3990548887898567, 0.40838227105366187, 0.41824770533872074, 0.4281131396237796, 0.4379785739088385, 0.44784400819389736, 0.45770944247895623, 0.4675748767640151, 0.47930684021008596, 0.4910388036561568, 0.5027707671022277, 0.5145027305482985, 0.5262346939943694, 0.5379666574404403, 0.5549182092705026, 0.571869761100565, 0.5888213129306273, 0.6057728647606897, 0.6227244165907521, 0.6477357283105909, 0.6727470400304297, 0.6977583517502686, 0.7227696634701074, 0.7477809751899462, 0.7760834366822535, 0.8043858981745609, 0.8326883596668682, 0.8609908211591755, 0.8892932826514828, 0.9226790433691101, 0.9560648040867374, 0.9894505648043648, 1.022836325521992, 1.0562220862396194, 1.096301965501784, 1.1363818447639487, 1.1764617240261133, 1.2165416032882779, 1.2566214825504425, 1.296701361812607, 1.3534844183049897, 1.4102674747973722, 1.4670505312897548, 1.5238335877821374, 1.58061664427452, 1.6373997007669026, 1.7017739160652945, 1.7661481313636864, 1.8305223466620784, 1.8948965619604703, 1.9592707772588622, 2.023644992557254, 2.1063976367643615, 2.189150280971469, 2.2719029251785763, 2.3546555693856837, 2.437408213592791, 2.5201608577998984, 2.6382329835854637, 2.756305109371029, 2.874377235156594, 2.9924493609421594, 3.1105214867277247, 3.22859361251329, 3.3952338191872387, 3.5618740258611874, 3.728514232535136, 3.895154439209085, 4.061794645883033, 4.2284348525569815, 4.492974906894636, 4.757514961232291, 5.022055015569945, 5.2865950699076, 5.5511351242452545, 5.815675178582909, 6.2761967505735115, 6.736718322564114, 7.197239894554716, 7.657761466545319, 8.118283038535921, 9.297563752261942, 10.0]</t>
+          <t>[0.0, 5.951017677552405e-07, 1.190203535510481e-06, 7.141221213062886e-06, 1.3092238890615292e-05, 3.09059839867918e-05, 4.8719729082968314e-05, 6.653347417914482e-05, 0.00011057094830448325, 0.00015460842242982168, 0.00019864589655516012, 0.0004154442680846075, 0.000632242639614055, 0.0008490410111435024, 0.001697023316121143, 0.0025450056210987834, 0.003392987926076424, 0.004240970231054065, 0.005860829396873031, 0.007480688562691996, 0.009100547728510962, 0.010720406894329928, 0.012340266060148894, 0.01785998472390468, 0.023379703387660468, 0.028899422051416254, 0.03441914071517204, 0.03993885937892783, 0.04752228812057948, 0.05510571686223113, 0.06268914560388278, 0.07027257434553442, 0.07785600308718607, 0.08543943182883772, 0.0929990297092784, 0.10055862758971908, 0.10811822547015976, 0.11567782335060044, 0.12323742123104112, 0.1303810115879818, 0.13752460194492247, 0.14466819230186315, 0.15181178265880382, 0.1589553730157445, 0.16609896337268518, 0.1729484470373888, 0.1797979307020924, 0.18664741436679602, 0.19349689803149964, 0.20034638169620325, 0.20719586536090687, 0.21385713858020333, 0.2205184117994998, 0.22717968501879626, 0.23384095823809273, 0.2405022314573892, 0.24716350467668566, 0.2521320249999463, 0.2571005453232069, 0.26206906564646754, 0.26703758596972815, 0.27200610629298877, 0.2769746266162494, 0.28328281484689705, 0.2895910030775447, 0.29589919130819237, 0.30220737953884, 0.3085155677694877, 0.31482375600013535, 0.32406679122098725, 0.33330982644183915, 0.34255286166269105, 0.35179589688354296, 0.36103893210439486, 0.3705345899618054, 0.3800302478192159, 0.3895259056766264, 0.39902156353403695, 0.40851722139144747, 0.418012879248858, 0.4302686364357399, 0.44252439362262186, 0.4547801508095038, 0.4670359079963857, 0.47929166518326766, 0.4915474223701496, 0.5081299240972547, 0.5247124258243597, 0.5412949275514648, 0.5578774292785699, 0.5744599310056749, 0.5982245559889052, 0.6219891809721355, 0.6457538059553658, 0.6695184309385961, 0.6932830559218264, 0.7278592772845788, 0.7624354986473312, 0.7970117200100836, 0.831587941372836, 0.8661641627355884, 0.9029840196458736, 0.9398038765561588, 0.976623733466444, 1.0134435903767294, 1.0502634472870147, 1.1103692138358865, 1.1704749803847583, 1.23058074693363, 1.2906865134825019, 1.3507922800313736, 1.4108980465802454, 1.4773463780343001, 1.5437947094883548, 1.6102430409424096, 1.6766913723964643, 1.743139703850519, 1.8461776906808296, 1.9492156775111402, 2.0522536643414506, 2.155291651171761, 2.2583296380020714, 2.361367624832382, 2.4898319671550877, 2.6182963094777936, 2.7467606518004994, 2.8752249941232053, 3.003689336445911, 3.132153678768617, 3.2801298649738353, 3.4281060511790535, 3.576082237384272, 3.72405842358949, 3.8720346097947083, 4.0200107959999265, 4.2555277128170035, 4.4910446296340805, 4.7265615464511574, 4.962078463268234, 5.197595380085311, 5.433112296902388, 5.717025924390912, 6.000939551879435, 6.284853179367959, 6.568766806856482, 6.852680434345006, 7.136594061833529, 7.524717694615871, 7.912841327398214, 8.300964960180556, 8.689088592962898, 9.07721222574524, 9.465335858527583, 10.0]</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>0.2988242846986245</v>
+        <v>0.5793214388330745</v>
       </c>
       <c r="D29" t="n">
         <v>9.81</v>
@@ -2376,13 +2376,13 @@
         <v>2</v>
       </c>
       <c r="L29" t="n">
-        <v>2.988242846986245</v>
+        <v>5.793214388330745</v>
       </c>
       <c r="M29" t="n">
-        <v>0.02239743157437252</v>
+        <v>0.005959238874777518</v>
       </c>
       <c r="N29" t="n">
-        <v>0.1119871578718626</v>
+        <v>0.02979619437388759</v>
       </c>
       <c r="O29" t="n">
         <v>19.56310133970982</v>
@@ -2412,11 +2412,11 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>[0.0, 5.95331064962098e-07, 1.190662129924196e-06, 7.143972779545177e-06, 1.3097283429166157e-05, 3.091790747224531e-05, 4.8738531515324456e-05, 6.655915555840361e-05, 0.00011061418617084459, 0.00015466921678328557, 0.00019872424739572655, 0.0004159433988700126, 0.0006331625503442986, 0.0008503817018185847, 0.0017242367196518105, 0.002598091737485036, 0.0034719467553182616, 0.004345801773151487, 0.005978652446736619, 0.007611503120321751, 0.009244353793906883, 0.010877204467492015, 0.012510055141077147, 0.018440249516943827, 0.024370443892810505, 0.030300638268677182, 0.03623083264454386, 0.04216102702041054, 0.05024266033796647, 0.0583242936555224, 0.06640592697307833, 0.07448756029063426, 0.08256919360819019, 0.09065082692574612, 0.09800181379280841, 0.1053528006598707, 0.11270378752693298, 0.12005477439399527, 0.12740576126105757, 0.13475674812811989, 0.141203250496812, 0.14764975286550414, 0.15409625523419626, 0.1605427576028884, 0.1669892599715805, 0.17343576234027264, 0.17929668397737167, 0.1851576056144707, 0.19101852725156973, 0.19687944888866876, 0.2027403705257678, 0.20934320582822596, 0.21594604113068414, 0.22023616567099966, 0.22452629021131518, 0.2288164147516307, 0.23310653929194622, 0.23739666383226174, 0.24168678837257726, 0.24697370861485632, 0.2522606288571354, 0.25754754909941446, 0.2628344693416935, 0.2681213895839726, 0.27340830982625164, 0.2786551029327063, 0.28390189603916094, 0.2891486891456156, 0.29439548225207024, 0.2996422753585249, 0.30488906846497954, 0.31514621555721284, 0.32540336264944614, 0.33263836208330466, 0.3398733615171632, 0.3471083609510217, 0.35434336038488023, 0.36157835981873876, 0.3700026989278142, 0.3784270380368896, 0.386851377145965, 0.39527571625504043, 0.40370005536411585, 0.41212439447319127, 0.4230593722731772, 0.4339943500731631, 0.44492932787314904, 0.45586430567313496, 0.4667992834731209, 0.4777342612731068, 0.4905954440323038, 0.5034566267915008, 0.5163178095506978, 0.5291789923098948, 0.5420401750690919, 0.5549013578282889, 0.5739580353287357, 0.5930147128291825, 0.6120713903296293, 0.6311280678300761, 0.650184745330523, 0.6747005109763979, 0.6992162766222729, 0.7237320422681479, 0.7482478079140229, 0.7727635735598979, 0.8024177516055295, 0.8320719296511612, 0.8617261076967928, 0.8913802857424244, 0.9210344637880561, 0.9559249107005343, 0.9908153576130125, 1.0257058045254908, 1.060596251437969, 1.0954866983504472, 1.1343726906360858, 1.1732586829217244, 1.212144675207363, 1.2510306674930016, 1.2899166597786402, 1.3288026520642788, 1.3880435291456963, 1.4472844062271137, 1.5065252833085312, 1.5657661603899486, 1.625007037471366, 1.6842479145527836, 1.7573097748967048, 1.830371635240626, 1.9034334955845473, 1.9764953559284686, 2.04955721627239, 2.122619076616311, 2.2187771866170833, 2.314935296617856, 2.4110934066186283, 2.5072515166194007, 2.603409626620173, 2.6995677366209456, 2.824982330071167, 2.9503969235213887, 3.0758115169716103, 3.201226110421832, 3.3266407038720534, 3.452055297322275, 3.6279064873586284, 3.803757677394982, 3.9796088674313355, 4.155460057467689, 4.3313112475040425, 4.507162437540396, 4.781666909274912, 5.0561713810094275, 5.330675852743943, 5.605180324478459, 5.879684796212975, 6.1541892679474905, 6.646603166354995, 7.1390170647625, 7.631430963170005, 8.12384486157751, 8.616258759985016, 9.931452545364298, 10.0]</t>
+          <t>[0.0, 5.95331064962098e-07, 1.190662129924196e-06, 7.143972779545177e-06, 1.3097283429166157e-05, 3.091790746959021e-05, 4.8738531510014264e-05, 6.655915555043832e-05, 0.00011061418563830342, 0.0001546692157261685, 0.00019872424581403357, 0.0004159423445660842, 0.0006331604433181348, 0.0008503785420701854, 0.0017233894257766681, 0.002596400309483151, 0.003469411193189634, 0.0043424220768961165, 0.005973979174262659, 0.007605536271629201, 0.009237093368995744, 0.010868650466362286, 0.012500207563728829, 0.018334586903023017, 0.024168966242317208, 0.0300033455816114, 0.03583772492090559, 0.04167210426019978, 0.04956103022807375, 0.05744995619594773, 0.0653388821638217, 0.07322780813169566, 0.08111673409956963, 0.08900566006744359, 0.09644722892954363, 0.10388879779164367, 0.11133036665374371, 0.11877193551584375, 0.1262135043779438, 0.13365507324004383, 0.14016357454693595, 0.14667207585382808, 0.1531805771607202, 0.15968907846761232, 0.16619757977450444, 0.17270608108139657, 0.17868540764868612, 0.18466473421597568, 0.19064406078326523, 0.1966233873505548, 0.20260271391784435, 0.20857283476739918, 0.21454295561695402, 0.22051307646650886, 0.2264831973160637, 0.23245331816561854, 0.23842343901517338, 0.24394553946122846, 0.24946763990728354, 0.25498974035333866, 0.26051184079939377, 0.2660339412454489, 0.271556041691504, 0.277359041336148, 0.28316204098079206, 0.2889650406254361, 0.29476804027008013, 0.30057103991472417, 0.3063740395593682, 0.31779741987893745, 0.3267474115640642, 0.335697403249191, 0.3446473949343178, 0.35359738661944456, 0.36254737830457134, 0.37255127210859645, 0.38255516591262156, 0.3925590597166467, 0.4025629535206718, 0.4125668473246969, 0.422570741128722, 0.43533071730705336, 0.4480906934853847, 0.4608506696637161, 0.47361064584204743, 0.4863706220203788, 0.49913059819871014, 0.5149849290971585, 0.5308392599956069, 0.5466935908940552, 0.5625479217925036, 0.5784022526909519, 0.6022976967112346, 0.6261931407315172, 0.6500885847517999, 0.6739840287720825, 0.6978794727923652, 0.7325525561984282, 0.7672256396044912, 0.8018987230105542, 0.8365718064166172, 0.8712448898226802, 0.9083937074855755, 0.9455425251484707, 0.9826913428113659, 1.0198401604742613, 1.0569889781371566, 1.1170203023782532, 1.1770516266193498, 1.2370829508604464, 1.297114275101543, 1.3571455993426396, 1.4171769235837361, 1.4840402953932252, 1.5509036672027143, 1.6177670390122034, 1.6846304108216925, 1.7514937826311816, 1.8552479370020338, 1.959002091372886, 2.0627562457437385, 2.166510400114591, 2.2702645544854434, 2.374018708856296, 2.503274743710057, 2.632530778563818, 2.761786813417579, 2.89104284827134, 3.020298883125101, 3.149554917978862, 3.298455799783234, 3.447356681587606, 3.596257563391978, 3.74515844519635, 3.894059327000722, 4.042960208805094, 4.279962995035639, 4.516965781266184, 4.753968567496729, 4.990971353727274, 5.227974139957819, 5.464976926188364, 5.750792751662, 6.0366085771356355, 6.322424402609271, 6.608240228082907, 6.894056053556542, 7.179871879030178, 7.570645652371523, 7.961419425712868, 8.352193199054213, 8.742966972395557, 9.133740745736901, 9.524514519078245, 10.0]</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>0.298417252320771</v>
+        <v>0.5690365453868939</v>
       </c>
       <c r="D30" t="n">
         <v>9.81</v>
@@ -2443,13 +2443,13 @@
         <v>2</v>
       </c>
       <c r="L30" t="n">
-        <v>2.98417252320771</v>
+        <v>5.690365453868938</v>
       </c>
       <c r="M30" t="n">
-        <v>0.02245857212215322</v>
+        <v>0.006176602849555329</v>
       </c>
       <c r="N30" t="n">
-        <v>0.1122928606107661</v>
+        <v>0.03088301424777664</v>
       </c>
       <c r="O30" t="n">
         <v>19.54803143269989</v>
@@ -2479,11 +2479,11 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>[0.0, 5.956214680830018e-07, 1.1912429361660037e-06, 7.147457616996022e-06, 1.310367229782604e-05, 3.0933008481037457e-05, 4.8762344664248874e-05, 6.659168084746029e-05, 0.00011066894635610388, 0.00015474621186474746, 0.00019882347737339105, 0.00041657741246989955, 0.0006343313475664081, 0.0008520852826629165, 0.001763712530165714, 0.0026753397776685117, 0.0035869670251713094, 0.004498594272674107, 0.006150826448041568, 0.007803058623409029, 0.009455290798776491, 0.011107522974143953, 0.012759755149511415, 0.019358231520236333, 0.02595670789096125, 0.032555184261686174, 0.039153660632411096, 0.04575213700313602, 0.05454846833751511, 0.0633447996718942, 0.07214113100627328, 0.08093746234065237, 0.08973379367503145, 0.09853012500941054, 0.10579673154644895, 0.11306333808348736, 0.12032994462052576, 0.1275965511575642, 0.1348631576946026, 0.14212976423164103, 0.1486079348080971, 0.15508610538455314, 0.1615642759610092, 0.16804244653746525, 0.1745206171139213, 0.18099878769037736, 0.18616382404486878, 0.1913288603993602, 0.19649389675385162, 0.20165893310834304, 0.20682396946283446, 0.21198900581732588, 0.2176203061790851, 0.2232516065408443, 0.22888290690260352, 0.23451420726436273, 0.24014550762612194, 0.24577680798788115, 0.2520203138406651, 0.258263819693449, 0.26450732554623296, 0.2707508313990169, 0.27699433725180084, 0.2832378431045848, 0.2881945464313923, 0.29315124975819984, 0.29810795308500737, 0.3030646564118149, 0.30802135973862244, 0.31297806306542997, 0.320351287889713, 0.32772451271399605, 0.3350977375382791, 0.34247096236256214, 0.3498441871868452, 0.35706121714469513, 0.3642782471025451, 0.37149527706039503, 0.378712307018245, 0.38592933697609494, 0.3931463669339449, 0.40283794056687117, 0.41252951419979744, 0.4222210878327237, 0.43191266146565, 0.44160423509857627, 0.45129580873150255, 0.4635095915490307, 0.47572337436655887, 0.48793715718408703, 0.5001509400016152, 0.5123647228191434, 0.5245785056366715, 0.5413274037207496, 0.5580763018048277, 0.5748251998889058, 0.5915740979729839, 0.608322996057062, 0.6332744974633627, 0.6582259988696635, 0.6831775002759642, 0.708129001682265, 0.7330805030885658, 0.7613965378627388, 0.7897125726369117, 0.8180286074110847, 0.8463446421852577, 0.8746606769594307, 0.9084509840757283, 0.9422412911920259, 0.9760315983083235, 1.0098219054246211, 1.0436122125409186, 1.0837266207278593, 1.1238410289148, 1.1639554371017407, 1.2040698452886813, 1.244184253475622, 1.2842986616625627, 1.341186274831662, 1.3980738880007615, 1.454961501169861, 1.5118491143389603, 1.5687367275080597, 1.625624340677159, 1.6839390333661146, 1.7422537260550701, 1.8005684187440256, 1.8588831114329811, 1.9171978041219366, 1.9755124968108921, 2.059921922210222, 2.144331347609552, 2.228740773008882, 2.313150198408212, 2.397559623807542, 2.481969049206872, 2.59535376404792, 2.708738478888968, 2.822123193730016, 2.935507908571064, 3.048892623412112, 3.16227733825316, 3.3154441579516702, 3.4686109776501803, 3.6217777973486904, 3.7749446170472005, 3.9281114367457106, 4.081278256444221, 4.301983883933135, 4.5226895114220484, 4.743395138910962, 4.964100766399876, 5.18480639388879, 5.405512021377704, 5.762938336907958, 6.120364652438211, 6.477790967968465, 6.835217283498719, 7.1926435990289725, 8.89089876034548, 10.0]</t>
+          <t>[0.0, 5.956214680830018e-07, 1.1912429361660037e-06, 7.147457616996022e-06, 1.310367229782604e-05, 3.093300847847101e-05, 4.876234465911598e-05, 6.659168083976094e-05, 0.00011066894582630225, 0.00015474621081284357, 0.00019882347579938488, 0.0004165763502250259, 0.0006343292246506669, 0.0008520820990763078, 0.001762670672470081, 0.0026732592458638543, 0.0035838478192576277, 0.004494436392651401, 0.006145238312321234, 0.007796040231991067, 0.0094468421516609, 0.011097644071330733, 0.012748445991000567, 0.019180384109018855, 0.025612322227037142, 0.032044260345055434, 0.03847619846307372, 0.04490813658109201, 0.05339715638482614, 0.061886176188560266, 0.07037519599229439, 0.07886421579602851, 0.08735323559976263, 0.09584225540349675, 0.10317633263097968, 0.11051040985846261, 0.11784448708594554, 0.12517856431342847, 0.1325126415409114, 0.13984671876839436, 0.14637651255062084, 0.15290630633284732, 0.1594361001150738, 0.1659658938973003, 0.17249568767952678, 0.17902548146175326, 0.1844721508339723, 0.18991882020619136, 0.1953654895784104, 0.20081215895062945, 0.2062588283228485, 0.21216049336359366, 0.21806215840433882, 0.22396382344508398, 0.22986548848582913, 0.2357671535265743, 0.24166881856731945, 0.24764112744535755, 0.2536134363233956, 0.2595857452014337, 0.26555805407947175, 0.2715303629575098, 0.2775026718355479, 0.28322113757390693, 0.288939603312266, 0.294658069050625, 0.3003765347889841, 0.3060950005273431, 0.31181346626570217, 0.31964399131198995, 0.32747451635827773, 0.3353050414045655, 0.3431355664508533, 0.3509660914971411, 0.36027819871294525, 0.3695903059287494, 0.3789024131445536, 0.38821452036035775, 0.3975266275761619, 0.4068387347919661, 0.41834957920724947, 0.42986042362253285, 0.44137126803781623, 0.4528821124530996, 0.464392956868383, 0.4759038012836664, 0.4919525485827266, 0.5080012958817868, 0.524050043180847, 0.5400987904799073, 0.5561475377789675, 0.5721962850780278, 0.594888363035098, 0.6175804409921681, 0.6402725189492383, 0.6629645969063085, 0.6856566748633787, 0.7198958387765193, 0.7541350026896599, 0.7883741666028006, 0.8226133305159412, 0.8568524944290818, 0.8934229760827734, 0.929993457736465, 0.9665639393901566, 1.0031344210438482, 1.0397049026975398, 1.0990600593648838, 1.1584152160322279, 1.217770372699572, 1.277125529366916, 1.33648068603426, 1.395835842701604, 1.4615764292981985, 1.527317015894793, 1.5930576024913876, 1.6587981890879822, 1.7245387756845767, 1.8279945059937002, 1.9314502363028236, 2.034905966611947, 2.138361696921071, 2.2418174272301945, 2.345273157539318, 2.451988913806541, 2.558704670073764, 2.665420426340987, 2.77213618260821, 2.878851938875433, 2.985567695142656, 3.1398977411202655, 3.294227787097875, 3.4485578330754847, 3.6028878790530943, 3.757217925030704, 3.9115479710083134, 4.122285717663795, 4.333023464319276, 4.543761210974758, 4.754498957630239, 4.96523670428572, 5.175974450941202, 5.490795418160398, 5.805616385379595, 6.120437352598791, 6.435258319817987, 6.750079287037184, 7.06490025425638, 7.437711017493068, 7.810521780729755, 8.183332543966443, 8.556143307203133, 8.928954070439822, 9.301764833676511, 9.814963631781977, 10.0]</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>0.2979028590318865</v>
+        <v>0.5571797818247779</v>
       </c>
       <c r="D31" t="n">
         <v>9.81</v>
@@ -2510,13 +2510,13 @@
         <v>2</v>
       </c>
       <c r="L31" t="n">
-        <v>2.979028590318864</v>
+        <v>5.571797818247779</v>
       </c>
       <c r="M31" t="n">
-        <v>0.02253619818311309</v>
+        <v>0.006442275567225818</v>
       </c>
       <c r="N31" t="n">
-        <v>0.1126809909155655</v>
+        <v>0.03221137783612909</v>
       </c>
       <c r="O31" t="n">
         <v>19.52897018220085</v>
@@ -2546,11 +2546,11 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>[0.0, 5.9598938799805e-07, 1.1919787759961e-06, 7.1518726559766e-06, 1.31117665359571e-05, 3.095214039330037e-05, 4.879251425064364e-05, 6.66328881079869e-05, 0.0001107383242911502, 0.0001548437604743135, 0.0001989491966574768, 0.00041738585934534585, 0.0006358225220332149, 0.0008542591847210839, 0.0018279101297022037, 0.0028015610746833235, 0.0037752120196644433, 0.004748862964645563, 0.0064357874228723015, 0.00812271188109904, 0.00980963633932578, 0.011496560797552518, 0.013183485255779257, 0.021848794069375763, 0.03051410288297227, 0.03917941169656877, 0.04784472051016528, 0.056510029323761785, 0.06531986025828099, 0.07412969119280019, 0.08293952212731939, 0.0917493530618386, 0.1005591839963578, 0.109369014930877, 0.11651295130715539, 0.12365688768343377, 0.13080082405971216, 0.13794476043599055, 0.14508869681226894, 0.15223263318854732, 0.15923339689041538, 0.16623416059228344, 0.1732349242941515, 0.1783827508925879, 0.1835305774910243, 0.1886784040894607, 0.19382623068789712, 0.19897405728633352, 0.20412188388476993, 0.21022541206462514, 0.21632894024448035, 0.22243246842433556, 0.22853599660419077, 0.23463952478404598, 0.2407430529639012, 0.24643475126009823, 0.25212644955629526, 0.2578181478524923, 0.26350984614868933, 0.26920154444488636, 0.2748932427410834, 0.2803142349146144, 0.28573522708814536, 0.29115621926167634, 0.2965772114352073, 0.3019982036087383, 0.3074191957822693, 0.31485399672744824, 0.3222887976726272, 0.32972359861780615, 0.3371583995629851, 0.34459320050816405, 0.35203906679550834, 0.3594849330828526, 0.3669307993701969, 0.3743766656575412, 0.38182253194488547, 0.38926839823222975, 0.39893674395431056, 0.40860508967639136, 0.41827343539847217, 0.427941781120553, 0.4376101268426338, 0.4472784725647146, 0.4596374795079953, 0.47199648645127595, 0.48435549339455664, 0.4967145003378373, 0.509073507281118, 0.5214325142243987, 0.538707704484922, 0.5559828947454453, 0.5732580850059685, 0.5905332752664918, 0.6078084655270151, 0.633254085489968, 0.6586997054529209, 0.6841453254158738, 0.7095909453788267, 0.7350365653417796, 0.7638688897920831, 0.7927012142423866, 0.8215335386926901, 0.8503658631429936, 0.879198187593297, 0.9137240216104187, 0.9482498556275403, 0.9827756896446619, 1.0173015236617835, 1.051827357678905, 1.09043980964081, 1.1290522616027152, 1.1676647135646203, 1.2062771655265254, 1.2448896174884305, 1.2835020694503356, 1.3399358206035292, 1.3963695717567228, 1.4528033229099164, 1.50923707406311, 1.5656708252163036, 1.6221045763694972, 1.6932102715451995, 1.7643159667209019, 1.8354216618966042, 1.9065273570723065, 1.9776330522480088, 2.048738747423711, 2.141769058877562, 2.234799370331413, 2.3278296817852637, 2.4208599932391146, 2.5138903046929655, 2.6069206161468164, 2.7262203967780523, 2.845520177409288, 2.964819958040524, 3.08411973867176, 3.203419519302996, 3.322719299934232, 3.48146208301409, 3.640204866093948, 3.798947649173806, 3.957690432253664, 4.116433215333522, 4.275175998413381, 4.50047906536624, 4.7257821323190985, 4.951085199271957, 5.176388266224816, 5.401691333177674, 5.626994400130533, 5.98577519338405, 6.344555986637568, 6.703336779891085, 7.062117573144603, 7.42089836639812, 7.7796791596516375, 8.433825740119728, 9.087972320587818, 9.742118901055909, 10.0]</t>
+          <t>[0.0, 5.9598938799805e-07, 1.1919787759961e-06, 7.1518726559766e-06, 1.31117665359571e-05, 3.09521403908463e-05, 4.8792514245735496e-05, 6.663288810062469e-05, 0.00011073832376481984, 0.000154843759429015, 0.00019894919509321016, 0.00041738478689668174, 0.0006358203787001533, 0.0008542559705036249, 0.001826473222294287, 0.002798690474084949, 0.0037709077258756113, 0.004743124977666274, 0.006428341956958664, 0.008113558936251054, 0.009798775915543444, 0.011483992894835834, 0.013169209874128224, 0.0213991971834412, 0.02962918449275418, 0.03785917180206716, 0.04608915911138014, 0.05431914642069312, 0.06332592473275349, 0.07233270304481386, 0.08133948135687423, 0.0903462596689346, 0.09764134384505929, 0.10493642802118398, 0.11223151219730867, 0.11952659637343337, 0.12682168054955806, 0.13411676472568274, 0.1406055875325877, 0.14709441033949266, 0.15358323314639763, 0.1600720559533026, 0.16656087876020756, 0.17304970156711252, 0.17875128417768654, 0.18445286678826056, 0.19015444939883458, 0.1958560320094086, 0.20155761461998262, 0.2077368509957374, 0.2139160873714922, 0.220095323747247, 0.2262745601230018, 0.23245379649875658, 0.23863303287451137, 0.2445264973340429, 0.25041996179357445, 0.256313426253106, 0.26220689071263753, 0.26810035517216907, 0.2739938196317006, 0.2797161182144794, 0.2854384167972582, 0.29116071538003696, 0.29688301396281574, 0.30260531254559453, 0.3083276111283733, 0.3161909031947113, 0.32405419526104934, 0.33191748732738735, 0.33978077939372536, 0.3476440714600634, 0.35693989662782444, 0.3662357217955855, 0.37553154696334656, 0.3848273721311076, 0.3941231972988687, 0.40341902246662975, 0.41494522093798103, 0.4264714194093323, 0.4379976178806836, 0.44952381635203487, 0.46105001482338615, 0.4725762132947374, 0.4886634165594803, 0.5047506198242232, 0.5208378230889661, 0.536925026353709, 0.5530122296184519, 0.5690994328831948, 0.5917941057592337, 0.6144887786352727, 0.6371834515113117, 0.6598781243873507, 0.6825727972633897, 0.7167482507227754, 0.750923704182161, 0.7850991576415467, 0.8192746111009324, 0.853450064560318, 0.8899043865605153, 0.9263587085607126, 0.9628130305609098, 0.9992673525611071, 1.0357216745613043, 1.0949475079560589, 1.1541733413508135, 1.2133991747455681, 1.2726250081403228, 1.3318508415350774, 1.391076674929832, 1.456631284663923, 1.5221858943980142, 1.5877405041321053, 1.6532951138661964, 1.7188497236002875, 1.821990132591995, 1.9251305415837023, 2.0282709505754095, 2.1314113595671165, 2.2345517685588234, 2.3376921775505304, 2.4441212024296566, 2.550550227308783, 2.656979252187909, 2.763408277067035, 2.8698373019461614, 2.9762663268252876, 3.1302310991841664, 3.2841958715430453, 3.438160643901924, 3.592125416260803, 3.746090188619682, 3.9000549609785606, 4.133980978248544, 4.367906995518527, 4.60183301278851, 4.835759030058493, 5.069685047328476, 5.303611064598459, 5.591099429130798, 5.878587793663137, 6.166076158195477, 6.453564522727816, 6.741052887260155, 7.028541251792494, 7.46045037909375, 7.892359506395006, 8.324268633696262, 8.756177760997517, 9.188086888298772, 9.619996015600027, 10.0]</t>
         </is>
       </c>
       <c r="C32" t="n">
-        <v>0.2972517737757087</v>
+        <v>0.5437081355180632</v>
       </c>
       <c r="D32" t="n">
         <v>9.81</v>
@@ -2577,13 +2577,13 @@
         <v>2</v>
       </c>
       <c r="L32" t="n">
-        <v>2.972517737757086</v>
+        <v>5.437081355180632</v>
       </c>
       <c r="M32" t="n">
-        <v>0.02263503060160117</v>
+        <v>0.006765475611947775</v>
       </c>
       <c r="N32" t="n">
-        <v>0.1131751530080058</v>
+        <v>0.03382737805973887</v>
       </c>
       <c r="O32" t="n">
         <v>19.50486046006736</v>
@@ -2613,11 +2613,11 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>[0.0, 5.964557196075114e-07, 1.1929114392150228e-06, 7.157468635290138e-06, 1.3122025831365253e-05, 3.097638976267404e-05, 4.883075369398283e-05, 6.668511762529162e-05, 0.00011082626066545523, 0.00015496740370561884, 0.00019910854674578247, 0.00041841904049549645, 0.0006377295342452104, 0.0008570400279949244, 0.0019530408746054966, 0.003049041721216069, 0.004145042567826641, 0.0052410434144372145, 0.007001585350075514, 0.008762127285713813, 0.010522669221352112, 0.01228321115699041, 0.01404375309262871, 0.02095970575595512, 0.02787565841928153, 0.03479161108260794, 0.04170756374593435, 0.04862351640926076, 0.05732992690498316, 0.06603633740070555, 0.07474274789642794, 0.08344915839215034, 0.09215556888787273, 0.10086197938359512, 0.1079926475177435, 0.11512331565189188, 0.12225398378604026, 0.12938465192018864, 0.13651532005433703, 0.14364598818848542, 0.15013077777100392, 0.15661556735352242, 0.1631003569360409, 0.1695851465185594, 0.1760699361010779, 0.1825547256835964, 0.18780355881085625, 0.1930523919381161, 0.19830122506537595, 0.2035500581926358, 0.20879889131989565, 0.2140477244471555, 0.2196551887759488, 0.2252626531047421, 0.23087011743353542, 0.23647758176232872, 0.24208504609112202, 0.2481572910222081, 0.2542295359532942, 0.2603017808843803, 0.2663740258154664, 0.2724462707465525, 0.2785185156776386, 0.2844052963862142, 0.2902920770947898, 0.29617885780336545, 0.30206563851194107, 0.3079524192205167, 0.3138391999290923, 0.3212828625939717, 0.3287265252588511, 0.3361701879237305, 0.3436138505886099, 0.3510575132534893, 0.35850117591836866, 0.3669017242615714, 0.37530227260477417, 0.3837028209479769, 0.39210336929117967, 0.4005039176343824, 0.4089044659775852, 0.4178165009488211, 0.42672853592005705, 0.435640570891293, 0.4445526058625289, 0.45346464083376486, 0.4623766758050008, 0.4750034303215754, 0.48763018483814996, 0.5002569393547245, 0.5128836938712991, 0.5255104483878736, 0.5458753638494223, 0.5662402793109709, 0.5866051947725195, 0.6069701102340681, 0.6273350256956167, 0.6547041066380624, 0.6820731875805082, 0.7094422685229539, 0.7368113494653996, 0.7641804304078453, 0.7949454873846985, 0.8257105443615517, 0.8564756013384048, 0.887240658315258, 0.9180057152921112, 0.9556739123205585, 0.9933421093490059, 1.0310103063774534, 1.0686785034059008, 1.1063467004343481, 1.1440148974627955, 1.194966038418882, 1.2459171793749686, 1.2968683203310551, 1.3478194612871417, 1.3987706022432282, 1.4497217431993148, 1.5023614487869532, 1.5550011543745916, 1.60764085996223, 1.6602805655498685, 1.712920271137507, 1.7655599767251453, 1.8397351083733027, 1.91391024002146, 1.9880853716696174, 2.0622605033177748, 2.136435634965932, 2.210610766614089, 2.311997630017918, 2.413384493421747, 2.5147713568255763, 2.6161582202294054, 2.7175450836332344, 2.8189319470370635, 2.950276676954555, 3.081621406872047, 3.2129661367895386, 3.3443108667070303, 3.475655596624522, 3.6070003265420136, 3.781145259406137, 3.9552901922702604, 4.129435125134384, 4.3035800579985075, 4.477724990862631, 4.651869923726755, 4.896960522957434, 5.1420511221881124, 5.387141721418791, 5.63223232064947, 5.877322919880148, 6.122413519110827, 6.507887630857723, 6.893361742604618, 7.278835854351514, 7.6643099660984095, 8.049784077845306, 8.435258189592203, 9.13428301253933, 9.833307835486456, 10.0]</t>
+          <t>[0.0, 5.964557196075114e-07, 1.1929114392150228e-06, 7.157468635290138e-06, 1.3122025831365253e-05, 3.09763897603625e-05, 4.883075368935974e-05, 6.668511761835698e-05, 0.00011082626014352877, 0.00015496740266870057, 0.00019910854519387237, 0.00041841795487560266, 0.0006377273645573329, 0.0008570367742390632, 0.0019504836267643941, 0.003043930479289725, 0.004137377331815056, 0.005230824184340387, 0.006988891286910877, 0.008746958389481366, 0.010505025492051855, 0.012263092594622344, 0.014021159697192833, 0.021193406293004244, 0.028365652888815655, 0.035537899484627065, 0.04271014608043848, 0.049882392676249894, 0.0586974261495974, 0.06751245962294491, 0.07632749309629243, 0.08514252656963994, 0.09395756004298746, 0.10277259351633497, 0.10995388458860283, 0.1171351756608707, 0.12431646673313856, 0.13149775780540643, 0.1386790488776743, 0.14586033994994216, 0.15240644704477635, 0.15895255413961054, 0.16549866123444473, 0.17204476832927892, 0.17859087542411312, 0.1851369825189473, 0.19051861307208653, 0.19590024362522576, 0.201281874178365, 0.20666350473150422, 0.21204513528464344, 0.21742676583778267, 0.22387400835831256, 0.23032125087884245, 0.23676849339937234, 0.24103500628812297, 0.2453015191768736, 0.24956803206562422, 0.25383454495437485, 0.2581010578431255, 0.26366254799020206, 0.26922403813727863, 0.2747855282843552, 0.2803470184314318, 0.28693540136877205, 0.2935237843061123, 0.3001121672434526, 0.30670055018079284, 0.3132889331181331, 0.32450312829618466, 0.3357173234742362, 0.3469315186522878, 0.35814571383033933, 0.3693599090083909, 0.38057410418644244, 0.38942231579577474, 0.39827052740510704, 0.40711873901443935, 0.41596695062377165, 0.42481516223310395, 0.43366337384243625, 0.4496004470594447, 0.4655375202764531, 0.48147459349346156, 0.49741166671047, 0.5133487399274784, 0.5379532514037988, 0.5625577628801192, 0.5871622743564395, 0.6117667858327599, 0.6363712973090803, 0.6660184859294569, 0.6956656745498335, 0.7253128631702102, 0.7549600517905868, 0.7846072404109634, 0.8292571198149351, 0.8739069992189068, 0.9185568786228785, 0.9632067580268502, 1.0078566374308218, 1.0525065168347933, 1.1060294864254696, 1.1595524560161459, 1.2130754256068221, 1.2665983951974984, 1.3201213647881747, 1.373644334378851, 1.4438379218107433, 1.5140315092426357, 1.5842250966745282, 1.6544186841064206, 1.724612271538313, 1.7948058589702054, 1.8844521151799183, 1.9740983713896312, 2.063744627599344, 2.1533908838090565, 2.243037140018769, 2.332683396228482, 2.4656206665324185, 2.598557936836355, 2.731495207140292, 2.8644324774442285, 2.997369747748165, 3.1303070180521018, 3.2768699660592686, 3.4234329140664355, 3.5699958620736023, 3.716558810080769, 3.863121758087936, 4.009684706095102, 4.220719110430707, 4.431753514766312, 4.642787919101917, 4.853822323437521, 5.064856727773126, 5.275891132108731, 5.565527008638501, 5.855162885168271, 6.144798761698041, 6.4344346382278115, 6.724070514757582, 7.013706391287352, 7.404321188275722, 7.794935985264091, 8.185550782252461, 8.576165579240831, 8.9667803762292, 9.35739517321757, 9.882155888313102, 10.0]</t>
         </is>
       </c>
       <c r="C33" t="n">
-        <v>0.2964281696164348</v>
+        <v>0.5286314530324919</v>
       </c>
       <c r="D33" t="n">
         <v>9.81</v>
@@ -2644,13 +2644,13 @@
         <v>2</v>
       </c>
       <c r="L33" t="n">
-        <v>2.964281696164348</v>
+        <v>5.286314530324919</v>
       </c>
       <c r="M33" t="n">
-        <v>0.02276098491639689</v>
+        <v>0.007156884300345036</v>
       </c>
       <c r="N33" t="n">
-        <v>0.1138049245819845</v>
+        <v>0.03578442150172518</v>
       </c>
       <c r="O33" t="n">
         <v>19.47436515224987</v>
@@ -2680,11 +2680,11 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>[0.0, 5.970471135409412e-07, 1.1940942270818823e-06, 7.164565362491294e-06, 1.3135036497900705e-05, 3.100714245233332e-05, 4.887924840676593e-05, 6.675135436119855e-05, 0.00011093778193276994, 0.00015512420950434134, 0.00019931063707591274, 0.00041974325246278715, 0.0006401758678496616, 0.000860608483236536, 0.0024186454793745436, 0.0036422141733070423, 0.004865782867239541, 0.006089351561172041, 0.0073129202551045405, 0.009792822905220735, 0.01227272555533693, 0.014752628205453124, 0.01723253085556932, 0.019712433505685516, 0.02651081398652434, 0.03330919446736316, 0.04010757494820198, 0.0469059554290408, 0.05370433590987962, 0.06122359127726599, 0.06874284664465236, 0.07626210201203873, 0.0837813573794251, 0.09130061274681148, 0.0983067481632721, 0.10531288357973273, 0.11231901899619336, 0.11932515441265398, 0.12633128982911462, 0.13333742524557526, 0.13983594592277435, 0.14633446659997343, 0.1528329872771725, 0.1593315079543716, 0.16583002863157068, 0.17232854930876976, 0.17746655380524715, 0.18260455830172453, 0.18774256279820192, 0.1928805672946793, 0.1980185717911567, 0.2031565762876341, 0.2082104314894503, 0.21326428669126649, 0.21831814189308268, 0.22337199709489888, 0.22842585229671508, 0.23347970749853128, 0.23949617358833805, 0.24551263967814482, 0.2515291057679516, 0.2575455718577584, 0.26356203794756516, 0.26957850403737194, 0.27505088325022853, 0.2805232624630851, 0.2859956416759417, 0.2914680208887983, 0.2969404001016549, 0.3024127793145115, 0.3095441594673424, 0.31667553962017325, 0.32380691977300413, 0.330938299925835, 0.3380696800786659, 0.34543279168918045, 0.352795903299695, 0.3601590149102096, 0.36752212652072414, 0.3748852381312387, 0.38224834974175326, 0.3919946301327394, 0.4017409105237255, 0.41148719091471164, 0.42123347130569777, 0.4309797516966839, 0.44072603208767, 0.45375028048451554, 0.46677452888136106, 0.4797987772782066, 0.4928230256750521, 0.5058472740718976, 0.518871522468743, 0.5375117173849074, 0.5561519123010719, 0.5747921072172363, 0.5934323021334007, 0.6120724970495651, 0.6307126919657295, 0.6572433203159324, 0.6837739486661352, 0.710304577016338, 0.7368352053665408, 0.7633658337167436, 0.7944725695544057, 0.8255793053920678, 0.8566860412297299, 0.887792777067392, 0.9188995129050541, 0.953321554735269, 0.9877435965654839, 1.0221656383956987, 1.0565876802259135, 1.0910097220561283, 1.1441058224269078, 1.1972019227976873, 1.2502980231684668, 1.3033941235392463, 1.3564902239100258, 1.4095863242808053, 1.474176446604711, 1.5387665689286165, 1.6033566912525221, 1.6679468135764277, 1.7325369359003333, 1.797127058224239, 1.8794614791209092, 1.9617959000175795, 2.04413032091425, 2.12646474181092, 2.2087991627075905, 2.291133583604261, 2.386450008610851, 2.4817664336174414, 2.5770828586240317, 2.672399283630622, 2.7677157086372124, 2.8630321336438027, 2.985380940816362, 3.107729747988921, 3.23007855516148, 3.3524273623340393, 3.4747761695065984, 3.5971249766791575, 3.7548801533283735, 3.9126353299775896, 4.070390506626806, 4.228145683276022, 4.385900859925238, 4.543656036574454, 4.754219745034734, 4.964783453495015, 5.175347161955295, 5.385910870415575, 5.596474578875855, 5.807038287336136, 6.135610646761997, 6.464183006187858, 6.7927553656137185, 7.1213277250395794, 7.44990008446544, 7.778472443891301, 8.359470068689227, 8.940467693487152, 9.521465318285077, 10.0]</t>
+          <t>[0.0, 5.970471135409412e-07, 1.1940942270818823e-06, 7.164565362491294e-06, 1.3135036497900705e-05, 3.1007142450202685e-05, 4.8879248402504665e-05, 6.675135435480665e-05, 0.00011093778141643541, 0.00015512420847806416, 0.0001993106355396929, 0.00041974214974495165, 0.0006401736639502104, 0.0008606051781554692, 0.0024052261622529094, 0.003624440603532196, 0.004843655044811483, 0.00606286948609077, 0.0072820839273700574, 0.009759909840918611, 0.012237735754467165, 0.01471556166801572, 0.017193387581564273, 0.019671213495112826, 0.026642881156408102, 0.03361454881770338, 0.040586216478998655, 0.04755788414029393, 0.05452955180158921, 0.06220730478723571, 0.06988505777288222, 0.07756281075852872, 0.08524056374417523, 0.09291831672982173, 0.09997591792452895, 0.10703351911923617, 0.11409112031394339, 0.12114872150865061, 0.12820632270335783, 0.13526392389806505, 0.14184091960038528, 0.1484179153027055, 0.15499491100502574, 0.16157190670734597, 0.1681489024096662, 0.17472589811198644, 0.17992283131069203, 0.18511976450939763, 0.19031669770810322, 0.19551363090680882, 0.2007105641055144, 0.20590749730422, 0.2109734703004658, 0.21603944329671157, 0.22110541629295735, 0.22617138928920313, 0.23123736228544892, 0.2363033352816947, 0.24293560402103606, 0.24956787276037742, 0.2562001414997188, 0.26283241023906023, 0.26946467897840165, 0.27609694771774307, 0.2814181581599987, 0.28673936860225435, 0.29206057904451, 0.29738178948676564, 0.3027029999290213, 0.3114877558577526, 0.32027251178648397, 0.3290572677152153, 0.33784202364394667, 0.346626779572678, 0.35571981749514403, 0.36481285541761005, 0.37390589334007607, 0.3829989312625421, 0.3920919691850081, 0.4011850071074741, 0.41367534003880074, 0.42616567297012736, 0.438656005901454, 0.4511463388327806, 0.4636366717641072, 0.47612700469543384, 0.4936174468520955, 0.5111078890087573, 0.528598331165419, 0.5460887733220807, 0.5635792154787425, 0.5810696576354042, 0.6032616051808479, 0.6254535527262917, 0.6476455002717354, 0.6698374478171791, 0.6920293953626229, 0.728265033417769, 0.7645006714729152, 0.8007363095280614, 0.8369719475832076, 0.8732075856383538, 0.9104637335536903, 0.9477198814690267, 0.9849760293843632, 1.0222321772996996, 1.059488325215036, 1.1201091684244209, 1.1807300116338058, 1.2413508548431906, 1.3019716980525755, 1.3625925412619604, 1.4232133844713453, 1.490658095065872, 1.558102805660399, 1.6255475162549258, 1.6929922268494526, 1.7604369374439794, 1.8651155594656699, 1.9697941814873603, 2.0744728035090505, 2.1791514255307405, 2.2838300475524305, 2.3885086695741204, 2.51904063675596, 2.6495726039377994, 2.780104571119639, 2.9106365383014783, 3.0411685054833177, 3.171700472665157, 3.3236157153620165, 3.475530958058876, 3.627446200755735, 3.7793614434525944, 3.9312766861494537, 4.083191928846313, 4.32172173805771, 4.560251547269107, 4.798781356480505, 5.037311165691902, 5.275840974903299, 5.514370784114696, 5.804150215433951, 6.093929646753205, 6.383709078072459, 6.673488509391714, 6.963267940710968, 7.253047372030222, 7.649002629103216, 8.04495788617621, 8.440913143249205, 8.8368684003222, 9.232823657395194, 9.628778914468189, 10.0]</t>
         </is>
       </c>
       <c r="C34" t="n">
-        <v>0.2953866325093481</v>
+        <v>0.5120137083934897</v>
       </c>
       <c r="D34" t="n">
         <v>9.81</v>
@@ -2711,13 +2711,13 @@
         <v>2</v>
       </c>
       <c r="L34" t="n">
-        <v>2.953866325093481</v>
+        <v>5.120137083934897</v>
       </c>
       <c r="M34" t="n">
-        <v>0.02292177895597923</v>
+        <v>0.007628986005694798</v>
       </c>
       <c r="N34" t="n">
-        <v>0.1146088947798962</v>
+        <v>0.03814493002847399</v>
       </c>
       <c r="O34" t="n">
         <v>19.43579300306733</v>
@@ -2747,11 +2747,11 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>[0.0, 5.977976368016702e-07, 1.1955952736033404e-06, 7.173571641620042e-06, 1.3151548009636744e-05, 3.1046169995682814e-05, 4.8940791981728885e-05, 6.683541396777496e-05, 0.00011107931373092981, 0.00015532321349408468, 0.00019956711325723955, 0.0004214468664832747, 0.0006433266197093099, 0.000865206372935345, 0.0020639051587923365, 0.0032626039446493277, 0.004461302730506319, 0.00566000151636331, 0.007482113601415358, 0.009304225686467407, 0.011126337771519456, 0.012948449856571505, 0.014770561941623555, 0.020112551211458368, 0.02545454048129318, 0.030796529751127993, 0.03613851902096281, 0.04148050829079762, 0.05042942989939086, 0.059378351507984095, 0.06832727311657733, 0.07727619472517055, 0.08444085469003469, 0.09160551465489883, 0.09877017461976297, 0.1059348345846271, 0.11309949454949124, 0.12026415451435538, 0.1266290869896943, 0.13299401946503323, 0.13935895194037215, 0.14572388441571107, 0.15208881689105, 0.15845374936638892, 0.1642242961149089, 0.1699948428634289, 0.17576538961194887, 0.18153593636046886, 0.18730648310898884, 0.19377397009218772, 0.2002414570753866, 0.20450789490663565, 0.2087743327378847, 0.21304077056913376, 0.2173072084003828, 0.22157364623163187, 0.22584008406288092, 0.23125693126361024, 0.23667377846433957, 0.2420906256650689, 0.24750747286579822, 0.25292432006652754, 0.25834116726725687, 0.2637293785466966, 0.2691175898261363, 0.27450580110557604, 0.27989401238501577, 0.2852822236644555, 0.2906704349438952, 0.29926849138799455, 0.3078665478320939, 0.3164646042761932, 0.32506266072029255, 0.3336607171643919, 0.3432038874380977, 0.35274705771180354, 0.36229022798550936, 0.3718333982592152, 0.381376568532921, 0.39091973880662684, 0.40181201866359006, 0.4127042985205533, 0.4235965783775165, 0.43448885823447975, 0.445381138091443, 0.4562734179484062, 0.4703700887112123, 0.48446675947401835, 0.4985634302368244, 0.5126601009996306, 0.5267567717624366, 0.5465861621787261, 0.5664155525950156, 0.5862449430113051, 0.6060743334275946, 0.6259037238438842, 0.6516618804578423, 0.6774200370718005, 0.7031781936857587, 0.7289363502997169, 0.7546945069136751, 0.7894040808904967, 0.8241136548673184, 0.85882322884414, 0.8935328028209616, 0.9282423767977832, 0.9664585820061914, 1.0046747872145996, 1.0428909924230076, 1.0811071976314157, 1.1193234028398238, 1.1705538850306823, 1.2217843672215407, 1.2730148494123992, 1.3242453316032576, 1.375475813794116, 1.4267062959849746, 1.485501393539165, 1.5442964910933554, 1.6030915886475459, 1.6618866862017363, 1.7206817837559267, 1.7794768813101172, 1.8565321755517512, 1.9335874697933852, 2.010642764035019, 2.087698058276653, 2.1647533525182867, 2.2418086467599205, 2.3470937120582906, 2.4523787773566608, 2.557663842655031, 2.662948907953401, 2.768233973251771, 2.8735190385501412, 3.0094677345188687, 3.1454164304875962, 3.2813651264563237, 3.417313822425051, 3.5532625183937787, 3.689211214362506, 3.867257440884571, 4.045303667406635, 4.2233498939287, 4.401396120450764, 4.5794423469728285, 4.757488573494893, 4.99656783037481, 5.235647087254726, 5.474726344134643, 5.71380560101456, 5.952884857894476, 6.191964114774393, 6.535238749760635, 6.878513384746876, 7.2217880197331175, 7.565062654719359, 7.9083372897056, 8.251611924691842, 8.806790856417752, 9.361969788143663, 9.917148719869573, 10.0]</t>
+          <t>[0.0, 5.977976368016702e-07, 1.1955952736033404e-06, 7.173571641620042e-06, 1.3151548009636744e-05, 3.104616999378204e-05, 4.894079197792733e-05, 6.683541396207263e-05, 0.00011107931322170125, 0.00015532321248132986, 0.00019956711174095847, 0.00042144574141047967, 0.0006433243710800008, 0.000865203000749522, 0.0020681510920384743, 0.0032710991833274266, 0.004474047274616378, 0.00567699536590533, 0.007500944660882868, 0.009324893955860405, 0.011148843250837943, 0.01297279254581548, 0.014796741840793017, 0.020188469830644793, 0.02558019782049657, 0.030971925810348345, 0.036363653800200124, 0.04175538179005191, 0.05087748155947834, 0.059999581328904775, 0.06912168109833121, 0.07650546225397685, 0.08388924340962249, 0.09127302456526813, 0.09865680572091377, 0.10604058687655941, 0.11342436803220506, 0.11979189702952048, 0.12615942602683589, 0.1325269550241513, 0.1388944840214667, 0.1452620130187821, 0.15162954201609752, 0.1579307705455992, 0.1642319990751009, 0.17053322760460257, 0.17513852650512868, 0.17974382540565478, 0.1843491243061809, 0.188954423206707, 0.1935597221072331, 0.20123947253060936, 0.20592107208284488, 0.2106026716350804, 0.2152842711873159, 0.21996587073955143, 0.22464747029178694, 0.22932906984402246, 0.23457210791047, 0.23981514597691755, 0.2450581840433651, 0.25030122210981265, 0.2555442601762602, 0.26078729824270774, 0.26640260941092575, 0.27201792057914376, 0.27763323174736176, 0.28324854291557977, 0.2888638540837978, 0.2944791652520158, 0.30255508281955984, 0.3106310003871039, 0.31870691795464795, 0.326782835522192, 0.33485875308973606, 0.34419517070186995, 0.35353158831400383, 0.3628680059261377, 0.3722044235382716, 0.3815408411504055, 0.39087725876253937, 0.40247284071674816, 0.41406842267095695, 0.42566400462516574, 0.4372595865793745, 0.4488551685335833, 0.4604507504877921, 0.4765919298390439, 0.4927331091902957, 0.5088742885415476, 0.5250154678927994, 0.5411566472440512, 0.5638161478028842, 0.5864756483617173, 0.6091351489205503, 0.6317946494793834, 0.6544541500382164, 0.6871850562695216, 0.7199159625008269, 0.7526468687321322, 0.7853777749634374, 0.8181086811947427, 0.8529126998240104, 0.8877167184532782, 0.9225207370825459, 0.9573247557118136, 0.9921287743410814, 1.0538443456102677, 1.115559916879454, 1.1772754881486405, 1.2389910594178268, 1.3007066306870132, 1.3624222019561996, 1.4266223742665018, 1.4908225465768041, 1.5550227188871064, 1.6192228911974087, 1.683423063507711, 1.7476232358180133, 1.8285638772447383, 1.9095045186714634, 1.9904451600981885, 2.0713858015249134, 2.1523264429516384, 2.2332670843783635, 2.347566844220698, 2.461866604063032, 2.5761663639053665, 2.6904661237477008, 2.804765883590035, 2.9190656434323694, 3.09023118335495, 3.2613967232775307, 3.4325622632001114, 3.603727803122692, 3.7748933430452727, 3.9460588829678533, 4.153941534327906, 4.361824185687959, 4.569706837048011, 4.777589488408064, 4.985472139768117, 5.1933547911281694, 5.507322105403, 5.821289419677831, 6.135256733952662, 6.449224048227493, 6.763191362502324, 7.077158676777155, 7.486211976020116, 7.895265275263077, 8.304318574506038, 8.713371873748997, 9.122425172991957, 9.531478472234916, 10.0]</t>
         </is>
       </c>
       <c r="C35" t="n">
-        <v>0.2940694343881703</v>
+        <v>0.4939682061568098</v>
       </c>
       <c r="D35" t="n">
         <v>9.81</v>
@@ -2778,13 +2778,13 @@
         <v>2</v>
       </c>
       <c r="L35" t="n">
-        <v>2.940694343881703</v>
+        <v>4.939682061568098</v>
       </c>
       <c r="M35" t="n">
-        <v>0.02312758166739389</v>
+        <v>0.008196567165833021</v>
       </c>
       <c r="N35" t="n">
-        <v>0.1156379083369694</v>
+        <v>0.04098283582916511</v>
       </c>
       <c r="O35" t="n">
         <v>19.38700481894847</v>
@@ -2814,11 +2814,11 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>[0.0, 5.987509583809791e-07, 1.1975019167619582e-06, 7.185011500571749e-06, 1.3172521084381541e-05, 3.1095743259981034e-05, 4.901896543558053e-05, 6.694218761118002e-05, 0.00011125909347240102, 0.000155575999333622, 0.000199892905194843, 0.00042364940518781105, 0.0006474059051807791, 0.0008711624051737471, 0.0018091512966774363, 0.0027471401881811255, 0.003685129079684815, 0.004623117971188504, 0.006267713192637614, 0.007912308414086723, 0.009556903635535833, 0.011201498856984942, 0.012846094078434052, 0.017534180531775367, 0.02222226698511668, 0.026910353438457994, 0.03159843989179931, 0.036286526345140624, 0.045325087856686395, 0.05436364936823217, 0.06340221087977793, 0.0724407723913237, 0.07959413228857957, 0.08674749218583545, 0.09390085208309133, 0.10105421198034721, 0.10820757187760309, 0.11536093177485897, 0.12170867209624373, 0.1280564124176285, 0.13440415273901327, 0.14075189306039804, 0.1470996333817828, 0.15344737370316758, 0.15923950450788332, 0.16503163531259907, 0.1708237661173148, 0.17661589692203056, 0.1824080277267463, 0.1883871655606183, 0.1943663033944903, 0.2003454412283623, 0.20632457906223428, 0.21230371689610628, 0.21828285472997827, 0.22381366067421093, 0.2293444666184436, 0.23487527256267626, 0.24040607850690893, 0.2459368844511416, 0.25146769039537425, 0.25703468870597157, 0.2626016870165689, 0.2681686853271662, 0.2737356836377635, 0.27930268194836083, 0.28486968025895815, 0.294917741256204, 0.3049658022534499, 0.3124806051228033, 0.3199954079921567, 0.3275102108615101, 0.3350250137308635, 0.34253981660021693, 0.3527662046857279, 0.36299259277123885, 0.3732189808567498, 0.3834453689422608, 0.39367175702777174, 0.4038981451132827, 0.41624697951409917, 0.42859581391491564, 0.4409446483157321, 0.45329348271654857, 0.46564231711736503, 0.4779911515181815, 0.4943453132471685, 0.5106994749761555, 0.5270536367051426, 0.5434077984341297, 0.5597619601631167, 0.5819846416554153, 0.6042073231477139, 0.6264300046400124, 0.648652686132311, 0.6708753676246095, 0.7018904157533147, 0.7329054638820198, 0.763920512010725, 0.7949355601394301, 0.8259506082681353, 0.8608250885026634, 0.8956995687371915, 0.9305740489717196, 0.9654485292062477, 1.0003230094407758, 1.0462678881416199, 1.092212766842464, 1.138157645543308, 1.184102524244152, 1.2300474029449961, 1.2759922816458402, 1.3304619593206015, 1.3849316369953628, 1.439401314670124, 1.4938709923448854, 1.5483406700196467, 1.602810347694408, 1.668853994051173, 1.7348976404079381, 1.8009412867647032, 1.8669849331214683, 1.9330285794782334, 1.9990722258349984, 2.0935834535107025, 2.1880946811864064, 2.2826059088621102, 2.377117136537814, 2.471628364213518, 2.566139591889222, 2.688334901555262, 2.8105302112213018, 2.9327255208873417, 3.0549208305533817, 3.1771161402194217, 3.2993114498854617, 3.4586921673765043, 3.618072884867547, 3.7774536023585896, 3.9368343198496323, 4.096215037340675, 4.2555957548317185, 4.464291271846711, 4.672986788861703, 4.881682305876695, 5.090377822891687, 5.29907333990668, 5.507768856921672, 5.788804796310431, 6.06984073569919, 6.350876675087949, 6.6319126144767075, 6.9129485538654665, 7.193984493254225, 7.599841678515209, 8.005698863776193, 8.411556049037177, 8.817413234298161, 9.223270419559146, 9.62912760482013, 10.0]</t>
+          <t>[0.0, 5.987509583809791e-07, 1.1975019167619582e-06, 7.185011500571749e-06, 1.3172521084381541e-05, 3.109574325837268e-05, 4.9018965432363825e-05, 6.694218760635497e-05, 0.00011125909297221616, 0.00015557599833807736, 0.00019989290370393855, 0.0004236482506064, 0.0006474035975088615, 0.0008711589444113229, 0.0018103548825863442, 0.0027495508207613655, 0.0036887467589363865, 0.004627942697111408, 0.006272639667313121, 0.007917336637514835, 0.009562033607716548, 0.011206730577918262, 0.012851427548119975, 0.017563392180811464, 0.022275356813502952, 0.02698732144619444, 0.03169928607888593, 0.03641125071157743, 0.04541147595821801, 0.054411701204858595, 0.06341192645149918, 0.07241215169813976, 0.07959977059050242, 0.08678738948286509, 0.09397500837522775, 0.10116262726759041, 0.10835024615995308, 0.11553786505231574, 0.12191822639165763, 0.1282985877309995, 0.1346789490703414, 0.14105931040968328, 0.14743967174902517, 0.15382003308836706, 0.15967832747925556, 0.16553662187014406, 0.17139491626103256, 0.17725321065192107, 0.18311150504280957, 0.18913751697132833, 0.1951635288998471, 0.20118954082836585, 0.2072155527568846, 0.21324156468540337, 0.21926757661392213, 0.2249317002840964, 0.23059582395427067, 0.23625994762444494, 0.2419240712946192, 0.24758819496479348, 0.2532523186349678, 0.25895748200471175, 0.2646626453744557, 0.2703678087441997, 0.27607297211394366, 0.28177813548368763, 0.2874832988534316, 0.29616797928293465, 0.3048526597124377, 0.31353734014194073, 0.3222220205714438, 0.3309067010009468, 0.34038255246364757, 0.3498584039263483, 0.35933425538904906, 0.3688101068517498, 0.37828595831445055, 0.3877618097771513, 0.39957094395286497, 0.41138007812857863, 0.4231892123042923, 0.43499834648000596, 0.4468074806557196, 0.4586166148314333, 0.4750511995471058, 0.4914857842627783, 0.5079203689784508, 0.5243549536941234, 0.540789538409796, 0.561771900656308, 0.58275426290282, 0.6037366251493319, 0.6247189873958439, 0.6457013496423558, 0.6782739012769959, 0.7108464529116361, 0.7434190045462762, 0.7759915561809163, 0.8085641078155564, 0.8429960441095969, 0.8774279804036375, 0.911859916697678, 0.9462918529917185, 0.980723789285759, 1.0415110303683934, 1.1022982714510279, 1.1630855125336623, 1.2238727536162968, 1.2846599946989312, 1.3454472357815657, 1.4089457327709847, 1.4724442297604037, 1.5359427267498227, 1.5994412237392417, 1.6629397207286607, 1.7264382177180797, 1.8064740565864637, 1.8865098954548476, 1.9665457343232315, 2.0465815731916157, 2.12661741206, 2.206653250928384, 2.3196182514643002, 2.4325832520002164, 2.5455482525361326, 2.6585132530720488, 2.771478253607965, 2.884443254143881, 3.053383991989681, 3.2223247298354805, 3.39126546768128, 3.56020620552708, 3.7291469433728794, 3.898087681218679, 4.103359878500927, 4.3086320757831755, 4.513904273065424, 4.719176470347672, 4.92444866762992, 5.129720864912168, 5.4394452468366135, 5.7491696287610585, 6.058894010685504, 6.368618392609949, 6.678342774534394, 6.988067156458839, 7.3926045469599355, 7.797141937461032, 8.201679327962129, 8.606216718463227, 9.010754108964324, 9.415291499465422, 9.88941401338664, 10.0]</t>
         </is>
       </c>
       <c r="C36" t="n">
-        <v>0.2924042906282585</v>
+        <v>0.4746469635961578</v>
       </c>
       <c r="D36" t="n">
         <v>9.81</v>
@@ -2845,13 +2845,13 @@
         <v>2</v>
       </c>
       <c r="L36" t="n">
-        <v>2.924042906282585</v>
+        <v>4.746469635961578</v>
       </c>
       <c r="M36" t="n">
-        <v>0.0233917392217865</v>
+        <v>0.008877457089465258</v>
       </c>
       <c r="N36" t="n">
-        <v>0.1169586961089325</v>
+        <v>0.04438728544732629</v>
       </c>
       <c r="O36" t="n">
         <v>19.32529482974482</v>
@@ -2881,11 +2881,11 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>[0.0, 5.99963253593378e-07, 1.199926507186756e-06, 7.1995590431205364e-06, 1.3199191579054317e-05, 3.1158783490870756e-05, 4.9118375402687194e-05, 6.707796731450364e-05, 0.00011148771875824559, 0.00015589747020198754, 0.00020030722164572949, 0.0004265156000559507, 0.0006527239784661719, 0.0008789323568763931, 0.0016922475378185868, 0.0025055627187607803, 0.003318877899702974, 0.004132193080645168, 0.0056758153139199975, 0.007219437547194827, 0.008763059780469658, 0.01030668201374449, 0.01185030424701932, 0.016100488468460676, 0.02035067268990203, 0.024600856911343387, 0.028851041132784742, 0.0331012253542261, 0.04178495870513753, 0.05046869205604896, 0.05915242540696039, 0.06783615875787183, 0.07651989210878327, 0.08352768734087955, 0.09053548257297583, 0.09754327780507212, 0.1045510730371684, 0.11155886826926469, 0.11856666350136097, 0.12496984394569849, 0.131373024390036, 0.13777620483437353, 0.14417938527871105, 0.15058256572304857, 0.1569857461673861, 0.16211730239750888, 0.16724885862763167, 0.17238041485775446, 0.17751197108787725, 0.18264352731800004, 0.18777508354812283, 0.19342798872203512, 0.1990808938959474, 0.2047337990698597, 0.21038670424377198, 0.21603960941768427, 0.22169251459159656, 0.2280572818870687, 0.23442204918254084, 0.24078681647801298, 0.24715158377348512, 0.25351635106895726, 0.2598811183644294, 0.26504716494373687, 0.27021321152304434, 0.2753792581023518, 0.2805453046816593, 0.28571135126096675, 0.2908773978402742, 0.2988647817724548, 0.30685216570463536, 0.31483954963681593, 0.3228269335689965, 0.33081431750117707, 0.33880170143335764, 0.34651611100602486, 0.3542305205786921, 0.3619449301513593, 0.36965933972402654, 0.37737374929669376, 0.385088158869361, 0.3949832083853874, 0.40487825790141385, 0.4147733074174403, 0.4246683569334667, 0.43456340644949315, 0.4444584559655196, 0.46041264399598175, 0.4763668320264439, 0.4923210200569061, 0.5082752080873683, 0.5242293961178304, 0.5401835841482925, 0.5651984678299066, 0.5902133515115207, 0.6152282351931347, 0.6402431188747488, 0.6652580025563629, 0.690272886237977, 0.718286189736758, 0.7462994932355389, 0.7743127967343199, 0.8023261002331008, 0.8303394037318818, 0.8642444083825243, 0.8981494130331668, 0.9320544176838093, 0.9659594223344518, 0.9998644269850943, 1.049544941495918, 1.0992254560067416, 1.1489059705175653, 1.198586485028389, 1.2482669995392126, 1.2979475140500363, 1.3553358711462316, 1.4127242282424268, 1.470112585338622, 1.5275009424348174, 1.5848892995310127, 1.642277656627208, 1.7160381268488498, 1.7897985970704917, 1.8635590672921336, 1.9373195375137755, 2.0110800077354174, 2.0848404779570595, 2.1687940443366713, 2.252747610716283, 2.336701177095895, 2.420654743475507, 2.5046083098551186, 2.5885618762347304, 2.71619367217319, 2.8438254681116497, 2.9714572640501093, 3.099089059988569, 3.2267208559270286, 3.3543526518654883, 3.519098812471216, 3.683844973076944, 3.848591133682672, 4.0133372942884, 4.178083454894128, 4.342829615499856, 4.560516419191696, 4.778203222883537, 4.995890026575378, 5.213576830267218, 5.431263633959059, 5.6489504376509, 5.94269247515542, 6.23643451265994, 6.530176550164461, 6.823918587668981, 7.117660625173501, 7.411402662678022, 7.825899135420261, 8.240395608162501, 8.654892080904741, 9.06938855364698, 9.48388502638922, 9.89838149913146, 10.0]</t>
+          <t>[0.0, 5.99963253593378e-07, 1.199926507186756e-06, 7.1995590431205364e-06, 1.3199191579054317e-05, 3.115878348963488e-05, 4.911837540021544e-05, 6.7077967310796e-05, 0.00011148771826958759, 0.0001558974692283792, 0.0002003072201871708, 0.0004265144060340599, 0.000652721591880949, 0.000878928777727838, 0.0016928264951161522, 0.0025067242125044664, 0.0033206219298927806, 0.004134519647281095, 0.0056821700700981255, 0.006841095381617932, 0.008000020693137738, 0.009158946004657545, 0.010742804025197252, 0.01232666204573696, 0.013910520066276667, 0.015494378086816375, 0.018293867489212433, 0.02109335689160849, 0.023892846294004545, 0.0266923356964006, 0.029491825098796658, 0.037554666048047816, 0.045617506997298975, 0.05368034794655013, 0.06174318889580129, 0.06980602984505245, 0.0778688707943036, 0.08487886234013375, 0.0918888538859639, 0.09889884543179406, 0.10590883697762421, 0.11291882852345436, 0.11992882006928451, 0.12638219730851763, 0.13283557454775075, 0.13928895178698386, 0.14574232902621698, 0.1521957062654501, 0.1586490835046832, 0.16381042131098095, 0.16897175911727869, 0.17413309692357642, 0.17929443472987416, 0.1844557725361719, 0.18961711034246964, 0.19474505395654243, 0.19987299757061522, 0.205000941184688, 0.2101288847987608, 0.21525682841283358, 0.22038477202690637, 0.22658508915212588, 0.2327854062773454, 0.2389857234025649, 0.24518604052778442, 0.25138635765300393, 0.25758667477822345, 0.2628335936990049, 0.2680805126197863, 0.27332743154056777, 0.2785743504613492, 0.28382126938213065, 0.2890681883029121, 0.2972343527777051, 0.3054005172524981, 0.31356668172729113, 0.32173284620208414, 0.32989901067687716, 0.33806517515167017, 0.34759959033439825, 0.3571340055171263, 0.3666684206998544, 0.37620283588258246, 0.38573725106531054, 0.3952716662480386, 0.40739918419802357, 0.4195267021480085, 0.4316542200979935, 0.44378173804797844, 0.4559092559979634, 0.46803677394794835, 0.4866723803361752, 0.5053079867244021, 0.5239435931126291, 0.542579199500856, 0.5612148058890829, 0.5798504122773098, 0.6019263620612305, 0.6240023118451512, 0.6460782616290719, 0.6681542114129926, 0.6902301611969133, 0.7263574805724281, 0.7624847999479429, 0.7986121193234578, 0.8347394386989726, 0.8708667580744874, 0.9156477408895827, 0.9604287237046779, 1.0052097065197731, 1.0499906893348685, 1.0947716721499638, 1.1483664007200078, 1.2019611292900518, 1.2555558578600958, 1.3091505864301398, 1.3627453150001838, 1.4163400435702278, 1.4922825827290378, 1.5682251218878478, 1.6441676610466578, 1.7201102002054678, 1.7960527393642778, 1.8936630092169684, 1.991273279069659, 2.0888835489223494, 2.18649381877504, 2.28410408862773, 2.3817143584804206, 2.5125320187260654, 2.64334967897171, 2.774167339217355, 2.9049849994629997, 3.0358026597086445, 3.1666203199542893, 3.31836002454068, 3.4700997291270705, 3.621839433713461, 3.773579138299852, 3.9253188428862424, 4.0770585474726335, 4.315911342113661, 4.554764136754688, 4.793616931395715, 5.032469726036743, 5.27132252067777, 5.510175315318797, 5.8091741378904445, 6.108172960462092, 6.407171783033739, 6.7061706056053865, 7.005169428177034, 7.304168250748681, 7.75319008519904, 8.202211919649399, 8.651233754099756, 9.100255588550114, 9.549277423000472, 9.99829925745083, 10.0]</t>
         </is>
       </c>
       <c r="C37" t="n">
-        <v>0.2902995666249751</v>
+        <v>0.4542241292660426</v>
       </c>
       <c r="D37" t="n">
         <v>9.81</v>
@@ -2912,13 +2912,13 @@
         <v>2</v>
       </c>
       <c r="L37" t="n">
-        <v>2.902995666249751</v>
+        <v>4.542241292660425</v>
       </c>
       <c r="M37" t="n">
-        <v>0.02373215743323485</v>
+        <v>0.009693700412141392</v>
       </c>
       <c r="N37" t="n">
-        <v>0.1186607871661742</v>
+        <v>0.04846850206070696</v>
       </c>
       <c r="O37" t="n">
         <v>19.24724062796851</v>
@@ -2948,11 +2948,11 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>[0.0, 6.015071089459949e-07, 1.2030142178919898e-06, 7.2180853073519385e-06, 1.3233156396811887e-05, 3.1239065396959e-05, 4.924497439710611e-05, 6.725088339725322e-05, 0.00011177888495463498, 0.00015630688651201673, 0.00020083488806939848, 0.0004302781506955035, 0.0006597214133216085, 0.0008891646759477136, 0.0016204472022617632, 0.002351729728575813, 0.0030830122548898622, 0.0038142947812039116, 0.005271951466013017, 0.006729608150822122, 0.008187264835631227, 0.009644921520440332, 0.011102578205249437, 0.015010496847379724, 0.01891841548951001, 0.022826334131640296, 0.026734252773770582, 0.03064217141590087, 0.03893514202034365, 0.047228112624786434, 0.05552108322922922, 0.063814053833672, 0.07210702443811479, 0.08039999504255757, 0.08733868458495891, 0.09427737412736026, 0.1012160636697616, 0.10815475321216295, 0.11509344275456429, 0.12203213229696563, 0.12845343264095518, 0.13487473298494473, 0.14129603332893428, 0.14771733367292383, 0.15413863401691338, 0.16055993436090293, 0.16582691954824763, 0.17109390473559233, 0.17636088992293703, 0.18162787511028172, 0.18689486029762642, 0.19216184548497112, 0.19798950725676084, 0.20381716902855057, 0.2096448308003403, 0.21547249257213003, 0.22130015434391975, 0.22814229050708615, 0.23498442667025254, 0.24182656283341894, 0.24866869899658534, 0.2555108351597517, 0.26235297132291807, 0.2679639002277914, 0.2735748291326647, 0.279185758037538, 0.2847966869424113, 0.2904076158472846, 0.2960185447521579, 0.3050478770015879, 0.31407720925101795, 0.323106541500448, 0.332135873749878, 0.34116520599930805, 0.3501945382487381, 0.3599581674955951, 0.36972179674245215, 0.3794854259893092, 0.3892490552361662, 0.39901268448302324, 0.40877631372988027, 0.4215324152760299, 0.43428851682217956, 0.4470446183683292, 0.45980071991447885, 0.4725568214606285, 0.48531292300677814, 0.5047793280984175, 0.524245733190057, 0.5437121382816964, 0.5631785433733358, 0.5826449484649753, 0.6021113535566147, 0.626340692370383, 0.6505700311841514, 0.6747993699979197, 0.699028708811688, 0.7232580476254563, 0.7582651064076646, 0.793272165189873, 0.8282792239720813, 0.8632862827542896, 0.898293341536498, 0.9373929120963101, 0.9764924826561223, 1.0155920532159346, 1.0546916237757469, 1.0937911943355592, 1.1434757616303903, 1.1931603289252215, 1.2428448962200527, 1.2925294635148838, 1.342214030809715, 1.3918985981045462, 1.446705757071052, 1.5015129160375578, 1.5563200750040636, 1.6111272339705693, 1.6659343929370751, 1.720741551903581, 1.8111986122432437, 1.9016556725829066, 1.9921127329225694, 2.0825697932622322, 2.173026853601895, 2.263483913941558, 2.3639942910520606, 2.4645046681625633, 2.565015045273066, 2.6655254223835687, 2.7660357994940714, 2.866546176604574, 2.9967760244341073, 3.1270058722636405, 3.2572357200931736, 3.387465567922707, 3.51769541575224, 3.647925263581773, 3.8155204879557556, 3.983115712329738, 4.150710936703721, 4.318306161077704, 4.485901385451687, 4.65349660982567, 4.867979913608996, 5.082463217392322, 5.296946521175648, 5.511429824958974, 5.7259131287423, 5.940396432525626, 6.21878925165588, 6.497182070786135, 6.775574889916389, 7.053967709046644, 7.332360528176898, 7.610753347307153, 7.981911071570033, 8.353068795832913, 8.724226520095794, 9.095384244358675, 9.466541968621556, 9.837699692884437, 10.0]</t>
+          <t>[0.0, 6.015071089459949e-07, 1.2030142178919898e-06, 7.2180853073519385e-06, 1.3233156396811887e-05, 3.123906539619873e-05, 4.924497439558557e-05, 6.725088339497242e-05, 0.00011177888448070118, 0.00015630688556642994, 0.0002008348866521587, 0.00043027690307861167, 0.0006597189195050646, 0.0008891609359315176, 0.0016207809338878469, 0.002352400931844176, 0.0030840209298005055, 0.003815640927756835, 0.005273140729223344, 0.006730640530689853, 0.008188140332156361, 0.00964564013362287, 0.011103139935089379, 0.015019428852110158, 0.018935717769130937, 0.022852006686151716, 0.026768295603172496, 0.030684584520193275, 0.03884993943626515, 0.04701529435233702, 0.05518064926840889, 0.06334600418448076, 0.07151135910055263, 0.0796767140166245, 0.0866276821266466, 0.09357865023666868, 0.10052961834669077, 0.10748058645671286, 0.11443155456673496, 0.12138252267675705, 0.12785129055355762, 0.1343200584303582, 0.1407888263071588, 0.1472575941839594, 0.15372636206075999, 0.16019512993756058, 0.16546228980931796, 0.17072944968107534, 0.17599660955283272, 0.1812637694245901, 0.1865309292963475, 0.19179808916810487, 0.19752284537411616, 0.20324760158012745, 0.20897235778613873, 0.21469711399215002, 0.2204218701981613, 0.22680967172592073, 0.23319747325368015, 0.23958527478143957, 0.24597307630919898, 0.2523608778369584, 0.2587486793647178, 0.2644559893958015, 0.2701632994268852, 0.27587060945796893, 0.28157791948905264, 0.28728522952013635, 0.29299253955122007, 0.3020443044393331, 0.31109606932744616, 0.3201478342155592, 0.32919959910367225, 0.3382513639917853, 0.34730312887989834, 0.3572686438008643, 0.3672341587218303, 0.3771996736427963, 0.38716518856376225, 0.39713070348472823, 0.4070962184056942, 0.42060258451177435, 0.4341089506178545, 0.4476153167239346, 0.46112168283001476, 0.4746280489360949, 0.48813441504217503, 0.5092086292371352, 0.5302828434320953, 0.5513570576270554, 0.5724312718220156, 0.5935054860169757, 0.6145797002119359, 0.638921643908616, 0.6632635876052962, 0.6876055313019764, 0.7119474749986566, 0.7362894186953368, 0.7754232423944047, 0.8145570660934727, 0.8536908897925406, 0.8928247134916085, 0.9319585371906765, 0.9800842509489388, 1.0282099647072012, 1.0763356784654636, 1.124461392223726, 1.1725871059819886, 1.2292998826615253, 1.2860126593410621, 1.342725436020599, 1.3994382127001357, 1.4561509893796725, 1.5128637660592092, 1.594166202601901, 1.6754686391445928, 1.7567710756872845, 1.8380735122299763, 1.919375948772668, 2.0233512956969206, 2.127326642621173, 2.231301989545426, 2.3352773364696784, 2.439252683393931, 2.5432280303181836, 2.660696932080215, 2.7781658338422464, 2.8956347356042778, 3.013103637366309, 3.1305725391283405, 3.248041440890372, 3.435438273272378, 3.622835105654384, 3.8102319380363903, 3.9976287704183964, 4.185025602800403, 4.3724224351824095, 4.606144176666581, 4.839865918150753, 5.073587659634925, 5.307309401119097, 5.541031142603269, 5.774752884087441, 6.126646864911463, 6.478540845735486, 6.830434826559508, 7.182328807383531, 7.534222788207553, 7.886116769031576, 8.320100913695889, 8.754085058360202, 9.188069203024515, 9.622053347688828, 10.0]</t>
         </is>
       </c>
       <c r="C38" t="n">
-        <v>0.2876399898857571</v>
+        <v>0.432879622606038</v>
       </c>
       <c r="D38" t="n">
         <v>9.81</v>
@@ -2979,13 +2979,13 @@
         <v>2</v>
       </c>
       <c r="L38" t="n">
-        <v>2.876399898857571</v>
+        <v>4.328796226060379</v>
       </c>
       <c r="M38" t="n">
-        <v>0.02417305087351897</v>
+        <v>0.01067322613729393</v>
       </c>
       <c r="N38" t="n">
-        <v>0.1208652543675948</v>
+        <v>0.05336613068646964</v>
       </c>
       <c r="O38" t="n">
         <v>19.14851336365426</v>
@@ -3015,11 +3015,11 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>[0.0, 6.034768471339253e-07, 1.2069536942678507e-06, 7.241722165607104e-06, 1.3276490636946357e-05, 3.134149410146507e-05, 4.9406497565983784e-05, 6.74715010305025e-05, 0.0001121503913925944, 0.0001568292817546863, 0.0002015081721167782, 0.00043527663163208145, 0.0006690450911473847, 0.000902813550662688, 0.001573075697737597, 0.002243337844812506, 0.0029135999918874153, 0.0035838621389623244, 0.004955472568744848, 0.006327082998527371, 0.007698693428309895, 0.009070303858092418, 0.010441914287874943, 0.014065364215978593, 0.017688814144082243, 0.021312264072185894, 0.024935714000289544, 0.028559163928393194, 0.03638861163792929, 0.04421805934746538, 0.05204750705700147, 0.059876954766537566, 0.06770640247607365, 0.07553585018560974, 0.08240453865173865, 0.08927322711786756, 0.09614191558399647, 0.10301060405012538, 0.10987929251625429, 0.1167479809823832, 0.12315155200328015, 0.1295551230241771, 0.13595869404507405, 0.142362265065971, 0.14876583608686794, 0.1551694071077649, 0.1604577850221086, 0.16574616293645233, 0.17103454085079606, 0.17632291876513978, 0.1816112966794835, 0.18689967459382723, 0.19278341499120985, 0.19866715538859248, 0.2045508957859751, 0.21043463618335773, 0.21631837658074035, 0.22331005504239285, 0.23030173350404534, 0.23729341196569784, 0.24428509042735033, 0.25127676888900286, 0.25826844735065535, 0.2639468756266538, 0.26962530390265227, 0.27530373217865073, 0.2809821604546492, 0.28666058873064765, 0.2923390170066461, 0.3016700556892573, 0.3110010943718685, 0.3203321330544797, 0.3296631717370909, 0.3389942104197021, 0.34832524910231333, 0.35828592259626985, 0.36824659609022636, 0.3782072695841829, 0.3881679430781394, 0.3981286165720959, 0.40808929006605243, 0.42146695626087244, 0.43484462245569244, 0.44822228865051245, 0.46159995484533245, 0.47497762104015245, 0.4956255919349419, 0.5162735628297312, 0.5369215337245206, 0.5575695046193099, 0.5782174755140992, 0.6010754131602917, 0.6239333508064842, 0.6467912884526766, 0.6696492260988691, 0.6925071637450616, 0.7263361543390991, 0.7601651449331367, 0.7939941355271742, 0.8278231261212118, 0.8616521167152493, 0.8995418245398447, 0.93743153236444, 0.9753212401890353, 1.0132109480136307, 1.0511006558382259, 1.099777906088893, 1.1484551563395602, 1.1971324065902273, 1.2458096568408945, 1.2944869070915617, 1.3431641573422288, 1.4083988839043067, 1.4736336104663845, 1.5388683370284624, 1.6041030635905402, 1.669337790152618, 1.734572516714696, 1.8147997596479843, 1.8950270025812728, 1.9752542455145612, 2.0554814884478496, 2.135708731381138, 2.2159359743144265, 2.3158929873046716, 2.415850000294917, 2.515807013285162, 2.615764026275407, 2.7157210392656523, 2.8156780522558975, 2.959456927202233, 3.1032358021485686, 3.247014677094904, 3.3907935520412398, 3.5345724269875753, 3.678351301933911, 3.8695270424895254, 4.06070278304514, 4.251878523600754, 4.443054264156369, 4.634230004711983, 4.825405745267598, 5.053344053263372, 5.281282361259147, 5.509220669254922, 5.737158977250696, 5.965097285246471, 6.193035593242246, 6.518756065608614, 6.844476537974983, 7.170197010341352, 7.49591748270772, 7.821637955074089, 8.147358427440459, 8.554446105567774, 8.961533783695089, 9.368621461822404, 9.775709139949718, 10.0]</t>
+          <t>[0.0, 6.034768471339253e-07, 1.2069536942678507e-06, 7.241722165607104e-06, 1.3276490636946357e-05, 3.134149410131338e-05, 4.940649756568041e-05, 6.747150103004744e-05, 0.00011215039093751558, 0.00015682928084498373, 0.00020150817075245187, 0.00043527530953939287, 0.0006690424483263339, 0.0009028095871132748, 0.0015732864719901025, 0.0022437633568669303, 0.002914240241743758, 0.003584717126620586, 0.004956233845862582, 0.006327750565104579, 0.007699267284346575, 0.009070784003588572, 0.01044230072283057, 0.014071125040447802, 0.017699949358065035, 0.02132877367568227, 0.024957597993299503, 0.028586422310916737, 0.036303980047284676, 0.044021537783652614, 0.05173909552002055, 0.05945665325638849, 0.06717421099275643, 0.07489176872912437, 0.08176891548781251, 0.08864606224650065, 0.09552320900518879, 0.10240035576387693, 0.10927750252256507, 0.11615464928125321, 0.12260354941619225, 0.1290524495511313, 0.13550134968607033, 0.14195024982100937, 0.1483991499559484, 0.15484805009088745, 0.16013417220173679, 0.16542029431258612, 0.17070641642343545, 0.1759925385342848, 0.18127866064513412, 0.18656478275598345, 0.19235042183530315, 0.19813606091462285, 0.20392169999394255, 0.20970733907326225, 0.21549297815258195, 0.2220997090300302, 0.22870643990747846, 0.23531317078492672, 0.24191990166237498, 0.24852663253982324, 0.2551333634172715, 0.26087553619779985, 0.2666177089783282, 0.27235988175885656, 0.2781020545393849, 0.28384422731991327, 0.2895864001004416, 0.2990843099972319, 0.3085822198940222, 0.31808012979081246, 0.32757803968760274, 0.337075949584393, 0.3465738594811833, 0.35670450642130974, 0.3668351533614362, 0.3769658003015626, 0.38709644724168907, 0.3972270941818155, 0.40735774112194195, 0.4213717007049371, 0.4353856602879323, 0.44939961987092747, 0.46341357945392264, 0.4774275390369178, 0.4972494556097859, 0.517071372182654, 0.536893288755522, 0.55671520532839, 0.576537121901258, 0.605231857314985, 0.6339265927287119, 0.6626213281424388, 0.6913160635561657, 0.7200107989698926, 0.7506157776327246, 0.7812207562955565, 0.8118257349583885, 0.8424307136212205, 0.8730356922840524, 0.928504458985463, 0.9839732256868735, 1.039441992388284, 1.0949107590896947, 1.1503795257911054, 1.205848292492516, 1.262200118872399, 1.318551945252282, 1.374903771632165, 1.431255598012048, 1.487607424391931, 1.543959250771814, 1.6268346819680848, 1.7097101131643555, 1.7925855443606262, 1.875460975556897, 1.9583364067531677, 2.0412118379494384, 2.146240600059736, 2.2512693621700333, 2.3562981242803307, 2.461326886390628, 2.5663556485009256, 2.671384410611223, 2.810342255102996, 2.949300099594769, 3.088257944086542, 3.227215788578315, 3.3661736330700878, 3.5051314775618607, 3.7118212290199355, 3.9185109804780103, 4.125200731936085, 4.331890483394159, 4.538580234852233, 4.745269986310308, 4.972017535287312, 5.198765084264317, 5.425512633241322, 5.652260182218327, 5.8790077311953315, 6.105755280172336, 6.471882951257965, 6.838010622343593, 7.204138293429222, 7.57026596451485, 7.936393635600479, 8.302521306686106, 8.764683386569274, 9.226845466452442, 9.68900754633561, 10.0]</t>
         </is>
       </c>
       <c r="C39" t="n">
-        <v>0.2842799809393754</v>
+        <v>0.4107841657322466</v>
       </c>
       <c r="D39" t="n">
         <v>9.81</v>
@@ -3046,13 +3046,13 @@
         <v>2</v>
       </c>
       <c r="L39" t="n">
-        <v>2.842799809393754</v>
+        <v>4.107841657322466</v>
       </c>
       <c r="M39" t="n">
-        <v>0.02474784802388053</v>
+        <v>0.01185229919686165</v>
       </c>
       <c r="N39" t="n">
-        <v>0.1237392401194026</v>
+        <v>0.05926149598430826</v>
       </c>
       <c r="O39" t="n">
         <v>19.02363766834054</v>
@@ -3082,11 +3082,11 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>[0.0, 6.059959132612402e-07, 1.2119918265224804e-06, 7.271950959134883e-06, 1.3331910091747286e-05, 3.1472489312316576e-05, 4.961306853288587e-05, 6.775364775345516e-05, 0.00011262553767134954, 0.00015749742758924392, 0.0002023693175071383, 0.00044202866992698055, 0.0006816880223468228, 0.0009213473747666651, 0.0015434319411494896, 0.002165516507532314, 0.0027876010739151386, 0.003409685640297963, 0.0046910341184540965, 0.00597238259661023, 0.0072537310747663635, 0.008535079552922497, 0.009816428031078631, 0.013197927445622967, 0.016579426860167303, 0.01996092627471164, 0.023342425689255975, 0.02672392510380031, 0.03399589037533453, 0.041267855646868745, 0.04853982091840296, 0.05581178618993718, 0.0630837514614714, 0.07035571673300561, 0.0771585858340626, 0.08396145493511958, 0.09076432403617657, 0.09756719313723355, 0.10437006223829054, 0.11117293133934752, 0.11755697616245998, 0.12394102098557244, 0.13032506580868491, 0.1367091106317974, 0.14309315545490986, 0.14947720027802233, 0.1547955163756223, 0.16011383247322228, 0.16543214857082225, 0.17075046466842222, 0.1760687807660222, 0.18138709686362217, 0.18732257345340372, 0.19325805004318528, 0.19919352663296683, 0.20512900322274838, 0.21106447981252993, 0.21819891635679015, 0.22533335290105036, 0.23246778944531057, 0.2396022259895708, 0.246736662533831, 0.25387109907809124, 0.2596741288117067, 0.26547715854532217, 0.27128018827893763, 0.2770832180125531, 0.28288624774616855, 0.29106348648321234, 0.29924072522025613, 0.3074179639572999, 0.3155952026943437, 0.3237724414313875, 0.3319496801684313, 0.34066662385493873, 0.34938356754144617, 0.3581005112279536, 0.36681745491446105, 0.3755343986009685, 0.3842513422874759, 0.39691579150764605, 0.4095802407278162, 0.4222446899479863, 0.43490913916815643, 0.44757358838832656, 0.4602380376084967, 0.47920119175035025, 0.4981643458922038, 0.5171275000340574, 0.536090654175911, 0.5550538083177645, 0.5740169624596181, 0.5974436850639473, 0.6208704076682765, 0.6442971302726057, 0.6677238528769349, 0.6911505754812641, 0.7199168869668255, 0.748683198452387, 0.7774495099379484, 0.8062158214235098, 0.8349821329090712, 0.8767135944172655, 0.9184450559254598, 0.9601765174336541, 1.0019079789418484, 1.0436394404500426, 1.0874516220996373, 1.131263803749232, 1.1750759853988266, 1.2188881670484213, 1.262700348698016, 1.3065125303476106, 1.3602588880968007, 1.4140052458459909, 1.467751603595181, 1.521497961344371, 1.5752443190935612, 1.659684519118954, 1.7441247191443467, 1.8285649191697395, 1.9130051191951323, 1.997445319220525, 2.081885519245918, 2.1775159265542703, 2.2731463338626225, 2.368776741170975, 2.464407148479327, 2.5600375557876793, 2.6556679630960316, 2.7784888297267596, 2.9013096963574876, 3.0241305629882156, 3.1469514296189436, 3.2697722962496716, 3.3925931628803996, 3.56986703651548, 3.74714091015056, 3.9244147837856405, 4.101688657420721, 4.278962531055801, 4.456236404690881, 4.689677255519517, 4.923118106348153, 5.156558957176789, 5.389999808005425, 5.623440658834061, 5.8568815096626965, 6.171135332049639, 6.485389154436581, 6.799642976823524, 7.113896799210466, 7.428150621597409, 7.742404443984351, 8.127933262734198, 8.513462081484043, 8.898990900233889, 9.284519718983734, 9.67004853773358, 10.0]</t>
+          <t>[0.0, 6.059959132612402e-07, 1.2119918265224804e-06, 7.271950959134883e-06, 1.3331910091747286e-05, 3.147248931294608e-05, 4.961306853414487e-05, 6.775364775534367e-05, 0.00011262553724049817, 0.00015749742672565268, 0.0002023693162108072, 0.0004420272411152594, 0.0006816851660197116, 0.0009213430909241637, 0.0015435725457180942, 0.0021658020005120245, 0.002788031455305955, 0.0034102609100998857, 0.004691589349699659, 0.005972917789299433, 0.007254246228899206, 0.008535574668498979, 0.009816903108098752, 0.013201957689602618, 0.016587012271106483, 0.019972066852610347, 0.02335712143411421, 0.026742176015618076, 0.033933733306735846, 0.041125290597853616, 0.048316847888971386, 0.055508405180089156, 0.06269996247120693, 0.06989151976232472, 0.07670147426819154, 0.08351142877405837, 0.0903213832799252, 0.09713133778579203, 0.10394129229165885, 0.11075124679752568, 0.1171763731356887, 0.12360149947385171, 0.13002662581201474, 0.13645175215017777, 0.1428768784883408, 0.14930200482650383, 0.15462069964607464, 0.15993939446564545, 0.16525808928521626, 0.17057678410478708, 0.1758954789243579, 0.1812141737439287, 0.1870886625885549, 0.19296315143318107, 0.19883764027780726, 0.20471212912243344, 0.21058661796705963, 0.21742865450535645, 0.22427069104365327, 0.2311127275819501, 0.2379547641202469, 0.24479680065854373, 0.25163883719684055, 0.2574447909532933, 0.2632507447097461, 0.26905669846619884, 0.2748626522226516, 0.28066860597910437, 0.28647455973555713, 0.2963213397275765, 0.3061681197195959, 0.3160148997116153, 0.32586167970363467, 0.33570845969565405, 0.34555523968767343, 0.35591046781533636, 0.3662656959429993, 0.3766209240706622, 0.38697615219832515, 0.3973313803259881, 0.407686608453651, 0.4223580260438096, 0.43702944363396823, 0.45170086122412684, 0.46637227881428545, 0.48104369640444405, 0.5013640468498998, 0.5216843972953555, 0.5420047477408113, 0.5623250981862671, 0.5826454486317229, 0.6118376805336472, 0.6410299124355715, 0.6702221443374958, 0.6994143762394202, 0.7286066081413445, 0.7596651708304939, 0.7907237335196433, 0.8217822962087927, 0.8528408588979421, 0.8838994215870916, 0.9398914965774948, 0.9958835715678981, 1.0518756465583015, 1.107867721548705, 1.1638597965391084, 1.219851871529512, 1.277021266086455, 1.3341906606433982, 1.3913600552003413, 1.4485294497572845, 1.5056988443142276, 1.5628682388711708, 1.6462282682982894, 1.729588297725408, 1.8129483271525266, 1.8963083565796452, 1.9796683860067639, 2.0630284154338825, 2.16619837314478, 2.2693683308556776, 2.372538288566575, 2.4757082462774727, 2.57887820398837, 2.6820481616992677, 2.8384988090296783, 2.994949456360089, 3.1514001036904995, 3.30785075102091, 3.4643013983513207, 3.6207520456817313, 3.825952915788954, 4.031153785896176, 4.236354656003399, 4.441555526110621, 4.646756396217843, 4.851957266325066, 5.0886533530317335, 5.325349439738401, 5.562045526445069, 5.798741613151737, 6.035437699858405, 6.272133786565073, 6.6491393334044, 7.026144880243727, 7.403150427083054, 7.780155973922382, 8.157161520761708, 8.534167067601034, 9.010159838769706, 9.486152609938378, 9.96214538110705, 10.0]</t>
         </is>
       </c>
       <c r="C40" t="n">
-        <v>0.2800354098774058</v>
+        <v>0.3880881323867191</v>
       </c>
       <c r="D40" t="n">
         <v>9.81</v>
@@ -3113,13 +3113,13 @@
         <v>2</v>
       </c>
       <c r="L40" t="n">
-        <v>2.800354098774057</v>
+        <v>3.880881323867191</v>
       </c>
       <c r="M40" t="n">
-        <v>0.02550375306825178</v>
+        <v>0.01327911924865743</v>
       </c>
       <c r="N40" t="n">
-        <v>0.1275187653412589</v>
+        <v>0.06639559624328713</v>
       </c>
       <c r="O40" t="n">
         <v>18.86568799366454</v>
@@ -3149,11 +3149,11 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>[0.0, 6.092273302409245e-07, 1.218454660481849e-06, 7.310727962891094e-06, 1.3403001265300338e-05, 3.1640529149146926e-05, 4.9878057032993514e-05, 6.811558491684011e-05, 0.00011323510117857467, 0.00015835461744030923, 0.00020347413370204378, 0.00045137197991435913, 0.0006992698261266744, 0.0009471676723389897, 0.0015302041832019986, 0.0021132406940650075, 0.0026962772049280164, 0.0032793137157910253, 0.004467158947829278, 0.005655004179867531, 0.0068428494119057845, 0.008030694643944038, 0.009218539875982291, 0.01239674074768345, 0.015574941619384608, 0.018753142491085766, 0.021931343362786924, 0.025109544234488083, 0.03178926126230625, 0.038468978290124425, 0.0451486953179426, 0.05182841234576077, 0.058508129373578945, 0.06518784640139712, 0.07194580253094043, 0.07870375866048375, 0.08546171479002707, 0.09221967091957038, 0.0989776270491137, 0.10573558317865701, 0.11271945940820154, 0.11970333563774606, 0.1266872118672906, 0.13367108809683514, 0.1406549643263797, 0.14763884055592424, 0.15311466159440948, 0.1585904826328947, 0.16406630367137995, 0.16954212470986518, 0.17501794574835042, 0.18049376678683565, 0.1875476741098825, 0.19228171847451428, 0.19701576283914607, 0.20174980720377786, 0.20648385156840965, 0.21121789593304144, 0.21763146623341476, 0.22404503653378807, 0.2304586068341614, 0.2368721771345347, 0.24328574743490802, 0.24969931773528134, 0.25652632619566684, 0.2633533346560524, 0.2701803431164379, 0.27700735157682344, 0.28383436003720897, 0.2928285768113098, 0.30182279358541064, 0.3108170103595115, 0.3198112271336123, 0.32880544390771316, 0.337799660681814, 0.34846556570079923, 0.35913147071978446, 0.3697973757387697, 0.38046328075775493, 0.39112918577674016, 0.4017950907957254, 0.4160176288413861, 0.4302401668870468, 0.4444627049327075, 0.4586852429783682, 0.4729077810240289, 0.4871303190696896, 0.5077955676465443, 0.528460816223399, 0.5491260648002537, 0.5697913133771084, 0.5904565619539631, 0.6142112919877983, 0.6379660220216335, 0.6617207520554688, 0.685475482089304, 0.7092302121231392, 0.7448654493878402, 0.7805006866525411, 0.8161359239172421, 0.8517711611819431, 0.887406398446644, 0.924120806811393, 0.9608352151761419, 0.9975496235408908, 1.0342640319056398, 1.0709784402703888, 1.123250438097871, 1.175522435925353, 1.2277944337528353, 1.2800664315803174, 1.3323384294077996, 1.3846104272352817, 1.4542092304336942, 1.5238080336321067, 1.5934068368305192, 1.6630056400289317, 1.7326044432273442, 1.8022032464257567, 1.8871258495494057, 1.9720484526730546, 2.0569710557967036, 2.1418936589203526, 2.2268162620440015, 2.3117388651676505, 2.434136070515491, 2.5565332758633312, 2.6789304812111716, 2.801327686559012, 2.9237248919068524, 3.0461220972546927, 3.190740021649699, 3.335357946044705, 3.479975870439711, 3.624593794834717, 3.769211719229723, 3.9138296436247293, 4.103294380224155, 4.292759116823581, 4.482223853423007, 4.671688590022433, 4.861153326621859, 5.050618063221285, 5.299329698986407, 5.548041334751528, 5.79675297051665, 6.045464606281771, 6.294176242046893, 6.5428878778120145, 6.90567153807838, 7.268455198344745, 7.631238858611111, 7.994022518877476, 8.356806179143842, 8.719589839410208, 9.212220404801803, 9.704850970193398, 10.0]</t>
+          <t>[0.0, 6.092273302409245e-07, 1.218454660481849e-06, 7.310727962891094e-06, 1.3403001265300338e-05, 3.1640529150783536e-05, 4.9878057036266734e-05, 6.811558492174993e-05, 0.00011323510077899071, 0.00015835461663623148, 0.00020347413249347223, 0.0004513703913922762, 0.0006992666502910801, 0.0009471629091898841, 0.0015303014229776737, 0.0021134399367654633, 0.002696578450553253, 0.0032797169643410426, 0.004467599216767598, 0.005655481469194153, 0.0068433637216207075, 0.008031245974047262, 0.009219128226473817, 0.012399733253404531, 0.015580338280335245, 0.018760943307265958, 0.02194154833419667, 0.02512215336112738, 0.03175244320834547, 0.03838273305556356, 0.045013022902781655, 0.05164331274999975, 0.05827360259721784, 0.06490389244443592, 0.0716688006929018, 0.07843370894136767, 0.08519861718983354, 0.09196352543829941, 0.09872843368676529, 0.10549334193523116, 0.11251629245089878, 0.1195392429665664, 0.12656219348223402, 0.13358514399790164, 0.14060809451356926, 0.14763104502923688, 0.1531057657039407, 0.1585804863786445, 0.1640552070533483, 0.16952992772805212, 0.17500464840275592, 0.18047936907745973, 0.1876016280626549, 0.19238716674935363, 0.19717270543605236, 0.2019582441227511, 0.20674378280944983, 0.21152932149614856, 0.2180847006349298, 0.22464007977371103, 0.23119545891249227, 0.2377508380512735, 0.24430621719005474, 0.250861596328836, 0.2573384341454948, 0.2638152719621536, 0.2702921097788124, 0.2767689475954712, 0.28324578541213, 0.29272775295937314, 0.30220972050661626, 0.3116916880538594, 0.3211736556011025, 0.3306556231483456, 0.34013759069558874, 0.35090225492014254, 0.36166691914469634, 0.37243158336925014, 0.38319624759380394, 0.39396091181835774, 0.40472557604291154, 0.41965304155341193, 0.4345805070639123, 0.4495079725744127, 0.4644354380849131, 0.4793629035954135, 0.4942903691059139, 0.514058853996015, 0.5338273388861161, 0.5535958237762172, 0.5733643086663183, 0.5931327935564193, 0.6180301060009757, 0.6429274184455321, 0.6678247308900885, 0.6927220433346449, 0.7176193557792013, 0.7550707471867734, 0.7925221385943454, 0.8299735300019174, 0.8674249214094895, 0.9048763128170615, 0.9524119621549445, 0.9999476114928275, 1.0474832608307105, 1.0950189101685934, 1.1425545595064763, 1.1900902088443592, 1.2464874744484795, 1.3028847400525998, 1.35928200565672, 1.4156792712608404, 1.4720765368649606, 1.5495925449202936, 1.6271085529756266, 1.7046245610309596, 1.7821405690862926, 1.8596565771416256, 1.9371725851969586, 2.024808602057972, 2.1124446189189854, 2.2000806357799987, 2.287716652641012, 2.3753526695020253, 2.4629886863630386, 2.6031957087967497, 2.7434027312304607, 2.883609753664172, 3.023816776097883, 3.164023798531594, 3.304230820965305, 3.495525571479053, 3.6868203219928013, 3.8781150725065494, 4.0694098230202975, 4.260704573534046, 4.451999324047794, 4.708601104239214, 4.965202884430635, 5.221804664622056, 5.478406444813476, 5.735008225004897, 5.991610005196318, 6.280883997991049, 6.5701579907857806, 6.859431983580512, 7.148705976375243, 7.437979969169975, 7.727253961964706, 8.198580287896167, 8.669906613827628, 9.141232939759089, 9.61255926569055, 10.0]</t>
         </is>
       </c>
       <c r="C41" t="n">
-        <v>0.2746776601614159</v>
+        <v>0.3649151029617267</v>
       </c>
       <c r="D41" t="n">
         <v>9.81</v>
@@ -3180,13 +3180,13 @@
         <v>2</v>
       </c>
       <c r="L41" t="n">
-        <v>2.746776601614159</v>
+        <v>3.649151029617267</v>
       </c>
       <c r="M41" t="n">
-        <v>0.02650838791291584</v>
+        <v>0.01501918336050952</v>
       </c>
       <c r="N41" t="n">
-        <v>0.1325419395645792</v>
+        <v>0.0750959168025476</v>
       </c>
       <c r="O41" t="n">
         <v>18.66590452365001</v>
@@ -3216,11 +3216,11 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>[0.0, 6.133888591916098e-07, 1.2267777183832196e-06, 7.360666310299317e-06, 1.3494554902215414e-05, 3.185693873441922e-05, 5.0219322566623024e-05, 6.858170639882683e-05, 0.0001140202061919182, 0.00015945870598500956, 0.00020489720577810094, 0.0004647825944696703, 0.0007246679831612396, 0.000984553371852809, 0.0015360336295066374, 0.002087513887160466, 0.002638994144814294, 0.0031904744024681226, 0.004284860390088742, 0.005379246377709362, 0.0064736323653299815, 0.007568018352950601, 0.00866240434057122, 0.011681489854121, 0.014700575367670778, 0.017719660881220557, 0.020738746394770337, 0.023757831908320117, 0.029889499595269778, 0.036021167282219435, 0.04215283496916909, 0.04828450265611875, 0.05441617034306841, 0.060547838030018064, 0.06731238645574841, 0.07407693488147876, 0.08084148330720911, 0.08760603173293946, 0.09437058015866981, 0.10113512858440016, 0.10802694985692485, 0.11491877112944954, 0.12181059240197423, 0.12870241367449892, 0.1355942349470236, 0.1424860562195483, 0.14812663242560925, 0.1537672086316702, 0.15940778483773116, 0.1650483610437921, 0.17068893724985307, 0.17632951345591402, 0.182981403082782, 0.18963329270964996, 0.19403651656317314, 0.19843974041669632, 0.2028429642702195, 0.20724618812374268, 0.21164941197726586, 0.21700467376772647, 0.2223599355581871, 0.2277151973486477, 0.23307045913910832, 0.23842572092956893, 0.24378098272002954, 0.25160705126268285, 0.2594331198053361, 0.2672591883479894, 0.27508525689064267, 0.28291132543329595, 0.29442481031247847, 0.305938295191661, 0.3174517800708435, 0.32896526495002604, 0.34047874982920856, 0.3519922347083911, 0.36220995520979204, 0.372427675711193, 0.38264539621259397, 0.39286311671399493, 0.4030808372153959, 0.41329855771679685, 0.43039250198789486, 0.44748644625899286, 0.46458039053009087, 0.4816743348011889, 0.4987682790722869, 0.5184484567562546, 0.5381286344402223, 0.55780881212419, 0.5774889898081577, 0.5971691674921253, 0.6270802528629107, 0.656991338233696, 0.6869024236044814, 0.7168135089752667, 0.7467245943460521, 0.7777841083633339, 0.8088436223806157, 0.8399031363978975, 0.8709626504151793, 0.9020221644324611, 0.9479466781876947, 0.9938711919429284, 1.039795705698162, 1.0857202194533955, 1.131644733208629, 1.1775692469638626, 1.2311277350644145, 1.2846862231649665, 1.3382447112655185, 1.3918031993660704, 1.4453616874666224, 1.4989201755671744, 1.5720737800207893, 1.6452273844744043, 1.7183809889280193, 1.7915345933816342, 1.8646881978352492, 1.9378418022888642, 2.0407671348008125, 2.1436924673127606, 2.2466177998247088, 2.349543132336657, 2.452468464848605, 2.555393797360553, 2.678071607420319, 2.800749417480085, 2.9234272275398507, 3.0461050375996166, 3.1687828476593825, 3.2914606577191483, 3.439676455493201, 3.5878922532672535, 3.736108051041306, 3.8843238488153586, 4.032539646589411, 4.180755444363464, 4.4090494038200445, 4.637343363276625, 4.865637322733206, 5.093931282189787, 5.322225241646367, 5.550519201102948, 5.854771767023404, 6.1590243329438605, 6.463276898864317, 6.767529464784773, 7.071782030705229, 7.3760345966256855, 7.753476402836901, 8.130918209048115, 8.50836001525933, 8.885801821470544, 9.263243627681758, 9.640685433892973, 10.0]</t>
+          <t>[0.0, 6.133888591916098e-07, 1.2267777183832196e-06, 7.360666310299317e-06, 1.3494554902215414e-05, 3.185693873736091e-05, 5.021932257250641e-05, 6.85817064076519e-05, 0.00011402020583290585, 0.0001594587052581598, 0.00020489720468341377, 0.0004647807511795227, 0.0007246642976756316, 0.0009845478441717404, 0.001536102554446801, 0.0020876572647218618, 0.0026392119749969224, 0.003190766685271983, 0.004285223022126313, 0.005379679358980644, 0.0064741356958349745, 0.007568592032689305, 0.008663048369543635, 0.01168379051119849, 0.014704532652853344, 0.017725274794508198, 0.020746016936163052, 0.023766759077817907, 0.02986999734815197, 0.03597323561848603, 0.04207647388882009, 0.04817971215915415, 0.054282950429488205, 0.06038618869982226, 0.06715774033012636, 0.07392929196043047, 0.08070084359073457, 0.08747239522103867, 0.09424394685134277, 0.10101549848164687, 0.1079397016036003, 0.11486390472555372, 0.12178810784750714, 0.12871231096946056, 0.13563651409141397, 0.14256071721336738, 0.1482031474335196, 0.1538455776536718, 0.159488007873824, 0.1651304380939762, 0.1707728683141284, 0.17641529853428062, 0.18312984105180902, 0.18984438356933742, 0.19427864317061946, 0.1987129027719015, 0.20314716237318356, 0.2075814219744656, 0.21201568157574766, 0.2174214911264904, 0.22282730067723314, 0.22823311022797588, 0.23363891977871862, 0.2393008255372873, 0.24496273129585597, 0.2506246370544246, 0.25628654281299323, 0.26194844857156185, 0.27165621435473325, 0.28136398013790465, 0.29107174592107604, 0.30077951170424744, 0.31048727748741883, 0.32019504327059023, 0.33000004381532905, 0.33980504436006786, 0.3496100449048067, 0.3594150454495455, 0.3692200459942843, 0.37902504653902314, 0.39272643074352614, 0.40642781494802915, 0.42012919915253216, 0.43383058335703517, 0.4475319675615382, 0.4664080590069837, 0.4852841504524292, 0.5041602418978747, 0.5230363333433201, 0.5419124247887656, 0.5691073938768312, 0.5963023629648968, 0.6234973320529624, 0.650692301141028, 0.6778872702290937, 0.7093388659611396, 0.7407904616931855, 0.7722420574252314, 0.8036936531572774, 0.8351452488893233, 0.8851666571744209, 0.9351880654595185, 0.9852094737446161, 1.0352308820297136, 1.085252290314811, 1.1352736985999083, 1.193388956974304, 1.2515042153486995, 1.309619473723095, 1.3677347320974906, 1.4258499904718862, 1.5004825558142665, 1.5751151211566468, 1.649747686499027, 1.7243802518414073, 1.7990128171837876, 1.8736453825261679, 1.9759133607112749, 2.078181338896382, 2.180449317081489, 2.282717295266596, 2.384985273451703, 2.48725325163681, 2.6034989237357755, 2.719744595834741, 2.8359902679337066, 2.952235940032672, 3.0684816121316376, 3.184727284230603, 3.368686279587995, 3.5526452749453865, 3.736604270302778, 3.92056326566017, 4.104522261017562, 4.288481256374953, 4.540915618941829, 4.7933499815087055, 5.045784344075582, 5.298218706642458, 5.550653069209334, 5.80308743177621, 6.1481040852858175, 6.493120738795425, 6.838137392305033, 7.18315404581464, 7.528170699324248, 7.873187352833855, 8.265014049578367, 8.656840746322878, 9.048667443067389, 9.4404941398119, 9.832320836556411, 10.0]</t>
         </is>
       </c>
       <c r="C42" t="n">
-        <v>0.2679407953170916</v>
+        <v>0.3413620667859624</v>
       </c>
       <c r="D42" t="n">
         <v>9.81</v>
@@ -3247,13 +3247,13 @@
         <v>2</v>
       </c>
       <c r="L42" t="n">
-        <v>2.679407953170916</v>
+        <v>3.413620667859623</v>
       </c>
       <c r="M42" t="n">
-        <v>0.02785815249617525</v>
+        <v>0.01716324796799101</v>
       </c>
       <c r="N42" t="n">
-        <v>0.1392907624808762</v>
+        <v>0.08581623983995502</v>
       </c>
       <c r="O42" t="n">
         <v>18.41320735936067</v>
@@ -3283,11 +3283,11 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>[0.0, 6.187756156509127e-07, 1.2375512313018254e-06, 7.425307387810952e-06, 1.361306354432008e-05, 3.213706667400045e-05, 5.0661069803680815e-05, 6.918507293336118e-05, 0.00011503660684440212, 0.00016088814075544306, 0.000206739674666484, 0.00048521478876809964, 0.0007636899028697153, 0.0010421650169713309, 0.0015694507971583862, 0.0020967365773454415, 0.002624022357532497, 0.003151308137719552, 0.004155970626062783, 0.005160633114406015, 0.006165295602749246, 0.007169958091092477, 0.008174620579435708, 0.011100625713733681, 0.014026630848031654, 0.016952635982329628, 0.019878641116627602, 0.022804646250925577, 0.02849071701693782, 0.034176787782950066, 0.03986285854896231, 0.04554892931497455, 0.05123500008098679, 0.05692107084699903, 0.06379453291343662, 0.07066799497987421, 0.0775414570463118, 0.08441491911274938, 0.09128838117918697, 0.09816184324562456, 0.10485924514230832, 0.11155664703899208, 0.11825404893567584, 0.1249514508323596, 0.13164885272904336, 0.13834625462572714, 0.1443889230422433, 0.15043159145875945, 0.1564742598752756, 0.16251692829179176, 0.16855959670830792, 0.17460226512482407, 0.1804579926416643, 0.1863137201585045, 0.19216944767534472, 0.19802517519218493, 0.20388090270902515, 0.2095134611122431, 0.21514601951546103, 0.22077857791867897, 0.2264111363218969, 0.23204369472511485, 0.2376762531283328, 0.24489772908262794, 0.2521192050369231, 0.2593406809912182, 0.26656215694551333, 0.27378363289980845, 0.28100510885410357, 0.2925554035479303, 0.30410569824175704, 0.3156559929355838, 0.3272062876294105, 0.33875658232323724, 0.350306877017064, 0.3620427086466613, 0.3737785402762587, 0.385514371905856, 0.3972502035354534, 0.4089860351650507, 0.42072186679464807, 0.4386770834985456, 0.45663230020244316, 0.4745875169063407, 0.49254273361023826, 0.5104979503141358, 0.5284531670180334, 0.5502333599758858, 0.5720135529337383, 0.5937937458915908, 0.6155739388494433, 0.6373541318072958, 0.6697685207011856, 0.7021829095950755, 0.7345972984889653, 0.7670116873828551, 0.7994260762767449, 0.8331292528039304, 0.8668324293311158, 0.9005356058583013, 0.9342387823854867, 0.9679419589126722, 1.0161434754615422, 1.0643449920104122, 1.1125465085592823, 1.1607480251081523, 1.2089495416570224, 1.2571510582058925, 1.3211281539923516, 1.3851052497788108, 1.44908234556527, 1.513059441351729, 1.5770365371381883, 1.6410136329246474, 1.7131088057301536, 1.7852039785356597, 1.8572991513411659, 1.929394324146672, 2.0014894969521784, 2.0735846697576847, 2.1870547932605233, 2.300524916763362, 2.4139950402662005, 2.527465163769039, 2.6409352872718777, 2.7544054107747162, 2.8885720258215017, 3.0227386408682873, 3.1569052559150728, 3.2910718709618583, 3.425238486008644, 3.5594051010554293, 3.722834463636385, 3.886263826217341, 4.0496931887982965, 4.213122551379252, 4.376551913960207, 4.5399812765411625, 4.792643108626237, 5.045304940711311, 5.297966772796386, 5.55062860488146, 5.803290436966535, 6.055952269051609, 6.363414048295393, 6.670875827539177, 6.9783376067829614, 7.285799386026746, 7.59326116527053, 7.900722944514314, 8.315787011505808, 8.730851078497302, 9.145915145488797, 9.56097921248029, 9.976043279471785, 10.0]</t>
+          <t>[0.0, 6.187756156509127e-07, 1.2375512313018254e-06, 7.425307387810952e-06, 1.361306354432008e-05, 3.2137066678644804e-05, 5.066106981296953e-05, 6.918507294729425e-05, 0.00011503660653841532, 0.00016088814012953637, 0.00020673967372065744, 0.00048521249666001097, 0.0007636853195993645, 0.001042158142538718, 0.001569500355395304, 0.00209684256825189, 0.0026241847811084755, 0.0031515269939650613, 0.004156273802520952, 0.0051610206110768424, 0.006165767419632733, 0.007170514228188624, 0.008175261036744513, 0.011102433328981767, 0.014029605621219021, 0.016956777913456275, 0.01988395020569353, 0.022811122497930783, 0.028480582272981298, 0.03415004204803181, 0.03981950182308233, 0.04548896159813285, 0.05115842137318337, 0.05682788114823389, 0.06370866162045352, 0.07058944209267315, 0.07747022256489278, 0.0843510030371124, 0.09123178350933203, 0.09811256398155166, 0.10483486059721357, 0.11155715721287549, 0.1182794538285374, 0.1250017504441993, 0.13172404705986124, 0.13844634367552316, 0.14449054133403613, 0.1505347389925491, 0.15657893665106207, 0.16262313430957503, 0.168667331968088, 0.17471152962660097, 0.1805989724144871, 0.18648641520237325, 0.19237385799025938, 0.19826130077814552, 0.20414874356603166, 0.20980830288487123, 0.2154678622037108, 0.22112742152255038, 0.22678698084138996, 0.23244654016022953, 0.2381060994790691, 0.2453927462636744, 0.2526793930482797, 0.25996603983288497, 0.26725268661749024, 0.2745393334020955, 0.2818259801867008, 0.29325562203632655, 0.3046852638859523, 0.31611490573557804, 0.3275445475852038, 0.33897418943482954, 0.3504038312844553, 0.36238021152097855, 0.3743565917575018, 0.38633297199402505, 0.3983093522305483, 0.41028573246707156, 0.4222621127035948, 0.4405683283070926, 0.45887454391059035, 0.4771807595140881, 0.4954869751175859, 0.5137931907210836, 0.5320994063245814, 0.5528317742271148, 0.5735641421296482, 0.5942965100321816, 0.6150288779347151, 0.6357612458372485, 0.6693461676259279, 0.7029310894146074, 0.7365160112032868, 0.7701009329919662, 0.8036858547806457, 0.8384094776253112, 0.8731331004699766, 0.9078567233146421, 0.9425803461593075, 0.977303969003973, 1.037607535982368, 1.0979111029607629, 1.1582146699391578, 1.2185182369175527, 1.2788218038959476, 1.3391253708743425, 1.4092726612892985, 1.4794199517042546, 1.5495672421192106, 1.6197145325341666, 1.6898618229491227, 1.7600091133640787, 1.8493359638936873, 1.9386628144232958, 2.027989664952904, 2.1173165154825124, 2.2066433660121207, 2.295970216541729, 2.4272687230105787, 2.5585672294794284, 2.689865735948278, 2.8211642424171277, 2.9524627488859774, 3.083761255354827, 3.2604349960389674, 3.4371087367231077, 3.613782477407248, 3.7904562180913883, 3.9671299587755287, 4.143803699459669, 4.383621951030065, 4.623440202600461, 4.8632584541708574, 5.103076705741254, 5.34289495731165, 5.582713208882046, 5.881909389407717, 6.181105569933388, 6.480301750459059, 6.77949793098473, 7.078694111510401, 7.3778902920360725, 7.82478895810839, 8.271687624180707, 8.718586290253025, 9.165484956325344, 9.612383622397662, 10.0]</t>
         </is>
       </c>
       <c r="C43" t="n">
-        <v>0.2595512482514927</v>
+        <v>0.3175069626377336</v>
       </c>
       <c r="D43" t="n">
         <v>9.81</v>
@@ -3314,13 +3314,13 @@
         <v>2</v>
       </c>
       <c r="L43" t="n">
-        <v>2.595512482514926</v>
+        <v>3.175069626377336</v>
       </c>
       <c r="M43" t="n">
-        <v>0.02968819213127778</v>
+        <v>0.01983916954171683</v>
       </c>
       <c r="N43" t="n">
-        <v>0.1484409606563889</v>
+        <v>0.09919584770858413</v>
       </c>
       <c r="O43" t="n">
         <v>18.09358203282477</v>
@@ -3350,11 +3350,11 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>[0.0, 6.257949578546094e-07, 1.2515899157092187e-06, 7.509539494255313e-06, 1.3767489072801408e-05, 3.25021000309464e-05, 5.123671098909139e-05, 6.997132194723638e-05, 0.00011636129909049325, 0.0001627512762337501, 0.00020914125337700697, 0.0005199632952951397, 0.0008307853372132724, 0.001141607379131405, 0.0016542567477732175, 0.00216690611641503, 0.002679555485056843, 0.0031922048536986557, 0.004145275495075569, 0.005098346136452483, 0.006051416777829397, 0.0070044874192063105, 0.00953374340668788, 0.01206299939416945, 0.01459225538165102, 0.01712151136913259, 0.01965076735661416, 0.02390387511009799, 0.02815698286358182, 0.03241009061706565, 0.03666319837054948, 0.04091630612403331, 0.04516941387751714, 0.052171193468342515, 0.05917297305916789, 0.06617475264999326, 0.07317653224081863, 0.080178311831644, 0.08718009142246938, 0.0940865778874153, 0.10099306435236122, 0.10789955081730714, 0.11480603728225305, 0.12171252374719897, 0.1286190102121449, 0.1343873126366375, 0.1401556150611301, 0.14592391748562272, 0.15169221991011533, 0.15746052233460794, 0.16322882475910055, 0.17041938124583483, 0.1776099377325691, 0.18219731919277982, 0.18678470065299052, 0.19137208211320123, 0.19595946357341193, 0.20054684503362263, 0.20596832097868134, 0.21138979692374005, 0.21681127286879875, 0.22223274881385746, 0.22765422475891617, 0.23307570070397488, 0.2411166272993523, 0.2491575538947297, 0.25719848049010713, 0.26523940708548455, 0.27328033368086196, 0.2813212602762394, 0.2913817846772333, 0.3014423090782272, 0.31150283347922114, 0.32156335788021506, 0.331623882281209, 0.3416844066822029, 0.3540552850456676, 0.36642616340913226, 0.37879704177259693, 0.3911679201360616, 0.4035387984995263, 0.41590967686299096, 0.43426559872789927, 0.4526215205928076, 0.4709774424577159, 0.4893333643226242, 0.5076892861875325, 0.5260452080524408, 0.5480292387612815, 0.5700132694701222, 0.5919973001789629, 0.6139813308878036, 0.6359653615966443, 0.668911584209746, 0.7018578068228476, 0.7348040294359492, 0.7677502520490509, 0.8006964746621525, 0.8377468961278814, 0.8747973175936103, 0.9118477390593392, 0.9488981605250681, 0.985948581990797, 1.0449636943449159, 1.1039788066990348, 1.1629939190531537, 1.2220090314072727, 1.2810241437613916, 1.3400392561155106, 1.4018443117407622, 1.4636493673660138, 1.5254544229912654, 1.587259478616517, 1.6490645342417687, 1.7108695898670203, 1.7884997082502365, 1.8661298266334527, 1.943759945016669, 2.021390063399885, 2.0990201817831013, 2.1766503001663176, 2.2952476109322006, 2.4138449216980837, 2.532442232463967, 2.65103954322985, 2.769636853995733, 2.888234164761616, 3.0310176121386885, 3.173801059515761, 3.3165845068928332, 3.4593679542699056, 3.602151401646978, 3.7449348490240504, 3.953785138153749, 4.162635427283448, 4.3714857164131455, 4.5803360055428435, 4.789186294672541, 4.998036583802239, 5.250883699200894, 5.503730814599548, 5.756577929998202, 6.009425045396856, 6.2622721607955105, 6.515119276194165, 6.854895795282145, 7.194672314370125, 7.5344488334581055, 7.874225352546086, 8.214001871634066, 8.553778390722046, 9.006110955644651, 9.458443520567256, 9.91077608548986, 10.0]</t>
+          <t>[0.0, 6.257949578546094e-07, 1.2515899157092187e-06, 7.509539494255313e-06, 1.3767489072801408e-05, 3.250210003783187e-05, 5.123671100286233e-05, 6.997132196789279e-05, 0.00011636129885445542, 0.00016275127574101806, 0.0002091412526275807, 0.0005199600679686504, 0.0008307788833097202, 0.0011415976986507898, 0.0016542921424863616, 0.0021669865863219334, 0.002679681030157505, 0.003192375473993077, 0.0041450200656975855, 0.005097664657402095, 0.006050309249106604, 0.007002953840811113, 0.009532745608971886, 0.012062537377132658, 0.014592329145293431, 0.017122120913454206, 0.01965191268161498, 0.02390188763241495, 0.02815186258321492, 0.03240183753401489, 0.03665181248481486, 0.04090178743561483, 0.0451517623864148, 0.052164806061107065, 0.05917784973579933, 0.06619089341049159, 0.07320393708518384, 0.0802169807598761, 0.08723002443456836, 0.09415361499644877, 0.10107720555832918, 0.10800079612020959, 0.11492438668209, 0.12184797724397041, 0.1287715678058508, 0.13455174095382977, 0.14033191410180873, 0.1461120872497877, 0.15189226039776665, 0.15767243354574562, 0.16345260669372458, 0.17064028979163362, 0.17782797288954266, 0.18243420611060396, 0.18704043933166525, 0.19164667255272655, 0.19625290577378784, 0.20085913899484914, 0.20633811520764947, 0.2118170914204498, 0.21729606763325013, 0.22277504384605046, 0.22863136203988968, 0.2344876802337289, 0.24034399842756812, 0.24620031662140734, 0.25205663481524654, 0.2637054815484045, 0.2753543282815625, 0.28700317501472045, 0.2986520217478784, 0.3103008684810364, 0.32194971521419435, 0.33136823286785244, 0.34078675052151053, 0.3502052681751686, 0.3596237858288267, 0.3690423034824848, 0.3784608211361429, 0.3955248938569741, 0.4125889665778053, 0.4296530392986365, 0.44671711201946773, 0.46378118474029895, 0.48279333658333173, 0.5018054884263645, 0.5208176402693974, 0.5398297921124302, 0.558841943955463, 0.5875903583003624, 0.6163387726452618, 0.6450871869901612, 0.6738356013350606, 0.70258401567996, 0.7326578060712834, 0.7627315964626068, 0.7928053868539302, 0.8228791772452536, 0.852952967636577, 0.9077328797006511, 0.9625127917647252, 1.017292703828799, 1.072072615892873, 1.126852527956947, 1.181632440021021, 1.232659072878516, 1.2836857057360112, 1.3347123385935062, 1.3857389714510013, 1.4367656043084964, 1.4877922371659915, 1.563598238406292, 1.6394042396465927, 1.7152102408868932, 1.7910162421271938, 1.8668222433674944, 1.942628244607795, 2.0429764965273773, 2.1433247484469597, 2.243673000366542, 2.3440212522861246, 2.444369504205707, 2.5447177561252894, 2.689331903317589, 2.8339460505098883, 2.978560197702188, 3.1231743448944873, 3.267788492086787, 3.4124026392790863, 3.590443894533535, 3.7684851497879834, 3.946526405042432, 4.124567660296881, 4.30260891555133, 4.480650170805779, 4.744804985084039, 5.008959799362298, 5.273114613640558, 5.537269427918817, 5.8014242421970765, 6.065579056475336, 6.365204981636936, 6.664830906798535, 6.964456831960135, 7.264082757121734, 7.563708682283334, 7.8633346074449335, 8.346004893388011, 8.82867517933109, 9.311345465274167, 9.794015751217245, 10.0]</t>
         </is>
       </c>
       <c r="C44" t="n">
-        <v>0.2492827936872632</v>
+        <v>0.2934259498071939</v>
       </c>
       <c r="D44" t="n">
         <v>9.81</v>
@@ -3381,13 +3381,13 @@
         <v>2</v>
       </c>
       <c r="L44" t="n">
-        <v>2.492827936872632</v>
+        <v>2.934259498071939</v>
       </c>
       <c r="M44" t="n">
-        <v>0.0321843979443279</v>
+        <v>0.02322913069960428</v>
       </c>
       <c r="N44" t="n">
-        <v>0.1609219897216395</v>
+        <v>0.1161456534980214</v>
       </c>
       <c r="O44" t="n">
         <v>17.68930227111675</v>
@@ -3417,11 +3417,11 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>[0.0, 6.350224816450632e-07, 1.2700449632901264e-06, 7.620269779740759e-06, 1.3970494596191392e-05, 3.29819775092253e-05, 5.1993460422259206e-05, 7.100494333529311e-05, 0.00011810314176575695, 0.00016520134019622077, 0.0002122995386266846, 0.0005965341634571191, 0.000878367259858237, 0.001160200356259355, 0.001442033452660473, 0.002175372402176562, 0.002908711351692651, 0.00364205030120874, 0.004375389250724829, 0.005835184672282372, 0.007294980093839915, 0.008754775515397458, 0.010214570936955002, 0.011674366358512546, 0.014578642155142494, 0.01748291795177244, 0.020387193748402387, 0.023291469545032334, 0.02619574534166228, 0.03124386318940093, 0.03629198103713958, 0.041340098884878225, 0.04638821673261687, 0.05143633458035552, 0.05648445242809417, 0.0637726502438613, 0.07106084805962845, 0.0783490458753956, 0.08563724369116274, 0.09292544150692988, 0.10021363932269703, 0.10630925462553728, 0.11240486992837753, 0.11850048523121778, 0.12459610053405804, 0.1306917158368983, 0.13770500523539547, 0.14471829463389266, 0.14937124949578776, 0.15402420435768285, 0.15867715921957795, 0.16333011408147305, 0.16798306894336815, 0.17263602380526324, 0.17866338759885314, 0.18469075139244304, 0.19071811518603293, 0.19674547897962283, 0.20277284277321272, 0.20880020656680262, 0.21491156749186735, 0.22102292841693208, 0.2271342893419968, 0.23324565026706154, 0.23935701119212627, 0.245468372117191, 0.25438998780292393, 0.2633116034886569, 0.27223321917438986, 0.2811548348601228, 0.2900764505458558, 0.3003436223507655, 0.3106107941556752, 0.32087796596058493, 0.33114513776549465, 0.34141230957040436, 0.3516794813753141, 0.3653354516808356, 0.3789914219863571, 0.3926473922918786, 0.40630336259740013, 0.41995933290292164, 0.43361530320844316, 0.4503864722189663, 0.4671576412294895, 0.48392881024001266, 0.5006999792505358, 0.5174711482610589, 0.534242317271582, 0.5583583025443668, 0.5824742878171516, 0.6065902730899364, 0.6307062583627212, 0.654822243635506, 0.6886274141093606, 0.7224325845832151, 0.7562377550570697, 0.7900429255309243, 0.8238480960047788, 0.8592068634759651, 0.8945656309471514, 0.9299243984183376, 0.9652831658895239, 1.0006419333607102, 1.0360007008318965, 1.080247410470636, 1.1244941201093757, 1.1687408297481152, 1.2129875393868548, 1.2572342490255943, 1.326329245433183, 1.3954242418407716, 1.4645192382483603, 1.533614234655949, 1.6027092310635376, 1.6718042274711262, 1.7461208105755117, 1.8204373936798972, 1.8947539767842827, 1.9690705598886682, 2.043387142993054, 2.1177037260974396, 2.216000531517543, 2.3142973369376465, 2.41259414235775, 2.5108909477778534, 2.609187753197957, 2.7074845586180603, 2.857551395100276, 3.0076182315824918, 3.1576850680647075, 3.3077519045469232, 3.457818741029139, 3.6078855775113547, 3.789624385445645, 3.9713631933799354, 4.153102001314226, 4.334840809248516, 4.516579617182806, 4.698318425117097, 4.921891152102837, 5.1454638790885765, 5.369036606074316, 5.592609333060056, 5.816182060045796, 6.039754787031536, 6.391236822306708, 6.74271885758188, 7.094200892857052, 7.445682928132224, 7.797164963407396, 8.148646998682569, 8.626897662604307, 9.105148326526045, 9.583398990447783, 10.0]</t>
+          <t>[0.0, 6.350224816450632e-07, 1.2700449632901264e-06, 7.620269779740759e-06, 1.3970494596191392e-05, 3.298197751909547e-05, 5.1993460441999546e-05, 7.100494336490362e-05, 0.00011810314162311481, 0.000165201339881326, 0.0002122995381395372, 0.000596528302389899, 0.0008783681967832332, 0.0011602080911765674, 0.0014420479855699016, 0.0021751878282804653, 0.002908327670991029, 0.0036414675137015923, 0.004374607356412156, 0.005833807216843195, 0.0072930070772742345, 0.008752206937705273, 0.010211406798136312, 0.01167060665856735, 0.014575086966340934, 0.017479567274114517, 0.020384047581888103, 0.023288527889661688, 0.026193008197435273, 0.031237635296345875, 0.036282262395256476, 0.041326889494167074, 0.04637151659307767, 0.05141614369198827, 0.05646077079089887, 0.06376438122915006, 0.07106799166740124, 0.07837160210565243, 0.08567521254390362, 0.0929788229821548, 0.10028243342040599, 0.10639536053812451, 0.11250828765584303, 0.11862121477356155, 0.12473414189128007, 0.1308470690089986, 0.13787143059020296, 0.14489579217140733, 0.14955927224883914, 0.15422275232627095, 0.15888623240370275, 0.16354971248113456, 0.16821319255856637, 0.17287667263599818, 0.17892788319268096, 0.18497909374936375, 0.19103030430604653, 0.19708151486272932, 0.2031327254194121, 0.2091839359760949, 0.21529769482819525, 0.2214114536802956, 0.22752521253239597, 0.23363897138449632, 0.23975273023659668, 0.24586648908869704, 0.25474750225157283, 0.26362851541444865, 0.27250952857732447, 0.2813905417402003, 0.2902715549030761, 0.300557172824728, 0.3108427907463799, 0.3211284086680318, 0.33141402658968366, 0.34169964451133555, 0.35198526243298744, 0.3657727313475908, 0.37956020026219417, 0.39334766917679753, 0.4071351380914009, 0.42092260700600426, 0.4347100759206076, 0.45173100601629695, 0.4687519361119863, 0.4857728662076756, 0.502793796303365, 0.5198147263990542, 0.5415754664421139, 0.5633362064851735, 0.5850969465282331, 0.6068576865712927, 0.6286184266143523, 0.6615504041855049, 0.6944823817566576, 0.7274143593278102, 0.7603463368989628, 0.7932783144701154, 0.8276540226115657, 0.862029730753016, 0.8964054388944663, 0.9307811470359166, 0.9651568551773669, 1.0239595118813785, 1.0827621685853899, 1.1415648252894013, 1.2003674819934127, 1.2591701386974241, 1.3179727954014355, 1.3870417519023166, 1.4561107084031977, 1.5251796649040787, 1.5942486214049598, 1.663317577905841, 1.732386534406722, 1.820846269024376, 1.9093060036420302, 1.9977657382596843, 2.0862254728773384, 2.1746852074949925, 2.2631449421126466, 2.3919450244344898, 2.520745106756333, 2.649545189078176, 2.778345271400019, 2.9071453537218623, 3.0359454360437055, 3.177363109697594, 3.318780783351482, 3.4601984570053705, 3.601616130659259, 3.7430338043131473, 3.8844514779670356, 4.111984660464474, 4.339517842961913, 4.567051025459351, 4.79458420795679, 5.022117390454229, 5.249650572951667, 5.501387944042798, 5.7531253151339286, 6.004862686225059, 6.25660005731619, 6.50833742840732, 6.760074799498451, 7.169328040930774, 7.578581282363096, 7.987834523795419, 8.397087765227742, 8.806341006660064, 9.215594248092387, 9.72916193224914, 10.0]</t>
         </is>
       </c>
       <c r="C45" t="n">
-        <v>0.2370205012290184</v>
+        <v>0.2692237827503345</v>
       </c>
       <c r="D45" t="n">
         <v>9.81</v>
@@ -3448,13 +3448,13 @@
         <v>2</v>
       </c>
       <c r="L45" t="n">
-        <v>2.370205012290184</v>
+        <v>2.692237827503345</v>
       </c>
       <c r="M45" t="n">
-        <v>0.03560066998855967</v>
+        <v>0.027593268794869</v>
       </c>
       <c r="N45" t="n">
-        <v>0.1780033499427983</v>
+        <v>0.137966343974345</v>
       </c>
       <c r="O45" t="n">
         <v>17.17794690545135</v>
@@ -3484,11 +3484,11 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>[0.0, 6.47296241088557e-07, 1.294592482177114e-06, 7.767554893062685e-06, 1.4240517303948256e-05, 3.3620291720375226e-05, 5.30000661368022e-05, 7.237984055322917e-05, 0.00012042074549797093, 0.0001684616504427127, 0.00021650255538745446, 0.00054726126776506, 0.0008073521078863862, 0.0010674429480077125, 0.0013275337881290387, 0.002155081620025385, 0.002982629451921731, 0.003810177283818077, 0.004637725115714423, 0.006240429028256203, 0.007843132940797984, 0.009445836853339764, 0.011048540765881545, 0.012651244678423325, 0.015536275474000206, 0.018421306269577088, 0.02130633706515397, 0.024191367860730853, 0.027076398656307735, 0.031833573822780556, 0.03659074898925338, 0.041347924155726204, 0.04610509932219903, 0.05086227448867185, 0.055619449655144676, 0.06238488776355783, 0.06915032587197098, 0.07591576398038413, 0.08268120208879728, 0.08944664019721044, 0.09621207830562359, 0.10192347021794072, 0.10763486213025786, 0.11334625404257499, 0.11905764595489213, 0.12476903786720926, 0.13131460876125364, 0.137860179655298, 0.14440575054934238, 0.15095132144338674, 0.1574968923374311, 0.16404246323147548, 0.17040237810800546, 0.17676229298453544, 0.18312220786106542, 0.1894821227375954, 0.19584203761412539, 0.20220195249065537, 0.20863835621466595, 0.21507475993867653, 0.2215111636626871, 0.2279475673866977, 0.23438397111070827, 0.24082037483471885, 0.2505740521493876, 0.26032772946405636, 0.2700814067787251, 0.27983508409339386, 0.2895887614080626, 0.3002270113460732, 0.3108652612840838, 0.3215035112220944, 0.332141761160105, 0.3427800110981156, 0.3534182610361262, 0.36802075091816466, 0.3826232408002031, 0.39722573068224154, 0.41182822056428, 0.4264307104463184, 0.44103320032835686, 0.45868479614882857, 0.4763363919693003, 0.493987987789772, 0.5116395836102436, 0.5292911794307154, 0.5469427752511871, 0.5722018119758273, 0.5974608487004676, 0.6227198854251078, 0.6479789221497481, 0.6732379588743883, 0.7083479572682395, 0.7434579556620907, 0.7785679540559419, 0.8136779524497931, 0.8487879508436443, 0.8860396989912017, 0.9232914471387591, 0.9605431952863165, 0.9977949434338739, 1.0350466915814311, 1.0722984397289883, 1.1186716460812391, 1.16504485243349, 1.2114180587857408, 1.2577912651379917, 1.3041644714902425, 1.3771516660173697, 1.450138860544497, 1.5231260550716241, 1.5961132495987513, 1.6691004441258785, 1.7420876386530058, 1.8199141388867266, 1.8977406391204474, 1.9755671393541683, 2.053393639587889, 2.13122013982161, 2.2090466400553312, 2.312047129393151, 2.415047618730971, 2.5180481080687906, 2.6210485974066104, 2.7240490867444302, 2.82704957608225, 2.985216348333031, 3.1433831205838123, 3.3015498928345934, 3.4597166650853746, 3.6178834373361557, 3.776050209586937, 3.9682693367421407, 4.1604884638973445, 4.352707591052548, 4.544926718207751, 4.737145845362955, 4.929364972518158, 5.188589168008564, 5.44781336349897, 5.707037558989375, 5.966261754479781, 6.225485949970187, 6.484710145460593, 6.866502851187313, 7.248295556914034, 7.630088262640754, 8.011880968367475, 8.393673674094195, 8.775466379820916, 9.305938554528094, 9.836410729235272, 10.0]</t>
+          <t>[0.0, 6.47296241088557e-07, 1.294592482177114e-06, 7.767554893062685e-06, 1.4240517303948256e-05, 3.362029173428261e-05, 5.300006616461697e-05, 7.237984059495133e-05, 0.00012042074548206309, 0.00016846165036917484, 0.0002165025552562866, 0.0005472666132808359, 0.0008073626719090571, 0.0010674587305372783, 0.0013275547891654995, 0.002154650399529113, 0.002981746009892727, 0.0038088416202563405, 0.004635937230619954, 0.006237397967581177, 0.0078388587045424, 0.009440319441503624, 0.011041780178464848, 0.012643240915426072, 0.01552785769054447, 0.018412474465662867, 0.021297091240781267, 0.024181708015899667, 0.027066324791018066, 0.03182138797763251, 0.03657645116424695, 0.041331514350861395, 0.04608657753747584, 0.05084164072409028, 0.055596703910704724, 0.06237190802693023, 0.06914711214315575, 0.07592231625938126, 0.08269752037560676, 0.08947272449183227, 0.09624792860805778, 0.10197365536781493, 0.10769938212757207, 0.11342510888732922, 0.11915083564708637, 0.12487656240684351, 0.13143231930155652, 0.13798807619626952, 0.1445438330909825, 0.1510995899856955, 0.1576553468804085, 0.1642111037751215, 0.1705933128206984, 0.1769755218662753, 0.1833577309118522, 0.1897399399574291, 0.196122149003006, 0.2025043580485829, 0.20896133267005643, 0.21541830729152994, 0.22187528191300346, 0.22833225653447697, 0.2347892311559505, 0.241246205777424, 0.25094884170268406, 0.2606514776279441, 0.27035411355320416, 0.2800567494784642, 0.28975938540372426, 0.30041276475333567, 0.3110661441029471, 0.3217195234525585, 0.3323729028021699, 0.3430262821517813, 0.35367966150139274, 0.3683968907434556, 0.3831141199855185, 0.39783134922758134, 0.4125485784696442, 0.4272658077117071, 0.44198303695376995, 0.45982265552624085, 0.47766227409871176, 0.49550189267118266, 0.5133415112436536, 0.5311811298161244, 0.5490207483885953, 0.5724676220617502, 0.5959144957349051, 0.61936136940806, 0.6428082430812149, 0.6662551167543698, 0.7016781281865887, 0.7371011396188076, 0.7725241510510266, 0.8079471624832455, 0.8433701739154644, 0.8801737115560395, 0.9169772491966146, 0.9537807868371897, 0.9905843244777648, 1.0273878621183399, 1.064191399758915, 1.1108124351995616, 1.1574334706402083, 1.204054506080855, 1.2506755415215016, 1.2972965769621483, 1.370829669401746, 1.444362761841344, 1.5178958542809418, 1.5914289467205396, 1.6649620391601374, 1.7384951315997352, 1.817220105027365, 1.895945078454995, 1.9746700518826248, 2.0533950253102544, 2.132119998737884, 2.2108449721655132, 2.336858551723055, 2.462872131280597, 2.588885710838139, 2.714899290395681, 2.8409128699532227, 2.9669264495107646, 3.1065496241426294, 3.246172798774494, 3.385795973406359, 3.5254191480382238, 3.6650423226700886, 3.8046654973019534, 4.027097955597434, 4.2495304138929155, 4.471962872188397, 4.694395330483878, 4.916827788779359, 5.13926024707484, 5.384909522518305, 5.630558797961769, 5.876208073405234, 6.121857348848699, 6.367506624292163, 6.613155899735628, 7.013667283844944, 7.41417866795426, 7.814690052063575, 8.21520143617289, 8.615712820282205, 9.01622420439152, 9.516023880605117, 10.0]</t>
         </is>
       </c>
       <c r="C46" t="n">
-        <v>0.222818994218676</v>
+        <v>0.2450823727545197</v>
       </c>
       <c r="D46" t="n">
         <v>9.81</v>
@@ -3515,13 +3515,13 @@
         <v>2</v>
       </c>
       <c r="L46" t="n">
-        <v>2.22818994218676</v>
+        <v>2.450823727545197</v>
       </c>
       <c r="M46" t="n">
-        <v>0.04028334971045119</v>
+        <v>0.03329705650382783</v>
       </c>
       <c r="N46" t="n">
-        <v>0.2014167485522559</v>
+        <v>0.1664852825191391</v>
       </c>
       <c r="O46" t="n">
         <v>16.53115640352251</v>
@@ -3551,11 +3551,11 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>[0.0, 6.638846307198666e-07, 1.3277692614397331e-06, 7.966615568638398e-06, 1.4605461875837063e-05, 3.448302476097977e-05, 5.436058764612247e-05, 7.423815053126518e-05, 0.0001235543827048418, 0.00017287061487841843, 0.00022218684705199506, 0.0005764312660070328, 0.0008226329239967989, 0.0010688345819865651, 0.0013150362399763312, 0.0019237689302548766, 0.002532501620533422, 0.003141234310811967, 0.003749967001090512, 0.004928501615532361, 0.00610703622997421, 0.0072855708444160595, 0.00846410545885791, 0.00964264007329976, 0.012205810844554254, 0.014768981615808748, 0.017332152387063243, 0.019895323158317737, 0.02245849392957223, 0.026583506408449687, 0.030708518887327143, 0.034833531366204595, 0.038958543845082044, 0.04308355632395949, 0.04720856880283694, 0.0533972911390126, 0.05958601347518826, 0.06577473581136392, 0.07196345814753959, 0.07815218048371525, 0.08434090281989091, 0.09087320945614219, 0.09740551609239347, 0.10393782272864474, 0.11047012936489602, 0.11700243600114729, 0.12354981661097408, 0.13009719722080088, 0.13664457783062767, 0.14319195844045446, 0.14973933905028125, 0.15628671966010804, 0.16297714753454395, 0.16966757540897986, 0.17635800328341578, 0.1830484311578517, 0.1897388590322876, 0.1964292869067235, 0.20308109364904423, 0.20973290039136494, 0.21638470713368566, 0.22303651387600637, 0.22968832061832709, 0.2363401273606478, 0.2468847929779396, 0.2574294585952314, 0.2679741242125232, 0.278518789829815, 0.28906345544710677, 0.30026506023373417, 0.3114666650203616, 0.322668269806989, 0.3338698745936164, 0.3450714793802438, 0.3562730841668712, 0.3718630888137089, 0.38745309346054657, 0.40304309810738426, 0.41863310275422194, 0.4342231074010596, 0.4498131120478973, 0.4684004354771938, 0.48698775890649026, 0.5055750823357867, 0.5241624057650832, 0.5427497291943797, 0.566045935119044, 0.5893421410437083, 0.6126383469683726, 0.6359345528930369, 0.6592307588177012, 0.6940282958853078, 0.7288258329529144, 0.7636233700205209, 0.7984209070881275, 0.8332184441557341, 0.8692616528784737, 0.9053048616012133, 0.9413480703239528, 0.9773912790466924, 1.0134344877694321, 1.0646372957548573, 1.1158401037402825, 1.1670429117257077, 1.218245719711133, 1.2694485276965581, 1.3206513356819833, 1.3900648437267669, 1.4594783517715504, 1.528891859816334, 1.5983053678611174, 1.667718875905901, 1.7371323839506845, 1.8139232340570821, 1.8907140841634797, 1.9675049342698774, 2.044295784376275, 2.1210866344826727, 2.1978774845890703, 2.2992175435648874, 2.4005576025407045, 2.5018976615165216, 2.6032377204923387, 2.704577779468156, 2.805917838443973, 2.963583008208278, 3.121248177972583, 3.278913347736888, 3.436578517501193, 3.594243687265498, 3.751908857029803, 3.9436625610306666, 4.13541626503153, 4.3271699690323935, 4.518923673033257, 4.71067737703412, 4.902431081034983, 5.156806185757565, 5.4111812904801475, 5.66555639520273, 5.919931499925312, 6.174306604647894, 6.428681709370476, 6.81080150115723, 7.192921292943984, 7.575041084730738, 7.9571608765174915, 8.339280668304244, 8.721400460090997, 9.255581837232857, 9.789763214374716, 10.0]</t>
+          <t>[0.0, 6.638846307198666e-07, 1.3277692614397331e-06, 7.966615568638398e-06, 1.4605461875837063e-05, 3.448302478046304e-05, 5.436058768508902e-05, 7.4238150589715e-05, 0.00012355438286464285, 0.0001728706151395707, 0.00022218684741449855, 0.0005764378267353429, 0.0008226437200346997, 0.0010688496133340565, 0.0013150555066334133, 0.0019236946868263602, 0.0025323338670193074, 0.0031409730472122545, 0.0037496122274052017, 0.004927896858840906, 0.00610618149027661, 0.007284466121712314, 0.008462750753148018, 0.009641035384583722, 0.012203992696861616, 0.01476695000913951, 0.017329907321417405, 0.0198928646336953, 0.022455821945973196, 0.02657974934153395, 0.030703676737094704, 0.034827604132655454, 0.038951531528216204, 0.043075458923776955, 0.047199386319337705, 0.05339249867400457, 0.05958561102867144, 0.0657787233833383, 0.07197183573800517, 0.07816494809267203, 0.0843580604473389, 0.09090476950150897, 0.09745147855567904, 0.10399818760984911, 0.11054489666401918, 0.11709160571818925, 0.12365080318240325, 0.13021000064661725, 0.13676919811083127, 0.1433283955750453, 0.1498875930392593, 0.15644679050347332, 0.1631574729540375, 0.1698681554046017, 0.1765788378551659, 0.1832895203057301, 0.19000020275629428, 0.19671088520685848, 0.20338047200256007, 0.21005005879826166, 0.21671964559396326, 0.22338923238966485, 0.23005881918536644, 0.23672840598106804, 0.24720916487650854, 0.25768992377194905, 0.2681706826673895, 0.27865144156283, 0.2891322004582705, 0.3003472885310183, 0.31156237660376607, 0.32277746467651386, 0.33399255274926165, 0.34520764082200944, 0.35642272889475723, 0.37209940924945883, 0.38777608960416043, 0.40345276995886203, 0.41912945031356363, 0.43480613066826523, 0.45048281102296683, 0.4692510692621241, 0.4880193275012814, 0.5067875857404387, 0.525555843979596, 0.5443241022187533, 0.5679164502867704, 0.5915087983547875, 0.6151011464228047, 0.6386934944908218, 0.6622858425588389, 0.6975876471705952, 0.7328894517823514, 0.7681912563941077, 0.8034930610058639, 0.8387948656176202, 0.8754787101340727, 0.9121625546505253, 0.9488463991669779, 0.9855302436834305, 1.022214088199883, 1.086734166472915, 1.1512542447459473, 1.2157743230189795, 1.2802944012920117, 1.3448144795650439, 1.409334557838076, 1.4711879879057699, 1.5330414179734637, 1.5948948480411576, 1.6567482781088514, 1.7186017081765452, 1.780455138244239, 1.8654759577684212, 1.9504967772926034, 2.035517596816786, 2.120538416340968, 2.2055592358651506, 2.290580055389333, 2.4203936822080956, 2.550207309026858, 2.680020935845621, 2.8098345626643835, 2.939648189483146, 3.0694618163019087, 3.211935927554185, 3.3544100388064613, 3.4968841500587375, 3.639358261311014, 3.78183237256329, 3.9243064838155663, 4.154137658219967, 4.383968832624367, 4.613800007028767, 4.843631181433167, 5.0734623558375676, 5.303293530241968, 5.585323942431992, 5.867354354622016, 6.14938476681204, 6.431415179002064, 6.713445591192088, 6.995476003382112, 7.386079873371949, 7.776683743361785, 8.167287613351622, 8.557891483341459, 8.948495353331296, 9.339099223321133, 9.924198751892302, 10.0]</t>
         </is>
       </c>
       <c r="C47" t="n">
-        <v>0.2069477336771379</v>
+        <v>0.221321738653843</v>
       </c>
       <c r="D47" t="n">
         <v>9.81</v>
@@ -3582,13 +3582,13 @@
         <v>2</v>
       </c>
       <c r="L47" t="n">
-        <v>2.069477336771378</v>
+        <v>2.213217386538429</v>
       </c>
       <c r="M47" t="n">
-        <v>0.04669911456282443</v>
+        <v>0.04083023214046797</v>
       </c>
       <c r="N47" t="n">
-        <v>0.2334955728141221</v>
+        <v>0.2041511607023399</v>
       </c>
       <c r="O47" t="n">
         <v>15.71306006294538</v>
@@ -3618,11 +3618,11 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>[0.0, 6.868075072921821e-07, 1.3736150145843641e-06, 8.241690087506185e-06, 1.5109765160428006e-05, 3.5675259067240384e-05, 5.624075297405276e-05, 7.680624688086514e-05, 0.00012788710524286293, 0.0001789679636048607, 0.00023004882196685849, 0.0005080409099551213, 0.0007860329979433842, 0.0010076179411405933, 0.0012292028843378026, 0.001450787827535012, 0.0019693692014954678, 0.0024879505754559234, 0.003006531949416379, 0.0035251133233768347, 0.004507694686202662, 0.005490276049028489, 0.0064728574118543165, 0.007455438774680144, 0.008438020137505971, 0.010845422427218046, 0.013252824716930121, 0.015660227006642196, 0.01806762929635427, 0.020475031586066342, 0.024248788795925857, 0.02802254600578537, 0.03179630321564489, 0.03557006042550441, 0.03934381763536393, 0.04311757484522345, 0.04879836220177871, 0.05447914955833397, 0.060159936914889224, 0.06584072427144448, 0.07152151162799975, 0.07720229898455501, 0.08359835644773297, 0.08999441391091094, 0.0963904713740889, 0.10278652883726687, 0.10918258630044483, 0.11554475620529857, 0.1219069261101523, 0.12826909601500602, 0.13463126591985974, 0.14099343582471346, 0.14735560572956719, 0.15428111856457327, 0.16120663139957936, 0.16813214423458545, 0.17505765706959153, 0.18198316990459762, 0.1889086827396037, 0.19579589861033583, 0.20268311448106796, 0.2095703303518001, 0.21645754622253222, 0.22334476209326434, 0.23023197796399647, 0.24293406605294424, 0.255636154141892, 0.2683382422308398, 0.2810403303197876, 0.2937424184087354, 0.30472358134566624, 0.3157047442825971, 0.32668590721952795, 0.3376670701564588, 0.34864823309338966, 0.3596293960303205, 0.3818393826129454, 0.3967341332248542, 0.41162888383676294, 0.4265236344486717, 0.44141838506058045, 0.4563131356724892, 0.47120788628439797, 0.5072383499447706, 0.5307790704845731, 0.5543197910243756, 0.5778605115641781, 0.6014012321039806, 0.624941952643783, 0.6506516868381524, 0.6763614210325218, 0.7020711552268912, 0.7277808894212606, 0.75349062361563, 0.7792003578099994, 0.8245853798677312, 0.8699704019254629, 0.9153554239831947, 0.9607404460409265, 1.0061254680986582, 1.0538798040248865, 1.1016341399511147, 1.149388475877343, 1.1971428118035712, 1.2448971477297994, 1.2926514836560277, 1.3545373970286068, 1.4164233104011859, 1.478309223773765, 1.540195137146344, 1.6020810505189231, 1.691876813199838, 1.781672575880753, 1.871468338561668, 1.9612641012425829, 2.0510598639234976, 2.140855626604412, 2.2467121341289054, 2.3525686416533986, 2.458425149177892, 2.564281656702385, 2.6701381642268784, 2.7759946717513717, 2.9034687972987614, 3.030942922846151, 3.1584170483935408, 3.2858911739409304, 3.41336529948832, 3.54083942503571, 3.7423054337286112, 3.9437714424215127, 4.145237451114414, 4.3467034598073155, 4.548169468500217, 4.749635477193118, 5.024768009280059, 5.299900541367, 5.575033073453941, 5.850165605540882, 6.125298137627823, 6.400430669714764, 6.74833267344933, 7.096234677183896, 7.4441366809184615, 7.792038684653027, 8.139940688387593, 8.48784269212216, 8.965339812254534, 9.442836932386909, 9.920334052519284, 10.0]</t>
+          <t>[0.0, 6.868075072921821e-07, 1.3736150145843641e-06, 8.241690087506185e-06, 1.5109765160428006e-05, 3.567525909465372e-05, 5.624075302887943e-05, 7.680624696310514e-05, 0.00012788710565362222, 0.0001789679643441393, 0.00023004882303465638, 0.0005080428904928885, 0.0007860369579511207, 0.00100762544891199, 0.0012292139398728595, 0.0014508024308337289, 0.00196935364922555, 0.002487904867617371, 0.003006456086009192, 0.003525007304401013, 0.004507519974115566, 0.005490032643830118, 0.006472545313544671, 0.007455057983259223, 0.008437570652973776, 0.010844636028540224, 0.013251701404106671, 0.01565876677967312, 0.018065832155239568, 0.020472897530806018, 0.02424583820074315, 0.028018778870680282, 0.031791719540617415, 0.035564660210554544, 0.03933760088049167, 0.0431105415504288, 0.04879341010451457, 0.054476278658600344, 0.060159147212686115, 0.06584201576677189, 0.07152488432085766, 0.07720775287494343, 0.08361600340854786, 0.09002425394215229, 0.09643250447575671, 0.10284075500936114, 0.10924900554296557, 0.11562133878160982, 0.12199367202025407, 0.12836600525889832, 0.13473833849754258, 0.14111067173618683, 0.14748300497483108, 0.15442812570441164, 0.1613732464339922, 0.16831836716357276, 0.17526348789315332, 0.1822086086227339, 0.18915372935231445, 0.19605858648015628, 0.20296344360799812, 0.20986830073583995, 0.2167731578636818, 0.22367801499152362, 0.23058287211936546, 0.2431295203559469, 0.25567616859252834, 0.26822281682910976, 0.28076946506569117, 0.2933161133022726, 0.30430591381484534, 0.3152957143274181, 0.32628551483999085, 0.3372753153525636, 0.34826511586513637, 0.3592549163777091, 0.3802569119240299, 0.40125890747035065, 0.4222609030166714, 0.44326289856299217, 0.46426489410931293, 0.4852668896556337, 0.5055580064084639, 0.5258491231612942, 0.5461402399141244, 0.5664313566669547, 0.5867224734197849, 0.6070135901726151, 0.6372850626389209, 0.6675565351052267, 0.6978280075715325, 0.7280994800378383, 0.7583709525041441, 0.7969827938682711, 0.8355946352323981, 0.8742064765965251, 0.912818317960652, 0.951430159324779, 0.990042000688906, 1.037619850630241, 1.0851977005715758, 1.1327755505129107, 1.1803534004542455, 1.2279312503955804, 1.2755091003369152, 1.335688959017265, 1.3958688176976146, 1.4560486763779643, 1.516228535058314, 1.5764083937386637, 1.6365882524190134, 1.7265849722975122, 1.816581692176011, 1.9065784120545097, 1.9965751319330085, 2.0865718518115073, 2.176568571690006, 2.275139600795321, 2.3737106299006356, 2.4722816590059504, 2.570852688111265, 2.66942371721658, 2.767994746321895, 2.8988765017814795, 3.029758257241064, 3.160640012700649, 3.2915217681602336, 3.4224035236198183, 3.553285279079403, 3.75969317710971, 3.966101075140017, 4.1725089731703235, 4.37891687120063, 4.585324769230937, 4.791732667261243, 5.0456178454672695, 5.299503023673296, 5.553388201879322, 5.807273380085348, 6.061158558291375, 6.315043736497401, 6.657760476144355, 7.000477215791308, 7.343193955438262, 7.685910695085216, 8.028627434732169, 8.371344174379121, 8.90022928998354, 9.42911440558796, 9.957999521192379, 10.0]</t>
         </is>
       </c>
       <c r="C48" t="n">
-        <v>0.1899162435070918</v>
+        <v>0.1984354002627979</v>
       </c>
       <c r="D48" t="n">
         <v>9.81</v>
@@ -3649,13 +3649,13 @@
         <v>2</v>
       </c>
       <c r="L48" t="n">
-        <v>1.899162435070918</v>
+        <v>1.984354002627979</v>
       </c>
       <c r="M48" t="n">
-        <v>0.05545053909213717</v>
+        <v>0.05079157646249891</v>
       </c>
       <c r="N48" t="n">
-        <v>0.2772526954606858</v>
+        <v>0.2539578823124946</v>
       </c>
       <c r="O48" t="n">
         <v>14.67828663867616</v>
@@ -3685,11 +3685,11 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>[0.0, 7.195087894027813e-07, 1.4390175788055626e-06, 8.634105472833376e-06, 1.582919336686119e-05, 3.7376182997027324e-05, 5.8923172627193456e-05, 8.047016225735959e-05, 0.00013407296636508306, 0.00018767577047280653, 0.00024127857458053, 0.00048177613729495454, 0.0007222737000093791, 0.0009627712627238036, 0.0013399909456695805, 0.0017172106286153575, 0.0020944303115611345, 0.0024716499945069115, 0.0032285030269324343, 0.003985356059357957, 0.004742209091783479, 0.0054990621242090015, 0.0071818228858191455, 0.00886458364742929, 0.010547344409039434, 0.01223010517064958, 0.013912865932259724, 0.016769537556191684, 0.019626209180123644, 0.022482880804055604, 0.025339552427987563, 0.028196224051919523, 0.031052895675851483, 0.035811171778238685, 0.040569447880625886, 0.04532772398301309, 0.05008600008540029, 0.05484427618778749, 0.05960255229017469, 0.0672923308378127, 0.07498210938545072, 0.08057901310689214, 0.08617591682833356, 0.09177282054977498, 0.0973697242712164, 0.10296662799265782, 0.11227211263100015, 0.11807824130453443, 0.1238843699780687, 0.12969049865160298, 0.13549662732513726, 0.14130275599867154, 0.14710888467220581, 0.15450395027560246, 0.1618990158789991, 0.16929408148239575, 0.1766891470857924, 0.18408421268918904, 0.19147927829258568, 0.19874765526626803, 0.20601603223995038, 0.21328440921363273, 0.22055278618731508, 0.22782116316099743, 0.23508954013467978, 0.24623449963831545, 0.25737945914195115, 0.26852441864558685, 0.27966937814922255, 0.29081433765285825, 0.3036038566610569, 0.3163933756692555, 0.32918289467745415, 0.3419724136856528, 0.3547619326938514, 0.36755145170205006, 0.3858038311276191, 0.4040562105531882, 0.42230858997875725, 0.4405609694043263, 0.4588133488298954, 0.47706572825546445, 0.4983269213697169, 0.5195881144839694, 0.5408493075982218, 0.5621105007124743, 0.5833716938267267, 0.6046328869409792, 0.6336780926340038, 0.6627232983270284, 0.691768504020053, 0.7208137097130776, 0.7498589154061022, 0.7901284813338654, 0.8303980472616286, 0.8706676131893918, 0.910937179117155, 0.9512067450449182, 0.9984653963671847, 1.0457240476894512, 1.0929826990117175, 1.1402413503339839, 1.1875000016562502, 1.2347586529785166, 1.2888062621309602, 1.3428538712834037, 1.3969014804358473, 1.4509490895882908, 1.5049966987407344, 1.5920543361058757, 1.679111973471017, 1.7661696108361582, 1.8532272482012995, 1.9402848855664407, 2.027342522931582, 2.1274936036697794, 2.2276446844079767, 2.327795765146174, 2.4279468458843714, 2.5280979266225687, 2.628249007360766, 2.7604578154415877, 2.8926666235224094, 3.024875431603231, 3.157084239684053, 3.2892930477648745, 3.421501855845696, 3.6177820753415566, 3.814062294837417, 4.010342514333278, 4.206622733829139, 4.402902953325, 4.599183172820862, 4.876542078603521, 5.15390098438618, 5.431259890168839, 5.708618795951498, 5.985977701734157, 6.263336607516816, 6.607977880199727, 6.952619152882638, 7.2972604255655495, 7.641901698248461, 7.986542970931372, 8.331184243614283, 8.845319422570888, 9.359454601527494, 9.8735897804841, 10.0]</t>
+          <t>[0.0, 7.195087894027813e-07, 1.4390175788055626e-06, 8.634105472833376e-06, 1.582919336686119e-05, 3.737618303619494e-05, 5.892317270552869e-05, 8.047016237486244e-05, 0.00013407296714960433, 0.00018767577192434622, 0.0002412785766990881, 0.0004817770496744477, 0.0007222755226498072, 0.0009627739956251667, 0.0013400026022211927, 0.0017172312088172188, 0.0020944598154132446, 0.0024716884220092705, 0.0032283820796659983, 0.0039850757373227266, 0.004741769394979455, 0.005498463052636184, 0.007181097021466018, 0.008863730990295852, 0.010546364959125688, 0.012228998927955523, 0.013911632896785358, 0.01676762187027691, 0.01962361084376846, 0.022479599817260013, 0.025335588790751564, 0.028191577764243116, 0.031047566737734667, 0.03580583975454306, 0.040564112771351454, 0.04532238578815985, 0.050080658804968245, 0.05483893182177664, 0.059597204838585036, 0.0673070652753267, 0.07501692571206837, 0.08062338178932042, 0.08622983786657247, 0.09183629394382452, 0.09744275002107657, 0.10304920609832861, 0.11235601551423484, 0.11816825463118563, 0.12398049374813642, 0.12979273286508722, 0.13560497198203803, 0.14141721109898883, 0.14722945021593964, 0.15464043307861663, 0.16205141594129363, 0.16946239880397063, 0.17687338166664762, 0.18428436452932462, 0.1916953473920016, 0.19898064383287375, 0.2062659402737459, 0.21355123671461804, 0.22083653315549018, 0.22812182959636232, 0.23540712603723446, 0.24655259446381161, 0.25769806289038877, 0.2688435313169659, 0.2799889997435431, 0.29113446817012023, 0.30395127601179417, 0.3167680838534681, 0.32958489169514205, 0.342401699536816, 0.3552185073784899, 0.36803531522016386, 0.3863901521642261, 0.4047449891082884, 0.42309982605235064, 0.4414546629964129, 0.45980949994047515, 0.4781643368845374, 0.499669679816573, 0.5211750227486086, 0.5426803656806443, 0.5641857086126799, 0.5856910515447156, 0.6071963944767512, 0.6366689386471107, 0.6661414828174702, 0.6956140269878297, 0.7250865711581892, 0.7545591153285487, 0.795300895184519, 0.8360426750404892, 0.8767844548964595, 0.9175262347524298, 0.9582680146084, 1.0019600561275144, 1.0456520976466286, 1.0893441391657428, 1.133036180684857, 1.1767282222039712, 1.2204202637230854, 1.2748218974766816, 1.3292235312302778, 1.383625164983874, 1.4380267987374702, 1.4924284324910664, 1.5784985474557705, 1.6645686624204745, 1.7506387773851786, 1.8367088923498827, 1.9227790073145867, 2.008849122279291, 2.109096965042299, 2.2093448078053073, 2.3095926505683155, 2.4098404933313238, 2.510088336094332, 2.6103361788573403, 2.7337800912986916, 2.857224003740043, 2.9806679161813943, 3.1041118286227456, 3.227555741064097, 3.3509996535054483, 3.5451378192030405, 3.7392759849006327, 3.933414150598225, 4.127552316295818, 4.321690481993411, 4.515828647691004, 4.755868405378014, 4.995908163065025, 5.235947920752035, 5.475987678439045, 5.716027436126056, 5.956067193813066, 6.28539531690239, 6.614723439991714, 6.944051563081038, 7.273379686170362, 7.602707809259686, 7.9320359323490095, 8.385022532220734, 8.83800913209246, 9.290995731964184, 9.743982331835909, 10.0]</t>
         </is>
       </c>
       <c r="C49" t="n">
-        <v>0.1724404715714122</v>
+        <v>0.1770146826388335</v>
       </c>
       <c r="D49" t="n">
         <v>9.81</v>
@@ -3716,13 +3716,13 @@
         <v>2</v>
       </c>
       <c r="L49" t="n">
-        <v>1.724404715714122</v>
+        <v>1.770146826388335</v>
       </c>
       <c r="M49" t="n">
-        <v>0.06725918367468382</v>
+        <v>0.06382802611750495</v>
       </c>
       <c r="N49" t="n">
-        <v>0.3362959183734191</v>
+        <v>0.3191401305875247</v>
       </c>
       <c r="O49" t="n">
         <v>13.36944807472602</v>
@@ -3752,11 +3752,11 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>[0.0, 7.684472056127673e-07, 1.5368944112255346e-06, 9.221366467353208e-06, 1.6905838523480884e-05, 3.9921894470631866e-05, 6.293795041778286e-05, 8.595400636493385e-05, 0.0001433409171356781, 0.00020072782790642236, 0.0002581147386771666, 0.00047666469048696894, 0.0006952146422967713, 0.0009137645941065737, 0.0012754308456223917, 0.0016370970971382097, 0.0019987633486540277, 0.002360429600169846, 0.0030826872099223063, 0.0038049448196747666, 0.004527202429427227, 0.005249460039179688, 0.006852509297313179, 0.00845555855544667, 0.01005860781358016, 0.011661657071713651, 0.013264706329847142, 0.0159209285323185, 0.018577150734789855, 0.02123337293726121, 0.023889595139732565, 0.02654581734220392, 0.029202039544675276, 0.03364776252032537, 0.038093485495975465, 0.04253920847162556, 0.046984931447275655, 0.05143065442292575, 0.055876377398575844, 0.06680776195442271, 0.07330150516275431, 0.07979524837108591, 0.08628899157941751, 0.09278273478774911, 0.0992764779960807, 0.10707099316783839, 0.11486550833959606, 0.12266002351135374, 0.1304545386831114, 0.13824905385486908, 0.14604356902662674, 0.15539445611091307, 0.1647453431951994, 0.17409623027948573, 0.18344711736377206, 0.1927980044480584, 0.20214889153234472, 0.2099665531767124, 0.21778421482108007, 0.22560187646544774, 0.23341953810981542, 0.2412371997541831, 0.25524390970199606, 0.269250619649809, 0.28325732959762195, 0.2972640395454349, 0.31127074949324784, 0.32602990706347673, 0.3407890646337056, 0.3555482222039345, 0.3703073797741634, 0.3850665373443923, 0.4032274779915137, 0.42138841863863513, 0.43954935928575656, 0.457710299932878, 0.4758712405799994, 0.49937968230824614, 0.5228881240364929, 0.5463965657647396, 0.5699050074929863, 0.5934134492212331, 0.6204077975237503, 0.6474021458262675, 0.6743964941287848, 0.701390842431302, 0.7283851907338192, 0.7701351403320553, 0.8118850899302914, 0.8536350395285275, 0.8953849891267636, 0.9371349387249996, 0.9788848883232357, 1.027712829817864, 1.0765407713124922, 1.1253687128071204, 1.1741966543017486, 1.2230245957963768, 1.271852537291005, 1.3365780988856, 1.401303660480195, 1.46602922207479, 1.5307547836693849, 1.5954803452639799, 1.6602059068585748, 1.7519461306324444, 1.843686354406314, 1.9354265781801836, 2.027166801954053, 2.118907025727923, 2.210647249501793, 2.3222778442389433, 2.433908438976094, 2.5455390337132444, 2.657169628450395, 2.7688002231875455, 2.880430817924696, 3.029631692134185, 3.1788325663436736, 3.3280334405531624, 3.477234314762651, 3.62643518897214, 3.775636063181629, 3.9760402220197446, 4.176444380857861, 4.3768485396959775, 4.577252698534094, 4.777656857372211, 4.978061016210328, 5.243935428618302, 5.509809841026277, 5.775684253434251, 6.041558665842226, 6.307433078250201, 6.573307490658175, 6.982815817072664, 7.392324143487153, 7.801832469901642, 8.211340796316131, 8.62084912273062, 9.030357449145109, 9.61590341845548, 10.0]</t>
+          <t>[0.0, 7.684472056127673e-07, 1.5368944112255346e-06, 9.221366467353208e-06, 1.6905838523480884e-05, 3.992189452834577e-05, 6.293795053321065e-05, 8.595400653807554e-05, 0.0001433409185124701, 0.00020072783048686465, 0.0002581147424612592, 0.0004766651885086167, 0.0006952156345559742, 0.0009137660806033316, 0.0012754388115050583, 0.001637111542406785, 0.0019987842733085117, 0.0023604570042102383, 0.0030825925336414738, 0.0038047280630727092, 0.004526863592503944, 0.00524899912193518, 0.006851894888869916, 0.008454790655804652, 0.010057686422739388, 0.011660582189674125, 0.01326347795660886, 0.015919128306646445, 0.01857477865668403, 0.021230429006721615, 0.0238860793567592, 0.026541729706796784, 0.02919738005683437, 0.033642750179895264, 0.03808812030295616, 0.04253349042601706, 0.04697886054907796, 0.05142423067213886, 0.05586960079519976, 0.06655260702127923, 0.07363939466637802, 0.08072618231147681, 0.0878129699565756, 0.09489975760167439, 0.10198654524677318, 0.1093370527563521, 0.11668756026593101, 0.12403806777550992, 0.13138857528508885, 0.1387390827946678, 0.14839063247521547, 0.15804218215576316, 0.16769373183631084, 0.17734528151685852, 0.1869968311974062, 0.1966483808779539, 0.20410989456442455, 0.2115714082508952, 0.21903292193736587, 0.22649443562383653, 0.2339559493103072, 0.24141746299677785, 0.2538103543012884, 0.26620324560579894, 0.2785961369103095, 0.29098902821482003, 0.3033819195193306, 0.3157748108238411, 0.328445574718965, 0.3411163386140889, 0.3537871025092128, 0.3664578664043367, 0.3791286302994606, 0.3917993941945845, 0.4108255725666482, 0.4298517509387119, 0.44887792931077564, 0.46790410768283935, 0.48693028605490307, 0.5135007788038283, 0.5400712715527535, 0.5666417643016787, 0.5932122570506039, 0.6197827497995291, 0.6505180667200824, 0.6812533836406357, 0.711988700561189, 0.7427240174817423, 0.7734593344022956, 0.8111896520461266, 0.8489199696899575, 0.8866502873337885, 0.9243806049776194, 0.9621109226214504, 0.9998412402652813, 1.0445527161458887, 1.089264192026496, 1.1339756679071034, 1.1786871437877107, 1.223398619668318, 1.2681100955489253, 1.3426782166710354, 1.4172463377931455, 1.4918144589152555, 1.5663825800373656, 1.6409507011594757, 1.7155188222815858, 1.801100806155716, 1.8866827900298464, 1.9722647739039767, 2.057846757778107, 2.1434287416522375, 2.229010725526368, 2.341207372636825, 2.4534040197472824, 2.5656006668577396, 2.6777973139681968, 2.789993961078654, 2.902190608189111, 3.068911623979194, 3.235632639769277, 3.40235365555936, 3.569074671349443, 3.7357956871395257, 3.9025167029296086, 4.136505744575877, 4.370494786222146, 4.604483827868415, 4.838472869514684, 5.072461911160953, 5.3064509528072215, 5.5981287837496305, 5.88980661469204, 6.181484445634449, 6.473162276576858, 6.764840107519267, 7.056517938461676, 7.492240923414765, 7.927963908367854, 8.363686893320942, 8.79940987827403, 9.235132863227118, 9.670855848180206, 10.0]</t>
         </is>
       </c>
       <c r="C50" t="n">
-        <v>0.1552956316138361</v>
+        <v>0.1575171711353884</v>
       </c>
       <c r="D50" t="n">
         <v>9.81</v>
@@ -3783,13 +3783,13 @@
         <v>2</v>
       </c>
       <c r="L50" t="n">
-        <v>1.552956316138361</v>
+        <v>1.575171711353884</v>
       </c>
       <c r="M50" t="n">
-        <v>0.08292997163221261</v>
+        <v>0.0806072654665056</v>
       </c>
       <c r="N50" t="n">
-        <v>0.414649858161063</v>
+        <v>0.4030363273325279</v>
       </c>
       <c r="O50" t="n">
         <v>11.7139567890923</v>
@@ -3819,11 +3819,11 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>[0.0, 8.475713663360658e-07, 1.6951427326721315e-06, 1.017085639603279e-05, 1.8646570059393445e-05, 4.403839350692338e-05, 6.943021695445331e-05, 9.482204040198324e-05, 0.0001583522359696596, 0.00022188243153733594, 0.0002854126271050123, 0.0004922845701542645, 0.0006991565132035166, 0.0009060284562527688, 0.001264186620519387, 0.0016223447847860052, 0.0019805029490526233, 0.0023386611133192413, 0.0030354587029694496, 0.003732256292619658, 0.004429053882269866, 0.005125851471920075, 0.006668119540338066, 0.008210387608756057, 0.009752655677174048, 0.01129492374559204, 0.01283719181401003, 0.015314552437591581, 0.017791913061173132, 0.02026927368475468, 0.02274663430833623, 0.02522399493191778, 0.027701355555499328, 0.031882758023525165, 0.036064160491551006, 0.04024556295957685, 0.04442696542760269, 0.04860836789562853, 0.05278977036365437, 0.059013261620500274, 0.06523675287734618, 0.07146024413419208, 0.07768373539103798, 0.08390722664788389, 0.09013071790472979, 0.09814236856631875, 0.10615401922790771, 0.11416566988949667, 0.12217732055108563, 0.1301889712126746, 0.13820062187426355, 0.14665421064933848, 0.1551077994244134, 0.16356138819948834, 0.17201497697456328, 0.1804685657496382, 0.18892215452471314, 0.19772745757866894, 0.20653276063262474, 0.21533806368658054, 0.22414336674053634, 0.23294866979449214, 0.24890266428375252, 0.2648566587730129, 0.2808106532622733, 0.29676464775153366, 0.31271864224079404, 0.32941886158374806, 0.34611908092670207, 0.3628193002696561, 0.3795195196126101, 0.3962197389555641, 0.41291995829851813, 0.43826711811881974, 0.46361427793912136, 0.48896143775942297, 0.5143085975797246, 0.5396557574000262, 0.5650029172203279, 0.5927421857346448, 0.6204814542489616, 0.6482207227632785, 0.6759599912775953, 0.7036992597919122, 0.731438528306229, 0.770957624528306, 0.8104767207503829, 0.8499958169724599, 0.8895149131945368, 0.9290340094166137, 0.9685531056386907, 1.0234344767497416, 1.0783158478607926, 1.1331972189718436, 1.1880785900828945, 1.2429599611939455, 1.2978413323049964, 1.362909076592247, 1.4279768208794974, 1.4930445651667479, 1.5581123094539984, 1.6231800537412489, 1.6882477980284993, 1.774379939924429, 1.8605120818203589, 1.9466442237162886, 2.0327763656122184, 2.118908507508148, 2.205040649404078, 2.3161976008029947, 2.4273545522019115, 2.5385115036008283, 2.649668454999745, 2.760825406398662, 2.8719823577975787, 3.038221242030718, 3.2044601262638577, 3.370699010496997, 3.5369378947301366, 3.703176778963276, 3.8694156631964156, 4.098840889905019, 4.328266116613623, 4.557691343322227, 4.787116570030831, 5.016541796739435, 5.2459670234480384, 5.56738958678317, 5.8888121501183015, 6.210234713453433, 6.531657276788565, 6.853079840123696, 7.174502403458828, 7.633668352657571, 8.092834301856314, 8.552000251055057, 9.0111662002538, 9.470332149452544, 9.929498098651287, 10.0]</t>
+          <t>[0.0, 8.475713663360658e-07, 1.6951427326721315e-06, 1.017085639603279e-05, 1.8646570059393445e-05, 4.403839359699854e-05, 6.943021713460364e-05, 9.482204067220873e-05, 0.00015835223838193721, 0.0002218824360916657, 0.00028541263380139415, 0.0004922848764268234, 0.0006991571190522527, 0.000906029361677682, 0.0012641926632400646, 0.0016223559648024472, 0.0019805192663648295, 0.002338682567927212, 0.003035389932622859, 0.003732097297318506, 0.004428804662014153, 0.005125512026709801, 0.006667603159510426, 0.00820969429231105, 0.009751785425111674, 0.011293876557912298, 0.012835967690712921, 0.01531283565315338, 0.01778970361559384, 0.020266571578034298, 0.022743439540474756, 0.025220307502915214, 0.02769717546535567, 0.0318779104682798, 0.03605864547120392, 0.04023938047412805, 0.04442011547705217, 0.048600850479976296, 0.05278158548290042, 0.05900285797225384, 0.06522413046160726, 0.07144540295096068, 0.0776666754403141, 0.08388794792966751, 0.09010922041902093, 0.09813478672646633, 0.10616035303391173, 0.11418591934135713, 0.12221148564880253, 0.13023705195624793, 0.13826261826369335, 0.14672278560015206, 0.15518295293661077, 0.1636431202730695, 0.1721032876095282, 0.1805634549459869, 0.18902362228244562, 0.19784831065093672, 0.20667299901942782, 0.2154976873879189, 0.22432237575641, 0.2331470641249011, 0.24911022656850193, 0.26507338901210276, 0.2810365514557036, 0.29699971389930446, 0.3129628763429053, 0.32970456682497884, 0.34644625730705236, 0.3631879477891259, 0.3799296382711994, 0.39667132875327293, 0.41341301923534646, 0.4388413148648016, 0.46426961049425675, 0.4896979061237119, 0.515126201753167, 0.5405544973826222, 0.5659827930120773, 0.5938351558514448, 0.6216875186908122, 0.6495398815301796, 0.677392244369547, 0.7052446072089145, 0.7330969700482819, 0.7729001916800771, 0.8127034133118722, 0.8525066349436674, 0.8923098565754626, 0.9321130782072578, 0.9719162998390529, 1.0270988964645344, 1.082281493090016, 1.1374640897154975, 1.192646686340979, 1.2478292829664606, 1.303011879591942, 1.3686279451317964, 1.4342440106716507, 1.499860076211505, 1.5654761417513594, 1.6310922072912137, 1.696708272831068, 1.7835656315519943, 1.8704229902729206, 1.9572803489938468, 2.044137707714773, 2.130995066435699, 2.217852425156625, 2.329588240888406, 2.4413240566201866, 2.5530598723519673, 2.664795688083748, 2.7765315038155287, 2.8882673195473094, 3.0567540273875, 3.2252407352276906, 3.393727443067881, 3.562214150908072, 3.7307008587482624, 3.899187566588453, 4.131110365484365, 4.363033164380277, 4.594955963276189, 4.826878762172101, 5.058801561068013, 5.290724359963925, 5.616016670112232, 5.941308980260538, 6.266601290408844, 6.5918936005571505, 6.917185910705457, 7.242478220853763, 7.709075973104904, 8.175673725356045, 8.642271477607187, 9.108869229858328, 9.57546698210947, 10.0]</t>
         </is>
       </c>
       <c r="C51" t="n">
-        <v>0.1390945427724638</v>
+        <v>0.1400708294490355</v>
       </c>
       <c r="D51" t="n">
         <v>9.81</v>
@@ -3850,13 +3850,13 @@
         <v>2</v>
       </c>
       <c r="L51" t="n">
-        <v>1.390945427724638</v>
+        <v>1.400708294490355</v>
       </c>
       <c r="M51" t="n">
-        <v>0.1033736410071521</v>
+        <v>0.1019376447030222</v>
       </c>
       <c r="N51" t="n">
-        <v>0.5168682050357603</v>
+        <v>0.5096882235151112</v>
       </c>
       <c r="O51" t="n">
         <v>9.620000000000001</v>

</xml_diff>